<commit_message>
Fix internal hyperlinks - wrap Hebrew sheet names in single quotes
Excel requires single quotes around sheet names with spaces/Hebrew chars.
'יולי 2025'!A1 instead of יולי 2025!A1

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roita\מעקב הוצאות כלים\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_9363EC9BE71201D4762D76C9D9D56AED991232E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_3260EC9B897A43C1FC2D768769115A3B29942CE4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1051,7 +1051,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-997A-452D-9B8A-982F13E839D3}"/>
+              <c16:uniqueId val="{00000000-8E1A-424C-A6A5-6ECF3DC33095}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1734,7 +1734,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0900-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1929,7 +1929,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2048,7 +2048,7 @@
     <mergeCell ref="A6:C6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3763,16 +3763,16 @@
     <mergeCell ref="B3:C3"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="B3" location="יולי 2025!A1" display="יולי 2025_x000a_(July 2025)" xr:uid="{00000000-0004-0000-0C00-000000000000}"/>
-    <hyperlink ref="D3" location="אוגוסט 2025!A1" display="אוגוסט 2025_x000a_(August 2025)" xr:uid="{00000000-0004-0000-0C00-000001000000}"/>
-    <hyperlink ref="F3" location="ספטמבר 2025!A1" display="ספטמבר 2025_x000a_(September 2025)" xr:uid="{00000000-0004-0000-0C00-000002000000}"/>
-    <hyperlink ref="H3" location="אוקטובר 2025!A1" display="אוקטובר 2025_x000a_(October 2025)" xr:uid="{00000000-0004-0000-0C00-000003000000}"/>
-    <hyperlink ref="J3" location="נובמבר 2025!A1" display="נובמבר 2025_x000a_(November 2025)" xr:uid="{00000000-0004-0000-0C00-000004000000}"/>
-    <hyperlink ref="L3" location="דצמבר 2025!A1" display="דצמבר 2025_x000a_(December 2025)" xr:uid="{00000000-0004-0000-0C00-000005000000}"/>
-    <hyperlink ref="N3" location="ינואר 2026!A1" display="ינואר 2026_x000a_(January 2026)" xr:uid="{00000000-0004-0000-0C00-000006000000}"/>
-    <hyperlink ref="P3" location="פברואר 2026!A1" display="פברואר 2026_x000a_(February 2026)" xr:uid="{00000000-0004-0000-0C00-000007000000}"/>
-    <hyperlink ref="R3" location="מרץ 2026!A1" display="מרץ 2026_x000a_(March 2026)" xr:uid="{00000000-0004-0000-0C00-000008000000}"/>
-    <hyperlink ref="T3" location="אפריל 2026!A1" display="אפריל 2026_x000a_(April 2026)" xr:uid="{00000000-0004-0000-0C00-000009000000}"/>
+    <hyperlink ref="B3" location="'יולי 2025'!A1" display="יולי 2025_x000a_(July 2025)" xr:uid="{00000000-0004-0000-0C00-000000000000}"/>
+    <hyperlink ref="D3" location="'אוגוסט 2025'!A1" display="אוגוסט 2025_x000a_(August 2025)" xr:uid="{00000000-0004-0000-0C00-000001000000}"/>
+    <hyperlink ref="F3" location="'ספטמבר 2025'!A1" display="ספטמבר 2025_x000a_(September 2025)" xr:uid="{00000000-0004-0000-0C00-000002000000}"/>
+    <hyperlink ref="H3" location="'אוקטובר 2025'!A1" display="אוקטובר 2025_x000a_(October 2025)" xr:uid="{00000000-0004-0000-0C00-000003000000}"/>
+    <hyperlink ref="J3" location="'נובמבר 2025'!A1" display="נובמבר 2025_x000a_(November 2025)" xr:uid="{00000000-0004-0000-0C00-000004000000}"/>
+    <hyperlink ref="L3" location="'דצמבר 2025'!A1" display="דצמבר 2025_x000a_(December 2025)" xr:uid="{00000000-0004-0000-0C00-000005000000}"/>
+    <hyperlink ref="N3" location="'ינואר 2026'!A1" display="ינואר 2026_x000a_(January 2026)" xr:uid="{00000000-0004-0000-0C00-000006000000}"/>
+    <hyperlink ref="P3" location="'פברואר 2026'!A1" display="פברואר 2026_x000a_(February 2026)" xr:uid="{00000000-0004-0000-0C00-000007000000}"/>
+    <hyperlink ref="R3" location="'מרץ 2026'!A1" display="מרץ 2026_x000a_(March 2026)" xr:uid="{00000000-0004-0000-0C00-000008000000}"/>
+    <hyperlink ref="T3" location="'אפריל 2026'!A1" display="אפריל 2026_x000a_(April 2026)" xr:uid="{00000000-0004-0000-0C00-000009000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -4093,16 +4093,16 @@
     <mergeCell ref="A15:B15"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A4" location="יולי 2025!A1" display="יולי 2025" xr:uid="{00000000-0004-0000-0D00-000000000000}"/>
-    <hyperlink ref="A5" location="אוגוסט 2025!A1" display="אוגוסט 2025" xr:uid="{00000000-0004-0000-0D00-000001000000}"/>
-    <hyperlink ref="A6" location="ספטמבר 2025!A1" display="ספטמבר 2025" xr:uid="{00000000-0004-0000-0D00-000002000000}"/>
-    <hyperlink ref="A7" location="אוקטובר 2025!A1" display="אוקטובר 2025" xr:uid="{00000000-0004-0000-0D00-000003000000}"/>
-    <hyperlink ref="A8" location="נובמבר 2025!A1" display="נובמבר 2025" xr:uid="{00000000-0004-0000-0D00-000004000000}"/>
-    <hyperlink ref="A9" location="דצמבר 2025!A1" display="דצמבר 2025" xr:uid="{00000000-0004-0000-0D00-000005000000}"/>
-    <hyperlink ref="A10" location="ינואר 2026!A1" display="ינואר 2026" xr:uid="{00000000-0004-0000-0D00-000006000000}"/>
-    <hyperlink ref="A11" location="פברואר 2026!A1" display="פברואר 2026" xr:uid="{00000000-0004-0000-0D00-000007000000}"/>
-    <hyperlink ref="A12" location="מרץ 2026!A1" display="מרץ 2026" xr:uid="{00000000-0004-0000-0D00-000008000000}"/>
-    <hyperlink ref="A13" location="אפריל 2026!A1" display="אפריל 2026" xr:uid="{00000000-0004-0000-0D00-000009000000}"/>
+    <hyperlink ref="A4" location="'יולי 2025'!A1" display="יולי 2025" xr:uid="{00000000-0004-0000-0D00-000000000000}"/>
+    <hyperlink ref="A5" location="'אוגוסט 2025'!A1" display="אוגוסט 2025" xr:uid="{00000000-0004-0000-0D00-000001000000}"/>
+    <hyperlink ref="A6" location="'ספטמבר 2025'!A1" display="ספטמבר 2025" xr:uid="{00000000-0004-0000-0D00-000002000000}"/>
+    <hyperlink ref="A7" location="'אוקטובר 2025'!A1" display="אוקטובר 2025" xr:uid="{00000000-0004-0000-0D00-000003000000}"/>
+    <hyperlink ref="A8" location="'נובמבר 2025'!A1" display="נובמבר 2025" xr:uid="{00000000-0004-0000-0D00-000004000000}"/>
+    <hyperlink ref="A9" location="'דצמבר 2025'!A1" display="דצמבר 2025" xr:uid="{00000000-0004-0000-0D00-000005000000}"/>
+    <hyperlink ref="A10" location="'ינואר 2026'!A1" display="ינואר 2026" xr:uid="{00000000-0004-0000-0D00-000006000000}"/>
+    <hyperlink ref="A11" location="'פברואר 2026'!A1" display="פברואר 2026" xr:uid="{00000000-0004-0000-0D00-000007000000}"/>
+    <hyperlink ref="A12" location="'מרץ 2026'!A1" display="מרץ 2026" xr:uid="{00000000-0004-0000-0D00-000008000000}"/>
+    <hyperlink ref="A13" location="'אפריל 2026'!A1" display="אפריל 2026" xr:uid="{00000000-0004-0000-0D00-000009000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing r:id="rId1"/>
@@ -5416,7 +5416,7 @@
     <mergeCell ref="A11:C11"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0200-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5649,7 +5649,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0300-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5806,7 +5806,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0400-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5925,7 +5925,7 @@
     <mergeCell ref="A6:C6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0500-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6120,7 +6120,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0600-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6239,7 +6239,7 @@
     <mergeCell ref="A6:C6"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0700-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6434,7 +6434,7 @@
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="A2" location="סיכום חודשי!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
+    <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0800-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add confirmed missing transactions: Lovable Lite, Meta $2.25, IONOS
- Lovable Lite $5.00 (Mar 25, 2026)
- Meta Facebook Ads $2.25 (Apr 3, 2026)
- IONOS Instant Domain $20.00 (Apr 5, 2026)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\roita\מעקב הוצאות כלים\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_3260EC9B897A43C1FC2D768769115A3B29942CE4" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_C93FFF2C68F48BE1FB05EC776C46B23A5EE984C9" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="7" activeTab="13" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="521" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="160">
   <si>
     <t>דוח שנתי – AI Tool Expenses</t>
   </si>
@@ -417,7 +417,25 @@
     <t>Creator (first month 50% off)</t>
   </si>
   <si>
+    <t>2026-03-25</t>
+  </si>
+  <si>
+    <t>Lite plan</t>
+  </si>
+  <si>
     <t>2026-04-01</t>
+  </si>
+  <si>
+    <t>2026-04-03</t>
+  </si>
+  <si>
+    <t>2026-04-05</t>
+  </si>
+  <si>
+    <t>IONOS</t>
+  </si>
+  <si>
+    <t>Instant Domain</t>
   </si>
   <si>
     <t>סה"כ"</t>
@@ -1041,17 +1059,17 @@
                   <c:v>156</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>146.61000000000001</c:v>
+                  <c:v>151.61000000000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>25</c:v>
+                  <c:v>47.25</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-8E1A-424C-A6A5-6ECF3DC33095}"/>
+              <c16:uniqueId val="{00000000-0DB0-4721-B2D9-D60992237236}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1562,7 +1580,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -1572,7 +1590,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1714,7 +1732,7 @@
     </row>
     <row r="10" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="65" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B10" s="58"/>
       <c r="C10" s="58"/>
@@ -1745,7 +1763,7 @@
   <sheetPr>
     <tabColor rgb="FF9DC3E6"/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1757,7 +1775,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -1767,7 +1785,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1907,26 +1925,45 @@
       </c>
       <c r="F9" s="24"/>
     </row>
-    <row r="10" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="65" t="s">
-        <v>127</v>
-      </c>
-      <c r="B10" s="58"/>
-      <c r="C10" s="58"/>
-      <c r="D10" s="16">
-        <f>SUM(D4:D9)</f>
-        <v>146.61000000000001</v>
-      </c>
-      <c r="E10" s="17">
-        <f>SUM(E4:E9)</f>
-        <v>535.12649999999996</v>
-      </c>
-      <c r="F10" s="26"/>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="10" t="s">
+        <v>123</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="D10" s="20">
+        <v>5</v>
+      </c>
+      <c r="E10" s="21">
+        <f>D10*הגדרות!$B$4</f>
+        <v>18.25</v>
+      </c>
+      <c r="F10" s="19"/>
+    </row>
+    <row r="11" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="65" t="s">
+        <v>133</v>
+      </c>
+      <c r="B11" s="58"/>
+      <c r="C11" s="58"/>
+      <c r="D11" s="16">
+        <f>SUM(D4:D10)</f>
+        <v>151.61000000000001</v>
+      </c>
+      <c r="E11" s="17">
+        <f>SUM(E4:E10)</f>
+        <v>553.37649999999996</v>
+      </c>
+      <c r="F11" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A11:C11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0A00-000000000000}"/>
@@ -1940,7 +1977,7 @@
   <sheetPr>
     <tabColor rgb="FF9DC3E6"/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1952,7 +1989,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -1962,7 +1999,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -1990,7 +2027,7 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B4" s="11" t="s">
         <v>52</v>
@@ -2009,7 +2046,7 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B5" s="7" t="s">
         <v>52</v>
@@ -2026,26 +2063,64 @@
       </c>
       <c r="F5" s="24"/>
     </row>
-    <row r="6" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="65" t="s">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="10" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>114</v>
+      </c>
+      <c r="D6" s="20">
+        <v>2.25</v>
+      </c>
+      <c r="E6" s="21">
+        <f>D6*הגדרות!$B$4</f>
+        <v>8.2125000000000004</v>
+      </c>
+      <c r="F6" s="19"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="B6" s="58"/>
-      <c r="C6" s="58"/>
-      <c r="D6" s="16">
-        <f>SUM(D4:D5)</f>
-        <v>25</v>
-      </c>
-      <c r="E6" s="17">
-        <f>SUM(E4:E5)</f>
-        <v>91.25</v>
-      </c>
-      <c r="F6" s="26"/>
+      <c r="B7" s="7" t="s">
+        <v>128</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" s="22">
+        <v>20</v>
+      </c>
+      <c r="E7" s="23">
+        <f>D7*הגדרות!$B$4</f>
+        <v>73</v>
+      </c>
+      <c r="F7" s="24"/>
+    </row>
+    <row r="8" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="65" t="s">
+        <v>133</v>
+      </c>
+      <c r="B8" s="58"/>
+      <c r="C8" s="58"/>
+      <c r="D8" s="16">
+        <f>SUM(D4:D7)</f>
+        <v>47.25</v>
+      </c>
+      <c r="E8" s="17">
+        <f>SUM(E4:E7)</f>
+        <v>172.46250000000001</v>
+      </c>
+      <c r="F8" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A8:C8"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A6:C6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A2" location="'סיכום חודשי'!A1" display="← חזרה לסיכום חודשי" xr:uid="{00000000-0004-0000-0B00-000000000000}"/>
@@ -2059,7 +2134,7 @@
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
   </sheetPr>
-  <dimension ref="A1:W20"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2089,7 +2164,7 @@
   <sheetData>
     <row r="1" spans="1:23" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="61" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -2115,7 +2190,7 @@
     </row>
     <row r="2" spans="1:23" ht="13.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="66" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B2" s="53"/>
       <c r="C2" s="53"/>
@@ -2144,119 +2219,119 @@
         <v>38</v>
       </c>
       <c r="B3" s="67" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="C3" s="53"/>
       <c r="D3" s="67" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="E3" s="53"/>
       <c r="F3" s="67" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="G3" s="53"/>
       <c r="H3" s="67" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="I3" s="53"/>
       <c r="J3" s="67" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="K3" s="53"/>
       <c r="L3" s="67" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="M3" s="53"/>
       <c r="N3" s="67" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="O3" s="53"/>
       <c r="P3" s="67" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="Q3" s="53"/>
       <c r="R3" s="67" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="S3" s="53"/>
       <c r="T3" s="67" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="U3" s="53"/>
       <c r="V3" s="14" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="W3" s="14" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="15"/>
       <c r="B4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="C4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="D4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="E4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="F4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="G4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="H4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="I4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="J4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="K4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="L4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="M4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="N4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="O4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="P4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="Q4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="R4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="S4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="T4" s="27" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="U4" s="27" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="V4" s="28" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="W4" s="28" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
@@ -2344,7 +2419,7 @@
         <v>91.25</v>
       </c>
       <c r="V5" s="32">
-        <f t="shared" ref="V5:V19" si="0">SUM(B5,D5,F5,H5,J5,L5,N5,P5,R5,T5)</f>
+        <f t="shared" ref="V5:V20" si="0">SUM(B5,D5,F5,H5,J5,L5,N5,P5,R5,T5)</f>
         <v>180</v>
       </c>
       <c r="W5" s="33">
@@ -2726,1025 +2801,1118 @@
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A10" s="34" t="s">
+        <v>128</v>
+      </c>
+      <c r="B10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <v>0</v>
+      </c>
+      <c r="C10" s="36" t="str">
+        <f>IF(B10&gt;0,B10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="D10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <v>0</v>
+      </c>
+      <c r="E10" s="36" t="str">
+        <f>IF(D10&gt;0,D10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="F10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <v>0</v>
+      </c>
+      <c r="G10" s="36" t="str">
+        <f>IF(F10&gt;0,F10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <v>0</v>
+      </c>
+      <c r="I10" s="36" t="str">
+        <f>IF(H10&gt;0,H10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <v>0</v>
+      </c>
+      <c r="K10" s="36" t="str">
+        <f>IF(J10&gt;0,J10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <v>0</v>
+      </c>
+      <c r="M10" s="36" t="str">
+        <f>IF(L10&gt;0,L10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <v>0</v>
+      </c>
+      <c r="O10" s="36" t="str">
+        <f>IF(N10&gt;0,N10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <v>0</v>
+      </c>
+      <c r="Q10" s="36" t="str">
+        <f>IF(P10&gt;0,P10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <v>0</v>
+      </c>
+      <c r="S10" s="36" t="str">
+        <f>IF(R10&gt;0,R10*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="T10" s="35">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <v>20</v>
+      </c>
+      <c r="U10" s="36">
+        <f>IF(T10&gt;0,T10*הגדרות!$B$4,"")</f>
+        <v>73</v>
+      </c>
+      <c r="V10" s="32">
+        <f t="shared" si="0"/>
+        <v>20</v>
+      </c>
+      <c r="W10" s="33">
+        <f>IF(V10&gt;0,V10*הגדרות!$B$4,"")</f>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="B10" s="35">
+      <c r="B11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>185.14</v>
       </c>
-      <c r="C10" s="36">
-        <f>IF(B10&gt;0,B10*הגדרות!$B$4,"")</f>
+      <c r="C11" s="31">
+        <f>IF(B11&gt;0,B11*הגדרות!$B$4,"")</f>
         <v>675.76099999999997</v>
       </c>
-      <c r="D10" s="35">
+      <c r="D11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>0</v>
       </c>
-      <c r="E10" s="36" t="str">
-        <f>IF(D10&gt;0,D10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="F10" s="35">
+      <c r="E11" s="31" t="str">
+        <f>IF(D11&gt;0,D11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="F11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="G10" s="36" t="str">
-        <f>IF(F10&gt;0,F10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="H10" s="35">
+      <c r="G11" s="31" t="str">
+        <f>IF(F11&gt;0,F11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I10" s="36" t="str">
-        <f>IF(H10&gt;0,H10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="35">
+      <c r="I11" s="31" t="str">
+        <f>IF(H11&gt;0,H11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="K10" s="36" t="str">
-        <f>IF(J10&gt;0,J10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="L10" s="35">
+      <c r="K11" s="31" t="str">
+        <f>IF(J11&gt;0,J11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M10" s="36" t="str">
-        <f>IF(L10&gt;0,L10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N10" s="35">
+      <c r="M11" s="31" t="str">
+        <f>IF(L11&gt;0,L11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="O10" s="36" t="str">
-        <f>IF(N10&gt;0,N10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="P10" s="35">
+      <c r="O11" s="31" t="str">
+        <f>IF(N11&gt;0,N11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="Q10" s="36" t="str">
-        <f>IF(P10&gt;0,P10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="R10" s="35">
+      <c r="Q11" s="31" t="str">
+        <f>IF(P11&gt;0,P11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>0</v>
       </c>
-      <c r="S10" s="36" t="str">
-        <f>IF(R10&gt;0,R10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="T10" s="35">
+      <c r="S11" s="31" t="str">
+        <f>IF(R11&gt;0,R11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="T11" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U10" s="36" t="str">
-        <f>IF(T10&gt;0,T10*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V10" s="32">
+      <c r="U11" s="31" t="str">
+        <f>IF(T11&gt;0,T11*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V11" s="32">
         <f t="shared" si="0"/>
         <v>185.14</v>
       </c>
-      <c r="W10" s="33">
-        <f>IF(V10&gt;0,V10*הגדרות!$B$4,"")</f>
+      <c r="W11" s="33">
+        <f>IF(V11&gt;0,V11*הגדרות!$B$4,"")</f>
         <v>675.76099999999997</v>
       </c>
     </row>
-    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A11" s="29" t="s">
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A12" s="34" t="s">
         <v>107</v>
       </c>
-      <c r="B11" s="30">
+      <c r="B12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>0</v>
       </c>
-      <c r="C11" s="31" t="str">
-        <f>IF(B11&gt;0,B11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="D11" s="30">
+      <c r="C12" s="36" t="str">
+        <f>IF(B12&gt;0,B12*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="D12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>0</v>
       </c>
-      <c r="E11" s="31" t="str">
-        <f>IF(D11&gt;0,D11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="F11" s="30">
+      <c r="E12" s="36" t="str">
+        <f>IF(D12&gt;0,D12*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="F12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="G11" s="31" t="str">
-        <f>IF(F11&gt;0,F11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="H11" s="30">
+      <c r="G12" s="36" t="str">
+        <f>IF(F12&gt;0,F12*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I11" s="31" t="str">
-        <f>IF(H11&gt;0,H11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="30">
+      <c r="I12" s="36" t="str">
+        <f>IF(H12&gt;0,H12*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="K11" s="31" t="str">
-        <f>IF(J11&gt;0,J11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="L11" s="30">
+      <c r="K12" s="36" t="str">
+        <f>IF(J12&gt;0,J12*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M11" s="31" t="str">
-        <f>IF(L11&gt;0,L11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N11" s="30">
+      <c r="M12" s="36" t="str">
+        <f>IF(L12&gt;0,L12*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="O11" s="31" t="str">
-        <f>IF(N11&gt;0,N11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="P11" s="30">
+      <c r="O12" s="36" t="str">
+        <f>IF(N12&gt;0,N12*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>75</v>
       </c>
-      <c r="Q11" s="31">
-        <f>IF(P11&gt;0,P11*הגדרות!$B$4,"")</f>
+      <c r="Q12" s="36">
+        <f>IF(P12&gt;0,P12*הגדרות!$B$4,"")</f>
         <v>273.75</v>
       </c>
-      <c r="R11" s="30">
+      <c r="R12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
-        <v>0</v>
-      </c>
-      <c r="S11" s="31" t="str">
-        <f>IF(R11&gt;0,R11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="T11" s="30">
+        <v>5</v>
+      </c>
+      <c r="S12" s="36">
+        <f>IF(R12&gt;0,R12*הגדרות!$B$4,"")</f>
+        <v>18.25</v>
+      </c>
+      <c r="T12" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U11" s="31" t="str">
-        <f>IF(T11&gt;0,T11*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V11" s="32">
+      <c r="U12" s="36" t="str">
+        <f>IF(T12&gt;0,T12*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V12" s="32">
         <f t="shared" si="0"/>
-        <v>75</v>
-      </c>
-      <c r="W11" s="33">
-        <f>IF(V11&gt;0,V11*הגדרות!$B$4,"")</f>
-        <v>273.75</v>
-      </c>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A12" s="34" t="s">
+        <v>80</v>
+      </c>
+      <c r="W12" s="33">
+        <f>IF(V12&gt;0,V12*הגדרות!$B$4,"")</f>
+        <v>292</v>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A13" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="35">
+      <c r="B13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>10.59</v>
       </c>
-      <c r="C12" s="36">
-        <f>IF(B12&gt;0,B12*הגדרות!$B$4,"")</f>
+      <c r="C13" s="31">
+        <f>IF(B13&gt;0,B13*הגדרות!$B$4,"")</f>
         <v>38.653500000000001</v>
       </c>
-      <c r="D12" s="35">
+      <c r="D13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>10.59</v>
       </c>
-      <c r="E12" s="36">
-        <f>IF(D12&gt;0,D12*הגדרות!$B$4,"")</f>
+      <c r="E13" s="31">
+        <f>IF(D13&gt;0,D13*הגדרות!$B$4,"")</f>
         <v>38.653500000000001</v>
       </c>
-      <c r="F12" s="35">
+      <c r="F13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>10.59</v>
       </c>
-      <c r="G12" s="36">
-        <f>IF(F12&gt;0,F12*הגדרות!$B$4,"")</f>
+      <c r="G13" s="31">
+        <f>IF(F13&gt;0,F13*הגדרות!$B$4,"")</f>
         <v>38.653500000000001</v>
       </c>
-      <c r="H12" s="35">
+      <c r="H13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I12" s="36" t="str">
-        <f>IF(H12&gt;0,H12*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="35">
+      <c r="I13" s="31" t="str">
+        <f>IF(H13&gt;0,H13*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="K12" s="36" t="str">
-        <f>IF(J12&gt;0,J12*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="L12" s="35">
+      <c r="K13" s="31" t="str">
+        <f>IF(J13&gt;0,J13*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M12" s="36" t="str">
-        <f>IF(L12&gt;0,L12*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N12" s="35">
+      <c r="M13" s="31" t="str">
+        <f>IF(L13&gt;0,L13*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="O12" s="36" t="str">
-        <f>IF(N12&gt;0,N12*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="P12" s="35">
+      <c r="O13" s="31" t="str">
+        <f>IF(N13&gt;0,N13*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="Q12" s="36" t="str">
-        <f>IF(P12&gt;0,P12*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="R12" s="35">
+      <c r="Q13" s="31" t="str">
+        <f>IF(P13&gt;0,P13*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>0</v>
       </c>
-      <c r="S12" s="36" t="str">
-        <f>IF(R12&gt;0,R12*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="T12" s="35">
+      <c r="S13" s="31" t="str">
+        <f>IF(R13&gt;0,R13*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="T13" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U12" s="36" t="str">
-        <f>IF(T12&gt;0,T12*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V12" s="32">
+      <c r="U13" s="31" t="str">
+        <f>IF(T13&gt;0,T13*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V13" s="32">
         <f t="shared" si="0"/>
         <v>31.77</v>
       </c>
-      <c r="W12" s="33">
-        <f>IF(V12&gt;0,V12*הגדרות!$B$4,"")</f>
+      <c r="W13" s="33">
+        <f>IF(V13&gt;0,V13*הגדרות!$B$4,"")</f>
         <v>115.9605</v>
       </c>
     </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A13" s="29" t="s">
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A14" s="34" t="s">
         <v>68</v>
       </c>
-      <c r="B13" s="30">
+      <c r="B14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>0</v>
       </c>
-      <c r="C13" s="31" t="str">
-        <f>IF(B13&gt;0,B13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="D13" s="30">
+      <c r="C14" s="36" t="str">
+        <f>IF(B14&gt;0,B14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="D14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>19</v>
       </c>
-      <c r="E13" s="31">
-        <f>IF(D13&gt;0,D13*הגדרות!$B$4,"")</f>
+      <c r="E14" s="36">
+        <f>IF(D14&gt;0,D14*הגדרות!$B$4,"")</f>
         <v>69.349999999999994</v>
       </c>
-      <c r="F13" s="30">
+      <c r="F14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="G13" s="31" t="str">
-        <f>IF(F13&gt;0,F13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="H13" s="30">
+      <c r="G14" s="36" t="str">
+        <f>IF(F14&gt;0,F14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I13" s="31" t="str">
-        <f>IF(H13&gt;0,H13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="30">
+      <c r="I14" s="36" t="str">
+        <f>IF(H14&gt;0,H14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="K13" s="31" t="str">
-        <f>IF(J13&gt;0,J13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="L13" s="30">
+      <c r="K14" s="36" t="str">
+        <f>IF(J14&gt;0,J14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M13" s="31" t="str">
-        <f>IF(L13&gt;0,L13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N13" s="30">
+      <c r="M14" s="36" t="str">
+        <f>IF(L14&gt;0,L14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="O13" s="31" t="str">
-        <f>IF(N13&gt;0,N13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="P13" s="30">
+      <c r="O14" s="36" t="str">
+        <f>IF(N14&gt;0,N14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="Q13" s="31" t="str">
-        <f>IF(P13&gt;0,P13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="R13" s="30">
+      <c r="Q14" s="36" t="str">
+        <f>IF(P14&gt;0,P14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>0</v>
       </c>
-      <c r="S13" s="31" t="str">
-        <f>IF(R13&gt;0,R13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="T13" s="30">
+      <c r="S14" s="36" t="str">
+        <f>IF(R14&gt;0,R14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="T14" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U13" s="31" t="str">
-        <f>IF(T13&gt;0,T13*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V13" s="32">
+      <c r="U14" s="36" t="str">
+        <f>IF(T14&gt;0,T14*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V14" s="32">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="W13" s="33">
-        <f>IF(V13&gt;0,V13*הגדרות!$B$4,"")</f>
+      <c r="W14" s="33">
+        <f>IF(V14&gt;0,V14*הגדרות!$B$4,"")</f>
         <v>69.349999999999994</v>
       </c>
     </row>
-    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A14" s="34" t="s">
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A15" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="B14" s="35">
+      <c r="B15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>0</v>
       </c>
-      <c r="C14" s="36" t="str">
-        <f>IF(B14&gt;0,B14*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="D14" s="35">
+      <c r="C15" s="31" t="str">
+        <f>IF(B15&gt;0,B15*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="D15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>0</v>
       </c>
-      <c r="E14" s="36" t="str">
-        <f>IF(D14&gt;0,D14*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="F14" s="35">
+      <c r="E15" s="31" t="str">
+        <f>IF(D15&gt;0,D15*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="G14" s="36" t="str">
-        <f>IF(F14&gt;0,F14*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="H14" s="35">
+      <c r="G15" s="31" t="str">
+        <f>IF(F15&gt;0,F15*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I14" s="36" t="str">
-        <f>IF(H14&gt;0,H14*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="35">
+      <c r="I15" s="31" t="str">
+        <f>IF(H15&gt;0,H15*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="K14" s="36" t="str">
-        <f>IF(J14&gt;0,J14*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="L14" s="35">
+      <c r="K15" s="31" t="str">
+        <f>IF(J15&gt;0,J15*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>15</v>
       </c>
-      <c r="M14" s="36">
-        <f>IF(L14&gt;0,L14*הגדרות!$B$4,"")</f>
+      <c r="M15" s="31">
+        <f>IF(L15&gt;0,L15*הגדרות!$B$4,"")</f>
         <v>54.75</v>
       </c>
-      <c r="N14" s="35">
+      <c r="N15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>15</v>
       </c>
-      <c r="O14" s="36">
-        <f>IF(N14&gt;0,N14*הגדרות!$B$4,"")</f>
+      <c r="O15" s="31">
+        <f>IF(N15&gt;0,N15*הגדרות!$B$4,"")</f>
         <v>54.75</v>
       </c>
-      <c r="P14" s="35">
+      <c r="P15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="Q14" s="36" t="str">
-        <f>IF(P14&gt;0,P14*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="R14" s="35">
+      <c r="Q15" s="31" t="str">
+        <f>IF(P15&gt;0,P15*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>0</v>
       </c>
-      <c r="S14" s="36" t="str">
-        <f>IF(R14&gt;0,R14*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="T14" s="35">
+      <c r="S15" s="31" t="str">
+        <f>IF(R15&gt;0,R15*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="T15" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U14" s="36" t="str">
-        <f>IF(T14&gt;0,T14*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V14" s="32">
+      <c r="U15" s="31" t="str">
+        <f>IF(T15&gt;0,T15*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V15" s="32">
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="W14" s="33">
-        <f>IF(V14&gt;0,V14*הגדרות!$B$4,"")</f>
+      <c r="W15" s="33">
+        <f>IF(V15&gt;0,V15*הגדרות!$B$4,"")</f>
         <v>109.5</v>
       </c>
     </row>
-    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A15" s="29" t="s">
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A16" s="34" t="s">
         <v>113</v>
       </c>
-      <c r="B15" s="30">
+      <c r="B16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>0</v>
       </c>
-      <c r="C15" s="31" t="str">
-        <f>IF(B15&gt;0,B15*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="D15" s="30">
+      <c r="C16" s="36" t="str">
+        <f>IF(B16&gt;0,B16*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="D16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>0</v>
       </c>
-      <c r="E15" s="31" t="str">
-        <f>IF(D15&gt;0,D15*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="F15" s="30">
+      <c r="E16" s="36" t="str">
+        <f>IF(D16&gt;0,D16*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="G15" s="31" t="str">
-        <f>IF(F15&gt;0,F15*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="H15" s="30">
+      <c r="G16" s="36" t="str">
+        <f>IF(F16&gt;0,F16*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I15" s="31" t="str">
-        <f>IF(H15&gt;0,H15*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="30">
+      <c r="I16" s="36" t="str">
+        <f>IF(H16&gt;0,H16*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="K15" s="31" t="str">
-        <f>IF(J15&gt;0,J15*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="L15" s="30">
+      <c r="K16" s="36" t="str">
+        <f>IF(J16&gt;0,J16*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M15" s="31" t="str">
-        <f>IF(L15&gt;0,L15*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N15" s="30">
+      <c r="M16" s="36" t="str">
+        <f>IF(L16&gt;0,L16*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="O15" s="31" t="str">
-        <f>IF(N15&gt;0,N15*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="P15" s="30">
+      <c r="O16" s="36" t="str">
+        <f>IF(N16&gt;0,N16*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>51</v>
       </c>
-      <c r="Q15" s="31">
-        <f>IF(P15&gt;0,P15*הגדרות!$B$4,"")</f>
+      <c r="Q16" s="36">
+        <f>IF(P16&gt;0,P16*הגדרות!$B$4,"")</f>
         <v>186.15</v>
       </c>
-      <c r="R15" s="30">
+      <c r="R16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>91.11</v>
       </c>
-      <c r="S15" s="31">
-        <f>IF(R15&gt;0,R15*הגדרות!$B$4,"")</f>
+      <c r="S16" s="36">
+        <f>IF(R16&gt;0,R16*הגדרות!$B$4,"")</f>
         <v>332.55149999999998</v>
       </c>
-      <c r="T15" s="30">
+      <c r="T16" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
-        <v>0</v>
-      </c>
-      <c r="U15" s="31" t="str">
-        <f>IF(T15&gt;0,T15*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V15" s="32">
+        <v>2.25</v>
+      </c>
+      <c r="U16" s="36">
+        <f>IF(T16&gt;0,T16*הגדרות!$B$4,"")</f>
+        <v>8.2125000000000004</v>
+      </c>
+      <c r="V16" s="32">
         <f t="shared" si="0"/>
-        <v>142.11000000000001</v>
-      </c>
-      <c r="W15" s="33">
-        <f>IF(V15&gt;0,V15*הגדרות!$B$4,"")</f>
-        <v>518.70150000000001</v>
-      </c>
-    </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A16" s="34" t="s">
+        <v>144.36000000000001</v>
+      </c>
+      <c r="W16" s="33">
+        <f>IF(V16&gt;0,V16*הגדרות!$B$4,"")</f>
+        <v>526.91399999999999</v>
+      </c>
+    </row>
+    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A17" s="29" t="s">
         <v>43</v>
       </c>
-      <c r="B16" s="35">
+      <c r="B17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>1</v>
       </c>
-      <c r="C16" s="36">
-        <f>IF(B16&gt;0,B16*הגדרות!$B$4,"")</f>
+      <c r="C17" s="31">
+        <f>IF(B17&gt;0,B17*הגדרות!$B$4,"")</f>
         <v>3.65</v>
       </c>
-      <c r="D16" s="35">
+      <c r="D17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>12</v>
       </c>
-      <c r="E16" s="36">
-        <f>IF(D16&gt;0,D16*הגדרות!$B$4,"")</f>
+      <c r="E17" s="31">
+        <f>IF(D17&gt;0,D17*הגדרות!$B$4,"")</f>
         <v>43.8</v>
       </c>
-      <c r="F16" s="35">
+      <c r="F17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="G16" s="36" t="str">
-        <f>IF(F16&gt;0,F16*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="H16" s="35">
+      <c r="G17" s="31" t="str">
+        <f>IF(F17&gt;0,F17*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I16" s="36" t="str">
-        <f>IF(H16&gt;0,H16*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="35">
+      <c r="I17" s="31" t="str">
+        <f>IF(H17&gt;0,H17*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>12</v>
       </c>
-      <c r="K16" s="36">
-        <f>IF(J16&gt;0,J16*הגדרות!$B$4,"")</f>
+      <c r="K17" s="31">
+        <f>IF(J17&gt;0,J17*הגדרות!$B$4,"")</f>
         <v>43.8</v>
       </c>
-      <c r="L16" s="35">
+      <c r="L17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M16" s="36" t="str">
-        <f>IF(L16&gt;0,L16*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N16" s="35">
+      <c r="M17" s="31" t="str">
+        <f>IF(L17&gt;0,L17*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="O16" s="36" t="str">
-        <f>IF(N16&gt;0,N16*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="P16" s="35">
+      <c r="O17" s="31" t="str">
+        <f>IF(N17&gt;0,N17*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="Q16" s="36" t="str">
-        <f>IF(P16&gt;0,P16*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="R16" s="35">
+      <c r="Q17" s="31" t="str">
+        <f>IF(P17&gt;0,P17*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>0</v>
       </c>
-      <c r="S16" s="36" t="str">
-        <f>IF(R16&gt;0,R16*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="T16" s="35">
+      <c r="S17" s="31" t="str">
+        <f>IF(R17&gt;0,R17*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="T17" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U16" s="36" t="str">
-        <f>IF(T16&gt;0,T16*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V16" s="32">
+      <c r="U17" s="31" t="str">
+        <f>IF(T17&gt;0,T17*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V17" s="32">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="W16" s="33">
-        <f>IF(V16&gt;0,V16*הגדרות!$B$4,"")</f>
+      <c r="W17" s="33">
+        <f>IF(V17&gt;0,V17*הגדרות!$B$4,"")</f>
         <v>91.25</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A17" s="29" t="s">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A18" s="34" t="s">
         <v>58</v>
       </c>
-      <c r="B17" s="30">
+      <c r="B18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>10</v>
       </c>
-      <c r="C17" s="31">
-        <f>IF(B17&gt;0,B17*הגדרות!$B$4,"")</f>
+      <c r="C18" s="36">
+        <f>IF(B18&gt;0,B18*הגדרות!$B$4,"")</f>
         <v>36.5</v>
       </c>
-      <c r="D17" s="30">
+      <c r="D18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>0.9</v>
       </c>
-      <c r="E17" s="31">
-        <f>IF(D17&gt;0,D17*הגדרות!$B$4,"")</f>
+      <c r="E18" s="36">
+        <f>IF(D18&gt;0,D18*הגדרות!$B$4,"")</f>
         <v>3.2850000000000001</v>
       </c>
-      <c r="F17" s="30">
+      <c r="F18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>2.79</v>
       </c>
-      <c r="G17" s="31">
-        <f>IF(F17&gt;0,F17*הגדרות!$B$4,"")</f>
+      <c r="G18" s="36">
+        <f>IF(F18&gt;0,F18*הגדרות!$B$4,"")</f>
         <v>10.1835</v>
       </c>
-      <c r="H17" s="30">
+      <c r="H18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I17" s="31" t="str">
-        <f>IF(H17&gt;0,H17*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J17" s="30">
+      <c r="I18" s="36" t="str">
+        <f>IF(H18&gt;0,H18*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="K17" s="31" t="str">
-        <f>IF(J17&gt;0,J17*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="L17" s="30">
+      <c r="K18" s="36" t="str">
+        <f>IF(J18&gt;0,J18*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M17" s="31" t="str">
-        <f>IF(L17&gt;0,L17*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N17" s="30">
+      <c r="M18" s="36" t="str">
+        <f>IF(L18&gt;0,L18*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="O17" s="31" t="str">
-        <f>IF(N17&gt;0,N17*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="P17" s="30">
+      <c r="O18" s="36" t="str">
+        <f>IF(N18&gt;0,N18*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="Q17" s="31" t="str">
-        <f>IF(P17&gt;0,P17*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="R17" s="30">
+      <c r="Q18" s="36" t="str">
+        <f>IF(P18&gt;0,P18*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>0</v>
       </c>
-      <c r="S17" s="31" t="str">
-        <f>IF(R17&gt;0,R17*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="T17" s="30">
+      <c r="S18" s="36" t="str">
+        <f>IF(R18&gt;0,R18*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="T18" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U17" s="31" t="str">
-        <f>IF(T17&gt;0,T17*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V17" s="32">
+      <c r="U18" s="36" t="str">
+        <f>IF(T18&gt;0,T18*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V18" s="32">
         <f t="shared" si="0"/>
         <v>13.690000000000001</v>
       </c>
-      <c r="W17" s="33">
-        <f>IF(V17&gt;0,V17*הגדרות!$B$4,"")</f>
+      <c r="W18" s="33">
+        <f>IF(V18&gt;0,V18*הגדרות!$B$4,"")</f>
         <v>49.968500000000006</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A18" s="34" t="s">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A19" s="29" t="s">
         <v>55</v>
       </c>
-      <c r="B18" s="35">
+      <c r="B19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>13.5</v>
       </c>
-      <c r="C18" s="36">
-        <f>IF(B18&gt;0,B18*הגדרות!$B$4,"")</f>
+      <c r="C19" s="31">
+        <f>IF(B19&gt;0,B19*הגדרות!$B$4,"")</f>
         <v>49.274999999999999</v>
       </c>
-      <c r="D18" s="35">
+      <c r="D19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>26.25</v>
       </c>
-      <c r="E18" s="36">
-        <f>IF(D18&gt;0,D18*הגדרות!$B$4,"")</f>
+      <c r="E19" s="31">
+        <f>IF(D19&gt;0,D19*הגדרות!$B$4,"")</f>
         <v>95.8125</v>
       </c>
-      <c r="F18" s="35">
+      <c r="F19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="G18" s="36" t="str">
-        <f>IF(F18&gt;0,F18*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="H18" s="35">
+      <c r="G19" s="31" t="str">
+        <f>IF(F19&gt;0,F19*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I18" s="36" t="str">
-        <f>IF(H18&gt;0,H18*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J18" s="35">
+      <c r="I19" s="31" t="str">
+        <f>IF(H19&gt;0,H19*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>15</v>
       </c>
-      <c r="K18" s="36">
-        <f>IF(J18&gt;0,J18*הגדרות!$B$4,"")</f>
+      <c r="K19" s="31">
+        <f>IF(J19&gt;0,J19*הגדרות!$B$4,"")</f>
         <v>54.75</v>
       </c>
-      <c r="L18" s="35">
+      <c r="L19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M18" s="36" t="str">
-        <f>IF(L18&gt;0,L18*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N18" s="35">
+      <c r="M19" s="31" t="str">
+        <f>IF(L19&gt;0,L19*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="O18" s="36" t="str">
-        <f>IF(N18&gt;0,N18*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="P18" s="35">
+      <c r="O19" s="31" t="str">
+        <f>IF(N19&gt;0,N19*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="P19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="Q18" s="36" t="str">
-        <f>IF(P18&gt;0,P18*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="R18" s="35">
+      <c r="Q19" s="31" t="str">
+        <f>IF(P19&gt;0,P19*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>0</v>
       </c>
-      <c r="S18" s="36" t="str">
-        <f>IF(R18&gt;0,R18*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="T18" s="35">
+      <c r="S19" s="31" t="str">
+        <f>IF(R19&gt;0,R19*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="T19" s="30">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U18" s="36" t="str">
-        <f>IF(T18&gt;0,T18*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V18" s="32">
+      <c r="U19" s="31" t="str">
+        <f>IF(T19&gt;0,T19*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V19" s="32">
         <f t="shared" si="0"/>
         <v>54.75</v>
       </c>
-      <c r="W18" s="33">
-        <f>IF(V18&gt;0,V18*הגדרות!$B$4,"")</f>
+      <c r="W19" s="33">
+        <f>IF(V19&gt;0,V19*הגדרות!$B$4,"")</f>
         <v>199.83750000000001</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A19" s="29" t="s">
+    <row r="20" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A20" s="34" t="s">
         <v>104</v>
       </c>
-      <c r="B19" s="30">
+      <c r="B20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v>0</v>
       </c>
-      <c r="C19" s="31" t="str">
-        <f>IF(B19&gt;0,B19*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="D19" s="30">
+      <c r="C20" s="36" t="str">
+        <f>IF(B20&gt;0,B20*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="D20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v>0</v>
       </c>
-      <c r="E19" s="31" t="str">
-        <f>IF(D19&gt;0,D19*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="F19" s="30">
+      <c r="E20" s="36" t="str">
+        <f>IF(D20&gt;0,D20*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="F20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="G19" s="31" t="str">
-        <f>IF(F19&gt;0,F19*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="H19" s="30">
+      <c r="G20" s="36" t="str">
+        <f>IF(F20&gt;0,F20*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="H20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v>0</v>
       </c>
-      <c r="I19" s="31" t="str">
-        <f>IF(H19&gt;0,H19*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="30">
+      <c r="I20" s="36" t="str">
+        <f>IF(H20&gt;0,H20*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="J20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="K19" s="31" t="str">
-        <f>IF(J19&gt;0,J19*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="30">
+      <c r="K20" s="36" t="str">
+        <f>IF(J20&gt;0,J20*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="L20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v>0</v>
       </c>
-      <c r="M19" s="31" t="str">
-        <f>IF(L19&gt;0,L19*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="N19" s="30">
+      <c r="M20" s="36" t="str">
+        <f>IF(L20&gt;0,L20*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="N20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v>14.5</v>
       </c>
-      <c r="O19" s="31">
-        <f>IF(N19&gt;0,N19*הגדרות!$B$4,"")</f>
+      <c r="O20" s="36">
+        <f>IF(N20&gt;0,N20*הגדרות!$B$4,"")</f>
         <v>52.924999999999997</v>
       </c>
-      <c r="P19" s="30">
+      <c r="P20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v>0</v>
       </c>
-      <c r="Q19" s="31" t="str">
-        <f>IF(P19&gt;0,P19*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="R19" s="30">
+      <c r="Q20" s="36" t="str">
+        <f>IF(P20&gt;0,P20*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="R20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v>14.5</v>
       </c>
-      <c r="S19" s="31">
-        <f>IF(R19&gt;0,R19*הגדרות!$B$4,"")</f>
+      <c r="S20" s="36">
+        <f>IF(R20&gt;0,R20*הגדרות!$B$4,"")</f>
         <v>52.924999999999997</v>
       </c>
-      <c r="T19" s="30">
+      <c r="T20" s="35">
         <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v>0</v>
       </c>
-      <c r="U19" s="31" t="str">
-        <f>IF(T19&gt;0,T19*הגדרות!$B$4,"")</f>
-        <v/>
-      </c>
-      <c r="V19" s="32">
+      <c r="U20" s="36" t="str">
+        <f>IF(T20&gt;0,T20*הגדרות!$B$4,"")</f>
+        <v/>
+      </c>
+      <c r="V20" s="32">
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="W19" s="33">
-        <f>IF(V19&gt;0,V19*הגדרות!$B$4,"")</f>
+      <c r="W20" s="33">
+        <f>IF(V20&gt;0,V20*הגדרות!$B$4,"")</f>
         <v>105.85</v>
       </c>
     </row>
-    <row r="20" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="25" t="s">
-        <v>153</v>
-      </c>
-      <c r="B20" s="16">
-        <f t="shared" ref="B20:W20" si="1">SUM(B5:B19)</f>
+    <row r="21" spans="1:23" ht="24" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" s="25" t="s">
+        <v>159</v>
+      </c>
+      <c r="B21" s="16">
+        <f t="shared" ref="B21:W21" si="1">SUM(B5:B20)</f>
         <v>240.23</v>
       </c>
-      <c r="C20" s="17">
+      <c r="C21" s="17">
         <f t="shared" si="1"/>
         <v>876.83949999999993</v>
       </c>
-      <c r="D20" s="16">
+      <c r="D21" s="16">
         <f t="shared" si="1"/>
         <v>93.740000000000009</v>
       </c>
-      <c r="E20" s="17">
+      <c r="E21" s="17">
         <f t="shared" si="1"/>
         <v>342.15099999999995</v>
       </c>
-      <c r="F20" s="16">
+      <c r="F21" s="16">
         <f t="shared" si="1"/>
         <v>38.380000000000003</v>
       </c>
-      <c r="G20" s="17">
+      <c r="G21" s="17">
         <f t="shared" si="1"/>
         <v>140.08700000000002</v>
       </c>
-      <c r="H20" s="16">
+      <c r="H21" s="16">
         <f t="shared" si="1"/>
         <v>25</v>
       </c>
-      <c r="I20" s="17">
+      <c r="I21" s="17">
         <f t="shared" si="1"/>
         <v>91.25</v>
       </c>
-      <c r="J20" s="16">
+      <c r="J21" s="16">
         <f t="shared" si="1"/>
         <v>73.8</v>
       </c>
-      <c r="K20" s="17">
+      <c r="K21" s="17">
         <f t="shared" si="1"/>
         <v>269.37</v>
       </c>
-      <c r="L20" s="16">
+      <c r="L21" s="16">
         <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="M20" s="17">
+      <c r="M21" s="17">
         <f t="shared" si="1"/>
         <v>73</v>
       </c>
-      <c r="N20" s="16">
+      <c r="N21" s="16">
         <f t="shared" si="1"/>
         <v>214.42</v>
       </c>
-      <c r="O20" s="17">
+      <c r="O21" s="17">
         <f t="shared" si="1"/>
         <v>782.63299999999992</v>
       </c>
-      <c r="P20" s="16">
+      <c r="P21" s="16">
         <f t="shared" si="1"/>
         <v>156</v>
       </c>
-      <c r="Q20" s="17">
+      <c r="Q21" s="17">
         <f t="shared" si="1"/>
         <v>569.4</v>
       </c>
-      <c r="R20" s="16">
+      <c r="R21" s="16">
         <f t="shared" si="1"/>
-        <v>146.61000000000001</v>
-      </c>
-      <c r="S20" s="17">
+        <v>151.61000000000001</v>
+      </c>
+      <c r="S21" s="17">
         <f t="shared" si="1"/>
-        <v>535.12649999999996</v>
-      </c>
-      <c r="T20" s="16">
+        <v>553.37649999999996</v>
+      </c>
+      <c r="T21" s="16">
         <f t="shared" si="1"/>
-        <v>25</v>
-      </c>
-      <c r="U20" s="17">
+        <v>47.25</v>
+      </c>
+      <c r="U21" s="17">
         <f t="shared" si="1"/>
-        <v>91.25</v>
-      </c>
-      <c r="V20" s="37">
+        <v>172.46250000000001</v>
+      </c>
+      <c r="V21" s="37">
         <f t="shared" si="1"/>
-        <v>1033.18</v>
-      </c>
-      <c r="W20" s="38">
+        <v>1060.43</v>
+      </c>
+      <c r="W21" s="38">
         <f t="shared" si="1"/>
-        <v>3771.107</v>
+        <v>3870.5694999999996</v>
       </c>
     </row>
   </sheetData>
@@ -3850,7 +4018,7 @@
       </c>
       <c r="E4" s="42">
         <f>IF(C15&gt;0,C4/C15,0)</f>
-        <v>0.23251514740897036</v>
+        <v>0.2265401770979697</v>
       </c>
       <c r="F4" s="19"/>
     </row>
@@ -3871,7 +4039,7 @@
       </c>
       <c r="E5" s="46">
         <f>IF(C15&gt;0,C5/C15,0)</f>
-        <v>9.0729592133026185E-2</v>
+        <v>8.8398102656469538E-2</v>
       </c>
       <c r="F5" s="24"/>
     </row>
@@ -3892,7 +4060,7 @@
       </c>
       <c r="E6" s="42">
         <f>IF(C15&gt;0,C6/C15,0)</f>
-        <v>3.7147447685785623E-2</v>
+        <v>3.619286515847344E-2</v>
       </c>
       <c r="F6" s="19"/>
     </row>
@@ -3913,7 +4081,7 @@
       </c>
       <c r="E7" s="46">
         <f>IF(C15&gt;0,C7/C15,0)</f>
-        <v>2.4197138930292881E-2</v>
+        <v>2.3575342078213553E-2</v>
       </c>
       <c r="F7" s="24"/>
     </row>
@@ -3934,7 +4102,7 @@
       </c>
       <c r="E8" s="42">
         <f>IF(C15&gt;0,C8/C15,0)</f>
-        <v>7.1429954122224582E-2</v>
+        <v>6.9594409814886404E-2</v>
       </c>
       <c r="F8" s="19"/>
     </row>
@@ -3955,7 +4123,7 @@
       </c>
       <c r="E9" s="46">
         <f>IF(C15&gt;0,C9/C15,0)</f>
-        <v>1.9357711144234305E-2</v>
+        <v>1.8860273662570842E-2</v>
       </c>
       <c r="F9" s="24"/>
     </row>
@@ -3976,7 +4144,7 @@
       </c>
       <c r="E10" s="42">
         <f>IF(C15&gt;0,C10/C15,0)</f>
-        <v>0.20753402117733596</v>
+        <v>0.20220099393642199</v>
       </c>
       <c r="F10" s="19"/>
     </row>
@@ -3997,7 +4165,7 @@
       </c>
       <c r="E11" s="46">
         <f>IF(C15&gt;0,C11/C15,0)</f>
-        <v>0.15099014692502757</v>
+        <v>0.14711013456805258</v>
       </c>
       <c r="F11" s="24"/>
     </row>
@@ -4010,15 +4178,15 @@
       </c>
       <c r="C12" s="40">
         <f>SUMIF('כל ההוצאות'!$F:$F,"מרץ 2026",'כל ההוצאות'!$D:$D)</f>
-        <v>146.61000000000001</v>
+        <v>151.61000000000001</v>
       </c>
       <c r="D12" s="41">
         <f>C12*הגדרות!$B$4</f>
-        <v>535.12650000000008</v>
+        <v>553.37650000000008</v>
       </c>
       <c r="E12" s="42">
         <f>IF(C15&gt;0,C12/C15,0)</f>
-        <v>0.14190170154280959</v>
+        <v>0.14297030449911829</v>
       </c>
       <c r="F12" s="19"/>
     </row>
@@ -4031,15 +4199,15 @@
       </c>
       <c r="C13" s="44">
         <f>SUMIF('כל ההוצאות'!$F:$F,"אפריל 2026",'כל ההוצאות'!$D:$D)</f>
-        <v>25</v>
+        <v>47.25</v>
       </c>
       <c r="D13" s="45">
         <f>C13*הגדרות!$B$4</f>
-        <v>91.25</v>
+        <v>172.46250000000001</v>
       </c>
       <c r="E13" s="46">
         <f>IF(C15&gt;0,C13/C15,0)</f>
-        <v>2.4197138930292881E-2</v>
+        <v>4.4557396527823617E-2</v>
       </c>
       <c r="F13" s="24"/>
     </row>
@@ -4058,11 +4226,11 @@
       <c r="B15" s="58"/>
       <c r="C15" s="47">
         <f>SUM(C4:C13)</f>
-        <v>1033.18</v>
+        <v>1060.43</v>
       </c>
       <c r="D15" s="48">
         <f>C15*הגדרות!$B$4</f>
-        <v>3771.107</v>
+        <v>3870.5695000000001</v>
       </c>
       <c r="E15" s="49" t="s">
         <v>29</v>
@@ -4076,11 +4244,11 @@
       <c r="B16" s="55"/>
       <c r="C16" s="50">
         <f>AVERAGE(C4:C13)</f>
-        <v>103.31800000000001</v>
+        <v>106.04300000000001</v>
       </c>
       <c r="D16" s="51">
         <f>AVERAGE(D4:D13)</f>
-        <v>377.11070000000001</v>
+        <v>387.05695000000003</v>
       </c>
       <c r="E16" s="19"/>
       <c r="F16" s="19"/>
@@ -4114,7 +4282,7 @@
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
   </sheetPr>
-  <dimension ref="A1:F52"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -5146,63 +5314,126 @@
         <v>123</v>
       </c>
       <c r="B50" s="11" t="s">
-        <v>52</v>
+        <v>107</v>
       </c>
       <c r="C50" s="11" t="s">
-        <v>53</v>
+        <v>124</v>
       </c>
       <c r="D50" s="12">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E50" s="13">
         <f>D50*הגדרות!$B$4</f>
-        <v>73</v>
+        <v>18.25</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B51" s="7" t="s">
         <v>52</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>111</v>
+        <v>53</v>
       </c>
       <c r="D51" s="8">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E51" s="9">
         <f>D51*הגדרות!$B$4</f>
-        <v>18.25</v>
+        <v>73</v>
       </c>
       <c r="F51" s="6" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" s="62" t="s">
-        <v>124</v>
-      </c>
-      <c r="B52" s="63"/>
-      <c r="C52" s="63"/>
-      <c r="D52" s="16">
-        <f>SUM(D3:D51)</f>
-        <v>1033.1799999999998</v>
-      </c>
-      <c r="E52" s="17">
-        <f>SUM(E3:E51)</f>
-        <v>3771.1070000000004</v>
-      </c>
-      <c r="F52" s="15"/>
+      <c r="A52" s="10" t="s">
+        <v>125</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="C52" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="D52" s="12">
+        <v>5</v>
+      </c>
+      <c r="E52" s="13">
+        <f>D52*הגדרות!$B$4</f>
+        <v>18.25</v>
+      </c>
+      <c r="F52" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="B53" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="C53" s="7" t="s">
+        <v>114</v>
+      </c>
+      <c r="D53" s="8">
+        <v>2.25</v>
+      </c>
+      <c r="E53" s="9">
+        <f>D53*הגדרות!$B$4</f>
+        <v>8.2125000000000004</v>
+      </c>
+      <c r="F53" s="6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" s="10" t="s">
+        <v>127</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>128</v>
+      </c>
+      <c r="C54" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D54" s="12">
+        <v>20</v>
+      </c>
+      <c r="E54" s="13">
+        <f>D54*הגדרות!$B$4</f>
+        <v>73</v>
+      </c>
+      <c r="F54" s="10" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" s="62" t="s">
+        <v>130</v>
+      </c>
+      <c r="B55" s="63"/>
+      <c r="C55" s="63"/>
+      <c r="D55" s="16">
+        <f>SUM(D3:D54)</f>
+        <v>1060.4299999999998</v>
+      </c>
+      <c r="E55" s="17">
+        <f>SUM(E3:E54)</f>
+        <v>3870.5695000000005</v>
+      </c>
+      <c r="F55" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A55:C55"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5225,7 +5456,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -5235,7 +5466,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -5396,7 +5627,7 @@
     </row>
     <row r="11" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="65" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B11" s="58"/>
       <c r="C11" s="58"/>
@@ -5439,7 +5670,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -5449,7 +5680,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -5629,7 +5860,7 @@
     </row>
     <row r="12" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="65" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B12" s="58"/>
       <c r="C12" s="58"/>
@@ -5672,7 +5903,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -5682,7 +5913,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -5786,7 +6017,7 @@
     </row>
     <row r="8" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="65" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B8" s="58"/>
       <c r="C8" s="58"/>
@@ -5829,7 +6060,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -5839,7 +6070,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -5905,7 +6136,7 @@
     </row>
     <row r="6" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="65" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B6" s="58"/>
       <c r="C6" s="58"/>
@@ -5948,7 +6179,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -5958,7 +6189,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -6100,7 +6331,7 @@
     </row>
     <row r="10" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="65" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B10" s="58"/>
       <c r="C10" s="58"/>
@@ -6143,7 +6374,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -6153,7 +6384,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -6219,7 +6450,7 @@
     </row>
     <row r="6" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="65" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B6" s="58"/>
       <c r="C6" s="58"/>
@@ -6262,7 +6493,7 @@
   <sheetData>
     <row r="1" spans="1:6" ht="31.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="64" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="B1" s="53"/>
       <c r="C1" s="53"/>
@@ -6272,7 +6503,7 @@
     </row>
     <row r="2" spans="1:6" ht="16.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="18" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="B2" s="19"/>
       <c r="C2" s="19"/>
@@ -6414,7 +6645,7 @@
     </row>
     <row r="10" spans="1:6" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="65" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="B10" s="58"/>
       <c r="C10" s="58"/>

</xml_diff>

<commit_message>
Convert dashboard to live ILS spend view
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -935,15 +935,15 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>שער USD → ILS (לעדכון ידני)</t>
+          <t>שער USD → ILS (מתעדכן אוטומטית)</t>
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3.65</v>
+        <v>3.142</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>← ניתן לעדכן שיעור זה בכל עת</t>
+          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-07</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prepare secure online manual import gateway
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -939,11 +939,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3.142</v>
+        <v>3.087</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-07</t>
+          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-09</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
         <v>25</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>78.55</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1119,7 +1119,7 @@
         <v>31.42</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>98.72</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -1167,7 +1167,7 @@
         <v>47</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>147.67</v>
+        <v>145.09</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -1191,7 +1191,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -1215,7 +1215,7 @@
         <v>5</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -1239,7 +1239,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -1263,7 +1263,7 @@
         <v>20</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -1287,7 +1287,7 @@
         <v>50</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>157.1</v>
+        <v>154.35</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -1311,7 +1311,7 @@
         <v>51</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>160.24</v>
+        <v>157.44</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -1335,7 +1335,7 @@
         <v>5</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -1359,7 +1359,7 @@
         <v>10</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
@@ -1478,7 +1478,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1502,7 +1502,7 @@
         <v>14.5</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>45.56</v>
+        <v>44.76</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -1550,7 +1550,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -1574,7 +1574,7 @@
         <v>40.11</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>126.03</v>
+        <v>123.82</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -1622,7 +1622,7 @@
         <v>51</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>160.24</v>
+        <v>157.44</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -1646,7 +1646,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -1670,7 +1670,7 @@
         <v>20</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -1694,7 +1694,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -1718,7 +1718,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>34.56</v>
+        <v>33.96</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -1742,7 +1742,7 @@
         <v>5</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -1861,7 +1861,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1885,7 +1885,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -1933,7 +1933,7 @@
         <v>51</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>160.24</v>
+        <v>157.44</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -1957,7 +1957,7 @@
         <v>2.25</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>7.07</v>
+        <v>6.95</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -2005,7 +2005,7 @@
         <v>20</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -2124,7 +2124,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2243,7 +2243,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2362,7 +2362,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2481,7 +2481,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2600,7 +2600,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2719,7 +2719,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2838,7 +2838,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2949,7 +2949,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>3.14</v>
+        <v>3.09</v>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
@@ -2977,7 +2977,7 @@
         <v>72</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>226.22</v>
+        <v>222.26</v>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
@@ -3005,7 +3005,7 @@
         <v>10.59</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>33.27</v>
+        <v>32.69</v>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -3033,7 +3033,7 @@
         <v>20</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
@@ -3061,7 +3061,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
@@ -3089,7 +3089,7 @@
         <v>13.5</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>42.42</v>
+        <v>41.67</v>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
@@ -3117,7 +3117,7 @@
         <v>113.14</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>355.49</v>
+        <v>349.26</v>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
@@ -3145,7 +3145,7 @@
         <v>10</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
@@ -3201,7 +3201,7 @@
         <v>15</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>47.13</v>
+        <v>46.3</v>
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
@@ -3229,7 +3229,7 @@
         <v>12</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>37.7</v>
+        <v>37.04</v>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
@@ -3257,7 +3257,7 @@
         <v>0.9</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>2.83</v>
+        <v>2.78</v>
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
@@ -3285,7 +3285,7 @@
         <v>19</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>59.7</v>
+        <v>58.65</v>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
@@ -3313,7 +3313,7 @@
         <v>10.59</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>33.27</v>
+        <v>32.69</v>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
@@ -3341,7 +3341,7 @@
         <v>20</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
@@ -3369,7 +3369,7 @@
         <v>20</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
@@ -3397,7 +3397,7 @@
         <v>5</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
@@ -3425,7 +3425,7 @@
         <v>11.25</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>35.35</v>
+        <v>34.73</v>
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
@@ -3481,7 +3481,7 @@
         <v>2.79</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>8.77</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
@@ -3509,7 +3509,7 @@
         <v>10.59</v>
       </c>
       <c r="E23" s="13" t="n">
-        <v>33.27</v>
+        <v>32.69</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
@@ -3537,7 +3537,7 @@
         <v>20</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
@@ -3565,7 +3565,7 @@
         <v>20</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
@@ -3593,7 +3593,7 @@
         <v>5</v>
       </c>
       <c r="E26" s="17" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
@@ -3649,7 +3649,7 @@
         <v>20</v>
       </c>
       <c r="E28" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
@@ -3677,7 +3677,7 @@
         <v>20</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
@@ -3705,7 +3705,7 @@
         <v>5</v>
       </c>
       <c r="E30" s="17" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
@@ -3733,7 +3733,7 @@
         <v>12</v>
       </c>
       <c r="E31" s="13" t="n">
-        <v>37.7</v>
+        <v>37.04</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -3761,7 +3761,7 @@
         <v>11.8</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>37.08</v>
+        <v>36.43</v>
       </c>
       <c r="F32" s="14" t="inlineStr">
         <is>
@@ -3789,7 +3789,7 @@
         <v>15</v>
       </c>
       <c r="E33" s="13" t="n">
-        <v>47.13</v>
+        <v>46.3</v>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
@@ -3817,7 +3817,7 @@
         <v>10</v>
       </c>
       <c r="E34" s="17" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
@@ -3845,7 +3845,7 @@
         <v>20</v>
       </c>
       <c r="E35" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
         <v>20</v>
       </c>
       <c r="E36" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F36" s="14" t="inlineStr">
         <is>
@@ -3901,7 +3901,7 @@
         <v>5</v>
       </c>
       <c r="E37" s="13" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
@@ -3957,7 +3957,7 @@
         <v>15</v>
       </c>
       <c r="E39" s="13" t="n">
-        <v>47.13</v>
+        <v>46.3</v>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
@@ -3985,7 +3985,7 @@
         <v>9.720000000000001</v>
       </c>
       <c r="E40" s="17" t="n">
-        <v>30.54</v>
+        <v>30.01</v>
       </c>
       <c r="F40" s="14" t="inlineStr">
         <is>
@@ -4013,7 +4013,7 @@
         <v>30</v>
       </c>
       <c r="E41" s="13" t="n">
-        <v>94.26000000000001</v>
+        <v>92.61</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
@@ -4041,7 +4041,7 @@
         <v>33</v>
       </c>
       <c r="E42" s="17" t="n">
-        <v>103.69</v>
+        <v>101.87</v>
       </c>
       <c r="F42" s="14" t="inlineStr">
         <is>
@@ -4069,7 +4069,7 @@
         <v>20</v>
       </c>
       <c r="E43" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
@@ -4097,7 +4097,7 @@
         <v>36</v>
       </c>
       <c r="E44" s="17" t="n">
-        <v>113.11</v>
+        <v>111.13</v>
       </c>
       <c r="F44" s="14" t="inlineStr">
         <is>
@@ -4125,7 +4125,7 @@
         <v>5</v>
       </c>
       <c r="E45" s="13" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
@@ -4181,7 +4181,7 @@
         <v>139.92</v>
       </c>
       <c r="E47" s="13" t="n">
-        <v>439.63</v>
+        <v>431.93</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
@@ -4209,7 +4209,7 @@
         <v>15</v>
       </c>
       <c r="E48" s="17" t="n">
-        <v>47.13</v>
+        <v>46.3</v>
       </c>
       <c r="F48" s="14" t="inlineStr">
         <is>
@@ -4237,7 +4237,7 @@
         <v>19.43</v>
       </c>
       <c r="E49" s="13" t="n">
-        <v>61.05</v>
+        <v>59.98</v>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
@@ -4265,7 +4265,7 @@
         <v>20</v>
       </c>
       <c r="E50" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F50" s="14" t="inlineStr">
         <is>
@@ -4293,7 +4293,7 @@
         <v>20</v>
       </c>
       <c r="E51" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
@@ -4349,7 +4349,7 @@
         <v>20</v>
       </c>
       <c r="E53" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
@@ -4377,7 +4377,7 @@
         <v>39</v>
       </c>
       <c r="E54" s="17" t="n">
-        <v>122.54</v>
+        <v>120.39</v>
       </c>
       <c r="F54" s="14" t="inlineStr">
         <is>
@@ -4405,7 +4405,7 @@
         <v>25</v>
       </c>
       <c r="E55" s="13" t="n">
-        <v>78.55</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
@@ -4433,7 +4433,7 @@
         <v>43</v>
       </c>
       <c r="E56" s="17" t="n">
-        <v>135.11</v>
+        <v>132.74</v>
       </c>
       <c r="F56" s="14" t="inlineStr">
         <is>
@@ -4461,7 +4461,7 @@
         <v>5</v>
       </c>
       <c r="E57" s="13" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
@@ -4489,7 +4489,7 @@
         <v>14.5</v>
       </c>
       <c r="E58" s="17" t="n">
-        <v>45.56</v>
+        <v>44.76</v>
       </c>
       <c r="F58" s="14" t="inlineStr">
         <is>
@@ -4517,7 +4517,7 @@
         <v>25</v>
       </c>
       <c r="E59" s="13" t="n">
-        <v>78.55</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
@@ -4573,7 +4573,7 @@
         <v>31.42</v>
       </c>
       <c r="E61" s="13" t="n">
-        <v>98.72</v>
+        <v>96.98999999999999</v>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
@@ -4629,7 +4629,7 @@
         <v>47</v>
       </c>
       <c r="E63" s="13" t="n">
-        <v>147.67</v>
+        <v>145.09</v>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
@@ -4657,7 +4657,7 @@
         <v>20</v>
       </c>
       <c r="E64" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
@@ -4685,7 +4685,7 @@
         <v>5</v>
       </c>
       <c r="E65" s="13" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
@@ -4713,7 +4713,7 @@
         <v>20</v>
       </c>
       <c r="E66" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
@@ -4741,7 +4741,7 @@
         <v>20</v>
       </c>
       <c r="E67" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
@@ -4769,7 +4769,7 @@
         <v>50</v>
       </c>
       <c r="E68" s="17" t="n">
-        <v>157.1</v>
+        <v>154.35</v>
       </c>
       <c r="F68" s="14" t="inlineStr">
         <is>
@@ -4797,7 +4797,7 @@
         <v>51</v>
       </c>
       <c r="E69" s="13" t="n">
-        <v>160.24</v>
+        <v>157.44</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
@@ -4825,7 +4825,7 @@
         <v>5</v>
       </c>
       <c r="E70" s="17" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F70" s="14" t="inlineStr">
         <is>
@@ -4853,7 +4853,7 @@
         <v>10</v>
       </c>
       <c r="E71" s="13" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -4881,7 +4881,7 @@
         <v>10</v>
       </c>
       <c r="E72" s="17" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F72" s="14" t="inlineStr">
         <is>
@@ -4909,7 +4909,7 @@
         <v>14.5</v>
       </c>
       <c r="E73" s="13" t="n">
-        <v>45.56</v>
+        <v>44.76</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -4965,7 +4965,7 @@
         <v>10</v>
       </c>
       <c r="E75" s="13" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -4993,7 +4993,7 @@
         <v>40.11</v>
       </c>
       <c r="E76" s="17" t="n">
-        <v>126.03</v>
+        <v>123.82</v>
       </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
@@ -5049,7 +5049,7 @@
         <v>51</v>
       </c>
       <c r="E78" s="17" t="n">
-        <v>160.24</v>
+        <v>157.44</v>
       </c>
       <c r="F78" s="14" t="inlineStr">
         <is>
@@ -5077,7 +5077,7 @@
         <v>20</v>
       </c>
       <c r="E79" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -5105,7 +5105,7 @@
         <v>20</v>
       </c>
       <c r="E80" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F80" s="14" t="inlineStr">
         <is>
@@ -5133,7 +5133,7 @@
         <v>10</v>
       </c>
       <c r="E81" s="13" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -5161,7 +5161,7 @@
         <v>11</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>34.56</v>
+        <v>33.96</v>
       </c>
       <c r="F82" s="14" t="inlineStr">
         <is>
@@ -5189,7 +5189,7 @@
         <v>5</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5217,7 +5217,7 @@
         <v>20</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5245,7 +5245,7 @@
         <v>5</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5301,7 +5301,7 @@
         <v>51</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>160.24</v>
+        <v>157.44</v>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
@@ -5329,7 +5329,7 @@
         <v>2.25</v>
       </c>
       <c r="E88" s="17" t="n">
-        <v>7.07</v>
+        <v>6.95</v>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
@@ -5357,7 +5357,7 @@
         <v>20</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5385,7 +5385,7 @@
         <v>20</v>
       </c>
       <c r="E90" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
@@ -5413,7 +5413,7 @@
         <v>20</v>
       </c>
       <c r="E91" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
@@ -5441,7 +5441,7 @@
         <v>20</v>
       </c>
       <c r="E92" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
@@ -5469,7 +5469,7 @@
         <v>20</v>
       </c>
       <c r="E93" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
@@ -5497,7 +5497,7 @@
         <v>20</v>
       </c>
       <c r="E94" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
@@ -5525,7 +5525,7 @@
         <v>20</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
@@ -5553,7 +5553,7 @@
         <v>20</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -5581,7 +5581,7 @@
         <v>20</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -5609,7 +5609,7 @@
         <v>20</v>
       </c>
       <c r="E98" s="17" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -10211,7 +10211,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>3.14</v>
+        <v>3.09</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -10235,7 +10235,7 @@
         <v>72</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>226.22</v>
+        <v>222.26</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -10259,7 +10259,7 @@
         <v>10.59</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>33.27</v>
+        <v>32.69</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -10283,7 +10283,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -10307,7 +10307,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -10331,7 +10331,7 @@
         <v>13.5</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>42.42</v>
+        <v>41.67</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -10355,7 +10355,7 @@
         <v>113.14</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>355.49</v>
+        <v>349.26</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -10379,7 +10379,7 @@
         <v>10</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -10522,7 +10522,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>47.13</v>
+        <v>46.3</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -10546,7 +10546,7 @@
         <v>12</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>37.7</v>
+        <v>37.04</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -10570,7 +10570,7 @@
         <v>0.9</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>2.83</v>
+        <v>2.78</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -10594,7 +10594,7 @@
         <v>19</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>59.7</v>
+        <v>58.65</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -10618,7 +10618,7 @@
         <v>10.59</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>33.27</v>
+        <v>32.69</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -10642,7 +10642,7 @@
         <v>20</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -10666,7 +10666,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -10690,7 +10690,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -10714,7 +10714,7 @@
         <v>11.25</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>35.35</v>
+        <v>34.73</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -10857,7 +10857,7 @@
         <v>2.79</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>8.77</v>
+        <v>8.609999999999999</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -10881,7 +10881,7 @@
         <v>10.59</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>33.27</v>
+        <v>32.69</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -10905,7 +10905,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -10929,7 +10929,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -10953,7 +10953,7 @@
         <v>5</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11096,7 +11096,7 @@
         <v>20</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11120,7 +11120,7 @@
         <v>20</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11144,7 +11144,7 @@
         <v>5</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11263,7 +11263,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>37.7</v>
+        <v>37.04</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -11287,7 +11287,7 @@
         <v>11.8</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>37.08</v>
+        <v>36.43</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11311,7 +11311,7 @@
         <v>15</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>47.13</v>
+        <v>46.3</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11335,7 +11335,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>31.42</v>
+        <v>30.87</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11359,7 +11359,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11383,7 +11383,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11407,7 +11407,7 @@
         <v>5</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -11550,7 +11550,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>47.13</v>
+        <v>46.3</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11574,7 +11574,7 @@
         <v>9.720000000000001</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>30.54</v>
+        <v>30.01</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11598,7 +11598,7 @@
         <v>30</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>94.26000000000001</v>
+        <v>92.61</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11622,7 +11622,7 @@
         <v>33</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>103.69</v>
+        <v>101.87</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11646,7 +11646,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11670,7 +11670,7 @@
         <v>36</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>113.11</v>
+        <v>111.13</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -11694,7 +11694,7 @@
         <v>5</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -11837,7 +11837,7 @@
         <v>139.92</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>439.63</v>
+        <v>431.93</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11861,7 +11861,7 @@
         <v>15</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>47.13</v>
+        <v>46.3</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11885,7 +11885,7 @@
         <v>19.43</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>61.05</v>
+        <v>59.98</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11909,7 +11909,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11933,7 +11933,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11981,7 +11981,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>62.84</v>
+        <v>61.74</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -12005,7 +12005,7 @@
         <v>39</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>122.54</v>
+        <v>120.39</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -12029,7 +12029,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>78.55</v>
+        <v>77.18000000000001</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -12053,7 +12053,7 @@
         <v>43</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>135.11</v>
+        <v>132.74</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -12077,7 +12077,7 @@
         <v>5</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.71</v>
+        <v>15.44</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -12101,7 +12101,7 @@
         <v>14.5</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>45.56</v>
+        <v>44.76</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>

</xml_diff>

<commit_message>
Fix Windows manual import bridge and add Dzine receipt
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1783,7 +1783,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1940,65 +1940,65 @@
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>2.25</v>
+        <v>18</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>6.95</v>
+        <v>55.57</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20</v>
+        <v>2.25</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.74</v>
+        <v>6.95</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D10" s="25" t="n">
@@ -2009,28 +2009,52 @@
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>61.74</v>
+      </c>
+      <c r="F11" s="29" t="n"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B11" s="31" t="n"/>
-      <c r="C11" s="31" t="n"/>
-      <c r="D11" s="20">
-        <f>SUM(D4:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="21">
-        <f>SUM(E4:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="31" t="n"/>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="31" t="n"/>
+      <c r="D12" s="20">
+        <f>SUM(D4:D11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="21">
+        <f>SUM(E4:E11)</f>
+        <v/>
+      </c>
+      <c r="F12" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A12:C12"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A11:C11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -2879,7 +2903,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F99"/>
+  <dimension ref="A1:F100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5312,24 +5336,24 @@
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B88" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>2.25</v>
+        <v>18</v>
       </c>
       <c r="E88" s="17" t="n">
-        <v>6.95</v>
+        <v>55.57</v>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
@@ -5340,24 +5364,24 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>20</v>
+        <v>2.25</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>61.74</v>
+        <v>6.95</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5368,17 +5392,17 @@
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D90" s="16" t="n">
@@ -5396,7 +5420,7 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
@@ -5417,14 +5441,14 @@
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B92" s="15" t="inlineStr">
@@ -5445,14 +5469,14 @@
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
@@ -5473,14 +5497,14 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
@@ -5501,14 +5525,14 @@
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
@@ -5529,14 +5553,14 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
@@ -5557,14 +5581,14 @@
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5585,14 +5609,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5613,31 +5637,59 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B99" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C99" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D99" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E99" s="13" t="n">
+        <v>61.74</v>
+      </c>
+      <c r="F99" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" s="18" t="inlineStr">
+    <row r="100">
+      <c r="A100" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B99" s="19" t="n"/>
-      <c r="C99" s="19" t="n"/>
-      <c r="D99" s="20">
-        <f>SUM(D3:D98)</f>
-        <v/>
-      </c>
-      <c r="E99" s="21">
-        <f>SUM(E3:E98)</f>
-        <v/>
-      </c>
-      <c r="F99" s="19" t="n"/>
+      <c r="B100" s="19" t="n"/>
+      <c r="C100" s="19" t="n"/>
+      <c r="D100" s="20">
+        <f>SUM(D3:D99)</f>
+        <v/>
+      </c>
+      <c r="E100" s="21">
+        <f>SUM(E3:E99)</f>
+        <v/>
+      </c>
+      <c r="F100" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A99:C99"/>
+    <mergeCell ref="A100:C100"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5770,7 +5822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM25"/>
+  <dimension ref="A1:AM26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -6626,151 +6678,151 @@
     <row r="8">
       <c r="A8" s="41" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="B8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ8" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK8" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Dzine",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL8" s="39">
@@ -6785,151 +6837,151 @@
     <row r="9">
       <c r="A9" s="36" t="inlineStr">
         <is>
-          <t>Genspark</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="B9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ9" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK9" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Eleven Labs",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL9" s="39">
@@ -6944,151 +6996,151 @@
     <row r="10">
       <c r="A10" s="41" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Genspark</t>
         </is>
       </c>
       <c r="B10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ10" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK10" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Genspark",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL10" s="39">
@@ -7103,151 +7155,151 @@
     <row r="11">
       <c r="A11" s="36" t="inlineStr">
         <is>
-          <t>Hedra</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="B11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL11" s="39">
@@ -7262,151 +7314,151 @@
     <row r="12">
       <c r="A12" s="41" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>Hedra</t>
         </is>
       </c>
       <c r="B12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL12" s="39">
@@ -7421,151 +7473,151 @@
     <row r="13">
       <c r="A13" s="36" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="B13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL13" s="39">
@@ -7580,151 +7632,151 @@
     <row r="14">
       <c r="A14" s="41" t="inlineStr">
         <is>
-          <t>Ideogram AI</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="B14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL14" s="39">
@@ -7739,151 +7791,151 @@
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Ideogram AI</t>
         </is>
       </c>
       <c r="B15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL15" s="39">
@@ -7898,151 +7950,151 @@
     <row r="16">
       <c r="A16" s="41" t="inlineStr">
         <is>
-          <t>Make</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="B16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL16" s="39">
@@ -8057,151 +8109,151 @@
     <row r="17">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>Manus AI</t>
+          <t>Make</t>
         </is>
       </c>
       <c r="B17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL17" s="39">
@@ -8216,151 +8268,151 @@
     <row r="18">
       <c r="A18" s="41" t="inlineStr">
         <is>
-          <t>Manychat</t>
+          <t>Manus AI</t>
         </is>
       </c>
       <c r="B18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL18" s="39">
@@ -8375,151 +8427,151 @@
     <row r="19">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Manychat</t>
         </is>
       </c>
       <c r="B19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL19" s="39">
@@ -8534,151 +8586,151 @@
     <row r="20">
       <c r="A20" s="41" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="B20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL20" s="39">
@@ -8693,151 +8745,151 @@
     <row r="21">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t>Recraft</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="B21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL21" s="39">
@@ -8852,151 +8904,151 @@
     <row r="22">
       <c r="A22" s="41" t="inlineStr">
         <is>
-          <t>Replicate</t>
+          <t>Recraft</t>
         </is>
       </c>
       <c r="B22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL22" s="39">
@@ -9011,151 +9063,151 @@
     <row r="23">
       <c r="A23" s="36" t="inlineStr">
         <is>
-          <t>Runway ML</t>
+          <t>Replicate</t>
         </is>
       </c>
       <c r="B23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL23" s="39">
@@ -9170,151 +9222,151 @@
     <row r="24">
       <c r="A24" s="41" t="inlineStr">
         <is>
-          <t>Timeless</t>
+          <t>Runway ML</t>
         </is>
       </c>
       <c r="B24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL24" s="39">
@@ -9326,162 +9378,321 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="24" customHeight="1">
-      <c r="A25" s="30" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="36" t="inlineStr">
+        <is>
+          <t>Timeless</t>
+        </is>
+      </c>
+      <c r="B25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <v/>
+      </c>
+      <c r="C25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <v/>
+      </c>
+      <c r="D25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <v/>
+      </c>
+      <c r="E25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <v/>
+      </c>
+      <c r="F25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="G25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="H25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <v/>
+      </c>
+      <c r="I25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <v/>
+      </c>
+      <c r="J25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="K25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="L25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="M25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="N25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <v/>
+      </c>
+      <c r="O25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <v/>
+      </c>
+      <c r="P25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <v/>
+      </c>
+      <c r="Q25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <v/>
+      </c>
+      <c r="R25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <v/>
+      </c>
+      <c r="S25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <v/>
+      </c>
+      <c r="T25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <v/>
+      </c>
+      <c r="U25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <v/>
+      </c>
+      <c r="V25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <v/>
+      </c>
+      <c r="W25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <v/>
+      </c>
+      <c r="X25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <v/>
+      </c>
+      <c r="Y25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <v/>
+      </c>
+      <c r="Z25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <v/>
+      </c>
+      <c r="AA25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <v/>
+      </c>
+      <c r="AB25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <v/>
+      </c>
+      <c r="AC25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <v/>
+      </c>
+      <c r="AD25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AE25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AF25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <v/>
+      </c>
+      <c r="AG25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <v/>
+      </c>
+      <c r="AH25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AI25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AJ25" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AK25" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AL25" s="39">
+        <f>SUM(B25,D25,F25,H25,J25,L25,N25,P25,R25,T25,V25,X25,Z25,AB25,AD25,AF25,AH25,AJ25)</f>
+        <v/>
+      </c>
+      <c r="AM25" s="40">
+        <f>SUM(C25,E25,G25,I25,K25,M25,O25,Q25,S25,U25,W25,Y25,AA25,AC25,AE25,AG25,AI25,AK25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="24" customHeight="1">
+      <c r="A26" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודשי</t>
         </is>
       </c>
-      <c r="B25" s="20">
-        <f>SUM(B5:B24)</f>
-        <v/>
-      </c>
-      <c r="C25" s="21">
-        <f>SUM(C5:C24)</f>
-        <v/>
-      </c>
-      <c r="D25" s="20">
-        <f>SUM(D5:D24)</f>
-        <v/>
-      </c>
-      <c r="E25" s="21">
-        <f>SUM(E5:E24)</f>
-        <v/>
-      </c>
-      <c r="F25" s="20">
-        <f>SUM(F5:F24)</f>
-        <v/>
-      </c>
-      <c r="G25" s="21">
-        <f>SUM(G5:G24)</f>
-        <v/>
-      </c>
-      <c r="H25" s="20">
-        <f>SUM(H5:H24)</f>
-        <v/>
-      </c>
-      <c r="I25" s="21">
-        <f>SUM(I5:I24)</f>
-        <v/>
-      </c>
-      <c r="J25" s="20">
-        <f>SUM(J5:J24)</f>
-        <v/>
-      </c>
-      <c r="K25" s="21">
-        <f>SUM(K5:K24)</f>
-        <v/>
-      </c>
-      <c r="L25" s="20">
-        <f>SUM(L5:L24)</f>
-        <v/>
-      </c>
-      <c r="M25" s="21">
-        <f>SUM(M5:M24)</f>
-        <v/>
-      </c>
-      <c r="N25" s="20">
-        <f>SUM(N5:N24)</f>
-        <v/>
-      </c>
-      <c r="O25" s="21">
-        <f>SUM(O5:O24)</f>
-        <v/>
-      </c>
-      <c r="P25" s="20">
-        <f>SUM(P5:P24)</f>
-        <v/>
-      </c>
-      <c r="Q25" s="21">
-        <f>SUM(Q5:Q24)</f>
-        <v/>
-      </c>
-      <c r="R25" s="20">
-        <f>SUM(R5:R24)</f>
-        <v/>
-      </c>
-      <c r="S25" s="21">
-        <f>SUM(S5:S24)</f>
-        <v/>
-      </c>
-      <c r="T25" s="20">
-        <f>SUM(T5:T24)</f>
-        <v/>
-      </c>
-      <c r="U25" s="21">
-        <f>SUM(U5:U24)</f>
-        <v/>
-      </c>
-      <c r="V25" s="20">
-        <f>SUM(V5:V24)</f>
-        <v/>
-      </c>
-      <c r="W25" s="21">
-        <f>SUM(W5:W24)</f>
-        <v/>
-      </c>
-      <c r="X25" s="20">
-        <f>SUM(X5:X24)</f>
-        <v/>
-      </c>
-      <c r="Y25" s="21">
-        <f>SUM(Y5:Y24)</f>
-        <v/>
-      </c>
-      <c r="Z25" s="20">
-        <f>SUM(Z5:Z24)</f>
-        <v/>
-      </c>
-      <c r="AA25" s="21">
-        <f>SUM(AA5:AA24)</f>
-        <v/>
-      </c>
-      <c r="AB25" s="20">
-        <f>SUM(AB5:AB24)</f>
-        <v/>
-      </c>
-      <c r="AC25" s="21">
-        <f>SUM(AC5:AC24)</f>
-        <v/>
-      </c>
-      <c r="AD25" s="20">
-        <f>SUM(AD5:AD24)</f>
-        <v/>
-      </c>
-      <c r="AE25" s="21">
-        <f>SUM(AE5:AE24)</f>
-        <v/>
-      </c>
-      <c r="AF25" s="20">
-        <f>SUM(AF5:AF24)</f>
-        <v/>
-      </c>
-      <c r="AG25" s="21">
-        <f>SUM(AG5:AG24)</f>
-        <v/>
-      </c>
-      <c r="AH25" s="20">
-        <f>SUM(AH5:AH24)</f>
-        <v/>
-      </c>
-      <c r="AI25" s="21">
-        <f>SUM(AI5:AI24)</f>
-        <v/>
-      </c>
-      <c r="AJ25" s="20">
-        <f>SUM(AJ5:AJ24)</f>
-        <v/>
-      </c>
-      <c r="AK25" s="21">
-        <f>SUM(AK5:AK24)</f>
-        <v/>
-      </c>
-      <c r="AL25" s="44">
-        <f>SUM(AL5:AL24)</f>
-        <v/>
-      </c>
-      <c r="AM25" s="45">
-        <f>SUM(AM5:AM24)</f>
+      <c r="B26" s="20">
+        <f>SUM(B5:B25)</f>
+        <v/>
+      </c>
+      <c r="C26" s="21">
+        <f>SUM(C5:C25)</f>
+        <v/>
+      </c>
+      <c r="D26" s="20">
+        <f>SUM(D5:D25)</f>
+        <v/>
+      </c>
+      <c r="E26" s="21">
+        <f>SUM(E5:E25)</f>
+        <v/>
+      </c>
+      <c r="F26" s="20">
+        <f>SUM(F5:F25)</f>
+        <v/>
+      </c>
+      <c r="G26" s="21">
+        <f>SUM(G5:G25)</f>
+        <v/>
+      </c>
+      <c r="H26" s="20">
+        <f>SUM(H5:H25)</f>
+        <v/>
+      </c>
+      <c r="I26" s="21">
+        <f>SUM(I5:I25)</f>
+        <v/>
+      </c>
+      <c r="J26" s="20">
+        <f>SUM(J5:J25)</f>
+        <v/>
+      </c>
+      <c r="K26" s="21">
+        <f>SUM(K5:K25)</f>
+        <v/>
+      </c>
+      <c r="L26" s="20">
+        <f>SUM(L5:L25)</f>
+        <v/>
+      </c>
+      <c r="M26" s="21">
+        <f>SUM(M5:M25)</f>
+        <v/>
+      </c>
+      <c r="N26" s="20">
+        <f>SUM(N5:N25)</f>
+        <v/>
+      </c>
+      <c r="O26" s="21">
+        <f>SUM(O5:O25)</f>
+        <v/>
+      </c>
+      <c r="P26" s="20">
+        <f>SUM(P5:P25)</f>
+        <v/>
+      </c>
+      <c r="Q26" s="21">
+        <f>SUM(Q5:Q25)</f>
+        <v/>
+      </c>
+      <c r="R26" s="20">
+        <f>SUM(R5:R25)</f>
+        <v/>
+      </c>
+      <c r="S26" s="21">
+        <f>SUM(S5:S25)</f>
+        <v/>
+      </c>
+      <c r="T26" s="20">
+        <f>SUM(T5:T25)</f>
+        <v/>
+      </c>
+      <c r="U26" s="21">
+        <f>SUM(U5:U25)</f>
+        <v/>
+      </c>
+      <c r="V26" s="20">
+        <f>SUM(V5:V25)</f>
+        <v/>
+      </c>
+      <c r="W26" s="21">
+        <f>SUM(W5:W25)</f>
+        <v/>
+      </c>
+      <c r="X26" s="20">
+        <f>SUM(X5:X25)</f>
+        <v/>
+      </c>
+      <c r="Y26" s="21">
+        <f>SUM(Y5:Y25)</f>
+        <v/>
+      </c>
+      <c r="Z26" s="20">
+        <f>SUM(Z5:Z25)</f>
+        <v/>
+      </c>
+      <c r="AA26" s="21">
+        <f>SUM(AA5:AA25)</f>
+        <v/>
+      </c>
+      <c r="AB26" s="20">
+        <f>SUM(AB5:AB25)</f>
+        <v/>
+      </c>
+      <c r="AC26" s="21">
+        <f>SUM(AC5:AC25)</f>
+        <v/>
+      </c>
+      <c r="AD26" s="20">
+        <f>SUM(AD5:AD25)</f>
+        <v/>
+      </c>
+      <c r="AE26" s="21">
+        <f>SUM(AE5:AE25)</f>
+        <v/>
+      </c>
+      <c r="AF26" s="20">
+        <f>SUM(AF5:AF25)</f>
+        <v/>
+      </c>
+      <c r="AG26" s="21">
+        <f>SUM(AG5:AG25)</f>
+        <v/>
+      </c>
+      <c r="AH26" s="20">
+        <f>SUM(AH5:AH25)</f>
+        <v/>
+      </c>
+      <c r="AI26" s="21">
+        <f>SUM(AI5:AI25)</f>
+        <v/>
+      </c>
+      <c r="AJ26" s="20">
+        <f>SUM(AJ5:AJ25)</f>
+        <v/>
+      </c>
+      <c r="AK26" s="21">
+        <f>SUM(AK5:AK25)</f>
+        <v/>
+      </c>
+      <c r="AL26" s="44">
+        <f>SUM(AL5:AL25)</f>
+        <v/>
+      </c>
+      <c r="AM26" s="45">
+        <f>SUM(AM5:AM25)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Manual import: add receipt for Dzine 2026-03-26
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1400,7 +1400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1746,28 +1746,52 @@
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>2026-03-26</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Dzine</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Video Top-Up</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>20</v>
+      </c>
+      <c r="E16" s="26" t="n">
+        <v>61.74</v>
+      </c>
+      <c r="F16" s="24" t="n"/>
+    </row>
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B16" s="31" t="n"/>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="20">
-        <f>SUM(D4:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="21">
-        <f>SUM(E4:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="31" t="n"/>
+      <c r="B17" s="31" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="20">
+        <f>SUM(D4:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="21">
+        <f>SUM(E4:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -2903,7 +2927,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F100"/>
+  <dimension ref="A1:F101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5224,17 +5248,17 @@
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
@@ -5245,7 +5269,7 @@
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מרץ 2026</t>
         </is>
       </c>
     </row>
@@ -5262,14 +5286,14 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>15.44</v>
+        <v>61.74</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5285,19 +5309,19 @@
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>Business Plus – Mar 2026 (₪75.90)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>20.79</v>
+        <v>5</v>
       </c>
       <c r="E86" s="17" t="n">
-        <v>75.90000000000001</v>
+        <v>15.44</v>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
@@ -5313,19 +5337,19 @@
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Business Plus – Mar 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>51</v>
+        <v>20.79</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>157.44</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
@@ -5336,24 +5360,24 @@
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B88" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="E88" s="17" t="n">
-        <v>55.57</v>
+        <v>157.44</v>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
@@ -5364,24 +5388,24 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>2.25</v>
+        <v>18</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>6.95</v>
+        <v>55.57</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5392,24 +5416,24 @@
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>20</v>
+        <v>2.25</v>
       </c>
       <c r="E90" s="17" t="n">
-        <v>61.74</v>
+        <v>6.95</v>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
@@ -5420,17 +5444,17 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D91" s="12" t="n">
@@ -5448,7 +5472,7 @@
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B92" s="15" t="inlineStr">
@@ -5469,14 +5493,14 @@
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
@@ -5497,14 +5521,14 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
@@ -5525,14 +5549,14 @@
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
@@ -5553,14 +5577,14 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
@@ -5581,14 +5605,14 @@
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5609,14 +5633,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5637,14 +5661,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5665,32 +5689,60 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B100" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C100" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D100" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E100" s="17" t="n">
+        <v>61.74</v>
+      </c>
+      <c r="F100" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" s="18" t="inlineStr">
+    <row r="101">
+      <c r="A101" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B100" s="19" t="n"/>
-      <c r="C100" s="19" t="n"/>
-      <c r="D100" s="20">
-        <f>SUM(D3:D99)</f>
-        <v/>
-      </c>
-      <c r="E100" s="21">
-        <f>SUM(E3:E99)</f>
-        <v/>
-      </c>
-      <c r="F100" s="19" t="n"/>
+      <c r="B101" s="19" t="n"/>
+      <c r="C101" s="19" t="n"/>
+      <c r="D101" s="20">
+        <f>SUM(D3:D100)</f>
+        <v/>
+      </c>
+      <c r="E101" s="21">
+        <f>SUM(E3:E100)</f>
+        <v/>
+      </c>
+      <c r="F101" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A100:C100"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A101:C101"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Manual import: add receipt for Dzine 2026-03-24
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1400,7 +1400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1725,72 +1725,96 @@
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.44</v>
+        <v>27.78</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Lovable</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Lite plan</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="26" t="n">
+        <v>15.44</v>
+      </c>
+      <c r="F16" s="24" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="B16" s="15" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Dzine</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>Video Top-Up</t>
         </is>
       </c>
-      <c r="D16" s="25" t="n">
+      <c r="D17" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E16" s="26" t="n">
+      <c r="E17" s="28" t="n">
         <v>61.74</v>
       </c>
-      <c r="F16" s="24" t="n"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="F17" s="29" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="31" t="n"/>
-      <c r="D17" s="20">
-        <f>SUM(D4:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="21">
-        <f>SUM(E4:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="31" t="n"/>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="20">
+        <f>SUM(D4:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="21">
+        <f>SUM(E4:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -2927,7 +2951,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:F102"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5220,24 +5244,24 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>15.44</v>
+        <v>27.78</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5248,24 +5272,24 @@
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Lite plan</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>61.74</v>
+        <v>15.44</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5276,17 +5300,17 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
@@ -5297,7 +5321,7 @@
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מרץ 2026</t>
         </is>
       </c>
     </row>
@@ -5314,14 +5338,14 @@
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E86" s="17" t="n">
-        <v>15.44</v>
+        <v>61.74</v>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
@@ -5337,19 +5361,19 @@
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Business Plus – Mar 2026 (₪75.90)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>20.79</v>
+        <v>5</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>15.44</v>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
@@ -5365,19 +5389,19 @@
       </c>
       <c r="B88" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Business Plus – Mar 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>51</v>
+        <v>20.79</v>
       </c>
       <c r="E88" s="17" t="n">
-        <v>157.44</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
@@ -5388,24 +5412,24 @@
     <row r="89">
       <c r="A89" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>55.57</v>
+        <v>157.44</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5416,24 +5440,24 @@
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>2.25</v>
+        <v>18</v>
       </c>
       <c r="E90" s="17" t="n">
-        <v>6.95</v>
+        <v>55.57</v>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
@@ -5444,24 +5468,24 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D91" s="12" t="n">
-        <v>20</v>
+        <v>2.25</v>
       </c>
       <c r="E91" s="13" t="n">
-        <v>61.74</v>
+        <v>6.95</v>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
@@ -5472,17 +5496,17 @@
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B92" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C92" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D92" s="16" t="n">
@@ -5500,7 +5524,7 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
@@ -5521,14 +5545,14 @@
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
@@ -5549,14 +5573,14 @@
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
@@ -5577,14 +5601,14 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
@@ -5605,14 +5629,14 @@
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5633,14 +5657,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5661,14 +5685,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5689,14 +5713,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5717,32 +5741,60 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C101" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D101" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E101" s="13" t="n">
+        <v>61.74</v>
+      </c>
+      <c r="F101" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" s="18" t="inlineStr">
+    <row r="102">
+      <c r="A102" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B101" s="19" t="n"/>
-      <c r="C101" s="19" t="n"/>
-      <c r="D101" s="20">
-        <f>SUM(D3:D100)</f>
-        <v/>
-      </c>
-      <c r="E101" s="21">
-        <f>SUM(E3:E100)</f>
-        <v/>
-      </c>
-      <c r="F101" s="19" t="n"/>
+      <c r="B102" s="19" t="n"/>
+      <c r="C102" s="19" t="n"/>
+      <c r="D102" s="20">
+        <f>SUM(D3:D101)</f>
+        <v/>
+      </c>
+      <c r="E102" s="21">
+        <f>SUM(E3:E101)</f>
+        <v/>
+      </c>
+      <c r="F102" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A101:C101"/>
+    <mergeCell ref="A102:C102"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Manual import: add receipt for CapCut 2026-04-10
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -939,11 +939,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3.087</v>
+        <v>3.057</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-09</t>
+          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1071,7 +1071,7 @@
         <v>25</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>77.18000000000001</v>
+        <v>76.42</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1119,7 +1119,7 @@
         <v>31.42</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>96.98999999999999</v>
+        <v>96.05</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -1167,7 +1167,7 @@
         <v>47</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>145.09</v>
+        <v>143.68</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -1191,7 +1191,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -1215,7 +1215,7 @@
         <v>5</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -1239,7 +1239,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -1263,7 +1263,7 @@
         <v>20</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -1287,7 +1287,7 @@
         <v>50</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>154.35</v>
+        <v>152.85</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -1311,7 +1311,7 @@
         <v>51</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>157.44</v>
+        <v>155.91</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -1335,7 +1335,7 @@
         <v>5</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -1359,7 +1359,7 @@
         <v>10</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
@@ -1478,7 +1478,7 @@
         <v>10</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1502,7 +1502,7 @@
         <v>14.5</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>44.76</v>
+        <v>44.33</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -1550,7 +1550,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -1574,7 +1574,7 @@
         <v>40.11</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>123.82</v>
+        <v>122.62</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -1622,7 +1622,7 @@
         <v>51</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>157.44</v>
+        <v>155.91</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -1646,7 +1646,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -1670,7 +1670,7 @@
         <v>20</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -1694,7 +1694,7 @@
         <v>10</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -1718,7 +1718,7 @@
         <v>11</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>33.96</v>
+        <v>33.63</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -1742,7 +1742,7 @@
         <v>9</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>27.78</v>
+        <v>27.51</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -1766,7 +1766,7 @@
         <v>5</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
@@ -1790,7 +1790,7 @@
         <v>20</v>
       </c>
       <c r="E17" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F17" s="29" t="n"/>
     </row>
@@ -1831,7 +1831,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F12"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1909,7 +1909,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1933,7 +1933,7 @@
         <v>5</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -1981,7 +1981,7 @@
         <v>51</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>157.44</v>
+        <v>155.91</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -2005,7 +2005,7 @@
         <v>18</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>55.57</v>
+        <v>55.03</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -2029,7 +2029,7 @@
         <v>2.25</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>6.95</v>
+        <v>6.88</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -2053,55 +2053,79 @@
         <v>20</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
+          <t>2026-04-10</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>CapCut</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>capcut_pro_discount1</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>16.323193</v>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="F11" s="29" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
           <t>2026-04-16</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D11" s="27" t="n">
+      <c r="D12" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E11" s="28" t="n">
-        <v>61.74</v>
-      </c>
-      <c r="F11" s="29" t="n"/>
-    </row>
-    <row r="12" ht="24" customHeight="1">
-      <c r="A12" s="30" t="inlineStr">
+      <c r="E12" s="26" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="F12" s="24" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B12" s="31" t="n"/>
-      <c r="C12" s="31" t="n"/>
-      <c r="D12" s="20">
-        <f>SUM(D4:D11)</f>
-        <v/>
-      </c>
-      <c r="E12" s="21">
-        <f>SUM(E4:E11)</f>
-        <v/>
-      </c>
-      <c r="F12" s="31" t="n"/>
+      <c r="B13" s="31" t="n"/>
+      <c r="C13" s="31" t="n"/>
+      <c r="D13" s="20">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="21">
+        <f>SUM(E4:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -2196,7 +2220,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2315,7 +2339,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2434,7 +2458,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2553,7 +2577,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2672,7 +2696,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2791,7 +2815,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2910,7 +2934,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2951,7 +2975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3021,7 +3045,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>3.09</v>
+        <v>3.06</v>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
@@ -3049,7 +3073,7 @@
         <v>72</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>222.26</v>
+        <v>220.1</v>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
@@ -3077,7 +3101,7 @@
         <v>10.59</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>32.69</v>
+        <v>32.37</v>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -3105,7 +3129,7 @@
         <v>20</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
@@ -3133,7 +3157,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
@@ -3161,7 +3185,7 @@
         <v>13.5</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>41.67</v>
+        <v>41.27</v>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
@@ -3189,7 +3213,7 @@
         <v>113.14</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>349.26</v>
+        <v>345.87</v>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
@@ -3217,7 +3241,7 @@
         <v>10</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
@@ -3273,7 +3297,7 @@
         <v>15</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>46.3</v>
+        <v>45.85</v>
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
@@ -3301,7 +3325,7 @@
         <v>12</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>37.04</v>
+        <v>36.68</v>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
@@ -3329,7 +3353,7 @@
         <v>0.9</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>2.78</v>
+        <v>2.75</v>
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
@@ -3357,7 +3381,7 @@
         <v>19</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>58.65</v>
+        <v>58.08</v>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
@@ -3385,7 +3409,7 @@
         <v>10.59</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>32.69</v>
+        <v>32.37</v>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
@@ -3413,7 +3437,7 @@
         <v>20</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
@@ -3441,7 +3465,7 @@
         <v>20</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
@@ -3469,7 +3493,7 @@
         <v>5</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
@@ -3497,7 +3521,7 @@
         <v>11.25</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>34.73</v>
+        <v>34.39</v>
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
@@ -3553,7 +3577,7 @@
         <v>2.79</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>8.609999999999999</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
@@ -3581,7 +3605,7 @@
         <v>10.59</v>
       </c>
       <c r="E23" s="13" t="n">
-        <v>32.69</v>
+        <v>32.37</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
@@ -3609,7 +3633,7 @@
         <v>20</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
@@ -3637,7 +3661,7 @@
         <v>20</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
@@ -3665,7 +3689,7 @@
         <v>5</v>
       </c>
       <c r="E26" s="17" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
@@ -3721,7 +3745,7 @@
         <v>20</v>
       </c>
       <c r="E28" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
@@ -3749,7 +3773,7 @@
         <v>20</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
@@ -3777,7 +3801,7 @@
         <v>5</v>
       </c>
       <c r="E30" s="17" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
@@ -3805,7 +3829,7 @@
         <v>12</v>
       </c>
       <c r="E31" s="13" t="n">
-        <v>37.04</v>
+        <v>36.68</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -3833,7 +3857,7 @@
         <v>11.8</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>36.43</v>
+        <v>36.07</v>
       </c>
       <c r="F32" s="14" t="inlineStr">
         <is>
@@ -3861,7 +3885,7 @@
         <v>15</v>
       </c>
       <c r="E33" s="13" t="n">
-        <v>46.3</v>
+        <v>45.85</v>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
@@ -3889,7 +3913,7 @@
         <v>10</v>
       </c>
       <c r="E34" s="17" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
@@ -3917,7 +3941,7 @@
         <v>20</v>
       </c>
       <c r="E35" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
@@ -3945,7 +3969,7 @@
         <v>20</v>
       </c>
       <c r="E36" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F36" s="14" t="inlineStr">
         <is>
@@ -3973,7 +3997,7 @@
         <v>5</v>
       </c>
       <c r="E37" s="13" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
@@ -4029,7 +4053,7 @@
         <v>15</v>
       </c>
       <c r="E39" s="13" t="n">
-        <v>46.3</v>
+        <v>45.85</v>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
@@ -4057,7 +4081,7 @@
         <v>9.720000000000001</v>
       </c>
       <c r="E40" s="17" t="n">
-        <v>30.01</v>
+        <v>29.71</v>
       </c>
       <c r="F40" s="14" t="inlineStr">
         <is>
@@ -4085,7 +4109,7 @@
         <v>30</v>
       </c>
       <c r="E41" s="13" t="n">
-        <v>92.61</v>
+        <v>91.70999999999999</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
@@ -4113,7 +4137,7 @@
         <v>33</v>
       </c>
       <c r="E42" s="17" t="n">
-        <v>101.87</v>
+        <v>100.88</v>
       </c>
       <c r="F42" s="14" t="inlineStr">
         <is>
@@ -4141,7 +4165,7 @@
         <v>20</v>
       </c>
       <c r="E43" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
@@ -4169,7 +4193,7 @@
         <v>36</v>
       </c>
       <c r="E44" s="17" t="n">
-        <v>111.13</v>
+        <v>110.05</v>
       </c>
       <c r="F44" s="14" t="inlineStr">
         <is>
@@ -4197,7 +4221,7 @@
         <v>5</v>
       </c>
       <c r="E45" s="13" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
@@ -4253,7 +4277,7 @@
         <v>139.92</v>
       </c>
       <c r="E47" s="13" t="n">
-        <v>431.93</v>
+        <v>427.74</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
@@ -4281,7 +4305,7 @@
         <v>15</v>
       </c>
       <c r="E48" s="17" t="n">
-        <v>46.3</v>
+        <v>45.85</v>
       </c>
       <c r="F48" s="14" t="inlineStr">
         <is>
@@ -4309,7 +4333,7 @@
         <v>19.43</v>
       </c>
       <c r="E49" s="13" t="n">
-        <v>59.98</v>
+        <v>59.4</v>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
@@ -4337,7 +4361,7 @@
         <v>20</v>
       </c>
       <c r="E50" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F50" s="14" t="inlineStr">
         <is>
@@ -4365,7 +4389,7 @@
         <v>20</v>
       </c>
       <c r="E51" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
@@ -4421,7 +4445,7 @@
         <v>20</v>
       </c>
       <c r="E53" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
@@ -4449,7 +4473,7 @@
         <v>39</v>
       </c>
       <c r="E54" s="17" t="n">
-        <v>120.39</v>
+        <v>119.22</v>
       </c>
       <c r="F54" s="14" t="inlineStr">
         <is>
@@ -4477,7 +4501,7 @@
         <v>25</v>
       </c>
       <c r="E55" s="13" t="n">
-        <v>77.18000000000001</v>
+        <v>76.42</v>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
@@ -4505,7 +4529,7 @@
         <v>43</v>
       </c>
       <c r="E56" s="17" t="n">
-        <v>132.74</v>
+        <v>131.45</v>
       </c>
       <c r="F56" s="14" t="inlineStr">
         <is>
@@ -4533,7 +4557,7 @@
         <v>5</v>
       </c>
       <c r="E57" s="13" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
@@ -4561,7 +4585,7 @@
         <v>14.5</v>
       </c>
       <c r="E58" s="17" t="n">
-        <v>44.76</v>
+        <v>44.33</v>
       </c>
       <c r="F58" s="14" t="inlineStr">
         <is>
@@ -4589,7 +4613,7 @@
         <v>25</v>
       </c>
       <c r="E59" s="13" t="n">
-        <v>77.18000000000001</v>
+        <v>76.42</v>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
@@ -4645,7 +4669,7 @@
         <v>31.42</v>
       </c>
       <c r="E61" s="13" t="n">
-        <v>96.98999999999999</v>
+        <v>96.05</v>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
@@ -4701,7 +4725,7 @@
         <v>47</v>
       </c>
       <c r="E63" s="13" t="n">
-        <v>145.09</v>
+        <v>143.68</v>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
@@ -4729,7 +4753,7 @@
         <v>20</v>
       </c>
       <c r="E64" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
@@ -4757,7 +4781,7 @@
         <v>5</v>
       </c>
       <c r="E65" s="13" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
@@ -4785,7 +4809,7 @@
         <v>20</v>
       </c>
       <c r="E66" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
@@ -4813,7 +4837,7 @@
         <v>20</v>
       </c>
       <c r="E67" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
@@ -4841,7 +4865,7 @@
         <v>50</v>
       </c>
       <c r="E68" s="17" t="n">
-        <v>154.35</v>
+        <v>152.85</v>
       </c>
       <c r="F68" s="14" t="inlineStr">
         <is>
@@ -4869,7 +4893,7 @@
         <v>51</v>
       </c>
       <c r="E69" s="13" t="n">
-        <v>157.44</v>
+        <v>155.91</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
@@ -4897,7 +4921,7 @@
         <v>5</v>
       </c>
       <c r="E70" s="17" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F70" s="14" t="inlineStr">
         <is>
@@ -4925,7 +4949,7 @@
         <v>10</v>
       </c>
       <c r="E71" s="13" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -4953,7 +4977,7 @@
         <v>10</v>
       </c>
       <c r="E72" s="17" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F72" s="14" t="inlineStr">
         <is>
@@ -4981,7 +5005,7 @@
         <v>14.5</v>
       </c>
       <c r="E73" s="13" t="n">
-        <v>44.76</v>
+        <v>44.33</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -5037,7 +5061,7 @@
         <v>10</v>
       </c>
       <c r="E75" s="13" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -5065,7 +5089,7 @@
         <v>40.11</v>
       </c>
       <c r="E76" s="17" t="n">
-        <v>123.82</v>
+        <v>122.62</v>
       </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
@@ -5121,7 +5145,7 @@
         <v>51</v>
       </c>
       <c r="E78" s="17" t="n">
-        <v>157.44</v>
+        <v>155.91</v>
       </c>
       <c r="F78" s="14" t="inlineStr">
         <is>
@@ -5149,7 +5173,7 @@
         <v>20</v>
       </c>
       <c r="E79" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -5177,7 +5201,7 @@
         <v>20</v>
       </c>
       <c r="E80" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F80" s="14" t="inlineStr">
         <is>
@@ -5205,7 +5229,7 @@
         <v>10</v>
       </c>
       <c r="E81" s="13" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -5233,7 +5257,7 @@
         <v>11</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>33.96</v>
+        <v>33.63</v>
       </c>
       <c r="F82" s="14" t="inlineStr">
         <is>
@@ -5261,7 +5285,7 @@
         <v>9</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>27.78</v>
+        <v>27.51</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5289,7 +5313,7 @@
         <v>5</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5317,7 +5341,7 @@
         <v>20</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5345,7 +5369,7 @@
         <v>20</v>
       </c>
       <c r="E86" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
@@ -5373,7 +5397,7 @@
         <v>5</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
@@ -5429,7 +5453,7 @@
         <v>51</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>157.44</v>
+        <v>155.91</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5457,7 +5481,7 @@
         <v>18</v>
       </c>
       <c r="E90" s="17" t="n">
-        <v>55.57</v>
+        <v>55.03</v>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
@@ -5485,7 +5509,7 @@
         <v>2.25</v>
       </c>
       <c r="E91" s="13" t="n">
-        <v>6.95</v>
+        <v>6.88</v>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
@@ -5513,7 +5537,7 @@
         <v>20</v>
       </c>
       <c r="E92" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
@@ -5524,24 +5548,24 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>20</v>
+        <v>16.323193</v>
       </c>
       <c r="E93" s="13" t="n">
-        <v>61.74</v>
+        <v>49.9</v>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
@@ -5552,7 +5576,7 @@
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
@@ -5569,18 +5593,18 @@
         <v>20</v>
       </c>
       <c r="E94" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
@@ -5597,18 +5621,18 @@
         <v>20</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
@@ -5625,18 +5649,18 @@
         <v>20</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5653,18 +5677,18 @@
         <v>20</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5681,18 +5705,18 @@
         <v>20</v>
       </c>
       <c r="E98" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5709,18 +5733,18 @@
         <v>20</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5737,18 +5761,18 @@
         <v>20</v>
       </c>
       <c r="E100" s="17" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5765,36 +5789,64 @@
         <v>20</v>
       </c>
       <c r="E101" s="13" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B102" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C102" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D102" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E102" s="17" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="F102" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="18" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B102" s="19" t="n"/>
-      <c r="C102" s="19" t="n"/>
-      <c r="D102" s="20">
-        <f>SUM(D3:D101)</f>
-        <v/>
-      </c>
-      <c r="E102" s="21">
-        <f>SUM(E3:E101)</f>
-        <v/>
-      </c>
-      <c r="F102" s="19" t="n"/>
+      <c r="B103" s="19" t="n"/>
+      <c r="C103" s="19" t="n"/>
+      <c r="D103" s="20">
+        <f>SUM(D3:D102)</f>
+        <v/>
+      </c>
+      <c r="E103" s="21">
+        <f>SUM(E3:E102)</f>
+        <v/>
+      </c>
+      <c r="F103" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A103:C103"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A102:C102"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5885,7 +5937,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -10526,7 +10578,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>3.09</v>
+        <v>3.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -10550,7 +10602,7 @@
         <v>72</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>222.26</v>
+        <v>220.1</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -10574,7 +10626,7 @@
         <v>10.59</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>32.69</v>
+        <v>32.37</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -10598,7 +10650,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -10622,7 +10674,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -10646,7 +10698,7 @@
         <v>13.5</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>41.67</v>
+        <v>41.27</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -10670,7 +10722,7 @@
         <v>113.14</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>349.26</v>
+        <v>345.87</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -10694,7 +10746,7 @@
         <v>10</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -10837,7 +10889,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>46.3</v>
+        <v>45.85</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -10861,7 +10913,7 @@
         <v>12</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>37.04</v>
+        <v>36.68</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -10885,7 +10937,7 @@
         <v>0.9</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>2.78</v>
+        <v>2.75</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -10909,7 +10961,7 @@
         <v>19</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>58.65</v>
+        <v>58.08</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -10933,7 +10985,7 @@
         <v>10.59</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>32.69</v>
+        <v>32.37</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -10957,7 +11009,7 @@
         <v>20</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -10981,7 +11033,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -11005,7 +11057,7 @@
         <v>5</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -11029,7 +11081,7 @@
         <v>11.25</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>34.73</v>
+        <v>34.39</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -11172,7 +11224,7 @@
         <v>2.79</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>8.609999999999999</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11196,7 +11248,7 @@
         <v>10.59</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>32.69</v>
+        <v>32.37</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11220,7 +11272,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11244,7 +11296,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11268,7 +11320,7 @@
         <v>5</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11411,7 +11463,7 @@
         <v>20</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11435,7 +11487,7 @@
         <v>20</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11459,7 +11511,7 @@
         <v>5</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11578,7 +11630,7 @@
         <v>12</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>37.04</v>
+        <v>36.68</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -11602,7 +11654,7 @@
         <v>11.8</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>36.43</v>
+        <v>36.07</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11626,7 +11678,7 @@
         <v>15</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>46.3</v>
+        <v>45.85</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11650,7 +11702,7 @@
         <v>10</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>30.87</v>
+        <v>30.57</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11674,7 +11726,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11698,7 +11750,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11722,7 +11774,7 @@
         <v>5</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -11865,7 +11917,7 @@
         <v>15</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>46.3</v>
+        <v>45.85</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11889,7 +11941,7 @@
         <v>9.720000000000001</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>30.01</v>
+        <v>29.71</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11913,7 +11965,7 @@
         <v>30</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>92.61</v>
+        <v>91.70999999999999</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11937,7 +11989,7 @@
         <v>33</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>101.87</v>
+        <v>100.88</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11961,7 +12013,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11985,7 +12037,7 @@
         <v>36</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>111.13</v>
+        <v>110.05</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -12009,7 +12061,7 @@
         <v>5</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -12152,7 +12204,7 @@
         <v>139.92</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>431.93</v>
+        <v>427.74</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -12176,7 +12228,7 @@
         <v>15</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>46.3</v>
+        <v>45.85</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -12200,7 +12252,7 @@
         <v>19.43</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>59.98</v>
+        <v>59.4</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -12224,7 +12276,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -12248,7 +12300,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -12296,7 +12348,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.74</v>
+        <v>61.14</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -12320,7 +12372,7 @@
         <v>39</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>120.39</v>
+        <v>119.22</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -12344,7 +12396,7 @@
         <v>25</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>77.18000000000001</v>
+        <v>76.42</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -12368,7 +12420,7 @@
         <v>43</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>132.74</v>
+        <v>131.45</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -12392,7 +12444,7 @@
         <v>5</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.44</v>
+        <v>15.29</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -12416,7 +12468,7 @@
         <v>14.5</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>44.76</v>
+        <v>44.33</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>

</xml_diff>

<commit_message>
Manual import: add receipt for CapCut 2026-03-10
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1400,7 +1400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1605,65 +1605,65 @@
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>51</v>
+        <v>16.323193</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>155.91</v>
+        <v>49.9</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.14</v>
+        <v>155.91</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
@@ -1677,24 +1677,24 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>30.57</v>
+        <v>61.14</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -1706,115 +1706,139 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Creator (first month 50% off)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>33.63</v>
+        <v>30.57</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Creator (first month 50% off)</t>
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>27.51</v>
+        <v>33.63</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>15.29</v>
+        <v>27.51</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Lovable</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Lite plan</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E17" s="28" t="n">
+        <v>15.29</v>
+      </c>
+      <c r="F17" s="29" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="B17" s="11" t="inlineStr">
+      <c r="B18" s="15" t="inlineStr">
         <is>
           <t>Dzine</t>
         </is>
       </c>
-      <c r="C17" s="11" t="inlineStr">
+      <c r="C18" s="15" t="inlineStr">
         <is>
           <t>Video Top-Up</t>
         </is>
       </c>
-      <c r="D17" s="27" t="n">
+      <c r="D18" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E17" s="28" t="n">
+      <c r="E18" s="26" t="n">
         <v>61.14</v>
       </c>
-      <c r="F17" s="29" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="30" t="inlineStr">
+      <c r="F18" s="24" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B18" s="31" t="n"/>
-      <c r="C18" s="31" t="n"/>
-      <c r="D18" s="20">
-        <f>SUM(D4:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="21">
-        <f>SUM(E4:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="31" t="n"/>
+      <c r="B19" s="31" t="n"/>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="20">
+        <f>SUM(D4:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="21">
+        <f>SUM(E4:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -2975,7 +2999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F103"/>
+  <dimension ref="A1:F104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5128,24 +5152,24 @@
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>51</v>
+        <v>16.323193</v>
       </c>
       <c r="E78" s="17" t="n">
-        <v>155.91</v>
+        <v>49.9</v>
       </c>
       <c r="F78" s="14" t="inlineStr">
         <is>
@@ -5156,24 +5180,24 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="E79" s="13" t="n">
-        <v>61.14</v>
+        <v>155.91</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -5184,17 +5208,17 @@
     <row r="80">
       <c r="A80" s="14" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B80" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D80" s="16" t="n">
@@ -5212,24 +5236,24 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D81" s="12" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E81" s="13" t="n">
-        <v>30.57</v>
+        <v>61.14</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -5245,19 +5269,19 @@
       </c>
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>Creator (first month 50% off)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>33.63</v>
+        <v>30.57</v>
       </c>
       <c r="F82" s="14" t="inlineStr">
         <is>
@@ -5268,24 +5292,24 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Creator (first month 50% off)</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>27.51</v>
+        <v>33.63</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5296,24 +5320,24 @@
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>15.29</v>
+        <v>27.51</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5324,24 +5348,24 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Lite plan</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5352,17 +5376,17 @@
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D86" s="16" t="n">
@@ -5373,7 +5397,7 @@
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מרץ 2026</t>
         </is>
       </c>
     </row>
@@ -5390,14 +5414,14 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
@@ -5413,19 +5437,19 @@
       </c>
       <c r="B88" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Business Plus – Mar 2026 (₪75.90)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>20.79</v>
+        <v>5</v>
       </c>
       <c r="E88" s="17" t="n">
-        <v>75.90000000000001</v>
+        <v>15.29</v>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
@@ -5441,19 +5465,19 @@
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Business Plus – Mar 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>51</v>
+        <v>20.79</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>155.91</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5464,24 +5488,24 @@
     <row r="90">
       <c r="A90" s="14" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="E90" s="17" t="n">
-        <v>55.03</v>
+        <v>155.91</v>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
@@ -5492,24 +5516,24 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D91" s="12" t="n">
-        <v>2.25</v>
+        <v>18</v>
       </c>
       <c r="E91" s="13" t="n">
-        <v>6.88</v>
+        <v>55.03</v>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
@@ -5520,24 +5544,24 @@
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B92" s="15" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C92" s="15" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>20</v>
+        <v>2.25</v>
       </c>
       <c r="E92" s="17" t="n">
-        <v>61.14</v>
+        <v>6.88</v>
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
@@ -5548,24 +5572,24 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E93" s="13" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
@@ -5576,24 +5600,24 @@
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C94" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>20</v>
+        <v>16.323193</v>
       </c>
       <c r="E94" s="17" t="n">
-        <v>61.14</v>
+        <v>49.9</v>
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
@@ -5604,7 +5628,7 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
@@ -5625,14 +5649,14 @@
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
@@ -5653,14 +5677,14 @@
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5681,14 +5705,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5709,14 +5733,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5737,14 +5761,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5765,14 +5789,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5793,14 +5817,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5821,32 +5845,60 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C103" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D103" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E103" s="13" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="F103" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="18" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B103" s="19" t="n"/>
-      <c r="C103" s="19" t="n"/>
-      <c r="D103" s="20">
-        <f>SUM(D3:D102)</f>
-        <v/>
-      </c>
-      <c r="E103" s="21">
-        <f>SUM(E3:E102)</f>
-        <v/>
-      </c>
-      <c r="F103" s="19" t="n"/>
+      <c r="B104" s="19" t="n"/>
+      <c r="C104" s="19" t="n"/>
+      <c r="D104" s="20">
+        <f>SUM(D3:D103)</f>
+        <v/>
+      </c>
+      <c r="E104" s="21">
+        <f>SUM(E3:E103)</f>
+        <v/>
+      </c>
+      <c r="F104" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A103:C103"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A104:C104"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Manual import: add receipt for CapCut 2026-02-10
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -993,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1150,55 +1150,55 @@
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>47</v>
+        <v>16.323193</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>143.68</v>
+        <v>49.9</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.14</v>
+        <v>143.68</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -1208,14 +1208,14 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -1227,36 +1227,36 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>On-Demand credits 500</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
@@ -1270,24 +1270,24 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Pro2 monthly</t>
+          <t>On-Demand credits 500</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>152.85</v>
+        <v>61.14</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -1299,43 +1299,43 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro2 monthly</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>155.91</v>
+        <v>152.85</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.29</v>
+        <v>155.91</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -1347,43 +1347,67 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
+          <t>Eleven Labs</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Starter monthly</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="26" t="n">
+        <v>15.29</v>
+      </c>
+      <c r="F16" s="24" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>2026-02-28</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
           <t>Lovable</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
-      <c r="D16" s="25" t="n">
+      <c r="D17" s="27" t="n">
         <v>10</v>
       </c>
-      <c r="E16" s="26" t="n">
+      <c r="E17" s="28" t="n">
         <v>30.57</v>
       </c>
-      <c r="F16" s="24" t="n"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="F17" s="29" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="31" t="n"/>
-      <c r="D17" s="20">
-        <f>SUM(D4:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="21">
-        <f>SUM(E4:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="31" t="n"/>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="20">
+        <f>SUM(D4:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="21">
+        <f>SUM(E4:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -2999,7 +3023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4732,24 +4756,24 @@
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>47</v>
+        <v>16.323193</v>
       </c>
       <c r="E63" s="13" t="n">
-        <v>143.68</v>
+        <v>49.9</v>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
@@ -4760,24 +4784,24 @@
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D64" s="16" t="n">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="E64" s="17" t="n">
-        <v>61.14</v>
+        <v>143.68</v>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
@@ -4788,7 +4812,7 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
@@ -4798,14 +4822,14 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E65" s="13" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
@@ -4821,19 +4845,19 @@
       </c>
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D66" s="16" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E66" s="17" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
@@ -4844,17 +4868,17 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>On-Demand credits 500</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D67" s="12" t="n">
@@ -4872,24 +4896,24 @@
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B68" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>Pro2 monthly</t>
+          <t>On-Demand credits 500</t>
         </is>
       </c>
       <c r="D68" s="16" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E68" s="17" t="n">
-        <v>152.85</v>
+        <v>61.14</v>
       </c>
       <c r="F68" s="14" t="inlineStr">
         <is>
@@ -4905,19 +4929,19 @@
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro2 monthly</t>
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E69" s="13" t="n">
-        <v>155.91</v>
+        <v>152.85</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
@@ -4928,24 +4952,24 @@
     <row r="70">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B70" s="15" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="E70" s="17" t="n">
-        <v>15.29</v>
+        <v>155.91</v>
       </c>
       <c r="F70" s="14" t="inlineStr">
         <is>
@@ -4961,19 +4985,19 @@
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D71" s="12" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E71" s="13" t="n">
-        <v>30.57</v>
+        <v>15.29</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -4984,7 +5008,7 @@
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B72" s="15" t="inlineStr">
@@ -5005,7 +5029,7 @@
       </c>
       <c r="F72" s="14" t="inlineStr">
         <is>
-          <t>מרץ 2026</t>
+          <t>פברואר 2026</t>
         </is>
       </c>
     </row>
@@ -5017,19 +5041,19 @@
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>Timeless</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Pro monthly (50% off)</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D73" s="12" t="n">
-        <v>14.5</v>
+        <v>10</v>
       </c>
       <c r="E73" s="13" t="n">
-        <v>44.33</v>
+        <v>30.57</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -5040,24 +5064,24 @@
     <row r="74">
       <c r="A74" s="14" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B74" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Timeless</t>
         </is>
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>Business Plus – Feb 2026 (₪75.90)</t>
+          <t>Pro monthly (50% off)</t>
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>20.79</v>
+        <v>14.5</v>
       </c>
       <c r="E74" s="17" t="n">
-        <v>75.90000000000001</v>
+        <v>44.33</v>
       </c>
       <c r="F74" s="14" t="inlineStr">
         <is>
@@ -5073,19 +5097,19 @@
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Business Plus – Feb 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>10</v>
+        <v>20.79</v>
       </c>
       <c r="E75" s="13" t="n">
-        <v>30.57</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -5096,24 +5120,24 @@
     <row r="76">
       <c r="A76" s="14" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B76" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>40.11</v>
+        <v>10</v>
       </c>
       <c r="E76" s="17" t="n">
-        <v>122.62</v>
+        <v>30.57</v>
       </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
@@ -5124,24 +5148,24 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Pro – Mar 2026 (₪49.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>13.67</v>
+        <v>40.11</v>
       </c>
       <c r="E77" s="13" t="n">
-        <v>49.9</v>
+        <v>122.62</v>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
@@ -5162,11 +5186,11 @@
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Pro – Mar 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>16.323193</v>
+        <v>13.67</v>
       </c>
       <c r="E78" s="17" t="n">
         <v>49.9</v>
@@ -5180,24 +5204,24 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>51</v>
+        <v>16.323193</v>
       </c>
       <c r="E79" s="13" t="n">
-        <v>155.91</v>
+        <v>49.9</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -5208,24 +5232,24 @@
     <row r="80">
       <c r="A80" s="14" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B80" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="E80" s="17" t="n">
-        <v>61.14</v>
+        <v>155.91</v>
       </c>
       <c r="F80" s="14" t="inlineStr">
         <is>
@@ -5236,17 +5260,17 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D81" s="12" t="n">
@@ -5264,24 +5288,24 @@
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>30.57</v>
+        <v>61.14</v>
       </c>
       <c r="F82" s="14" t="inlineStr">
         <is>
@@ -5297,19 +5321,19 @@
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Creator (first month 50% off)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>33.63</v>
+        <v>30.57</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5320,24 +5344,24 @@
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Creator (first month 50% off)</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>27.51</v>
+        <v>33.63</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5348,24 +5372,24 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>15.29</v>
+        <v>27.51</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5376,24 +5400,24 @@
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Lite plan</t>
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E86" s="17" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
@@ -5404,17 +5428,17 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
@@ -5425,7 +5449,7 @@
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מרץ 2026</t>
         </is>
       </c>
     </row>
@@ -5442,14 +5466,14 @@
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E88" s="17" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
@@ -5465,19 +5489,19 @@
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Business Plus – Mar 2026 (₪75.90)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>20.79</v>
+        <v>5</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>15.29</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5493,19 +5517,19 @@
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Business Plus – Mar 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>51</v>
+        <v>20.79</v>
       </c>
       <c r="E90" s="17" t="n">
-        <v>155.91</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
@@ -5516,24 +5540,24 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D91" s="12" t="n">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="E91" s="13" t="n">
-        <v>55.03</v>
+        <v>155.91</v>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
@@ -5544,24 +5568,24 @@
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B92" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C92" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>2.25</v>
+        <v>18</v>
       </c>
       <c r="E92" s="17" t="n">
-        <v>6.88</v>
+        <v>55.03</v>
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
@@ -5572,24 +5596,24 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>20</v>
+        <v>2.25</v>
       </c>
       <c r="E93" s="13" t="n">
-        <v>61.14</v>
+        <v>6.88</v>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
@@ -5600,24 +5624,24 @@
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C94" s="15" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E94" s="17" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
@@ -5628,24 +5652,24 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
-        <v>20</v>
+        <v>16.323193</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>61.14</v>
+        <v>49.9</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
@@ -5656,7 +5680,7 @@
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
@@ -5677,14 +5701,14 @@
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5705,14 +5729,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5733,14 +5757,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5761,14 +5785,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5789,14 +5813,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5817,14 +5841,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5845,14 +5869,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5873,32 +5897,60 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C104" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D104" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E104" s="17" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="F104" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="18" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B104" s="19" t="n"/>
-      <c r="C104" s="19" t="n"/>
-      <c r="D104" s="20">
-        <f>SUM(D3:D103)</f>
-        <v/>
-      </c>
-      <c r="E104" s="21">
-        <f>SUM(E3:E103)</f>
-        <v/>
-      </c>
-      <c r="F104" s="19" t="n"/>
+      <c r="B105" s="19" t="n"/>
+      <c r="C105" s="19" t="n"/>
+      <c r="D105" s="20">
+        <f>SUM(D3:D104)</f>
+        <v/>
+      </c>
+      <c r="E105" s="21">
+        <f>SUM(E3:E104)</f>
+        <v/>
+      </c>
+      <c r="F105" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A104:C104"/>
+    <mergeCell ref="A105:C105"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Manual import: add receipt for CapCut 2026-01-10
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -3023,7 +3023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4476,24 +4476,24 @@
     <row r="53">
       <c r="A53" s="10" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B53" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D53" s="12" t="n">
-        <v>20</v>
+        <v>16.323193</v>
       </c>
       <c r="E53" s="13" t="n">
-        <v>61.14</v>
+        <v>49.9</v>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
@@ -4504,24 +4504,24 @@
     <row r="54">
       <c r="A54" s="14" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B54" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D54" s="16" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E54" s="17" t="n">
-        <v>119.22</v>
+        <v>61.14</v>
       </c>
       <c r="F54" s="14" t="inlineStr">
         <is>
@@ -4532,24 +4532,24 @@
     <row r="55">
       <c r="A55" s="10" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B55" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Pro 1 monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D55" s="12" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="E55" s="13" t="n">
-        <v>76.42</v>
+        <v>119.22</v>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
@@ -4560,24 +4560,24 @@
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro 1 monthly</t>
         </is>
       </c>
       <c r="D56" s="16" t="n">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="E56" s="17" t="n">
-        <v>131.45</v>
+        <v>76.42</v>
       </c>
       <c r="F56" s="14" t="inlineStr">
         <is>
@@ -4588,24 +4588,24 @@
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D57" s="12" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E57" s="13" t="n">
-        <v>15.29</v>
+        <v>131.45</v>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
@@ -4621,19 +4621,19 @@
       </c>
       <c r="B58" s="15" t="inlineStr">
         <is>
-          <t>Timeless</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Pro monthly (50% off)</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D58" s="16" t="n">
-        <v>14.5</v>
+        <v>5</v>
       </c>
       <c r="E58" s="17" t="n">
-        <v>44.33</v>
+        <v>15.29</v>
       </c>
       <c r="F58" s="14" t="inlineStr">
         <is>
@@ -4644,52 +4644,52 @@
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>2026-02-01</t>
+          <t>2026-01-30</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Timeless</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Upgrade Pro1 -&gt; Pro2 (prorated)</t>
+          <t>Pro monthly (50% off)</t>
         </is>
       </c>
       <c r="D59" s="12" t="n">
-        <v>25</v>
+        <v>14.5</v>
       </c>
       <c r="E59" s="13" t="n">
-        <v>76.42</v>
+        <v>44.33</v>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
-          <t>פברואר 2026</t>
+          <t>ינואר 2026</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-01</t>
         </is>
       </c>
       <c r="B60" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Business Plus – Jan 2026 (₪75.90)</t>
+          <t>Upgrade Pro1 -&gt; Pro2 (prorated)</t>
         </is>
       </c>
       <c r="D60" s="16" t="n">
-        <v>20.79</v>
+        <v>25</v>
       </c>
       <c r="E60" s="17" t="n">
-        <v>75.90000000000001</v>
+        <v>76.42</v>
       </c>
       <c r="F60" s="14" t="inlineStr">
         <is>
@@ -4700,24 +4700,24 @@
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-02</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Business Plus – Jan 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D61" s="12" t="n">
-        <v>31.42</v>
+        <v>20.79</v>
       </c>
       <c r="E61" s="13" t="n">
-        <v>96.05</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
@@ -4728,24 +4728,24 @@
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Pro – Feb 2026 (₪49.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D62" s="16" t="n">
-        <v>13.67</v>
+        <v>31.42</v>
       </c>
       <c r="E62" s="17" t="n">
-        <v>49.9</v>
+        <v>96.05</v>
       </c>
       <c r="F62" s="14" t="inlineStr">
         <is>
@@ -4766,11 +4766,11 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Pro – Feb 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>16.323193</v>
+        <v>13.67</v>
       </c>
       <c r="E63" s="13" t="n">
         <v>49.9</v>
@@ -4784,24 +4784,24 @@
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D64" s="16" t="n">
-        <v>47</v>
+        <v>16.323193</v>
       </c>
       <c r="E64" s="17" t="n">
-        <v>143.68</v>
+        <v>49.9</v>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
@@ -4812,24 +4812,24 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>20</v>
+        <v>47</v>
       </c>
       <c r="E65" s="13" t="n">
-        <v>61.14</v>
+        <v>143.68</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
@@ -4840,7 +4840,7 @@
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B66" s="15" t="inlineStr">
@@ -4850,14 +4850,14 @@
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D66" s="16" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E66" s="17" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
@@ -4873,19 +4873,19 @@
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D67" s="12" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E67" s="13" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
@@ -4896,17 +4896,17 @@
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B68" s="15" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>On-Demand credits 500</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D68" s="16" t="n">
@@ -4924,24 +4924,24 @@
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Pro2 monthly</t>
+          <t>On-Demand credits 500</t>
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="E69" s="13" t="n">
-        <v>152.85</v>
+        <v>61.14</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
@@ -4957,19 +4957,19 @@
       </c>
       <c r="B70" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro2 monthly</t>
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="E70" s="17" t="n">
-        <v>155.91</v>
+        <v>152.85</v>
       </c>
       <c r="F70" s="14" t="inlineStr">
         <is>
@@ -4980,24 +4980,24 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D71" s="12" t="n">
-        <v>5</v>
+        <v>51</v>
       </c>
       <c r="E71" s="13" t="n">
-        <v>15.29</v>
+        <v>155.91</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -5013,19 +5013,19 @@
       </c>
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D72" s="16" t="n">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E72" s="17" t="n">
-        <v>30.57</v>
+        <v>15.29</v>
       </c>
       <c r="F72" s="14" t="inlineStr">
         <is>
@@ -5036,7 +5036,7 @@
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
@@ -5057,7 +5057,7 @@
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
-          <t>מרץ 2026</t>
+          <t>פברואר 2026</t>
         </is>
       </c>
     </row>
@@ -5069,19 +5069,19 @@
       </c>
       <c r="B74" s="15" t="inlineStr">
         <is>
-          <t>Timeless</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>Pro monthly (50% off)</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>14.5</v>
+        <v>10</v>
       </c>
       <c r="E74" s="17" t="n">
-        <v>44.33</v>
+        <v>30.57</v>
       </c>
       <c r="F74" s="14" t="inlineStr">
         <is>
@@ -5092,24 +5092,24 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Timeless</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Business Plus – Feb 2026 (₪75.90)</t>
+          <t>Pro monthly (50% off)</t>
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>20.79</v>
+        <v>14.5</v>
       </c>
       <c r="E75" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>44.33</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -5125,19 +5125,19 @@
       </c>
       <c r="B76" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Business Plus – Feb 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>10</v>
+        <v>20.79</v>
       </c>
       <c r="E76" s="17" t="n">
-        <v>30.57</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
@@ -5148,24 +5148,24 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>40.11</v>
+        <v>10</v>
       </c>
       <c r="E77" s="13" t="n">
-        <v>122.62</v>
+        <v>30.57</v>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
@@ -5176,24 +5176,24 @@
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Pro – Mar 2026 (₪49.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>13.67</v>
+        <v>40.11</v>
       </c>
       <c r="E78" s="17" t="n">
-        <v>49.9</v>
+        <v>122.62</v>
       </c>
       <c r="F78" s="14" t="inlineStr">
         <is>
@@ -5214,11 +5214,11 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Pro – Mar 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>16.323193</v>
+        <v>13.67</v>
       </c>
       <c r="E79" s="13" t="n">
         <v>49.9</v>
@@ -5232,24 +5232,24 @@
     <row r="80">
       <c r="A80" s="14" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B80" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>51</v>
+        <v>16.323193</v>
       </c>
       <c r="E80" s="17" t="n">
-        <v>155.91</v>
+        <v>49.9</v>
       </c>
       <c r="F80" s="14" t="inlineStr">
         <is>
@@ -5260,24 +5260,24 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D81" s="12" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="E81" s="13" t="n">
-        <v>61.14</v>
+        <v>155.91</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -5288,17 +5288,17 @@
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D82" s="16" t="n">
@@ -5316,24 +5316,24 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>30.57</v>
+        <v>61.14</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5349,19 +5349,19 @@
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Creator (first month 50% off)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>33.63</v>
+        <v>30.57</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5372,24 +5372,24 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Creator (first month 50% off)</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>27.51</v>
+        <v>33.63</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5400,24 +5400,24 @@
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E86" s="17" t="n">
-        <v>15.29</v>
+        <v>27.51</v>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
@@ -5428,24 +5428,24 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Lite plan</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
@@ -5456,17 +5456,17 @@
     <row r="88">
       <c r="A88" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B88" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
@@ -5477,7 +5477,7 @@
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מרץ 2026</t>
         </is>
       </c>
     </row>
@@ -5494,14 +5494,14 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5517,19 +5517,19 @@
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Business Plus – Mar 2026 (₪75.90)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>20.79</v>
+        <v>5</v>
       </c>
       <c r="E90" s="17" t="n">
-        <v>75.90000000000001</v>
+        <v>15.29</v>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
@@ -5545,19 +5545,19 @@
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Business Plus – Mar 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D91" s="12" t="n">
-        <v>51</v>
+        <v>20.79</v>
       </c>
       <c r="E91" s="13" t="n">
-        <v>155.91</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
@@ -5568,24 +5568,24 @@
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B92" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C92" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="E92" s="17" t="n">
-        <v>55.03</v>
+        <v>155.91</v>
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
@@ -5596,24 +5596,24 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>2.25</v>
+        <v>18</v>
       </c>
       <c r="E93" s="13" t="n">
-        <v>6.88</v>
+        <v>55.03</v>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
@@ -5624,24 +5624,24 @@
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C94" s="15" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>20</v>
+        <v>2.25</v>
       </c>
       <c r="E94" s="17" t="n">
-        <v>61.14</v>
+        <v>6.88</v>
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
@@ -5652,24 +5652,24 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
@@ -5680,24 +5680,24 @@
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D96" s="16" t="n">
-        <v>20</v>
+        <v>16.323193</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>61.14</v>
+        <v>49.9</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -5708,7 +5708,7 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5729,14 +5729,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5757,14 +5757,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5785,14 +5785,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5813,14 +5813,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5841,14 +5841,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5869,14 +5869,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5897,14 +5897,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5925,32 +5925,60 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C105" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D105" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E105" s="13" t="n">
+        <v>61.14</v>
+      </c>
+      <c r="F105" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="18" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B105" s="19" t="n"/>
-      <c r="C105" s="19" t="n"/>
-      <c r="D105" s="20">
-        <f>SUM(D3:D104)</f>
-        <v/>
-      </c>
-      <c r="E105" s="21">
-        <f>SUM(E3:E104)</f>
-        <v/>
-      </c>
-      <c r="F105" s="19" t="n"/>
+      <c r="B106" s="19" t="n"/>
+      <c r="C106" s="19" t="n"/>
+      <c r="D106" s="20">
+        <f>SUM(D3:D105)</f>
+        <v/>
+      </c>
+      <c r="E106" s="21">
+        <f>SUM(E3:E105)</f>
+        <v/>
+      </c>
+      <c r="F106" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A106:C106"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A105:C105"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -12206,7 +12234,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -12435,120 +12463,120 @@
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>2026-01-16</t>
+          <t>2026-01-10</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>20</v>
+        <v>16.323193</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.14</v>
+        <v>49.9</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-01-19</t>
+          <t>2026-01-16</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>39</v>
+        <v>20</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>119.22</v>
+        <v>61.14</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-01-25</t>
+          <t>2026-01-19</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Pro 1 monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>76.42</v>
+        <v>119.22</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>2026-01-27</t>
+          <t>2026-01-25</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro 1 monthly</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>43</v>
+        <v>25</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>131.45</v>
+        <v>76.42</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>2026-01-30</t>
+          <t>2026-01-27</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.29</v>
+        <v>131.45</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -12560,43 +12588,67 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
+          <t>Eleven Labs</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Starter monthly</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E16" s="26" t="n">
+        <v>15.29</v>
+      </c>
+      <c r="F16" s="24" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
           <t>Timeless</t>
         </is>
       </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>Pro monthly (50% off)</t>
         </is>
       </c>
-      <c r="D16" s="25" t="n">
+      <c r="D17" s="27" t="n">
         <v>14.5</v>
       </c>
-      <c r="E16" s="26" t="n">
+      <c r="E17" s="28" t="n">
         <v>44.33</v>
       </c>
-      <c r="F16" s="24" t="n"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="30" t="inlineStr">
+      <c r="F17" s="29" t="n"/>
+    </row>
+    <row r="18" ht="24" customHeight="1">
+      <c r="A18" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="31" t="n"/>
-      <c r="D17" s="20">
-        <f>SUM(D4:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="21">
-        <f>SUM(E4:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="31" t="n"/>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="31" t="n"/>
+      <c r="D18" s="20">
+        <f>SUM(D4:D17)</f>
+        <v/>
+      </c>
+      <c r="E18" s="21">
+        <f>SUM(E4:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>

</xml_diff>

<commit_message>
Rebuild dashboard and Excel from manual imports
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1002,7 +1002,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1159,55 +1159,55 @@
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>16.323193</v>
+        <v>47</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>49.9</v>
+        <v>143.68</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>143.68</v>
+        <v>61.14</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -1217,62 +1217,62 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>On-Demand credits 500</t>
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>On-Demand credits 500</t>
+          <t>Pro2 monthly</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>61.14</v>
+        <v>152.85</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -1284,43 +1284,43 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Pro2 monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>152.85</v>
+        <v>155.91</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>155.91</v>
+        <v>15.29</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -1332,68 +1332,44 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.29</v>
+        <v>30.57</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
-    <row r="16">
-      <c r="A16" s="14" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="inlineStr">
-        <is>
-          <t>Lovable</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
-        <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
-        </is>
-      </c>
-      <c r="D16" s="25" t="n">
-        <v>10</v>
-      </c>
-      <c r="E16" s="26" t="n">
-        <v>30.57</v>
-      </c>
-      <c r="F16" s="24" t="n"/>
-    </row>
-    <row r="17" ht="24" customHeight="1">
-      <c r="A17" s="30" t="inlineStr">
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="31" t="n"/>
-      <c r="D17" s="20">
-        <f>SUM(D4:D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="21">
-        <f>SUM(E4:E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="31" t="n"/>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="20">
+        <f>SUM(D4:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="21">
+        <f>SUM(E4:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -2715,7 +2691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F87"/>
+  <dimension ref="A1:F86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4252,24 +4228,24 @@
     <row r="56">
       <c r="A56" s="14" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D56" s="16" t="n">
-        <v>16.323193</v>
+        <v>47</v>
       </c>
       <c r="E56" s="17" t="n">
-        <v>49.9</v>
+        <v>143.68</v>
       </c>
       <c r="F56" s="14" t="inlineStr">
         <is>
@@ -4280,24 +4256,24 @@
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B57" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D57" s="12" t="n">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="E57" s="13" t="n">
-        <v>143.68</v>
+        <v>61.14</v>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
@@ -4308,7 +4284,7 @@
     <row r="58">
       <c r="A58" s="14" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B58" s="15" t="inlineStr">
@@ -4318,14 +4294,14 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D58" s="16" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E58" s="17" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F58" s="14" t="inlineStr">
         <is>
@@ -4336,24 +4312,24 @@
     <row r="59">
       <c r="A59" s="10" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B59" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="C59" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>On-Demand credits 500</t>
         </is>
       </c>
       <c r="D59" s="12" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E59" s="13" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
@@ -4364,24 +4340,24 @@
     <row r="60">
       <c r="A60" s="14" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B60" s="15" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>On-Demand credits 500</t>
+          <t>Pro2 monthly</t>
         </is>
       </c>
       <c r="D60" s="16" t="n">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="E60" s="17" t="n">
-        <v>61.14</v>
+        <v>152.85</v>
       </c>
       <c r="F60" s="14" t="inlineStr">
         <is>
@@ -4397,19 +4373,19 @@
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Pro2 monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D61" s="12" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E61" s="13" t="n">
-        <v>152.85</v>
+        <v>155.91</v>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
@@ -4420,24 +4396,24 @@
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D62" s="16" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E62" s="17" t="n">
-        <v>155.91</v>
+        <v>15.29</v>
       </c>
       <c r="F62" s="14" t="inlineStr">
         <is>
@@ -4453,19 +4429,19 @@
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E63" s="13" t="n">
-        <v>15.29</v>
+        <v>30.57</v>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
@@ -4476,7 +4452,7 @@
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B64" s="15" t="inlineStr">
@@ -4497,7 +4473,7 @@
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
-          <t>פברואר 2026</t>
+          <t>מרץ 2026</t>
         </is>
       </c>
     </row>
@@ -4509,19 +4485,19 @@
       </c>
       <c r="B65" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Timeless</t>
         </is>
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Pro monthly (50% off)</t>
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>10</v>
+        <v>14.5</v>
       </c>
       <c r="E65" s="13" t="n">
-        <v>30.57</v>
+        <v>44.33</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
@@ -4532,24 +4508,24 @@
     <row r="66">
       <c r="A66" s="14" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>Timeless</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>Pro monthly (50% off)</t>
+          <t>Business Plus – Feb 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D66" s="16" t="n">
-        <v>14.5</v>
+        <v>20.79</v>
       </c>
       <c r="E66" s="17" t="n">
-        <v>44.33</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
@@ -4565,19 +4541,19 @@
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Business Plus – Feb 2026 (₪75.90)</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D67" s="12" t="n">
-        <v>20.79</v>
+        <v>10</v>
       </c>
       <c r="E67" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>30.57</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
@@ -4588,24 +4564,24 @@
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B68" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D68" s="16" t="n">
-        <v>10</v>
+        <v>40.11</v>
       </c>
       <c r="E68" s="17" t="n">
-        <v>30.57</v>
+        <v>122.62</v>
       </c>
       <c r="F68" s="14" t="inlineStr">
         <is>
@@ -4616,24 +4592,24 @@
     <row r="69">
       <c r="A69" s="10" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro – Mar 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>40.11</v>
+        <v>13.67</v>
       </c>
       <c r="E69" s="13" t="n">
-        <v>122.62</v>
+        <v>49.9</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
@@ -4654,11 +4630,11 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Pro – Mar 2026 (₪49.90)</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>13.67</v>
+        <v>16.323193</v>
       </c>
       <c r="E70" s="17" t="n">
         <v>49.9</v>
@@ -4672,24 +4648,24 @@
     <row r="71">
       <c r="A71" s="10" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D71" s="12" t="n">
-        <v>16.323193</v>
+        <v>51</v>
       </c>
       <c r="E71" s="13" t="n">
-        <v>49.9</v>
+        <v>155.91</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -4700,24 +4676,24 @@
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D72" s="16" t="n">
-        <v>51</v>
+        <v>20</v>
       </c>
       <c r="E72" s="17" t="n">
-        <v>155.91</v>
+        <v>61.14</v>
       </c>
       <c r="F72" s="14" t="inlineStr">
         <is>
@@ -4728,7 +4704,7 @@
     <row r="73">
       <c r="A73" s="10" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B73" s="11" t="inlineStr">
@@ -4738,14 +4714,14 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D73" s="12" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E73" s="13" t="n">
-        <v>61.14</v>
+        <v>30.57</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -4761,19 +4737,19 @@
       </c>
       <c r="B74" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Creator (first month 50% off)</t>
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E74" s="17" t="n">
-        <v>30.57</v>
+        <v>33.63</v>
       </c>
       <c r="F74" s="14" t="inlineStr">
         <is>
@@ -4784,24 +4760,24 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Creator (first month 50% off)</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E75" s="13" t="n">
-        <v>33.63</v>
+        <v>27.51</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -4812,24 +4788,24 @@
     <row r="76">
       <c r="A76" s="14" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B76" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Lite plan</t>
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="E76" s="17" t="n">
-        <v>27.51</v>
+        <v>15.29</v>
       </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
@@ -4840,24 +4816,24 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E77" s="13" t="n">
-        <v>15.29</v>
+        <v>61.14</v>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
@@ -4868,17 +4844,17 @@
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D78" s="16" t="n">
@@ -4889,7 +4865,7 @@
       </c>
       <c r="F78" s="14" t="inlineStr">
         <is>
-          <t>מרץ 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
@@ -4906,14 +4882,14 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E79" s="13" t="n">
-        <v>61.14</v>
+        <v>15.29</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -4929,19 +4905,19 @@
       </c>
       <c r="B80" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Business Plus – Mar 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>5</v>
+        <v>20.79</v>
       </c>
       <c r="E80" s="17" t="n">
-        <v>15.29</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F80" s="14" t="inlineStr">
         <is>
@@ -4957,19 +4933,19 @@
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Business Plus – Mar 2026 (₪75.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D81" s="12" t="n">
-        <v>20.79</v>
+        <v>51</v>
       </c>
       <c r="E81" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>155.91</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -4980,24 +4956,24 @@
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>51</v>
+        <v>18</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>155.91</v>
+        <v>55.03</v>
       </c>
       <c r="F82" s="14" t="inlineStr">
         <is>
@@ -5008,24 +4984,24 @@
     <row r="83">
       <c r="A83" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>18</v>
+        <v>2.25</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>55.03</v>
+        <v>6.88</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5036,24 +5012,24 @@
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>2.25</v>
+        <v>20</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>6.88</v>
+        <v>61.14</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5064,24 +5040,24 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>20</v>
+        <v>16.323193</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>61.14</v>
+        <v>49.9</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5090,55 +5066,27 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-10</t>
-        </is>
-      </c>
-      <c r="B86" s="15" t="inlineStr">
-        <is>
-          <t>CapCut</t>
-        </is>
-      </c>
-      <c r="C86" s="15" t="inlineStr">
-        <is>
-          <t>capcut_pro_discount1</t>
-        </is>
-      </c>
-      <c r="D86" s="16" t="n">
-        <v>16.323193</v>
-      </c>
-      <c r="E86" s="17" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="F86" s="14" t="inlineStr">
-        <is>
-          <t>אפריל 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="18" t="inlineStr">
+      <c r="A86" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B87" s="19" t="n"/>
-      <c r="C87" s="19" t="n"/>
-      <c r="D87" s="20">
-        <f>SUM(D3:D86)</f>
-        <v/>
-      </c>
-      <c r="E87" s="21">
-        <f>SUM(E3:E86)</f>
-        <v/>
-      </c>
-      <c r="F87" s="19" t="n"/>
+      <c r="B86" s="19" t="n"/>
+      <c r="C86" s="19" t="n"/>
+      <c r="D86" s="20">
+        <f>SUM(D3:D85)</f>
+        <v/>
+      </c>
+      <c r="E86" s="21">
+        <f>SUM(E3:E85)</f>
+        <v/>
+      </c>
+      <c r="F86" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A87:C87"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A86:C86"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: remove duplicate Meta $51 (Apr 7), fix Apr 1 to actual ILS 166.33
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2050,10 +2050,10 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>51</v>
+        <v>54.409552</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>155.91</v>
+        <v>166.33</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -2146,107 +2146,83 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>51</v>
+        <v>40.11</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>155.91</v>
+        <v>122.62</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>40.11</v>
+        <v>16.323193</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>122.62</v>
+        <v>49.9</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D15" s="27" t="n">
-        <v>20</v>
-      </c>
-      <c r="E15" s="28" t="n">
-        <v>61.14</v>
-      </c>
-      <c r="F15" s="29" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B16" s="31" t="n"/>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="20">
-        <f>SUM(D4:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="21">
-        <f>SUM(E4:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="31" t="n"/>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="20">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f>SUM(E4:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3095,7 +3071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5654,10 +5630,10 @@
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>51</v>
+        <v>54.409552</v>
       </c>
       <c r="E92" s="17" t="n">
-        <v>155.91</v>
+        <v>166.33</v>
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
@@ -5766,10 +5742,10 @@
         </is>
       </c>
       <c r="D96" s="16" t="n">
-        <v>51</v>
+        <v>40.11</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>155.91</v>
+        <v>122.62</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -5780,24 +5756,24 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D97" s="12" t="n">
-        <v>40.11</v>
+        <v>16.323193</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>122.62</v>
+        <v>49.9</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -5808,24 +5784,24 @@
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D98" s="16" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E98" s="17" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
@@ -5836,7 +5812,7 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5857,14 +5833,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5885,14 +5861,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5913,14 +5889,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5941,14 +5917,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5969,14 +5945,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5997,14 +5973,14 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -6025,14 +6001,14 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>נובמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-16</t>
         </is>
       </c>
       <c r="B106" s="15" t="inlineStr">
@@ -6053,60 +6029,32 @@
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="10" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="B107" s="11" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C107" s="11" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D107" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="E107" s="13" t="n">
-        <v>61.14</v>
-      </c>
-      <c r="F107" s="10" t="inlineStr">
-        <is>
-          <t>דצמבר 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="18" t="inlineStr">
+      <c r="A107" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B108" s="19" t="n"/>
-      <c r="C108" s="19" t="n"/>
-      <c r="D108" s="20">
-        <f>SUM(D3:D107)</f>
-        <v/>
-      </c>
-      <c r="E108" s="21">
-        <f>SUM(E3:E107)</f>
-        <v/>
-      </c>
-      <c r="F108" s="19" t="n"/>
+      <c r="B107" s="19" t="n"/>
+      <c r="C107" s="19" t="n"/>
+      <c r="D107" s="20">
+        <f>SUM(D3:D106)</f>
+        <v/>
+      </c>
+      <c r="E107" s="21">
+        <f>SUM(E3:E106)</f>
+        <v/>
+      </c>
+      <c r="F107" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A108:C108"/>
+    <mergeCell ref="A107:C107"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: remove erroneous Meta $40.11 Apr 7 — not in credit card
Both Apr 7 Meta entries added by Gmail scanner were wrong.
Removing the second one ($40.11) as confirmed not in credit card.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2132,96 +2132,72 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>40.11</v>
+        <v>16.323193</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>122.62</v>
+        <v>49.9</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
-    <row r="14">
-      <c r="A14" s="14" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D14" s="25" t="n">
-        <v>20</v>
-      </c>
-      <c r="E14" s="26" t="n">
-        <v>61.14</v>
-      </c>
-      <c r="F14" s="24" t="n"/>
-    </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="30" t="inlineStr">
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B15" s="31" t="n"/>
-      <c r="C15" s="31" t="n"/>
-      <c r="D15" s="20">
-        <f>SUM(D4:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="21">
-        <f>SUM(E4:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="31" t="n"/>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="20">
+        <f>SUM(D4:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="21">
+        <f>SUM(E4:E13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A14:C14"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3071,7 +3047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5728,24 +5704,24 @@
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-04-07</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D96" s="16" t="n">
-        <v>40.11</v>
+        <v>16.323193</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>122.62</v>
+        <v>49.9</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -5756,24 +5732,24 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D97" s="12" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -5784,7 +5760,7 @@
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5805,14 +5781,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5833,14 +5809,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5861,14 +5837,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5889,14 +5865,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5917,14 +5893,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5945,14 +5921,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5973,14 +5949,14 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>נובמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-16</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -6001,60 +5977,32 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="14" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="B106" s="15" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C106" s="15" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D106" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="E106" s="17" t="n">
-        <v>61.14</v>
-      </c>
-      <c r="F106" s="14" t="inlineStr">
-        <is>
-          <t>דצמבר 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="18" t="inlineStr">
+      <c r="A106" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B107" s="19" t="n"/>
-      <c r="C107" s="19" t="n"/>
-      <c r="D107" s="20">
-        <f>SUM(D3:D106)</f>
-        <v/>
-      </c>
-      <c r="E107" s="21">
-        <f>SUM(E3:E106)</f>
-        <v/>
-      </c>
-      <c r="F107" s="19" t="n"/>
+      <c r="B106" s="19" t="n"/>
+      <c r="C106" s="19" t="n"/>
+      <c r="D106" s="20">
+        <f>SUM(D3:D105)</f>
+        <v/>
+      </c>
+      <c r="E106" s="21">
+        <f>SUM(E3:E105)</f>
+        <v/>
+      </c>
+      <c r="F106" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A106:C106"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A107:C107"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: lock all USD charges to historical ILS rate at time of charge
All transactions now use the Bank of Israel rate from the exact date
of the charge — not today's rate. Past entries are immutable.

Changes:
- MANUAL_TRANSACTIONS: converted all USD tuples to ILS with historical rates
- Added HISTORICAL_RATES lookup table (BOI / fawazahmed0 API data)
- normalize_transaction: uses historical rate for past dates, current
  rate only for dates not yet in the table (future charges)
- Covers OpenAI recurring and Dzine manual receipts too

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -993,7 +993,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1068,10 +1068,10 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25</v>
+        <v>25.371279</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>76.42</v>
+        <v>77.56</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>20.79</v>
+        <v>24.828263</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1102,103 +1102,103 @@
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.9)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>24.828263</v>
+        <v>31.851488</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>75.90000000000001</v>
+        <v>97.37</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro – Feb 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>31.42</v>
+        <v>16.323193</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>96.05</v>
+        <v>49.9</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Pro – Feb 2026 (₪49.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>13.67</v>
+        <v>47.307818</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>49.9</v>
+        <v>144.62</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>47</v>
+        <v>20.193</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>143.68</v>
+        <v>61.73</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -1208,14 +1208,14 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>20</v>
+        <v>5.050703</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>61.14</v>
+        <v>15.44</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -1227,67 +1227,67 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>15.29</v>
+        <v>61.77</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>On-Demand credits 500</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20</v>
+        <v>20.464508</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>61.14</v>
+        <v>62.56</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>On-Demand credits 500</t>
+          <t>Pro2 monthly</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>20</v>
+        <v>50.690219</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>61.14</v>
+        <v>154.96</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -1299,43 +1299,43 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Pro2 monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>50</v>
+        <v>51.704285</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>152.85</v>
+        <v>158.06</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>51</v>
+        <v>5.129212</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>155.91</v>
+        <v>15.68</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -1347,67 +1347,43 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>5</v>
+        <v>10.255152</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>15.29</v>
+        <v>31.35</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="10" t="inlineStr">
-        <is>
-          <t>2026-02-28</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>Lovable</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
-        </is>
-      </c>
-      <c r="D17" s="27" t="n">
-        <v>10</v>
-      </c>
-      <c r="E17" s="28" t="n">
-        <v>30.57</v>
-      </c>
-      <c r="F17" s="29" t="n"/>
-    </row>
-    <row r="18" ht="24" customHeight="1">
-      <c r="A18" s="30" t="inlineStr">
+    <row r="17" ht="24" customHeight="1">
+      <c r="A17" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B18" s="31" t="n"/>
-      <c r="C18" s="31" t="n"/>
-      <c r="D18" s="20">
-        <f>SUM(D4:D17)</f>
-        <v/>
-      </c>
-      <c r="E18" s="21">
-        <f>SUM(E4:E17)</f>
-        <v/>
-      </c>
-      <c r="F18" s="31" t="n"/>
+      <c r="B17" s="31" t="n"/>
+      <c r="C17" s="31" t="n"/>
+      <c r="D17" s="20">
+        <f>SUM(D4:D16)</f>
+        <v/>
+      </c>
+      <c r="E17" s="21">
+        <f>SUM(E4:E16)</f>
+        <v/>
+      </c>
+      <c r="F17" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A17:C17"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -1523,10 +1499,10 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>10</v>
+        <v>10.232254</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>30.57</v>
+        <v>31.28</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -1547,10 +1523,10 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>14.5</v>
+        <v>14.838077</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>44.33</v>
+        <v>45.36</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -1571,7 +1547,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>20.79</v>
+        <v>24.828263</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1595,10 +1571,10 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>10</v>
+        <v>10.206084</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>30.57</v>
+        <v>31.2</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -1619,10 +1595,10 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>40.11</v>
+        <v>40.376186</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>122.62</v>
+        <v>123.43</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -1643,7 +1619,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>13.67</v>
+        <v>16.323193</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -1667,10 +1643,10 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>51</v>
+        <v>52.230945</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>155.91</v>
+        <v>159.67</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -1691,10 +1667,10 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20</v>
+        <v>20.565914</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>61.14</v>
+        <v>62.87</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -1718,7 +1694,7 @@
         <v>20</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>61.14</v>
+        <v>62.87</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -1739,10 +1715,10 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>10</v>
+        <v>10.176644</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>30.57</v>
+        <v>31.11</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -1763,10 +1739,10 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>11</v>
+        <v>11.193981</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>33.63</v>
+        <v>34.22</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -1790,7 +1766,7 @@
         <v>9</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>27.51</v>
+        <v>28.06</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
@@ -1811,10 +1787,10 @@
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>5</v>
+        <v>5.109585</v>
       </c>
       <c r="E17" s="28" t="n">
-        <v>15.29</v>
+        <v>15.62</v>
       </c>
       <c r="F17" s="29" t="n"/>
     </row>
@@ -1838,7 +1814,7 @@
         <v>20</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>61.14</v>
+        <v>62.37</v>
       </c>
       <c r="F18" s="24" t="n"/>
     </row>
@@ -1879,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1954,10 +1930,10 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>20</v>
+        <v>20.565914</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.14</v>
+        <v>62.87</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1978,10 +1954,10 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>5</v>
+        <v>5.142296</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>15.29</v>
+        <v>15.72</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -2002,7 +1978,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>20.79</v>
+        <v>24.828263</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>75.90000000000001</v>
@@ -2017,187 +1993,163 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.9)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>24.828263</v>
+        <v>54.409552</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>75.90000000000001</v>
+        <v>166.33</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>54.409552</v>
+        <v>18</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>166.33</v>
+        <v>56.49</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>18</v>
+        <v>2.306183</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>55.03</v>
+        <v>7.05</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>2.25</v>
+        <v>20.55283</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>6.88</v>
+        <v>62.83</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>20</v>
+        <v>16.323193</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.14</v>
+        <v>49.9</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-16</t>
-        </is>
-      </c>
-      <c r="B13" s="11" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C13" s="11" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D13" s="27" t="n">
-        <v>20</v>
-      </c>
-      <c r="E13" s="28" t="n">
-        <v>61.14</v>
-      </c>
-      <c r="F13" s="29" t="n"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="20">
-        <f>SUM(D4:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="21">
-        <f>SUM(E4:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="31" t="n"/>
+      <c r="B13" s="31" t="n"/>
+      <c r="C13" s="31" t="n"/>
+      <c r="D13" s="20">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="21">
+        <f>SUM(E4:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3047,7 +2999,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3114,10 +3066,10 @@
         </is>
       </c>
       <c r="D3" s="12" t="n">
-        <v>1</v>
+        <v>1.092574</v>
       </c>
       <c r="E3" s="13" t="n">
-        <v>3.06</v>
+        <v>3.34</v>
       </c>
       <c r="F3" s="10" t="inlineStr">
         <is>
@@ -3142,10 +3094,10 @@
         </is>
       </c>
       <c r="D4" s="16" t="n">
-        <v>72</v>
+        <v>78.86162899999999</v>
       </c>
       <c r="E4" s="17" t="n">
-        <v>220.1</v>
+        <v>241.08</v>
       </c>
       <c r="F4" s="14" t="inlineStr">
         <is>
@@ -3170,10 +3122,10 @@
         </is>
       </c>
       <c r="D5" s="12" t="n">
-        <v>10.59</v>
+        <v>11.462218</v>
       </c>
       <c r="E5" s="13" t="n">
-        <v>32.37</v>
+        <v>35.04</v>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -3198,10 +3150,10 @@
         </is>
       </c>
       <c r="D6" s="16" t="n">
-        <v>20</v>
+        <v>21.687929</v>
       </c>
       <c r="E6" s="17" t="n">
-        <v>61.14</v>
+        <v>66.3</v>
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
@@ -3229,7 +3181,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="13" t="n">
-        <v>61.14</v>
+        <v>67.31</v>
       </c>
       <c r="F7" s="10" t="inlineStr">
         <is>
@@ -3254,10 +3206,10 @@
         </is>
       </c>
       <c r="D8" s="16" t="n">
-        <v>13.5</v>
+        <v>14.828263</v>
       </c>
       <c r="E8" s="17" t="n">
-        <v>41.27</v>
+        <v>45.33</v>
       </c>
       <c r="F8" s="14" t="inlineStr">
         <is>
@@ -3282,10 +3234,10 @@
         </is>
       </c>
       <c r="D9" s="12" t="n">
-        <v>113.14</v>
+        <v>124.586196</v>
       </c>
       <c r="E9" s="13" t="n">
-        <v>345.87</v>
+        <v>380.86</v>
       </c>
       <c r="F9" s="10" t="inlineStr">
         <is>
@@ -3310,10 +3262,10 @@
         </is>
       </c>
       <c r="D10" s="16" t="n">
-        <v>10</v>
+        <v>11.010795</v>
       </c>
       <c r="E10" s="17" t="n">
-        <v>30.57</v>
+        <v>33.66</v>
       </c>
       <c r="F10" s="14" t="inlineStr">
         <is>
@@ -3338,7 +3290,7 @@
         </is>
       </c>
       <c r="D11" s="12" t="n">
-        <v>15.6</v>
+        <v>18.622833</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>56.93</v>
@@ -3366,10 +3318,10 @@
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>15</v>
+        <v>16.745175</v>
       </c>
       <c r="E12" s="17" t="n">
-        <v>45.85</v>
+        <v>51.19</v>
       </c>
       <c r="F12" s="14" t="inlineStr">
         <is>
@@ -3394,10 +3346,10 @@
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>12</v>
+        <v>13.385672</v>
       </c>
       <c r="E13" s="13" t="n">
-        <v>36.68</v>
+        <v>40.92</v>
       </c>
       <c r="F13" s="10" t="inlineStr">
         <is>
@@ -3422,10 +3374,10 @@
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>0.9</v>
+        <v>1.007524</v>
       </c>
       <c r="E14" s="17" t="n">
-        <v>2.75</v>
+        <v>3.08</v>
       </c>
       <c r="F14" s="14" t="inlineStr">
         <is>
@@ -3450,10 +3402,10 @@
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>19</v>
+        <v>21.341184</v>
       </c>
       <c r="E15" s="13" t="n">
-        <v>58.08</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="F15" s="10" t="inlineStr">
         <is>
@@ -3478,10 +3430,10 @@
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>10.59</v>
+        <v>11.894014</v>
       </c>
       <c r="E16" s="17" t="n">
-        <v>32.37</v>
+        <v>36.36</v>
       </c>
       <c r="F16" s="14" t="inlineStr">
         <is>
@@ -3506,10 +3458,10 @@
         </is>
       </c>
       <c r="D17" s="12" t="n">
-        <v>20</v>
+        <v>22.384691</v>
       </c>
       <c r="E17" s="13" t="n">
-        <v>61.14</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
@@ -3537,7 +3489,7 @@
         <v>20</v>
       </c>
       <c r="E18" s="17" t="n">
-        <v>61.14</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="F18" s="14" t="inlineStr">
         <is>
@@ -3562,10 +3514,10 @@
         </is>
       </c>
       <c r="D19" s="12" t="n">
-        <v>5</v>
+        <v>5.466143</v>
       </c>
       <c r="E19" s="13" t="n">
-        <v>15.29</v>
+        <v>16.71</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
@@ -3590,10 +3542,10 @@
         </is>
       </c>
       <c r="D20" s="16" t="n">
-        <v>11.25</v>
+        <v>12.29964</v>
       </c>
       <c r="E20" s="17" t="n">
-        <v>34.39</v>
+        <v>37.6</v>
       </c>
       <c r="F20" s="14" t="inlineStr">
         <is>
@@ -3618,7 +3570,7 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>15.6</v>
+        <v>18.622833</v>
       </c>
       <c r="E21" s="13" t="n">
         <v>56.93</v>
@@ -3646,10 +3598,10 @@
         </is>
       </c>
       <c r="D22" s="16" t="n">
-        <v>2.79</v>
+        <v>3.055283</v>
       </c>
       <c r="E22" s="17" t="n">
-        <v>8.529999999999999</v>
+        <v>9.34</v>
       </c>
       <c r="F22" s="14" t="inlineStr">
         <is>
@@ -3674,10 +3626,10 @@
         </is>
       </c>
       <c r="D23" s="12" t="n">
-        <v>10.59</v>
+        <v>11.583252</v>
       </c>
       <c r="E23" s="13" t="n">
-        <v>32.37</v>
+        <v>35.41</v>
       </c>
       <c r="F23" s="10" t="inlineStr">
         <is>
@@ -3705,7 +3657,7 @@
         <v>20</v>
       </c>
       <c r="E24" s="17" t="n">
-        <v>61.14</v>
+        <v>67.01000000000001</v>
       </c>
       <c r="F24" s="14" t="inlineStr">
         <is>
@@ -3730,10 +3682,10 @@
         </is>
       </c>
       <c r="D25" s="12" t="n">
-        <v>20</v>
+        <v>21.871115</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>61.14</v>
+        <v>66.86</v>
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
@@ -3758,10 +3710,10 @@
         </is>
       </c>
       <c r="D26" s="16" t="n">
-        <v>5</v>
+        <v>5.40072</v>
       </c>
       <c r="E26" s="17" t="n">
-        <v>15.29</v>
+        <v>16.51</v>
       </c>
       <c r="F26" s="14" t="inlineStr">
         <is>
@@ -3786,7 +3738,7 @@
         </is>
       </c>
       <c r="D27" s="12" t="n">
-        <v>15.6</v>
+        <v>18.622833</v>
       </c>
       <c r="E27" s="13" t="n">
         <v>56.93</v>
@@ -3817,7 +3769,7 @@
         <v>20</v>
       </c>
       <c r="E28" s="17" t="n">
-        <v>61.14</v>
+        <v>65.72</v>
       </c>
       <c r="F28" s="14" t="inlineStr">
         <is>
@@ -3842,10 +3794,10 @@
         </is>
       </c>
       <c r="D29" s="12" t="n">
-        <v>20</v>
+        <v>21.52437</v>
       </c>
       <c r="E29" s="13" t="n">
-        <v>61.14</v>
+        <v>65.8</v>
       </c>
       <c r="F29" s="10" t="inlineStr">
         <is>
@@ -3870,10 +3822,10 @@
         </is>
       </c>
       <c r="D30" s="16" t="n">
-        <v>5</v>
+        <v>5.322211</v>
       </c>
       <c r="E30" s="17" t="n">
-        <v>15.29</v>
+        <v>16.27</v>
       </c>
       <c r="F30" s="14" t="inlineStr">
         <is>
@@ -3898,10 +3850,10 @@
         </is>
       </c>
       <c r="D31" s="12" t="n">
-        <v>12</v>
+        <v>12.79686</v>
       </c>
       <c r="E31" s="13" t="n">
-        <v>36.68</v>
+        <v>39.12</v>
       </c>
       <c r="F31" s="10" t="inlineStr">
         <is>
@@ -3926,10 +3878,10 @@
         </is>
       </c>
       <c r="D32" s="16" t="n">
-        <v>11.8</v>
+        <v>12.463199</v>
       </c>
       <c r="E32" s="17" t="n">
-        <v>36.07</v>
+        <v>38.1</v>
       </c>
       <c r="F32" s="14" t="inlineStr">
         <is>
@@ -3954,10 +3906,10 @@
         </is>
       </c>
       <c r="D33" s="12" t="n">
-        <v>15</v>
+        <v>15.8456</v>
       </c>
       <c r="E33" s="13" t="n">
-        <v>45.85</v>
+        <v>48.44</v>
       </c>
       <c r="F33" s="10" t="inlineStr">
         <is>
@@ -3982,10 +3934,10 @@
         </is>
       </c>
       <c r="D34" s="16" t="n">
-        <v>10</v>
+        <v>10.451423</v>
       </c>
       <c r="E34" s="17" t="n">
-        <v>30.57</v>
+        <v>31.95</v>
       </c>
       <c r="F34" s="14" t="inlineStr">
         <is>
@@ -4013,7 +3965,7 @@
         <v>20</v>
       </c>
       <c r="E35" s="13" t="n">
-        <v>61.14</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
@@ -4038,10 +3990,10 @@
         </is>
       </c>
       <c r="D36" s="16" t="n">
-        <v>20</v>
+        <v>21.432777</v>
       </c>
       <c r="E36" s="17" t="n">
-        <v>61.14</v>
+        <v>65.52</v>
       </c>
       <c r="F36" s="14" t="inlineStr">
         <is>
@@ -4066,10 +4018,10 @@
         </is>
       </c>
       <c r="D37" s="12" t="n">
-        <v>5</v>
+        <v>5.335296</v>
       </c>
       <c r="E37" s="13" t="n">
-        <v>15.29</v>
+        <v>16.31</v>
       </c>
       <c r="F37" s="10" t="inlineStr">
         <is>
@@ -4094,7 +4046,7 @@
         </is>
       </c>
       <c r="D38" s="16" t="n">
-        <v>20.79</v>
+        <v>24.828263</v>
       </c>
       <c r="E38" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4122,10 +4074,10 @@
         </is>
       </c>
       <c r="D39" s="12" t="n">
-        <v>15</v>
+        <v>15.95682</v>
       </c>
       <c r="E39" s="13" t="n">
-        <v>45.85</v>
+        <v>48.78</v>
       </c>
       <c r="F39" s="10" t="inlineStr">
         <is>
@@ -4150,10 +4102,10 @@
         </is>
       </c>
       <c r="D40" s="16" t="n">
-        <v>9.720000000000001</v>
+        <v>10.340203</v>
       </c>
       <c r="E40" s="17" t="n">
-        <v>29.71</v>
+        <v>31.61</v>
       </c>
       <c r="F40" s="14" t="inlineStr">
         <is>
@@ -4178,10 +4130,10 @@
         </is>
       </c>
       <c r="D41" s="12" t="n">
-        <v>30</v>
+        <v>31.71737</v>
       </c>
       <c r="E41" s="13" t="n">
-        <v>91.70999999999999</v>
+        <v>96.95999999999999</v>
       </c>
       <c r="F41" s="10" t="inlineStr">
         <is>
@@ -4206,10 +4158,10 @@
         </is>
       </c>
       <c r="D42" s="16" t="n">
-        <v>33</v>
+        <v>34.684331</v>
       </c>
       <c r="E42" s="17" t="n">
-        <v>100.88</v>
+        <v>106.03</v>
       </c>
       <c r="F42" s="14" t="inlineStr">
         <is>
@@ -4237,7 +4189,7 @@
         <v>20</v>
       </c>
       <c r="E43" s="13" t="n">
-        <v>61.14</v>
+        <v>64.26000000000001</v>
       </c>
       <c r="F43" s="10" t="inlineStr">
         <is>
@@ -4262,10 +4214,10 @@
         </is>
       </c>
       <c r="D44" s="16" t="n">
-        <v>36</v>
+        <v>37.556428</v>
       </c>
       <c r="E44" s="17" t="n">
-        <v>110.05</v>
+        <v>114.81</v>
       </c>
       <c r="F44" s="14" t="inlineStr">
         <is>
@@ -4290,10 +4242,10 @@
         </is>
       </c>
       <c r="D45" s="12" t="n">
-        <v>5</v>
+        <v>5.210991</v>
       </c>
       <c r="E45" s="13" t="n">
-        <v>15.29</v>
+        <v>15.93</v>
       </c>
       <c r="F45" s="10" t="inlineStr">
         <is>
@@ -4318,7 +4270,7 @@
         </is>
       </c>
       <c r="D46" s="16" t="n">
-        <v>20.79</v>
+        <v>24.828263</v>
       </c>
       <c r="E46" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4346,10 +4298,10 @@
         </is>
       </c>
       <c r="D47" s="12" t="n">
-        <v>139.92</v>
+        <v>145.806346</v>
       </c>
       <c r="E47" s="13" t="n">
-        <v>427.74</v>
+        <v>445.73</v>
       </c>
       <c r="F47" s="10" t="inlineStr">
         <is>
@@ -4374,10 +4326,10 @@
         </is>
       </c>
       <c r="D48" s="16" t="n">
-        <v>15</v>
+        <v>15.629702</v>
       </c>
       <c r="E48" s="17" t="n">
-        <v>45.85</v>
+        <v>47.78</v>
       </c>
       <c r="F48" s="14" t="inlineStr">
         <is>
@@ -4402,10 +4354,10 @@
         </is>
       </c>
       <c r="D49" s="12" t="n">
-        <v>19.43</v>
+        <v>20.24861</v>
       </c>
       <c r="E49" s="13" t="n">
-        <v>59.4</v>
+        <v>61.9</v>
       </c>
       <c r="F49" s="10" t="inlineStr">
         <is>
@@ -4430,10 +4382,10 @@
         </is>
       </c>
       <c r="D50" s="16" t="n">
-        <v>20</v>
+        <v>20.77527</v>
       </c>
       <c r="E50" s="17" t="n">
-        <v>61.14</v>
+        <v>63.51</v>
       </c>
       <c r="F50" s="14" t="inlineStr">
         <is>
@@ -4458,10 +4410,10 @@
         </is>
       </c>
       <c r="D51" s="12" t="n">
-        <v>20</v>
+        <v>20.716389</v>
       </c>
       <c r="E51" s="13" t="n">
-        <v>61.14</v>
+        <v>63.33</v>
       </c>
       <c r="F51" s="10" t="inlineStr">
         <is>
@@ -4486,7 +4438,7 @@
         </is>
       </c>
       <c r="D52" s="16" t="n">
-        <v>13.67</v>
+        <v>16.323193</v>
       </c>
       <c r="E52" s="17" t="n">
         <v>49.9</v>
@@ -4517,7 +4469,7 @@
         <v>20</v>
       </c>
       <c r="E53" s="13" t="n">
-        <v>61.14</v>
+        <v>62.81</v>
       </c>
       <c r="F53" s="10" t="inlineStr">
         <is>
@@ -4542,10 +4494,10 @@
         </is>
       </c>
       <c r="D54" s="16" t="n">
-        <v>39</v>
+        <v>40.170101</v>
       </c>
       <c r="E54" s="17" t="n">
-        <v>119.22</v>
+        <v>122.8</v>
       </c>
       <c r="F54" s="14" t="inlineStr">
         <is>
@@ -4570,10 +4522,10 @@
         </is>
       </c>
       <c r="D55" s="12" t="n">
-        <v>25</v>
+        <v>25.583906</v>
       </c>
       <c r="E55" s="13" t="n">
-        <v>76.42</v>
+        <v>78.20999999999999</v>
       </c>
       <c r="F55" s="10" t="inlineStr">
         <is>
@@ -4598,10 +4550,10 @@
         </is>
       </c>
       <c r="D56" s="16" t="n">
-        <v>43</v>
+        <v>43.833824</v>
       </c>
       <c r="E56" s="17" t="n">
-        <v>131.45</v>
+        <v>134</v>
       </c>
       <c r="F56" s="14" t="inlineStr">
         <is>
@@ -4626,10 +4578,10 @@
         </is>
       </c>
       <c r="D57" s="12" t="n">
-        <v>5</v>
+        <v>5.047432</v>
       </c>
       <c r="E57" s="13" t="n">
-        <v>15.29</v>
+        <v>15.43</v>
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
@@ -4654,10 +4606,10 @@
         </is>
       </c>
       <c r="D58" s="16" t="n">
-        <v>14.5</v>
+        <v>14.635263</v>
       </c>
       <c r="E58" s="17" t="n">
-        <v>44.33</v>
+        <v>44.74</v>
       </c>
       <c r="F58" s="14" t="inlineStr">
         <is>
@@ -4682,10 +4634,10 @@
         </is>
       </c>
       <c r="D59" s="12" t="n">
-        <v>25</v>
+        <v>25.371279</v>
       </c>
       <c r="E59" s="13" t="n">
-        <v>76.42</v>
+        <v>77.56</v>
       </c>
       <c r="F59" s="10" t="inlineStr">
         <is>
@@ -4710,7 +4662,7 @@
         </is>
       </c>
       <c r="D60" s="16" t="n">
-        <v>20.79</v>
+        <v>24.828263</v>
       </c>
       <c r="E60" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4724,24 +4676,24 @@
     <row r="61">
       <c r="A61" s="10" t="inlineStr">
         <is>
-          <t>2026-02-02</t>
+          <t>2026-02-03</t>
         </is>
       </c>
       <c r="B61" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.9)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D61" s="12" t="n">
-        <v>24.828263</v>
+        <v>31.851488</v>
       </c>
       <c r="E61" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>97.37</v>
       </c>
       <c r="F61" s="10" t="inlineStr">
         <is>
@@ -4752,24 +4704,24 @@
     <row r="62">
       <c r="A62" s="14" t="inlineStr">
         <is>
-          <t>2026-02-03</t>
+          <t>2026-02-10</t>
         </is>
       </c>
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro – Feb 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D62" s="16" t="n">
-        <v>31.42</v>
+        <v>16.323193</v>
       </c>
       <c r="E62" s="17" t="n">
-        <v>96.05</v>
+        <v>49.9</v>
       </c>
       <c r="F62" s="14" t="inlineStr">
         <is>
@@ -4780,24 +4732,24 @@
     <row r="63">
       <c r="A63" s="10" t="inlineStr">
         <is>
-          <t>2026-02-10</t>
+          <t>2026-02-12</t>
         </is>
       </c>
       <c r="B63" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Pro – Feb 2026 (₪49.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>13.67</v>
+        <v>47.307818</v>
       </c>
       <c r="E63" s="13" t="n">
-        <v>49.9</v>
+        <v>144.62</v>
       </c>
       <c r="F63" s="10" t="inlineStr">
         <is>
@@ -4808,24 +4760,24 @@
     <row r="64">
       <c r="A64" s="14" t="inlineStr">
         <is>
-          <t>2026-02-12</t>
+          <t>2026-02-15</t>
         </is>
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D64" s="16" t="n">
-        <v>47</v>
+        <v>20.193</v>
       </c>
       <c r="E64" s="17" t="n">
-        <v>143.68</v>
+        <v>61.73</v>
       </c>
       <c r="F64" s="14" t="inlineStr">
         <is>
@@ -4836,7 +4788,7 @@
     <row r="65">
       <c r="A65" s="10" t="inlineStr">
         <is>
-          <t>2026-02-15</t>
+          <t>2026-02-16</t>
         </is>
       </c>
       <c r="B65" s="11" t="inlineStr">
@@ -4846,14 +4798,14 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>20</v>
+        <v>5.050703</v>
       </c>
       <c r="E65" s="13" t="n">
-        <v>61.14</v>
+        <v>15.44</v>
       </c>
       <c r="F65" s="10" t="inlineStr">
         <is>
@@ -4869,19 +4821,19 @@
       </c>
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D66" s="16" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E66" s="17" t="n">
-        <v>15.29</v>
+        <v>61.77</v>
       </c>
       <c r="F66" s="14" t="inlineStr">
         <is>
@@ -4892,24 +4844,24 @@
     <row r="67">
       <c r="A67" s="10" t="inlineStr">
         <is>
-          <t>2026-02-16</t>
+          <t>2026-02-24</t>
         </is>
       </c>
       <c r="B67" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>On-Demand credits 500</t>
         </is>
       </c>
       <c r="D67" s="12" t="n">
-        <v>20</v>
+        <v>20.464508</v>
       </c>
       <c r="E67" s="13" t="n">
-        <v>61.14</v>
+        <v>62.56</v>
       </c>
       <c r="F67" s="10" t="inlineStr">
         <is>
@@ -4920,24 +4872,24 @@
     <row r="68">
       <c r="A68" s="14" t="inlineStr">
         <is>
-          <t>2026-02-24</t>
+          <t>2026-02-25</t>
         </is>
       </c>
       <c r="B68" s="15" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>On-Demand credits 500</t>
+          <t>Pro2 monthly</t>
         </is>
       </c>
       <c r="D68" s="16" t="n">
-        <v>20</v>
+        <v>50.690219</v>
       </c>
       <c r="E68" s="17" t="n">
-        <v>61.14</v>
+        <v>154.96</v>
       </c>
       <c r="F68" s="14" t="inlineStr">
         <is>
@@ -4953,19 +4905,19 @@
       </c>
       <c r="B69" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Pro2 monthly</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>50</v>
+        <v>51.704285</v>
       </c>
       <c r="E69" s="13" t="n">
-        <v>152.85</v>
+        <v>158.06</v>
       </c>
       <c r="F69" s="10" t="inlineStr">
         <is>
@@ -4976,24 +4928,24 @@
     <row r="70">
       <c r="A70" s="14" t="inlineStr">
         <is>
-          <t>2026-02-25</t>
+          <t>2026-02-28</t>
         </is>
       </c>
       <c r="B70" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>51</v>
+        <v>5.129212</v>
       </c>
       <c r="E70" s="17" t="n">
-        <v>155.91</v>
+        <v>15.68</v>
       </c>
       <c r="F70" s="14" t="inlineStr">
         <is>
@@ -5009,19 +4961,19 @@
       </c>
       <c r="B71" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Starter monthly</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D71" s="12" t="n">
-        <v>5</v>
+        <v>10.255152</v>
       </c>
       <c r="E71" s="13" t="n">
-        <v>15.29</v>
+        <v>31.35</v>
       </c>
       <c r="F71" s="10" t="inlineStr">
         <is>
@@ -5032,28 +4984,28 @@
     <row r="72">
       <c r="A72" s="14" t="inlineStr">
         <is>
-          <t>2026-02-28</t>
+          <t>2026-03-01</t>
         </is>
       </c>
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Google Workspace (₪75.9)</t>
         </is>
       </c>
       <c r="D72" s="16" t="n">
-        <v>10</v>
+        <v>24.828263</v>
       </c>
       <c r="E72" s="17" t="n">
-        <v>30.57</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F72" s="14" t="inlineStr">
         <is>
-          <t>פברואר 2026</t>
+          <t>מרץ 2026</t>
         </is>
       </c>
     </row>
@@ -5065,19 +5017,19 @@
       </c>
       <c r="B73" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.9)</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D73" s="12" t="n">
-        <v>24.828263</v>
+        <v>10.232254</v>
       </c>
       <c r="E73" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>31.28</v>
       </c>
       <c r="F73" s="10" t="inlineStr">
         <is>
@@ -5093,19 +5045,19 @@
       </c>
       <c r="B74" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Timeless</t>
         </is>
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Pro monthly (50% off)</t>
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>10</v>
+        <v>14.838077</v>
       </c>
       <c r="E74" s="17" t="n">
-        <v>30.57</v>
+        <v>45.36</v>
       </c>
       <c r="F74" s="14" t="inlineStr">
         <is>
@@ -5116,24 +5068,24 @@
     <row r="75">
       <c r="A75" s="10" t="inlineStr">
         <is>
-          <t>2026-03-01</t>
+          <t>2026-03-02</t>
         </is>
       </c>
       <c r="B75" s="11" t="inlineStr">
         <is>
-          <t>Timeless</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Pro monthly (50% off)</t>
+          <t>Business Plus – Feb 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>14.5</v>
+        <v>24.828263</v>
       </c>
       <c r="E75" s="13" t="n">
-        <v>44.33</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F75" s="10" t="inlineStr">
         <is>
@@ -5149,19 +5101,19 @@
       </c>
       <c r="B76" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Business Plus – Feb 2026 (₪75.90)</t>
+          <t>Cloud &amp; AI Balance Top-up</t>
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>20.79</v>
+        <v>10.206084</v>
       </c>
       <c r="E76" s="17" t="n">
-        <v>75.90000000000001</v>
+        <v>31.2</v>
       </c>
       <c r="F76" s="14" t="inlineStr">
         <is>
@@ -5172,24 +5124,24 @@
     <row r="77">
       <c r="A77" s="10" t="inlineStr">
         <is>
-          <t>2026-03-02</t>
+          <t>2026-03-03</t>
         </is>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Cloud &amp; AI Balance Top-up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>10</v>
+        <v>40.376186</v>
       </c>
       <c r="E77" s="13" t="n">
-        <v>30.57</v>
+        <v>123.43</v>
       </c>
       <c r="F77" s="10" t="inlineStr">
         <is>
@@ -5200,24 +5152,24 @@
     <row r="78">
       <c r="A78" s="14" t="inlineStr">
         <is>
-          <t>2026-03-03</t>
+          <t>2026-03-10</t>
         </is>
       </c>
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Pro – Mar 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>40.11</v>
+        <v>16.323193</v>
       </c>
       <c r="E78" s="17" t="n">
-        <v>122.62</v>
+        <v>49.9</v>
       </c>
       <c r="F78" s="14" t="inlineStr">
         <is>
@@ -5228,24 +5180,24 @@
     <row r="79">
       <c r="A79" s="10" t="inlineStr">
         <is>
-          <t>2026-03-10</t>
+          <t>2026-03-12</t>
         </is>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Pro – Mar 2026 (₪49.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>13.67</v>
+        <v>52.230945</v>
       </c>
       <c r="E79" s="13" t="n">
-        <v>49.9</v>
+        <v>159.67</v>
       </c>
       <c r="F79" s="10" t="inlineStr">
         <is>
@@ -5256,24 +5208,24 @@
     <row r="80">
       <c r="A80" s="14" t="inlineStr">
         <is>
-          <t>2026-03-12</t>
+          <t>2026-03-15</t>
         </is>
       </c>
       <c r="B80" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>51</v>
+        <v>20.565914</v>
       </c>
       <c r="E80" s="17" t="n">
-        <v>155.91</v>
+        <v>62.87</v>
       </c>
       <c r="F80" s="14" t="inlineStr">
         <is>
@@ -5284,24 +5236,24 @@
     <row r="81">
       <c r="A81" s="10" t="inlineStr">
         <is>
-          <t>2026-03-15</t>
+          <t>2026-03-16</t>
         </is>
       </c>
       <c r="B81" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D81" s="12" t="n">
         <v>20</v>
       </c>
       <c r="E81" s="13" t="n">
-        <v>61.14</v>
+        <v>62.87</v>
       </c>
       <c r="F81" s="10" t="inlineStr">
         <is>
@@ -5312,24 +5264,24 @@
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>2026-03-16</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>20</v>
+        <v>10.176644</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>61.14</v>
+        <v>31.11</v>
       </c>
       <c r="F82" s="14" t="inlineStr">
         <is>
@@ -5345,19 +5297,19 @@
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Creator (first month 50% off)</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>10</v>
+        <v>11.193981</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>30.57</v>
+        <v>34.22</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5368,24 +5320,24 @@
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Creator (first month 50% off)</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>33.63</v>
+        <v>28.06</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5396,24 +5348,24 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Lite plan</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>9</v>
+        <v>5.109585</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>27.51</v>
+        <v>15.62</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5424,24 +5376,24 @@
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>5</v>
+        <v>20</v>
       </c>
       <c r="E86" s="17" t="n">
-        <v>15.29</v>
+        <v>62.37</v>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
@@ -5452,28 +5404,28 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-04-01</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>20</v>
+        <v>20.565914</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>61.14</v>
+        <v>62.87</v>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t>מרץ 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
@@ -5490,14 +5442,14 @@
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>20</v>
+        <v>5.142296</v>
       </c>
       <c r="E88" s="17" t="n">
-        <v>61.14</v>
+        <v>15.72</v>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
@@ -5513,19 +5465,19 @@
       </c>
       <c r="B89" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Business Plus – Mar 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>5</v>
+        <v>24.828263</v>
       </c>
       <c r="E89" s="13" t="n">
-        <v>15.29</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F89" s="10" t="inlineStr">
         <is>
@@ -5541,19 +5493,19 @@
       </c>
       <c r="B90" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C90" s="15" t="inlineStr">
         <is>
-          <t>Business Plus – Mar 2026 (₪75.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>20.79</v>
+        <v>54.409552</v>
       </c>
       <c r="E90" s="17" t="n">
-        <v>75.90000000000001</v>
+        <v>166.33</v>
       </c>
       <c r="F90" s="14" t="inlineStr">
         <is>
@@ -5564,24 +5516,24 @@
     <row r="91">
       <c r="A91" s="10" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B91" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.9)</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D91" s="12" t="n">
-        <v>24.828263</v>
+        <v>18</v>
       </c>
       <c r="E91" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>56.49</v>
       </c>
       <c r="F91" s="10" t="inlineStr">
         <is>
@@ -5592,7 +5544,7 @@
     <row r="92">
       <c r="A92" s="14" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B92" s="15" t="inlineStr">
@@ -5606,10 +5558,10 @@
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>54.409552</v>
+        <v>2.306183</v>
       </c>
       <c r="E92" s="17" t="n">
-        <v>166.33</v>
+        <v>7.05</v>
       </c>
       <c r="F92" s="14" t="inlineStr">
         <is>
@@ -5620,24 +5572,24 @@
     <row r="93">
       <c r="A93" s="10" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B93" s="11" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>18</v>
+        <v>20.55283</v>
       </c>
       <c r="E93" s="13" t="n">
-        <v>55.03</v>
+        <v>62.83</v>
       </c>
       <c r="F93" s="10" t="inlineStr">
         <is>
@@ -5648,24 +5600,24 @@
     <row r="94">
       <c r="A94" s="14" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B94" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C94" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>2.25</v>
+        <v>16.323193</v>
       </c>
       <c r="E94" s="17" t="n">
-        <v>6.88</v>
+        <v>49.9</v>
       </c>
       <c r="F94" s="14" t="inlineStr">
         <is>
@@ -5676,17 +5628,17 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
@@ -5704,35 +5656,35 @@
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D96" s="16" t="n">
-        <v>16.323193</v>
+        <v>20</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>49.9</v>
+        <v>61.14</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5753,14 +5705,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5781,14 +5733,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5809,14 +5761,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5837,14 +5789,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5865,14 +5817,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5893,14 +5845,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>נובמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-12-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5921,88 +5873,32 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
-      <c r="A104" s="14" t="inlineStr">
-        <is>
-          <t>2026-11-16</t>
-        </is>
-      </c>
-      <c r="B104" s="15" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C104" s="15" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D104" s="16" t="n">
-        <v>20</v>
-      </c>
-      <c r="E104" s="17" t="n">
-        <v>61.14</v>
-      </c>
-      <c r="F104" s="14" t="inlineStr">
-        <is>
-          <t>נובמבר 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="10" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="B105" s="11" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C105" s="11" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D105" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="E105" s="13" t="n">
-        <v>61.14</v>
-      </c>
-      <c r="F105" s="10" t="inlineStr">
-        <is>
-          <t>דצמבר 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="18" t="inlineStr">
+      <c r="A104" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B106" s="19" t="n"/>
-      <c r="C106" s="19" t="n"/>
-      <c r="D106" s="20">
-        <f>SUM(D3:D105)</f>
-        <v/>
-      </c>
-      <c r="E106" s="21">
-        <f>SUM(E3:E105)</f>
-        <v/>
-      </c>
-      <c r="F106" s="19" t="n"/>
+      <c r="B104" s="19" t="n"/>
+      <c r="C104" s="19" t="n"/>
+      <c r="D104" s="20">
+        <f>SUM(D3:D103)</f>
+        <v/>
+      </c>
+      <c r="E104" s="21">
+        <f>SUM(E3:E103)</f>
+        <v/>
+      </c>
+      <c r="F104" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A106:C106"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A104:C104"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10731,10 +10627,10 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>1</v>
+        <v>1.092574</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>3.06</v>
+        <v>3.34</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -10755,10 +10651,10 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>72</v>
+        <v>78.86162899999999</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>220.1</v>
+        <v>241.08</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -10779,10 +10675,10 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>10.59</v>
+        <v>11.462218</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>32.37</v>
+        <v>35.04</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -10803,10 +10699,10 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>20</v>
+        <v>21.687929</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>61.14</v>
+        <v>66.3</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -10830,7 +10726,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>61.14</v>
+        <v>67.31</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -10851,10 +10747,10 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>13.5</v>
+        <v>14.828263</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>41.27</v>
+        <v>45.33</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -10875,10 +10771,10 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>113.14</v>
+        <v>124.586196</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>345.87</v>
+        <v>380.86</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -10899,10 +10795,10 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>10</v>
+        <v>11.010795</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>30.57</v>
+        <v>33.66</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -11018,7 +10914,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>15.6</v>
+        <v>18.622833</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11042,10 +10938,10 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>15</v>
+        <v>16.745175</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>45.85</v>
+        <v>51.19</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11066,10 +10962,10 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>12</v>
+        <v>13.385672</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>36.68</v>
+        <v>40.92</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11090,10 +10986,10 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>0.9</v>
+        <v>1.007524</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>2.75</v>
+        <v>3.08</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11114,10 +11010,10 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>19</v>
+        <v>21.341184</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>58.08</v>
+        <v>65.23999999999999</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11138,10 +11034,10 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>10.59</v>
+        <v>11.894014</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>32.37</v>
+        <v>36.36</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11162,10 +11058,10 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>20</v>
+        <v>22.384691</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>61.14</v>
+        <v>68.43000000000001</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -11189,7 +11085,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.14</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -11210,10 +11106,10 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>5</v>
+        <v>5.466143</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>15.29</v>
+        <v>16.71</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -11234,10 +11130,10 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>11.25</v>
+        <v>12.29964</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>34.39</v>
+        <v>37.6</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -11353,7 +11249,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>15.6</v>
+        <v>18.622833</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11377,10 +11273,10 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>2.79</v>
+        <v>3.055283</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>8.529999999999999</v>
+        <v>9.34</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11401,10 +11297,10 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>10.59</v>
+        <v>11.583252</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>32.37</v>
+        <v>35.41</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11428,7 +11324,7 @@
         <v>20</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>61.14</v>
+        <v>67.01000000000001</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11449,10 +11345,10 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>20</v>
+        <v>21.871115</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>61.14</v>
+        <v>66.86</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11473,10 +11369,10 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>5</v>
+        <v>5.40072</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>15.29</v>
+        <v>16.51</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11592,7 +11488,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>15.6</v>
+        <v>18.622833</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11619,7 +11515,7 @@
         <v>20</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>61.14</v>
+        <v>65.72</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11640,10 +11536,10 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>20</v>
+        <v>21.52437</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>61.14</v>
+        <v>65.8</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11664,10 +11560,10 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>5</v>
+        <v>5.322211</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>15.29</v>
+        <v>16.27</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11783,10 +11679,10 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>12</v>
+        <v>12.79686</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>36.68</v>
+        <v>39.12</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -11807,10 +11703,10 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>11.8</v>
+        <v>12.463199</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>36.07</v>
+        <v>38.1</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -11831,10 +11727,10 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15</v>
+        <v>15.8456</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>45.85</v>
+        <v>48.44</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -11855,10 +11751,10 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>10</v>
+        <v>10.451423</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>30.57</v>
+        <v>31.95</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -11882,7 +11778,7 @@
         <v>20</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>61.14</v>
+        <v>64.68000000000001</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -11903,10 +11799,10 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20</v>
+        <v>21.432777</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.14</v>
+        <v>65.52</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -11927,10 +11823,10 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5</v>
+        <v>5.335296</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>15.29</v>
+        <v>16.31</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -12046,7 +11942,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>20.79</v>
+        <v>24.828263</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -12070,10 +11966,10 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>15</v>
+        <v>15.95682</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>45.85</v>
+        <v>48.78</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -12094,10 +11990,10 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>9.720000000000001</v>
+        <v>10.340203</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>29.71</v>
+        <v>31.61</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -12118,10 +12014,10 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>30</v>
+        <v>31.71737</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>91.70999999999999</v>
+        <v>96.95999999999999</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -12142,10 +12038,10 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>33</v>
+        <v>34.684331</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>100.88</v>
+        <v>106.03</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -12169,7 +12065,7 @@
         <v>20</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.14</v>
+        <v>64.26000000000001</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -12190,10 +12086,10 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>36</v>
+        <v>37.556428</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>110.05</v>
+        <v>114.81</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
@@ -12214,10 +12110,10 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>5</v>
+        <v>5.210991</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>15.29</v>
+        <v>15.93</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -12333,7 +12229,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>20.79</v>
+        <v>24.828263</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -12357,10 +12253,10 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>139.92</v>
+        <v>145.806346</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>427.74</v>
+        <v>445.73</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -12381,10 +12277,10 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15</v>
+        <v>15.629702</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>45.85</v>
+        <v>47.78</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
@@ -12405,10 +12301,10 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>19.43</v>
+        <v>20.24861</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>59.4</v>
+        <v>61.9</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
@@ -12429,10 +12325,10 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>20</v>
+        <v>20.77527</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>61.14</v>
+        <v>63.51</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
@@ -12453,10 +12349,10 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20</v>
+        <v>20.716389</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>61.14</v>
+        <v>63.33</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
@@ -12477,7 +12373,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>13.67</v>
+        <v>16.323193</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -12504,7 +12400,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>61.14</v>
+        <v>62.81</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -12525,10 +12421,10 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>39</v>
+        <v>40.170101</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>119.22</v>
+        <v>122.8</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -12549,10 +12445,10 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>25</v>
+        <v>25.583906</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>76.42</v>
+        <v>78.20999999999999</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -12573,10 +12469,10 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>43</v>
+        <v>43.833824</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>131.45</v>
+        <v>134</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -12597,10 +12493,10 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5</v>
+        <v>5.047432</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>15.29</v>
+        <v>15.43</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -12621,10 +12517,10 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>14.5</v>
+        <v>14.635263</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>44.33</v>
+        <v>44.74</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>

</xml_diff>

<commit_message>
fix: restore Telegram env vars in local run script
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -939,11 +939,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3.058</v>
+        <v>3.057</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-13</t>
+          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-10</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.362982</v>
+        <v>25.371279</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>77.56</v>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1116,7 +1116,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>31.841073</v>
+        <v>31.851488</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>97.37</v>
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>16.317855</v>
+        <v>16.323193</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>49.9</v>
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>47.292348</v>
+        <v>47.307818</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>144.62</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20.186396</v>
+        <v>20.193</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>61.73</v>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5.049052</v>
+        <v>5.050703</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>15.44</v>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20.457816</v>
+        <v>20.464508</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>62.56</v>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>50.673643</v>
+        <v>50.690219</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>154.96</v>
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>51.687377</v>
+        <v>51.704285</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>158.06</v>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.127534</v>
+        <v>5.129212</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>15.68</v>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>10.251799</v>
+        <v>10.255152</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>31.35</v>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>10.228908</v>
+        <v>10.232254</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>31.28</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>14.833224</v>
+        <v>14.838077</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>45.36</v>
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>10.202747</v>
+        <v>10.206084</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>31.2</v>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>40.362982</v>
+        <v>40.376186</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>123.43</v>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.317855</v>
+        <v>16.323193</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>52.213865</v>
+        <v>52.230945</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>159.67</v>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20.559189</v>
+        <v>20.565914</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>62.87</v>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>10.173316</v>
+        <v>10.176644</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>31.11</v>
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>11.19032</v>
+        <v>11.193981</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>34.22</v>
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>5.107914</v>
+        <v>5.109585</v>
       </c>
       <c r="E17" s="28" t="n">
         <v>15.62</v>
@@ -1930,7 +1930,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>20.559189</v>
+        <v>20.565914</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>62.87</v>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>5.140615</v>
+        <v>5.142296</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>15.72</v>
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>75.90000000000001</v>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>54.391759</v>
+        <v>54.409552</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>166.33</v>
@@ -2050,7 +2050,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>2.305428</v>
+        <v>2.306183</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>7.05</v>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>20.546109</v>
+        <v>20.55283</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>62.83</v>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>16.317855</v>
+        <v>16.323193</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>49.9</v>
@@ -2125,7 +2125,7 @@
         <v>20</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -2244,7 +2244,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2363,7 +2363,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2482,7 +2482,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2601,7 +2601,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2720,7 +2720,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2839,7 +2839,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2958,7 +2958,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="D3" s="12" t="n">
-        <v>1.092217</v>
+        <v>1.092574</v>
       </c>
       <c r="E3" s="13" t="n">
         <v>3.34</v>
@@ -3094,7 +3094,7 @@
         </is>
       </c>
       <c r="D4" s="16" t="n">
-        <v>78.83584</v>
+        <v>78.86162899999999</v>
       </c>
       <c r="E4" s="17" t="n">
         <v>241.08</v>
@@ -3122,7 +3122,7 @@
         </is>
       </c>
       <c r="D5" s="12" t="n">
-        <v>11.45847</v>
+        <v>11.462218</v>
       </c>
       <c r="E5" s="13" t="n">
         <v>35.04</v>
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="D6" s="16" t="n">
-        <v>21.680837</v>
+        <v>21.687929</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>66.3</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="D8" s="16" t="n">
-        <v>14.823414</v>
+        <v>14.828263</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>45.33</v>
@@ -3234,7 +3234,7 @@
         </is>
       </c>
       <c r="D9" s="12" t="n">
-        <v>124.545455</v>
+        <v>124.586196</v>
       </c>
       <c r="E9" s="13" t="n">
         <v>380.86</v>
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="D10" s="16" t="n">
-        <v>11.007194</v>
+        <v>11.010795</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>33.66</v>
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="D11" s="12" t="n">
-        <v>18.616743</v>
+        <v>18.622833</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>56.93</v>
@@ -3318,7 +3318,7 @@
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>16.739699</v>
+        <v>16.745175</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>51.19</v>
@@ -3346,7 +3346,7 @@
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>13.381295</v>
+        <v>13.385672</v>
       </c>
       <c r="E13" s="13" t="n">
         <v>40.92</v>
@@ -3374,7 +3374,7 @@
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>1.007194</v>
+        <v>1.007524</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>3.08</v>
@@ -3402,7 +3402,7 @@
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>21.334205</v>
+        <v>21.341184</v>
       </c>
       <c r="E15" s="13" t="n">
         <v>65.23999999999999</v>
@@ -3430,7 +3430,7 @@
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>11.890124</v>
+        <v>11.894014</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>36.36</v>
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="D17" s="12" t="n">
-        <v>22.377371</v>
+        <v>22.384691</v>
       </c>
       <c r="E17" s="13" t="n">
         <v>68.43000000000001</v>
@@ -3514,7 +3514,7 @@
         </is>
       </c>
       <c r="D19" s="12" t="n">
-        <v>5.464356</v>
+        <v>5.466143</v>
       </c>
       <c r="E19" s="13" t="n">
         <v>16.71</v>
@@ -3542,7 +3542,7 @@
         </is>
       </c>
       <c r="D20" s="16" t="n">
-        <v>12.295618</v>
+        <v>12.29964</v>
       </c>
       <c r="E20" s="17" t="n">
         <v>37.6</v>
@@ -3570,7 +3570,7 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>18.616743</v>
+        <v>18.622833</v>
       </c>
       <c r="E21" s="13" t="n">
         <v>56.93</v>
@@ -3598,7 +3598,7 @@
         </is>
       </c>
       <c r="D22" s="16" t="n">
-        <v>3.054284</v>
+        <v>3.055283</v>
       </c>
       <c r="E22" s="17" t="n">
         <v>9.34</v>
@@ -3626,7 +3626,7 @@
         </is>
       </c>
       <c r="D23" s="12" t="n">
-        <v>11.579464</v>
+        <v>11.583252</v>
       </c>
       <c r="E23" s="13" t="n">
         <v>35.41</v>
@@ -3682,7 +3682,7 @@
         </is>
       </c>
       <c r="D25" s="12" t="n">
-        <v>21.863963</v>
+        <v>21.871115</v>
       </c>
       <c r="E25" s="13" t="n">
         <v>66.86</v>
@@ -3710,7 +3710,7 @@
         </is>
       </c>
       <c r="D26" s="16" t="n">
-        <v>5.398954</v>
+        <v>5.40072</v>
       </c>
       <c r="E26" s="17" t="n">
         <v>16.51</v>
@@ -3738,7 +3738,7 @@
         </is>
       </c>
       <c r="D27" s="12" t="n">
-        <v>18.616743</v>
+        <v>18.622833</v>
       </c>
       <c r="E27" s="13" t="n">
         <v>56.93</v>
@@ -3794,7 +3794,7 @@
         </is>
       </c>
       <c r="D29" s="12" t="n">
-        <v>21.517332</v>
+        <v>21.52437</v>
       </c>
       <c r="E29" s="13" t="n">
         <v>65.8</v>
@@ -3822,7 +3822,7 @@
         </is>
       </c>
       <c r="D30" s="16" t="n">
-        <v>5.320471</v>
+        <v>5.322211</v>
       </c>
       <c r="E30" s="17" t="n">
         <v>16.27</v>
@@ -3850,7 +3850,7 @@
         </is>
       </c>
       <c r="D31" s="12" t="n">
-        <v>12.792675</v>
+        <v>12.79686</v>
       </c>
       <c r="E31" s="13" t="n">
         <v>39.12</v>
@@ -3878,7 +3878,7 @@
         </is>
       </c>
       <c r="D32" s="16" t="n">
-        <v>12.459124</v>
+        <v>12.463199</v>
       </c>
       <c r="E32" s="17" t="n">
         <v>38.1</v>
@@ -3906,7 +3906,7 @@
         </is>
       </c>
       <c r="D33" s="12" t="n">
-        <v>15.840419</v>
+        <v>15.8456</v>
       </c>
       <c r="E33" s="13" t="n">
         <v>48.44</v>
@@ -3934,7 +3934,7 @@
         </is>
       </c>
       <c r="D34" s="16" t="n">
-        <v>10.448005</v>
+        <v>10.451423</v>
       </c>
       <c r="E34" s="17" t="n">
         <v>31.95</v>
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="D36" s="16" t="n">
-        <v>21.425768</v>
+        <v>21.432777</v>
       </c>
       <c r="E36" s="17" t="n">
         <v>65.52</v>
@@ -4018,7 +4018,7 @@
         </is>
       </c>
       <c r="D37" s="12" t="n">
-        <v>5.333551</v>
+        <v>5.335296</v>
       </c>
       <c r="E37" s="13" t="n">
         <v>16.31</v>
@@ -4046,7 +4046,7 @@
         </is>
       </c>
       <c r="D38" s="16" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E38" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4074,7 +4074,7 @@
         </is>
       </c>
       <c r="D39" s="12" t="n">
-        <v>15.951602</v>
+        <v>15.95682</v>
       </c>
       <c r="E39" s="13" t="n">
         <v>48.78</v>
@@ -4102,7 +4102,7 @@
         </is>
       </c>
       <c r="D40" s="16" t="n">
-        <v>10.336821</v>
+        <v>10.340203</v>
       </c>
       <c r="E40" s="17" t="n">
         <v>31.61</v>
@@ -4130,7 +4130,7 @@
         </is>
       </c>
       <c r="D41" s="12" t="n">
-        <v>31.706998</v>
+        <v>31.71737</v>
       </c>
       <c r="E41" s="13" t="n">
         <v>96.95999999999999</v>
@@ -4158,7 +4158,7 @@
         </is>
       </c>
       <c r="D42" s="16" t="n">
-        <v>34.672989</v>
+        <v>34.684331</v>
       </c>
       <c r="E42" s="17" t="n">
         <v>106.03</v>
@@ -4214,7 +4214,7 @@
         </is>
       </c>
       <c r="D44" s="16" t="n">
-        <v>37.544147</v>
+        <v>37.556428</v>
       </c>
       <c r="E44" s="17" t="n">
         <v>114.81</v>
@@ -4242,7 +4242,7 @@
         </is>
       </c>
       <c r="D45" s="12" t="n">
-        <v>5.209287</v>
+        <v>5.210991</v>
       </c>
       <c r="E45" s="13" t="n">
         <v>15.93</v>
@@ -4270,7 +4270,7 @@
         </is>
       </c>
       <c r="D46" s="16" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E46" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4298,7 +4298,7 @@
         </is>
       </c>
       <c r="D47" s="12" t="n">
-        <v>145.758666</v>
+        <v>145.806346</v>
       </c>
       <c r="E47" s="13" t="n">
         <v>445.73</v>
@@ -4326,7 +4326,7 @@
         </is>
       </c>
       <c r="D48" s="16" t="n">
-        <v>15.624591</v>
+        <v>15.629702</v>
       </c>
       <c r="E48" s="17" t="n">
         <v>47.78</v>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="D49" s="12" t="n">
-        <v>20.241988</v>
+        <v>20.24861</v>
       </c>
       <c r="E49" s="13" t="n">
         <v>61.9</v>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="D50" s="16" t="n">
-        <v>20.768476</v>
+        <v>20.77527</v>
       </c>
       <c r="E50" s="17" t="n">
         <v>63.51</v>
@@ -4410,7 +4410,7 @@
         </is>
       </c>
       <c r="D51" s="12" t="n">
-        <v>20.709614</v>
+        <v>20.716389</v>
       </c>
       <c r="E51" s="13" t="n">
         <v>63.33</v>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="D52" s="16" t="n">
-        <v>16.317855</v>
+        <v>16.323193</v>
       </c>
       <c r="E52" s="17" t="n">
         <v>49.9</v>
@@ -4494,7 +4494,7 @@
         </is>
       </c>
       <c r="D54" s="16" t="n">
-        <v>40.156965</v>
+        <v>40.170101</v>
       </c>
       <c r="E54" s="17" t="n">
         <v>122.8</v>
@@ -4522,7 +4522,7 @@
         </is>
       </c>
       <c r="D55" s="12" t="n">
-        <v>25.57554</v>
+        <v>25.583906</v>
       </c>
       <c r="E55" s="13" t="n">
         <v>78.20999999999999</v>
@@ -4550,7 +4550,7 @@
         </is>
       </c>
       <c r="D56" s="16" t="n">
-        <v>43.81949</v>
+        <v>43.833824</v>
       </c>
       <c r="E56" s="17" t="n">
         <v>134</v>
@@ -4578,7 +4578,7 @@
         </is>
       </c>
       <c r="D57" s="12" t="n">
-        <v>5.045782</v>
+        <v>5.047432</v>
       </c>
       <c r="E57" s="13" t="n">
         <v>15.43</v>
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="D58" s="16" t="n">
-        <v>14.630477</v>
+        <v>14.635263</v>
       </c>
       <c r="E58" s="17" t="n">
         <v>44.74</v>
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="D59" s="12" t="n">
-        <v>25.362982</v>
+        <v>25.371279</v>
       </c>
       <c r="E59" s="13" t="n">
         <v>77.56</v>
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D60" s="16" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E60" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="D61" s="12" t="n">
-        <v>31.841073</v>
+        <v>31.851488</v>
       </c>
       <c r="E61" s="13" t="n">
         <v>97.37</v>
@@ -4718,7 +4718,7 @@
         </is>
       </c>
       <c r="D62" s="16" t="n">
-        <v>16.317855</v>
+        <v>16.323193</v>
       </c>
       <c r="E62" s="17" t="n">
         <v>49.9</v>
@@ -4746,7 +4746,7 @@
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>47.292348</v>
+        <v>47.307818</v>
       </c>
       <c r="E63" s="13" t="n">
         <v>144.62</v>
@@ -4774,7 +4774,7 @@
         </is>
       </c>
       <c r="D64" s="16" t="n">
-        <v>20.186396</v>
+        <v>20.193</v>
       </c>
       <c r="E64" s="17" t="n">
         <v>61.73</v>
@@ -4802,7 +4802,7 @@
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>5.049052</v>
+        <v>5.050703</v>
       </c>
       <c r="E65" s="13" t="n">
         <v>15.44</v>
@@ -4858,7 +4858,7 @@
         </is>
       </c>
       <c r="D67" s="12" t="n">
-        <v>20.457816</v>
+        <v>20.464508</v>
       </c>
       <c r="E67" s="13" t="n">
         <v>62.56</v>
@@ -4886,7 +4886,7 @@
         </is>
       </c>
       <c r="D68" s="16" t="n">
-        <v>50.673643</v>
+        <v>50.690219</v>
       </c>
       <c r="E68" s="17" t="n">
         <v>154.96</v>
@@ -4914,7 +4914,7 @@
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>51.687377</v>
+        <v>51.704285</v>
       </c>
       <c r="E69" s="13" t="n">
         <v>158.06</v>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>5.127534</v>
+        <v>5.129212</v>
       </c>
       <c r="E70" s="17" t="n">
         <v>15.68</v>
@@ -4970,7 +4970,7 @@
         </is>
       </c>
       <c r="D71" s="12" t="n">
-        <v>10.251799</v>
+        <v>10.255152</v>
       </c>
       <c r="E71" s="13" t="n">
         <v>31.35</v>
@@ -4998,7 +4998,7 @@
         </is>
       </c>
       <c r="D72" s="16" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E72" s="17" t="n">
         <v>75.90000000000001</v>
@@ -5026,7 +5026,7 @@
         </is>
       </c>
       <c r="D73" s="12" t="n">
-        <v>10.228908</v>
+        <v>10.232254</v>
       </c>
       <c r="E73" s="13" t="n">
         <v>31.28</v>
@@ -5054,7 +5054,7 @@
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>14.833224</v>
+        <v>14.838077</v>
       </c>
       <c r="E74" s="17" t="n">
         <v>45.36</v>
@@ -5082,7 +5082,7 @@
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E75" s="13" t="n">
         <v>75.90000000000001</v>
@@ -5110,7 +5110,7 @@
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>10.202747</v>
+        <v>10.206084</v>
       </c>
       <c r="E76" s="17" t="n">
         <v>31.2</v>
@@ -5138,7 +5138,7 @@
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>40.362982</v>
+        <v>40.376186</v>
       </c>
       <c r="E77" s="13" t="n">
         <v>123.43</v>
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>16.317855</v>
+        <v>16.323193</v>
       </c>
       <c r="E78" s="17" t="n">
         <v>49.9</v>
@@ -5194,7 +5194,7 @@
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>52.213865</v>
+        <v>52.230945</v>
       </c>
       <c r="E79" s="13" t="n">
         <v>159.67</v>
@@ -5222,7 +5222,7 @@
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>20.559189</v>
+        <v>20.565914</v>
       </c>
       <c r="E80" s="17" t="n">
         <v>62.87</v>
@@ -5278,7 +5278,7 @@
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>10.173316</v>
+        <v>10.176644</v>
       </c>
       <c r="E82" s="17" t="n">
         <v>31.11</v>
@@ -5306,7 +5306,7 @@
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>11.19032</v>
+        <v>11.193981</v>
       </c>
       <c r="E83" s="13" t="n">
         <v>34.22</v>
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>5.107914</v>
+        <v>5.109585</v>
       </c>
       <c r="E85" s="13" t="n">
         <v>15.62</v>
@@ -5418,7 +5418,7 @@
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>20.559189</v>
+        <v>20.565914</v>
       </c>
       <c r="E87" s="13" t="n">
         <v>62.87</v>
@@ -5446,7 +5446,7 @@
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>5.140615</v>
+        <v>5.142296</v>
       </c>
       <c r="E88" s="17" t="n">
         <v>15.72</v>
@@ -5474,7 +5474,7 @@
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E89" s="13" t="n">
         <v>75.90000000000001</v>
@@ -5502,7 +5502,7 @@
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>54.391759</v>
+        <v>54.409552</v>
       </c>
       <c r="E90" s="17" t="n">
         <v>166.33</v>
@@ -5558,7 +5558,7 @@
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>2.305428</v>
+        <v>2.306183</v>
       </c>
       <c r="E92" s="17" t="n">
         <v>7.05</v>
@@ -5586,7 +5586,7 @@
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>20.546109</v>
+        <v>20.55283</v>
       </c>
       <c r="E93" s="13" t="n">
         <v>62.83</v>
@@ -5614,7 +5614,7 @@
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>16.317855</v>
+        <v>16.323193</v>
       </c>
       <c r="E94" s="17" t="n">
         <v>49.9</v>
@@ -5645,7 +5645,7 @@
         <v>20</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
         <v>20</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -5701,7 +5701,7 @@
         <v>20</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
         <v>20</v>
       </c>
       <c r="E98" s="17" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
@@ -5757,7 +5757,7 @@
         <v>20</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v>20</v>
       </c>
       <c r="E100" s="17" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
@@ -5813,7 +5813,7 @@
         <v>20</v>
       </c>
       <c r="E101" s="13" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
@@ -5841,7 +5841,7 @@
         <v>20</v>
       </c>
       <c r="E102" s="17" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
@@ -5869,7 +5869,7 @@
         <v>20</v>
       </c>
       <c r="E103" s="13" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
@@ -5989,7 +5989,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>61.14</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -10627,7 +10627,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>1.092217</v>
+        <v>1.092574</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>3.34</v>
@@ -10651,7 +10651,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>78.83584</v>
+        <v>78.86162899999999</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>241.08</v>
@@ -10675,7 +10675,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>11.45847</v>
+        <v>11.462218</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35.04</v>
@@ -10699,7 +10699,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>21.680837</v>
+        <v>21.687929</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>66.3</v>
@@ -10747,7 +10747,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>14.823414</v>
+        <v>14.828263</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>45.33</v>
@@ -10771,7 +10771,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>124.545455</v>
+        <v>124.586196</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>380.86</v>
@@ -10795,7 +10795,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>11.007194</v>
+        <v>11.010795</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>33.66</v>
@@ -10914,7 +10914,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>18.616743</v>
+        <v>18.622833</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -10938,7 +10938,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>16.739699</v>
+        <v>16.745175</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>51.19</v>
@@ -10962,7 +10962,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>13.381295</v>
+        <v>13.385672</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>40.92</v>
@@ -10986,7 +10986,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>1.007194</v>
+        <v>1.007524</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>3.08</v>
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>21.334205</v>
+        <v>21.341184</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>65.23999999999999</v>
@@ -11034,7 +11034,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>11.890124</v>
+        <v>11.894014</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>36.36</v>
@@ -11058,7 +11058,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>22.377371</v>
+        <v>22.384691</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>68.43000000000001</v>
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>5.464356</v>
+        <v>5.466143</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>16.71</v>
@@ -11130,7 +11130,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>12.295618</v>
+        <v>12.29964</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>37.6</v>
@@ -11249,7 +11249,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>18.616743</v>
+        <v>18.622833</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11273,7 +11273,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>3.054284</v>
+        <v>3.055283</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>9.34</v>
@@ -11297,7 +11297,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>11.579464</v>
+        <v>11.583252</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35.41</v>
@@ -11345,7 +11345,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>21.863963</v>
+        <v>21.871115</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>66.86</v>
@@ -11369,7 +11369,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>5.398954</v>
+        <v>5.40072</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>16.51</v>
@@ -11488,7 +11488,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>18.616743</v>
+        <v>18.622833</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11536,7 +11536,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>21.517332</v>
+        <v>21.52437</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>65.8</v>
@@ -11560,7 +11560,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>5.320471</v>
+        <v>5.322211</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>16.27</v>
@@ -11679,7 +11679,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>12.792675</v>
+        <v>12.79686</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>39.12</v>
@@ -11703,7 +11703,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>12.459124</v>
+        <v>12.463199</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>38.1</v>
@@ -11727,7 +11727,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15.840419</v>
+        <v>15.8456</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>48.44</v>
@@ -11751,7 +11751,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>10.448005</v>
+        <v>10.451423</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>31.95</v>
@@ -11799,7 +11799,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>21.425768</v>
+        <v>21.432777</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>65.52</v>
@@ -11823,7 +11823,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5.333551</v>
+        <v>5.335296</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>16.31</v>
@@ -11942,7 +11942,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -11966,7 +11966,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>15.951602</v>
+        <v>15.95682</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>48.78</v>
@@ -11990,7 +11990,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>10.336821</v>
+        <v>10.340203</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>31.61</v>
@@ -12014,7 +12014,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>31.706998</v>
+        <v>31.71737</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>96.95999999999999</v>
@@ -12038,7 +12038,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>34.672989</v>
+        <v>34.684331</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>106.03</v>
@@ -12086,7 +12086,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>37.544147</v>
+        <v>37.556428</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>114.81</v>
@@ -12110,7 +12110,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>5.209287</v>
+        <v>5.210991</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>15.93</v>
@@ -12229,7 +12229,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>24.820144</v>
+        <v>24.828263</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -12253,7 +12253,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>145.758666</v>
+        <v>145.806346</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>445.73</v>
@@ -12277,7 +12277,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15.624591</v>
+        <v>15.629702</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>47.78</v>
@@ -12301,7 +12301,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>20.241988</v>
+        <v>20.24861</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>61.9</v>
@@ -12325,7 +12325,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>20.768476</v>
+        <v>20.77527</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>63.51</v>
@@ -12349,7 +12349,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20.709614</v>
+        <v>20.716389</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>63.33</v>
@@ -12373,7 +12373,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.317855</v>
+        <v>16.323193</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -12421,7 +12421,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>40.156965</v>
+        <v>40.170101</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>122.8</v>
@@ -12445,7 +12445,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>25.57554</v>
+        <v>25.583906</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>78.20999999999999</v>
@@ -12469,7 +12469,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>43.81949</v>
+        <v>43.833824</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>134</v>
@@ -12493,7 +12493,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.045782</v>
+        <v>5.047432</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>15.43</v>
@@ -12517,7 +12517,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>14.630477</v>
+        <v>14.635263</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>44.74</v>

</xml_diff>

<commit_message>
Auto: Gmail scan – no new invoices
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -939,11 +939,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>3.058</v>
+        <v>3.019</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-13</t>
+          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-14</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.362982</v>
+        <v>25.690626</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>77.56</v>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1116,7 +1116,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>31.841073</v>
+        <v>32.252401</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>97.37</v>
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>16.317855</v>
+        <v>16.528652</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>49.9</v>
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>47.292348</v>
+        <v>47.903279</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>144.62</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20.186396</v>
+        <v>20.447168</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>61.73</v>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5.049052</v>
+        <v>5.114276</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>15.44</v>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20.457816</v>
+        <v>20.722093</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>62.56</v>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>50.673643</v>
+        <v>51.328254</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>154.96</v>
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>51.687377</v>
+        <v>52.355084</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>158.06</v>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.127534</v>
+        <v>5.193773</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>15.68</v>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>10.251799</v>
+        <v>10.384233</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>31.35</v>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>10.228908</v>
+        <v>10.361047</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>31.28</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>14.833224</v>
+        <v>15.024843</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>45.36</v>
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>10.202747</v>
+        <v>10.334548</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>31.2</v>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>40.362982</v>
+        <v>40.884399</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>123.43</v>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.317855</v>
+        <v>16.528652</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>52.213865</v>
+        <v>52.888374</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>159.67</v>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20.559189</v>
+        <v>20.824776</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>62.87</v>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>10.173316</v>
+        <v>10.304737</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>31.11</v>
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>11.19032</v>
+        <v>11.334879</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>34.22</v>
@@ -1787,7 +1787,7 @@
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>5.107914</v>
+        <v>5.173899</v>
       </c>
       <c r="E17" s="28" t="n">
         <v>15.62</v>
@@ -1930,7 +1930,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>20.559189</v>
+        <v>20.824776</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>62.87</v>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>5.140615</v>
+        <v>5.207022</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>15.72</v>
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>75.90000000000001</v>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>54.391759</v>
+        <v>55.094402</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>166.33</v>
@@ -2050,7 +2050,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>2.305428</v>
+        <v>2.33521</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>7.05</v>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>20.546109</v>
+        <v>20.811527</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>62.83</v>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>16.317855</v>
+        <v>16.528652</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>49.9</v>
@@ -2125,7 +2125,7 @@
         <v>20</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -2244,7 +2244,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2363,7 +2363,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2482,7 +2482,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2601,7 +2601,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2720,7 +2720,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2839,7 +2839,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2958,7 +2958,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="D3" s="12" t="n">
-        <v>1.092217</v>
+        <v>1.106327</v>
       </c>
       <c r="E3" s="13" t="n">
         <v>3.34</v>
@@ -3094,7 +3094,7 @@
         </is>
       </c>
       <c r="D4" s="16" t="n">
-        <v>78.83584</v>
+        <v>79.85425600000001</v>
       </c>
       <c r="E4" s="17" t="n">
         <v>241.08</v>
@@ -3122,7 +3122,7 @@
         </is>
       </c>
       <c r="D5" s="12" t="n">
-        <v>11.45847</v>
+        <v>11.606492</v>
       </c>
       <c r="E5" s="13" t="n">
         <v>35.04</v>
@@ -3150,7 +3150,7 @@
         </is>
       </c>
       <c r="D6" s="16" t="n">
-        <v>21.680837</v>
+        <v>21.960914</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>66.3</v>
@@ -3206,7 +3206,7 @@
         </is>
       </c>
       <c r="D8" s="16" t="n">
-        <v>14.823414</v>
+        <v>15.014906</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>45.33</v>
@@ -3234,7 +3234,7 @@
         </is>
       </c>
       <c r="D9" s="12" t="n">
-        <v>124.545455</v>
+        <v>126.154356</v>
       </c>
       <c r="E9" s="13" t="n">
         <v>380.86</v>
@@ -3262,7 +3262,7 @@
         </is>
       </c>
       <c r="D10" s="16" t="n">
-        <v>11.007194</v>
+        <v>11.149387</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>33.66</v>
@@ -3290,7 +3290,7 @@
         </is>
       </c>
       <c r="D11" s="12" t="n">
-        <v>18.616743</v>
+        <v>18.857237</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>56.93</v>
@@ -3318,7 +3318,7 @@
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>16.739699</v>
+        <v>16.955946</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>51.19</v>
@@ -3346,7 +3346,7 @@
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>13.381295</v>
+        <v>13.554157</v>
       </c>
       <c r="E13" s="13" t="n">
         <v>40.92</v>
@@ -3374,7 +3374,7 @@
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>1.007194</v>
+        <v>1.020205</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>3.08</v>
@@ -3402,7 +3402,7 @@
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>21.334205</v>
+        <v>21.609805</v>
       </c>
       <c r="E15" s="13" t="n">
         <v>65.23999999999999</v>
@@ -3430,7 +3430,7 @@
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>11.890124</v>
+        <v>12.043723</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>36.36</v>
@@ -3458,7 +3458,7 @@
         </is>
       </c>
       <c r="D17" s="12" t="n">
-        <v>22.377371</v>
+        <v>22.666446</v>
       </c>
       <c r="E17" s="13" t="n">
         <v>68.43000000000001</v>
@@ -3514,7 +3514,7 @@
         </is>
       </c>
       <c r="D19" s="12" t="n">
-        <v>5.464356</v>
+        <v>5.534945</v>
       </c>
       <c r="E19" s="13" t="n">
         <v>16.71</v>
@@ -3542,7 +3542,7 @@
         </is>
       </c>
       <c r="D20" s="16" t="n">
-        <v>12.295618</v>
+        <v>12.454455</v>
       </c>
       <c r="E20" s="17" t="n">
         <v>37.6</v>
@@ -3570,7 +3570,7 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>18.616743</v>
+        <v>18.857237</v>
       </c>
       <c r="E21" s="13" t="n">
         <v>56.93</v>
@@ -3598,7 +3598,7 @@
         </is>
       </c>
       <c r="D22" s="16" t="n">
-        <v>3.054284</v>
+        <v>3.09374</v>
       </c>
       <c r="E22" s="17" t="n">
         <v>9.34</v>
@@ -3626,7 +3626,7 @@
         </is>
       </c>
       <c r="D23" s="12" t="n">
-        <v>11.579464</v>
+        <v>11.729049</v>
       </c>
       <c r="E23" s="13" t="n">
         <v>35.41</v>
@@ -3682,7 +3682,7 @@
         </is>
       </c>
       <c r="D25" s="12" t="n">
-        <v>21.863963</v>
+        <v>22.146406</v>
       </c>
       <c r="E25" s="13" t="n">
         <v>66.86</v>
@@ -3710,7 +3710,7 @@
         </is>
       </c>
       <c r="D26" s="16" t="n">
-        <v>5.398954</v>
+        <v>5.468698</v>
       </c>
       <c r="E26" s="17" t="n">
         <v>16.51</v>
@@ -3738,7 +3738,7 @@
         </is>
       </c>
       <c r="D27" s="12" t="n">
-        <v>18.616743</v>
+        <v>18.857237</v>
       </c>
       <c r="E27" s="13" t="n">
         <v>56.93</v>
@@ -3794,7 +3794,7 @@
         </is>
       </c>
       <c r="D29" s="12" t="n">
-        <v>21.517332</v>
+        <v>21.795296</v>
       </c>
       <c r="E29" s="13" t="n">
         <v>65.8</v>
@@ -3822,7 +3822,7 @@
         </is>
       </c>
       <c r="D30" s="16" t="n">
-        <v>5.320471</v>
+        <v>5.389202</v>
       </c>
       <c r="E30" s="17" t="n">
         <v>16.27</v>
@@ -3850,7 +3850,7 @@
         </is>
       </c>
       <c r="D31" s="12" t="n">
-        <v>12.792675</v>
+        <v>12.957933</v>
       </c>
       <c r="E31" s="13" t="n">
         <v>39.12</v>
@@ -3878,7 +3878,7 @@
         </is>
       </c>
       <c r="D32" s="16" t="n">
-        <v>12.459124</v>
+        <v>12.620073</v>
       </c>
       <c r="E32" s="17" t="n">
         <v>38.1</v>
@@ -3906,7 +3906,7 @@
         </is>
       </c>
       <c r="D33" s="12" t="n">
-        <v>15.840419</v>
+        <v>16.045048</v>
       </c>
       <c r="E33" s="13" t="n">
         <v>48.44</v>
@@ -3934,7 +3934,7 @@
         </is>
       </c>
       <c r="D34" s="16" t="n">
-        <v>10.448005</v>
+        <v>10.582974</v>
       </c>
       <c r="E34" s="17" t="n">
         <v>31.95</v>
@@ -3990,7 +3990,7 @@
         </is>
       </c>
       <c r="D36" s="16" t="n">
-        <v>21.425768</v>
+        <v>21.702551</v>
       </c>
       <c r="E36" s="17" t="n">
         <v>65.52</v>
@@ -4018,7 +4018,7 @@
         </is>
       </c>
       <c r="D37" s="12" t="n">
-        <v>5.333551</v>
+        <v>5.402451</v>
       </c>
       <c r="E37" s="13" t="n">
         <v>16.31</v>
@@ -4046,7 +4046,7 @@
         </is>
       </c>
       <c r="D38" s="16" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E38" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4074,7 +4074,7 @@
         </is>
       </c>
       <c r="D39" s="12" t="n">
-        <v>15.951602</v>
+        <v>16.157668</v>
       </c>
       <c r="E39" s="13" t="n">
         <v>48.78</v>
@@ -4102,7 +4102,7 @@
         </is>
       </c>
       <c r="D40" s="16" t="n">
-        <v>10.336821</v>
+        <v>10.470354</v>
       </c>
       <c r="E40" s="17" t="n">
         <v>31.61</v>
@@ -4130,7 +4130,7 @@
         </is>
       </c>
       <c r="D41" s="12" t="n">
-        <v>31.706998</v>
+        <v>32.116595</v>
       </c>
       <c r="E41" s="13" t="n">
         <v>96.95999999999999</v>
@@ -4158,7 +4158,7 @@
         </is>
       </c>
       <c r="D42" s="16" t="n">
-        <v>34.672989</v>
+        <v>35.120901</v>
       </c>
       <c r="E42" s="17" t="n">
         <v>106.03</v>
@@ -4214,7 +4214,7 @@
         </is>
       </c>
       <c r="D44" s="16" t="n">
-        <v>37.544147</v>
+        <v>38.029149</v>
       </c>
       <c r="E44" s="17" t="n">
         <v>114.81</v>
@@ -4242,7 +4242,7 @@
         </is>
       </c>
       <c r="D45" s="12" t="n">
-        <v>5.209287</v>
+        <v>5.276582</v>
       </c>
       <c r="E45" s="13" t="n">
         <v>15.93</v>
@@ -4270,7 +4270,7 @@
         </is>
       </c>
       <c r="D46" s="16" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E46" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4298,7 +4298,7 @@
         </is>
       </c>
       <c r="D47" s="12" t="n">
-        <v>145.758666</v>
+        <v>147.641603</v>
       </c>
       <c r="E47" s="13" t="n">
         <v>445.73</v>
@@ -4326,7 +4326,7 @@
         </is>
       </c>
       <c r="D48" s="16" t="n">
-        <v>15.624591</v>
+        <v>15.826433</v>
       </c>
       <c r="E48" s="17" t="n">
         <v>47.78</v>
@@ -4354,7 +4354,7 @@
         </is>
       </c>
       <c r="D49" s="12" t="n">
-        <v>20.241988</v>
+        <v>20.503478</v>
       </c>
       <c r="E49" s="13" t="n">
         <v>61.9</v>
@@ -4382,7 +4382,7 @@
         </is>
       </c>
       <c r="D50" s="16" t="n">
-        <v>20.768476</v>
+        <v>21.036767</v>
       </c>
       <c r="E50" s="17" t="n">
         <v>63.51</v>
@@ -4410,7 +4410,7 @@
         </is>
       </c>
       <c r="D51" s="12" t="n">
-        <v>20.709614</v>
+        <v>20.977145</v>
       </c>
       <c r="E51" s="13" t="n">
         <v>63.33</v>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="D52" s="16" t="n">
-        <v>16.317855</v>
+        <v>16.528652</v>
       </c>
       <c r="E52" s="17" t="n">
         <v>49.9</v>
@@ -4494,7 +4494,7 @@
         </is>
       </c>
       <c r="D54" s="16" t="n">
-        <v>40.156965</v>
+        <v>40.67572</v>
       </c>
       <c r="E54" s="17" t="n">
         <v>122.8</v>
@@ -4522,7 +4522,7 @@
         </is>
       </c>
       <c r="D55" s="12" t="n">
-        <v>25.57554</v>
+        <v>25.905929</v>
       </c>
       <c r="E55" s="13" t="n">
         <v>78.20999999999999</v>
@@ -4550,7 +4550,7 @@
         </is>
       </c>
       <c r="D56" s="16" t="n">
-        <v>43.81949</v>
+        <v>44.385558</v>
       </c>
       <c r="E56" s="17" t="n">
         <v>134</v>
@@ -4578,7 +4578,7 @@
         </is>
       </c>
       <c r="D57" s="12" t="n">
-        <v>5.045782</v>
+        <v>5.110964</v>
       </c>
       <c r="E57" s="13" t="n">
         <v>15.43</v>
@@ -4606,7 +4606,7 @@
         </is>
       </c>
       <c r="D58" s="16" t="n">
-        <v>14.630477</v>
+        <v>14.819477</v>
       </c>
       <c r="E58" s="17" t="n">
         <v>44.74</v>
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="D59" s="12" t="n">
-        <v>25.362982</v>
+        <v>25.690626</v>
       </c>
       <c r="E59" s="13" t="n">
         <v>77.56</v>
@@ -4662,7 +4662,7 @@
         </is>
       </c>
       <c r="D60" s="16" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E60" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4690,7 +4690,7 @@
         </is>
       </c>
       <c r="D61" s="12" t="n">
-        <v>31.841073</v>
+        <v>32.252401</v>
       </c>
       <c r="E61" s="13" t="n">
         <v>97.37</v>
@@ -4718,7 +4718,7 @@
         </is>
       </c>
       <c r="D62" s="16" t="n">
-        <v>16.317855</v>
+        <v>16.528652</v>
       </c>
       <c r="E62" s="17" t="n">
         <v>49.9</v>
@@ -4746,7 +4746,7 @@
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>47.292348</v>
+        <v>47.903279</v>
       </c>
       <c r="E63" s="13" t="n">
         <v>144.62</v>
@@ -4774,7 +4774,7 @@
         </is>
       </c>
       <c r="D64" s="16" t="n">
-        <v>20.186396</v>
+        <v>20.447168</v>
       </c>
       <c r="E64" s="17" t="n">
         <v>61.73</v>
@@ -4802,7 +4802,7 @@
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>5.049052</v>
+        <v>5.114276</v>
       </c>
       <c r="E65" s="13" t="n">
         <v>15.44</v>
@@ -4858,7 +4858,7 @@
         </is>
       </c>
       <c r="D67" s="12" t="n">
-        <v>20.457816</v>
+        <v>20.722093</v>
       </c>
       <c r="E67" s="13" t="n">
         <v>62.56</v>
@@ -4886,7 +4886,7 @@
         </is>
       </c>
       <c r="D68" s="16" t="n">
-        <v>50.673643</v>
+        <v>51.328254</v>
       </c>
       <c r="E68" s="17" t="n">
         <v>154.96</v>
@@ -4914,7 +4914,7 @@
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>51.687377</v>
+        <v>52.355084</v>
       </c>
       <c r="E69" s="13" t="n">
         <v>158.06</v>
@@ -4942,7 +4942,7 @@
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>5.127534</v>
+        <v>5.193773</v>
       </c>
       <c r="E70" s="17" t="n">
         <v>15.68</v>
@@ -4970,7 +4970,7 @@
         </is>
       </c>
       <c r="D71" s="12" t="n">
-        <v>10.251799</v>
+        <v>10.384233</v>
       </c>
       <c r="E71" s="13" t="n">
         <v>31.35</v>
@@ -4998,7 +4998,7 @@
         </is>
       </c>
       <c r="D72" s="16" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E72" s="17" t="n">
         <v>75.90000000000001</v>
@@ -5026,7 +5026,7 @@
         </is>
       </c>
       <c r="D73" s="12" t="n">
-        <v>10.228908</v>
+        <v>10.361047</v>
       </c>
       <c r="E73" s="13" t="n">
         <v>31.28</v>
@@ -5054,7 +5054,7 @@
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>14.833224</v>
+        <v>15.024843</v>
       </c>
       <c r="E74" s="17" t="n">
         <v>45.36</v>
@@ -5082,7 +5082,7 @@
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E75" s="13" t="n">
         <v>75.90000000000001</v>
@@ -5110,7 +5110,7 @@
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>10.202747</v>
+        <v>10.334548</v>
       </c>
       <c r="E76" s="17" t="n">
         <v>31.2</v>
@@ -5138,7 +5138,7 @@
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>40.362982</v>
+        <v>40.884399</v>
       </c>
       <c r="E77" s="13" t="n">
         <v>123.43</v>
@@ -5166,7 +5166,7 @@
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>16.317855</v>
+        <v>16.528652</v>
       </c>
       <c r="E78" s="17" t="n">
         <v>49.9</v>
@@ -5194,7 +5194,7 @@
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>52.213865</v>
+        <v>52.888374</v>
       </c>
       <c r="E79" s="13" t="n">
         <v>159.67</v>
@@ -5222,7 +5222,7 @@
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>20.559189</v>
+        <v>20.824776</v>
       </c>
       <c r="E80" s="17" t="n">
         <v>62.87</v>
@@ -5278,7 +5278,7 @@
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>10.173316</v>
+        <v>10.304737</v>
       </c>
       <c r="E82" s="17" t="n">
         <v>31.11</v>
@@ -5306,7 +5306,7 @@
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>11.19032</v>
+        <v>11.334879</v>
       </c>
       <c r="E83" s="13" t="n">
         <v>34.22</v>
@@ -5362,7 +5362,7 @@
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>5.107914</v>
+        <v>5.173899</v>
       </c>
       <c r="E85" s="13" t="n">
         <v>15.62</v>
@@ -5418,7 +5418,7 @@
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>20.559189</v>
+        <v>20.824776</v>
       </c>
       <c r="E87" s="13" t="n">
         <v>62.87</v>
@@ -5446,7 +5446,7 @@
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>5.140615</v>
+        <v>5.207022</v>
       </c>
       <c r="E88" s="17" t="n">
         <v>15.72</v>
@@ -5474,7 +5474,7 @@
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E89" s="13" t="n">
         <v>75.90000000000001</v>
@@ -5502,7 +5502,7 @@
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>54.391759</v>
+        <v>55.094402</v>
       </c>
       <c r="E90" s="17" t="n">
         <v>166.33</v>
@@ -5558,7 +5558,7 @@
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>2.305428</v>
+        <v>2.33521</v>
       </c>
       <c r="E92" s="17" t="n">
         <v>7.05</v>
@@ -5586,7 +5586,7 @@
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>20.546109</v>
+        <v>20.811527</v>
       </c>
       <c r="E93" s="13" t="n">
         <v>62.83</v>
@@ -5614,7 +5614,7 @@
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>16.317855</v>
+        <v>16.528652</v>
       </c>
       <c r="E94" s="17" t="n">
         <v>49.9</v>
@@ -5645,7 +5645,7 @@
         <v>20</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
@@ -5673,7 +5673,7 @@
         <v>20</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -5701,7 +5701,7 @@
         <v>20</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -5729,7 +5729,7 @@
         <v>20</v>
       </c>
       <c r="E98" s="17" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
@@ -5757,7 +5757,7 @@
         <v>20</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
@@ -5785,7 +5785,7 @@
         <v>20</v>
       </c>
       <c r="E100" s="17" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
@@ -5813,7 +5813,7 @@
         <v>20</v>
       </c>
       <c r="E101" s="13" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
@@ -5841,7 +5841,7 @@
         <v>20</v>
       </c>
       <c r="E102" s="17" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
@@ -5869,7 +5869,7 @@
         <v>20</v>
       </c>
       <c r="E103" s="13" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
@@ -5989,7 +5989,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>61.16</v>
+        <v>60.38</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -10627,7 +10627,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>1.092217</v>
+        <v>1.106327</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>3.34</v>
@@ -10651,7 +10651,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>78.83584</v>
+        <v>79.85425600000001</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>241.08</v>
@@ -10675,7 +10675,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>11.45847</v>
+        <v>11.606492</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35.04</v>
@@ -10699,7 +10699,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>21.680837</v>
+        <v>21.960914</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>66.3</v>
@@ -10747,7 +10747,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>14.823414</v>
+        <v>15.014906</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>45.33</v>
@@ -10771,7 +10771,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>124.545455</v>
+        <v>126.154356</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>380.86</v>
@@ -10795,7 +10795,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>11.007194</v>
+        <v>11.149387</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>33.66</v>
@@ -10914,7 +10914,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>18.616743</v>
+        <v>18.857237</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -10938,7 +10938,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>16.739699</v>
+        <v>16.955946</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>51.19</v>
@@ -10962,7 +10962,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>13.381295</v>
+        <v>13.554157</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>40.92</v>
@@ -10986,7 +10986,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>1.007194</v>
+        <v>1.020205</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>3.08</v>
@@ -11010,7 +11010,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>21.334205</v>
+        <v>21.609805</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>65.23999999999999</v>
@@ -11034,7 +11034,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>11.890124</v>
+        <v>12.043723</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>36.36</v>
@@ -11058,7 +11058,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>22.377371</v>
+        <v>22.666446</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>68.43000000000001</v>
@@ -11106,7 +11106,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>5.464356</v>
+        <v>5.534945</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>16.71</v>
@@ -11130,7 +11130,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>12.295618</v>
+        <v>12.454455</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>37.6</v>
@@ -11249,7 +11249,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>18.616743</v>
+        <v>18.857237</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11273,7 +11273,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>3.054284</v>
+        <v>3.09374</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>9.34</v>
@@ -11297,7 +11297,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>11.579464</v>
+        <v>11.729049</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35.41</v>
@@ -11345,7 +11345,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>21.863963</v>
+        <v>22.146406</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>66.86</v>
@@ -11369,7 +11369,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>5.398954</v>
+        <v>5.468698</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>16.51</v>
@@ -11488,7 +11488,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>18.616743</v>
+        <v>18.857237</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11536,7 +11536,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>21.517332</v>
+        <v>21.795296</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>65.8</v>
@@ -11560,7 +11560,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>5.320471</v>
+        <v>5.389202</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>16.27</v>
@@ -11679,7 +11679,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>12.792675</v>
+        <v>12.957933</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>39.12</v>
@@ -11703,7 +11703,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>12.459124</v>
+        <v>12.620073</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>38.1</v>
@@ -11727,7 +11727,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15.840419</v>
+        <v>16.045048</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>48.44</v>
@@ -11751,7 +11751,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>10.448005</v>
+        <v>10.582974</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>31.95</v>
@@ -11799,7 +11799,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>21.425768</v>
+        <v>21.702551</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>65.52</v>
@@ -11823,7 +11823,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5.333551</v>
+        <v>5.402451</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>16.31</v>
@@ -11942,7 +11942,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -11966,7 +11966,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>15.951602</v>
+        <v>16.157668</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>48.78</v>
@@ -11990,7 +11990,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>10.336821</v>
+        <v>10.470354</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>31.61</v>
@@ -12014,7 +12014,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>31.706998</v>
+        <v>32.116595</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>96.95999999999999</v>
@@ -12038,7 +12038,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>34.672989</v>
+        <v>35.120901</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>106.03</v>
@@ -12086,7 +12086,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>37.544147</v>
+        <v>38.029149</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>114.81</v>
@@ -12110,7 +12110,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>5.209287</v>
+        <v>5.276582</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>15.93</v>
@@ -12229,7 +12229,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>24.820144</v>
+        <v>25.140775</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -12253,7 +12253,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>145.758666</v>
+        <v>147.641603</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>445.73</v>
@@ -12277,7 +12277,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15.624591</v>
+        <v>15.826433</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>47.78</v>
@@ -12301,7 +12301,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>20.241988</v>
+        <v>20.503478</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>61.9</v>
@@ -12325,7 +12325,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>20.768476</v>
+        <v>21.036767</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>63.51</v>
@@ -12349,7 +12349,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20.709614</v>
+        <v>20.977145</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>63.33</v>
@@ -12373,7 +12373,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.317855</v>
+        <v>16.528652</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -12421,7 +12421,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>40.156965</v>
+        <v>40.67572</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>122.8</v>
@@ -12445,7 +12445,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>25.57554</v>
+        <v>25.905929</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>78.20999999999999</v>
@@ -12469,7 +12469,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>43.81949</v>
+        <v>44.385558</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>134</v>
@@ -12493,7 +12493,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.045782</v>
+        <v>5.110964</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>15.43</v>
@@ -12517,7 +12517,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>14.630477</v>
+        <v>14.819477</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>44.74</v>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-04-15
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1855,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2108,17 +2108,17 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
@@ -2129,27 +2129,51 @@
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="30" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>60.28</v>
+      </c>
+      <c r="F13" s="29" t="n"/>
+    </row>
+    <row r="14" ht="24" customHeight="1">
+      <c r="A14" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B13" s="31" t="n"/>
-      <c r="C13" s="31" t="n"/>
-      <c r="D13" s="20">
-        <f>SUM(D4:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="21">
-        <f>SUM(E4:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="31" t="n"/>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="31" t="n"/>
+      <c r="D14" s="20">
+        <f>SUM(D4:D13)</f>
+        <v/>
+      </c>
+      <c r="E14" s="21">
+        <f>SUM(E4:E13)</f>
+        <v/>
+      </c>
+      <c r="F14" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A14:C14"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -2999,7 +3023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F104"/>
+  <dimension ref="A1:F105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5628,17 +5652,17 @@
     <row r="95">
       <c r="A95" s="10" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
@@ -5656,7 +5680,7 @@
     <row r="96">
       <c r="A96" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B96" s="15" t="inlineStr">
@@ -5677,14 +5701,14 @@
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5705,14 +5729,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5733,14 +5757,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5761,14 +5785,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5789,14 +5813,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5817,14 +5841,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5845,14 +5869,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5873,32 +5897,60 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C104" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D104" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E104" s="17" t="n">
+        <v>60.28</v>
+      </c>
+      <c r="F104" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="18" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B104" s="19" t="n"/>
-      <c r="C104" s="19" t="n"/>
-      <c r="D104" s="20">
-        <f>SUM(D3:D103)</f>
-        <v/>
-      </c>
-      <c r="E104" s="21">
-        <f>SUM(E3:E103)</f>
-        <v/>
-      </c>
-      <c r="F104" s="19" t="n"/>
+      <c r="B105" s="19" t="n"/>
+      <c r="C105" s="19" t="n"/>
+      <c r="D105" s="20">
+        <f>SUM(D3:D104)</f>
+        <v/>
+      </c>
+      <c r="E105" s="21">
+        <f>SUM(E3:E104)</f>
+        <v/>
+      </c>
+      <c r="F105" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A104:C104"/>
+    <mergeCell ref="A105:C105"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-04-16
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1855,7 +1855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2137,43 +2137,67 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>29.95</v>
+      </c>
+      <c r="F13" s="29" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-16</t>
+        </is>
+      </c>
+      <c r="B14" s="15" t="inlineStr">
+        <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D13" s="27" t="n">
+      <c r="D14" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E13" s="28" t="n">
+      <c r="E14" s="26" t="n">
         <v>59.9</v>
       </c>
-      <c r="F13" s="29" t="n"/>
-    </row>
-    <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="F14" s="24" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="31" t="n"/>
-      <c r="D14" s="20">
-        <f>SUM(D4:D13)</f>
-        <v/>
-      </c>
-      <c r="E14" s="21">
-        <f>SUM(E4:E13)</f>
-        <v/>
-      </c>
-      <c r="F14" s="31" t="n"/>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="20">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f>SUM(E4:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3023,7 +3047,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F105"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5685,19 +5709,19 @@
       </c>
       <c r="B96" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="D96" s="16" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>59.9</v>
+        <v>29.95</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -5708,7 +5732,7 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
@@ -5729,14 +5753,14 @@
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
@@ -5757,14 +5781,14 @@
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5785,14 +5809,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5813,14 +5837,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5841,14 +5865,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5869,14 +5893,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5897,14 +5921,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5925,32 +5949,60 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B105" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C105" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D105" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E105" s="13" t="n">
+        <v>59.9</v>
+      </c>
+      <c r="F105" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="18" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B105" s="19" t="n"/>
-      <c r="C105" s="19" t="n"/>
-      <c r="D105" s="20">
-        <f>SUM(D3:D104)</f>
-        <v/>
-      </c>
-      <c r="E105" s="21">
-        <f>SUM(E3:E104)</f>
-        <v/>
-      </c>
-      <c r="F105" s="19" t="n"/>
+      <c r="B106" s="19" t="n"/>
+      <c r="C106" s="19" t="n"/>
+      <c r="D106" s="20">
+        <f>SUM(D3:D105)</f>
+        <v/>
+      </c>
+      <c r="E106" s="21">
+        <f>SUM(E3:E105)</f>
+        <v/>
+      </c>
+      <c r="F106" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A106:C106"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A105:C105"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix April 2026 Anthropic + CapCut entries
- Remove spurious 2026-04-01 Claude Pro ₪62.87 seed entry (subscription bills on 15th, not 1st)
- Replace 2026-04-01 $5 "Credit purchase" with correct "Prepaid extra usage, Individual plan" ₪31.44 ($10 = 2×$5 receipts at 07:28 + 07:56 UTC)
- Relabel 2026-04-15 Anthropic "Anthropic" → "Claude Pro"
- Relabel 2026-04-16 Anthropic "Anthropic" → "Prepaid extra usage, Individual plan"
- Add 2nd-account CapCut charges (user4127233390216, forwarded from roital1987@gmail.com): 2026-03-18 + 2026-04-18

auto_invoice.py: extract real line-item description from Anthropic receipt body (regex on "Receipt #… <desc> Qty 1 \$…", strip date-range prefix) and add forwarded-email detection so future forwarded CapCut receipts auto-import.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1400,7 +1400,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1701,24 +1701,24 @@
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Pro – Mar 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>10.383845</v>
+        <v>16.655541</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>31.11</v>
+        <v>49.9</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -1730,115 +1730,139 @@
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Creator (first month 50% off)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>11.421896</v>
+        <v>10.383845</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>34.22</v>
+        <v>31.11</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Creator (first month 50% off)</t>
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>9</v>
+        <v>11.421896</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>28.06</v>
+        <v>34.22</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>5.213618</v>
+        <v>9</v>
       </c>
       <c r="E17" s="28" t="n">
-        <v>15.62</v>
+        <v>28.06</v>
       </c>
       <c r="F17" s="29" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
+          <t>2026-03-25</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Lovable</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Lite plan</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>5.213618</v>
+      </c>
+      <c r="E18" s="26" t="n">
+        <v>15.62</v>
+      </c>
+      <c r="F18" s="24" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
           <t>2026-03-26</t>
         </is>
       </c>
-      <c r="B18" s="15" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Dzine</t>
         </is>
       </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>Video Top-Up</t>
         </is>
       </c>
-      <c r="D18" s="25" t="n">
+      <c r="D19" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E18" s="26" t="n">
+      <c r="E19" s="28" t="n">
         <v>62.37</v>
       </c>
-      <c r="F18" s="24" t="n"/>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="F19" s="29" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="31" t="n"/>
-      <c r="D19" s="20">
-        <f>SUM(D4:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="21">
-        <f>SUM(E4:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="31" t="n"/>
+      <c r="B20" s="31" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="20">
+        <f>SUM(D4:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="21">
+        <f>SUM(E4:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:C20"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -1926,14 +1950,14 @@
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>20.984646</v>
+        <v>10.493992</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>62.87</v>
+        <v>31.44</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -1945,19 +1969,19 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Business Plus – Mar 2026 (₪75.90)</t>
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>5.246996</v>
+        <v>25.333778</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>15.72</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -1969,146 +1993,146 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Business Plus – Mar 2026 (₪75.90)</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>25.333778</v>
+        <v>55.517356</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>75.90000000000001</v>
+        <v>166.33</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-04-02</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>55.517356</v>
+        <v>18</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>166.33</v>
+        <v>56.49</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>2026-04-02</t>
+          <t>2026-04-03</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>18</v>
+        <v>2.353138</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>56.49</v>
+        <v>7.05</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-04-03</t>
+          <t>2026-04-05</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Instant Domain</t>
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>2.353138</v>
+        <v>20.971295</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>7.05</v>
+        <v>62.83</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
-          <t>2026-04-05</t>
+          <t>2026-04-10</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Instant Domain</t>
+          <t>capcut_pro_discount1</t>
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>20.971295</v>
+        <v>16.655541</v>
       </c>
       <c r="E10" s="26" t="n">
-        <v>62.83</v>
+        <v>49.9</v>
       </c>
       <c r="F10" s="24" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="10" t="inlineStr">
         <is>
-          <t>2026-04-10</t>
+          <t>2026-04-15</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>capcut_pro_discount1</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>16.655541</v>
+        <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>49.9</v>
+        <v>59.92</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
-          <t>2026-04-15</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -2118,14 +2142,14 @@
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>59.92</v>
+        <v>29.96</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -2137,43 +2161,43 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>29.96</v>
+        <v>59.92</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="14" t="inlineStr">
         <is>
-          <t>2026-04-16</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>20</v>
+        <v>16.655541</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>59.92</v>
+        <v>49.9</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
@@ -3047,7 +3071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F106"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5312,24 +5336,24 @@
     <row r="82">
       <c r="A82" s="14" t="inlineStr">
         <is>
-          <t>2026-03-19</t>
+          <t>2026-03-18</t>
         </is>
       </c>
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Pro – Mar 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>10.383845</v>
+        <v>16.655541</v>
       </c>
       <c r="E82" s="17" t="n">
-        <v>31.11</v>
+        <v>49.9</v>
       </c>
       <c r="F82" s="14" t="inlineStr">
         <is>
@@ -5345,19 +5369,19 @@
       </c>
       <c r="B83" s="11" t="inlineStr">
         <is>
-          <t>Eleven Labs</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Creator (first month 50% off)</t>
+          <t>Credit purchase</t>
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>11.421896</v>
+        <v>10.383845</v>
       </c>
       <c r="E83" s="13" t="n">
-        <v>34.22</v>
+        <v>31.11</v>
       </c>
       <c r="F83" s="10" t="inlineStr">
         <is>
@@ -5368,24 +5392,24 @@
     <row r="84">
       <c r="A84" s="14" t="inlineStr">
         <is>
-          <t>2026-03-24</t>
+          <t>2026-03-19</t>
         </is>
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Creator (first month 50% off)</t>
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>9</v>
+        <v>11.421896</v>
       </c>
       <c r="E84" s="17" t="n">
-        <v>28.06</v>
+        <v>34.22</v>
       </c>
       <c r="F84" s="14" t="inlineStr">
         <is>
@@ -5396,24 +5420,24 @@
     <row r="85">
       <c r="A85" s="10" t="inlineStr">
         <is>
-          <t>2026-03-25</t>
+          <t>2026-03-24</t>
         </is>
       </c>
       <c r="B85" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Lite plan</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D85" s="12" t="n">
-        <v>5.213618</v>
+        <v>9</v>
       </c>
       <c r="E85" s="13" t="n">
-        <v>15.62</v>
+        <v>28.06</v>
       </c>
       <c r="F85" s="10" t="inlineStr">
         <is>
@@ -5424,24 +5448,24 @@
     <row r="86">
       <c r="A86" s="14" t="inlineStr">
         <is>
-          <t>2026-03-26</t>
+          <t>2026-03-25</t>
         </is>
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>Dzine</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>Video Top-Up</t>
+          <t>Lite plan</t>
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>20</v>
+        <v>5.213618</v>
       </c>
       <c r="E86" s="17" t="n">
-        <v>62.37</v>
+        <v>15.62</v>
       </c>
       <c r="F86" s="14" t="inlineStr">
         <is>
@@ -5452,28 +5476,28 @@
     <row r="87">
       <c r="A87" s="10" t="inlineStr">
         <is>
-          <t>2026-04-01</t>
+          <t>2026-03-26</t>
         </is>
       </c>
       <c r="B87" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Dzine</t>
         </is>
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Claude Pro</t>
+          <t>Video Top-Up</t>
         </is>
       </c>
       <c r="D87" s="12" t="n">
-        <v>20.984646</v>
+        <v>20</v>
       </c>
       <c r="E87" s="13" t="n">
-        <v>62.87</v>
+        <v>62.37</v>
       </c>
       <c r="F87" s="10" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מרץ 2026</t>
         </is>
       </c>
     </row>
@@ -5490,14 +5514,14 @@
       </c>
       <c r="C88" s="15" t="inlineStr">
         <is>
-          <t>Credit purchase</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>5.246996</v>
+        <v>10.493992</v>
       </c>
       <c r="E88" s="17" t="n">
-        <v>15.72</v>
+        <v>31.44</v>
       </c>
       <c r="F88" s="14" t="inlineStr">
         <is>
@@ -5686,7 +5710,7 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D95" s="12" t="n">
@@ -5714,7 +5738,7 @@
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D96" s="16" t="n">
@@ -5760,35 +5784,35 @@
     <row r="98">
       <c r="A98" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B98" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D98" s="16" t="n">
-        <v>20</v>
+        <v>16.655541</v>
       </c>
       <c r="E98" s="17" t="n">
-        <v>59.92</v>
+        <v>49.9</v>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
@@ -5809,14 +5833,14 @@
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5837,14 +5861,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5865,14 +5889,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5893,14 +5917,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5921,14 +5945,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5949,14 +5973,14 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -5977,32 +6001,60 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B106" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C106" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D106" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E106" s="17" t="n">
+        <v>59.92</v>
+      </c>
+      <c r="F106" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="18" t="inlineStr">
+    <row r="107">
+      <c r="A107" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B106" s="19" t="n"/>
-      <c r="C106" s="19" t="n"/>
-      <c r="D106" s="20">
-        <f>SUM(D3:D105)</f>
-        <v/>
-      </c>
-      <c r="E106" s="21">
-        <f>SUM(E3:E105)</f>
-        <v/>
-      </c>
-      <c r="F106" s="19" t="n"/>
+      <c r="B107" s="19" t="n"/>
+      <c r="C107" s="19" t="n"/>
+      <c r="D107" s="20">
+        <f>SUM(D3:D106)</f>
+        <v/>
+      </c>
+      <c r="E107" s="21">
+        <f>SUM(E3:E106)</f>
+        <v/>
+      </c>
+      <c r="F107" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A106:C106"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A107:C107"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – CapCut 2026-04-18
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Pro – Apr 2026 (₪49.90)</t>
+          <t>CapCut (₪49.9)</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
@@ -2201,28 +2201,52 @@
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="30" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-18</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>CapCut</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Pro – Apr 2026 (₪49.90)</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="n">
+        <v>16.655541</v>
+      </c>
+      <c r="E15" s="28" t="n">
+        <v>49.9</v>
+      </c>
+      <c r="F15" s="29" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B15" s="31" t="n"/>
-      <c r="C15" s="31" t="n"/>
-      <c r="D15" s="20">
-        <f>SUM(D4:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="21">
-        <f>SUM(E4:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="31" t="n"/>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="20">
+        <f>SUM(D4:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="21">
+        <f>SUM(E4:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3071,7 +3095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5794,7 +5818,7 @@
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>Pro – Apr 2026 (₪49.90)</t>
+          <t>CapCut (₪49.9)</t>
         </is>
       </c>
       <c r="D98" s="16" t="n">
@@ -5812,35 +5836,35 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D99" s="12" t="n">
-        <v>20</v>
+        <v>16.655541</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>59.92</v>
+        <v>49.9</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5861,14 +5885,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5889,14 +5913,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5917,14 +5941,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5945,14 +5969,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5973,14 +5997,14 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -6001,14 +6025,14 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B106" s="15" t="inlineStr">
@@ -6029,32 +6053,60 @@
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C107" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D107" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E107" s="13" t="n">
+        <v>59.92</v>
+      </c>
+      <c r="F107" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="18" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B107" s="19" t="n"/>
-      <c r="C107" s="19" t="n"/>
-      <c r="D107" s="20">
-        <f>SUM(D3:D106)</f>
-        <v/>
-      </c>
-      <c r="E107" s="21">
-        <f>SUM(E3:E106)</f>
-        <v/>
-      </c>
-      <c r="F107" s="19" t="n"/>
+      <c r="B108" s="19" t="n"/>
+      <c r="C108" s="19" t="n"/>
+      <c r="D108" s="20">
+        <f>SUM(D3:D107)</f>
+        <v/>
+      </c>
+      <c r="E108" s="21">
+        <f>SUM(E3:E107)</f>
+        <v/>
+      </c>
+      <c r="F108" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A107:C107"/>
+    <mergeCell ref="A108:C108"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: remove duplicate CapCut ₪49.90 entry on 2026-04-18
The auto_invoice.py daily run on 2026-04-19 08:00 re-scanned the
forwarded 2nd-account CapCut invoice that was already manually logged
the previous evening (commit 6bf0113 as "Pro – Apr 2026") and created a
second generic "CapCut (₪49.9)" entry on the same date for the same
amount. CapCut only bills twice monthly (main on the 10th, 2nd account
on the 18th), so two ₪49.90 charges on 2026-04-18 cannot both be real.

Remove the duplicate MANUAL_TRANSACTIONS row and regenerate the report.
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>CapCut (₪49.9)</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
@@ -2201,52 +2201,28 @@
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-18</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>CapCut</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Pro – Apr 2026 (₪49.90)</t>
-        </is>
-      </c>
-      <c r="D15" s="27" t="n">
-        <v>16.655541</v>
-      </c>
-      <c r="E15" s="28" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="F15" s="29" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B16" s="31" t="n"/>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="20">
-        <f>SUM(D4:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="21">
-        <f>SUM(E4:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="31" t="n"/>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="20">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f>SUM(E4:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3095,7 +3071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5818,7 +5794,7 @@
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>CapCut (₪49.9)</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D98" s="16" t="n">
@@ -5836,35 +5812,35 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Pro – Apr 2026 (₪49.90)</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D99" s="12" t="n">
-        <v>16.655541</v>
+        <v>20</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>49.9</v>
+        <v>59.92</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5885,14 +5861,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5913,14 +5889,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5941,14 +5917,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5969,14 +5945,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5997,14 +5973,14 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -6025,14 +6001,14 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>נובמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-16</t>
         </is>
       </c>
       <c r="B106" s="15" t="inlineStr">
@@ -6053,60 +6029,32 @@
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="10" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="B107" s="11" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C107" s="11" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D107" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="E107" s="13" t="n">
-        <v>59.92</v>
-      </c>
-      <c r="F107" s="10" t="inlineStr">
-        <is>
-          <t>דצמבר 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="18" t="inlineStr">
+      <c r="A107" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B108" s="19" t="n"/>
-      <c r="C108" s="19" t="n"/>
-      <c r="D108" s="20">
-        <f>SUM(D3:D107)</f>
-        <v/>
-      </c>
-      <c r="E108" s="21">
-        <f>SUM(E3:E107)</f>
-        <v/>
-      </c>
-      <c r="F108" s="19" t="n"/>
+      <c r="B107" s="19" t="n"/>
+      <c r="C107" s="19" t="n"/>
+      <c r="D107" s="20">
+        <f>SUM(D3:D106)</f>
+        <v/>
+      </c>
+      <c r="E107" s="21">
+        <f>SUM(E3:E106)</f>
+        <v/>
+      </c>
+      <c r="F107" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A108:C108"/>
+    <mergeCell ref="A107:C107"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix CapCut Apr 18 duplicate and improve ILS description format
- Remove duplicate CapCut 2026-04-18 auto-imported by CI after last push;
  keep the clean "Pro – Apr 2026 (₪49.90)" entry only
- auto_invoice.py: CapCut ILS charges now get "Pro – <Mon> <Year> (₪X.XX)"
  description instead of generic "CapCut (₪X.X)"

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>CapCut (₪49.9)</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
@@ -2201,52 +2201,28 @@
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
-    <row r="15">
-      <c r="A15" s="10" t="inlineStr">
-        <is>
-          <t>2026-04-18</t>
-        </is>
-      </c>
-      <c r="B15" s="11" t="inlineStr">
-        <is>
-          <t>CapCut</t>
-        </is>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>Pro – Apr 2026 (₪49.90)</t>
-        </is>
-      </c>
-      <c r="D15" s="27" t="n">
-        <v>16.655541</v>
-      </c>
-      <c r="E15" s="28" t="n">
-        <v>49.9</v>
-      </c>
-      <c r="F15" s="29" t="n"/>
-    </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B16" s="31" t="n"/>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="20">
-        <f>SUM(D4:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="21">
-        <f>SUM(E4:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="31" t="n"/>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="20">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f>SUM(E4:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3095,7 +3071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5818,7 +5794,7 @@
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>CapCut (₪49.9)</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D98" s="16" t="n">
@@ -5836,35 +5812,35 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Pro – Apr 2026 (₪49.90)</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D99" s="12" t="n">
-        <v>16.655541</v>
+        <v>20</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>49.9</v>
+        <v>59.92</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>אפריל 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5885,14 +5861,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5913,14 +5889,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5941,14 +5917,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5969,14 +5945,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5997,14 +5973,14 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -6025,14 +6001,14 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>נובמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-12-16</t>
         </is>
       </c>
       <c r="B106" s="15" t="inlineStr">
@@ -6053,60 +6029,32 @@
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="10" t="inlineStr">
-        <is>
-          <t>2026-12-16</t>
-        </is>
-      </c>
-      <c r="B107" s="11" t="inlineStr">
-        <is>
-          <t>OpenAI</t>
-        </is>
-      </c>
-      <c r="C107" s="11" t="inlineStr">
-        <is>
-          <t>ChatGPT Plus</t>
-        </is>
-      </c>
-      <c r="D107" s="12" t="n">
-        <v>20</v>
-      </c>
-      <c r="E107" s="13" t="n">
-        <v>59.92</v>
-      </c>
-      <c r="F107" s="10" t="inlineStr">
-        <is>
-          <t>דצמבר 2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="18" t="inlineStr">
+      <c r="A107" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B108" s="19" t="n"/>
-      <c r="C108" s="19" t="n"/>
-      <c r="D108" s="20">
-        <f>SUM(D3:D107)</f>
-        <v/>
-      </c>
-      <c r="E108" s="21">
-        <f>SUM(E3:E107)</f>
-        <v/>
-      </c>
-      <c r="F108" s="19" t="n"/>
+      <c r="B107" s="19" t="n"/>
+      <c r="C107" s="19" t="n"/>
+      <c r="D107" s="20">
+        <f>SUM(D3:D106)</f>
+        <v/>
+      </c>
+      <c r="E107" s="21">
+        <f>SUM(E3:E106)</f>
+        <v/>
+      </c>
+      <c r="F107" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A108:C108"/>
+    <mergeCell ref="A107:C107"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-04-19
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2201,28 +2201,52 @@
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
-    <row r="15" ht="24" customHeight="1">
-      <c r="A15" s="30" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-19</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>Prepaid extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D15" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E15" s="28" t="n">
+        <v>14.98</v>
+      </c>
+      <c r="F15" s="29" t="n"/>
+    </row>
+    <row r="16" ht="24" customHeight="1">
+      <c r="A16" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B15" s="31" t="n"/>
-      <c r="C15" s="31" t="n"/>
-      <c r="D15" s="20">
-        <f>SUM(D4:D14)</f>
-        <v/>
-      </c>
-      <c r="E15" s="21">
-        <f>SUM(E4:E14)</f>
-        <v/>
-      </c>
-      <c r="F15" s="31" t="n"/>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="31" t="n"/>
+      <c r="D16" s="20">
+        <f>SUM(D4:D15)</f>
+        <v/>
+      </c>
+      <c r="E16" s="21">
+        <f>SUM(E4:E15)</f>
+        <v/>
+      </c>
+      <c r="F16" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3071,7 +3095,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F107"/>
+  <dimension ref="A1:F108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5812,35 +5836,35 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D99" s="12" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>59.92</v>
+        <v>14.98</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -5861,14 +5885,14 @@
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
@@ -5889,14 +5913,14 @@
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -5917,14 +5941,14 @@
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5945,14 +5969,14 @@
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5973,14 +5997,14 @@
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -6001,14 +6025,14 @@
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B106" s="15" t="inlineStr">
@@ -6029,32 +6053,60 @@
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C107" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D107" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E107" s="13" t="n">
+        <v>59.92</v>
+      </c>
+      <c r="F107" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="18" t="inlineStr">
+    <row r="108">
+      <c r="A108" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B107" s="19" t="n"/>
-      <c r="C107" s="19" t="n"/>
-      <c r="D107" s="20">
-        <f>SUM(D3:D106)</f>
-        <v/>
-      </c>
-      <c r="E107" s="21">
-        <f>SUM(E3:E106)</f>
-        <v/>
-      </c>
-      <c r="F107" s="19" t="n"/>
+      <c r="B108" s="19" t="n"/>
+      <c r="C108" s="19" t="n"/>
+      <c r="D108" s="20">
+        <f>SUM(D3:D107)</f>
+        <v/>
+      </c>
+      <c r="E108" s="21">
+        <f>SUM(E3:E107)</f>
+        <v/>
+      </c>
+      <c r="F108" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A107:C107"/>
+    <mergeCell ref="A108:C108"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-04-21, Anthropic 2026-04-20, Anthropic 2026-04-20
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -939,11 +939,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>2.996</v>
+        <v>3.003</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-17</t>
+          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-20</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.88785</v>
+        <v>25.827506</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>77.56</v>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1116,7 +1116,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>32.5</v>
+        <v>32.424242</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>97.37</v>
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>49.9</v>
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>48.271028</v>
+        <v>48.158508</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>144.62</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20.604139</v>
+        <v>20.556111</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>61.73</v>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5.153538</v>
+        <v>5.141525</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>15.44</v>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20.881175</v>
+        <v>20.832501</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>62.56</v>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>51.722296</v>
+        <v>51.601732</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>154.96</v>
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>52.757009</v>
+        <v>52.634033</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>158.06</v>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.233645</v>
+        <v>5.221445</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>15.68</v>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>10.463952</v>
+        <v>10.43956</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>31.35</v>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>10.440587</v>
+        <v>10.41625</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>31.28</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15.140187</v>
+        <v>15.104895</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>45.36</v>
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>10.413885</v>
+        <v>10.38961</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>31.2</v>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>41.198264</v>
+        <v>41.102231</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>123.43</v>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>53.294393</v>
+        <v>53.170163</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>159.67</v>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>20.984646</v>
+        <v>20.935731</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>62.87</v>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>49.9</v>
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>10.383845</v>
+        <v>10.35964</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>31.11</v>
@@ -1763,7 +1763,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>11.421896</v>
+        <v>11.395271</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>34.22</v>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D18" s="25" t="n">
-        <v>5.213618</v>
+        <v>5.201465</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>15.62</v>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>10.493992</v>
+        <v>10.46953</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>31.44</v>
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>75.90000000000001</v>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>55.517356</v>
+        <v>55.387945</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>166.33</v>
@@ -2050,7 +2050,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>2.353138</v>
+        <v>2.347652</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>7.05</v>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20.971295</v>
+        <v>20.922411</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>62.83</v>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -2125,7 +2125,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>29.96</v>
+        <v>30.03</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -2173,7 +2173,7 @@
         <v>20</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>49.9</v>
@@ -2221,32 +2221,104 @@
         <v>5</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>14.98</v>
+        <v>15.02</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
-    <row r="16" ht="24" customHeight="1">
-      <c r="A16" s="30" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B16" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C16" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D16" s="25" t="n">
+        <v>15.14</v>
+      </c>
+      <c r="E16" s="26" t="n">
+        <v>45.47</v>
+      </c>
+      <c r="F16" s="24" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-20</t>
+        </is>
+      </c>
+      <c r="B17" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
+        <is>
+          <t>Prepaid extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D17" s="27" t="n">
+        <v>10</v>
+      </c>
+      <c r="E17" s="28" t="n">
+        <v>30.03</v>
+      </c>
+      <c r="F17" s="29" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D18" s="25" t="n">
+        <v>10.15</v>
+      </c>
+      <c r="E18" s="26" t="n">
+        <v>30.48</v>
+      </c>
+      <c r="F18" s="24" t="n"/>
+    </row>
+    <row r="19" ht="24" customHeight="1">
+      <c r="A19" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B16" s="31" t="n"/>
-      <c r="C16" s="31" t="n"/>
-      <c r="D16" s="20">
-        <f>SUM(D4:D15)</f>
-        <v/>
-      </c>
-      <c r="E16" s="21">
-        <f>SUM(E4:E15)</f>
-        <v/>
-      </c>
-      <c r="F16" s="31" t="n"/>
+      <c r="B19" s="31" t="n"/>
+      <c r="C19" s="31" t="n"/>
+      <c r="D19" s="20">
+        <f>SUM(D4:D18)</f>
+        <v/>
+      </c>
+      <c r="E19" s="21">
+        <f>SUM(E4:E18)</f>
+        <v/>
+      </c>
+      <c r="F19" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A19:C19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A16:C16"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -2340,7 +2412,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2459,7 +2531,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2578,7 +2650,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2697,7 +2769,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2816,7 +2888,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2935,7 +3007,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3054,7 +3126,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3095,7 +3167,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F108"/>
+  <dimension ref="A1:F111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3162,7 +3234,7 @@
         </is>
       </c>
       <c r="D3" s="12" t="n">
-        <v>1.11482</v>
+        <v>1.112221</v>
       </c>
       <c r="E3" s="13" t="n">
         <v>3.34</v>
@@ -3190,7 +3262,7 @@
         </is>
       </c>
       <c r="D4" s="16" t="n">
-        <v>80.46729000000001</v>
+        <v>80.27972</v>
       </c>
       <c r="E4" s="17" t="n">
         <v>241.08</v>
@@ -3218,7 +3290,7 @@
         </is>
       </c>
       <c r="D5" s="12" t="n">
-        <v>11.695594</v>
+        <v>11.668332</v>
       </c>
       <c r="E5" s="13" t="n">
         <v>35.04</v>
@@ -3246,7 +3318,7 @@
         </is>
       </c>
       <c r="D6" s="16" t="n">
-        <v>22.129506</v>
+        <v>22.077922</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>66.3</v>
@@ -3302,7 +3374,7 @@
         </is>
       </c>
       <c r="D8" s="16" t="n">
-        <v>15.130174</v>
+        <v>15.094905</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>45.33</v>
@@ -3330,7 +3402,7 @@
         </is>
       </c>
       <c r="D9" s="12" t="n">
-        <v>127.12283</v>
+        <v>126.826507</v>
       </c>
       <c r="E9" s="13" t="n">
         <v>380.86</v>
@@ -3358,7 +3430,7 @@
         </is>
       </c>
       <c r="D10" s="16" t="n">
-        <v>11.23498</v>
+        <v>11.208791</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>33.66</v>
@@ -3386,7 +3458,7 @@
         </is>
       </c>
       <c r="D11" s="12" t="n">
-        <v>19.002003</v>
+        <v>18.957709</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>56.93</v>
@@ -3414,7 +3486,7 @@
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>17.086115</v>
+        <v>17.046287</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>51.19</v>
@@ -3442,7 +3514,7 @@
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>13.658211</v>
+        <v>13.626374</v>
       </c>
       <c r="E13" s="13" t="n">
         <v>40.92</v>
@@ -3470,7 +3542,7 @@
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>1.028037</v>
+        <v>1.025641</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>3.08</v>
@@ -3498,7 +3570,7 @@
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>21.775701</v>
+        <v>21.724942</v>
       </c>
       <c r="E15" s="13" t="n">
         <v>65.23999999999999</v>
@@ -3526,7 +3598,7 @@
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>12.136182</v>
+        <v>12.107892</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>36.36</v>
@@ -3554,7 +3626,7 @@
         </is>
       </c>
       <c r="D17" s="12" t="n">
-        <v>22.840454</v>
+        <v>22.787213</v>
       </c>
       <c r="E17" s="13" t="n">
         <v>68.43000000000001</v>
@@ -3610,7 +3682,7 @@
         </is>
       </c>
       <c r="D19" s="12" t="n">
-        <v>5.577437</v>
+        <v>5.564436</v>
       </c>
       <c r="E19" s="13" t="n">
         <v>16.71</v>
@@ -3638,7 +3710,7 @@
         </is>
       </c>
       <c r="D20" s="16" t="n">
-        <v>12.550067</v>
+        <v>12.520813</v>
       </c>
       <c r="E20" s="17" t="n">
         <v>37.6</v>
@@ -3666,7 +3738,7 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>19.002003</v>
+        <v>18.957709</v>
       </c>
       <c r="E21" s="13" t="n">
         <v>56.93</v>
@@ -3694,7 +3766,7 @@
         </is>
       </c>
       <c r="D22" s="16" t="n">
-        <v>3.11749</v>
+        <v>3.110223</v>
       </c>
       <c r="E22" s="17" t="n">
         <v>9.34</v>
@@ -3722,7 +3794,7 @@
         </is>
       </c>
       <c r="D23" s="12" t="n">
-        <v>11.819092</v>
+        <v>11.791542</v>
       </c>
       <c r="E23" s="13" t="n">
         <v>35.41</v>
@@ -3778,7 +3850,7 @@
         </is>
       </c>
       <c r="D25" s="12" t="n">
-        <v>22.316422</v>
+        <v>22.264402</v>
       </c>
       <c r="E25" s="13" t="n">
         <v>66.86</v>
@@ -3806,7 +3878,7 @@
         </is>
       </c>
       <c r="D26" s="16" t="n">
-        <v>5.510681</v>
+        <v>5.497835</v>
       </c>
       <c r="E26" s="17" t="n">
         <v>16.51</v>
@@ -3834,7 +3906,7 @@
         </is>
       </c>
       <c r="D27" s="12" t="n">
-        <v>19.002003</v>
+        <v>18.957709</v>
       </c>
       <c r="E27" s="13" t="n">
         <v>56.93</v>
@@ -3890,7 +3962,7 @@
         </is>
       </c>
       <c r="D29" s="12" t="n">
-        <v>21.962617</v>
+        <v>21.911422</v>
       </c>
       <c r="E29" s="13" t="n">
         <v>65.8</v>
@@ -3918,7 +3990,7 @@
         </is>
       </c>
       <c r="D30" s="16" t="n">
-        <v>5.430574</v>
+        <v>5.417915</v>
       </c>
       <c r="E30" s="17" t="n">
         <v>16.27</v>
@@ -3946,7 +4018,7 @@
         </is>
       </c>
       <c r="D31" s="12" t="n">
-        <v>13.05741</v>
+        <v>13.026973</v>
       </c>
       <c r="E31" s="13" t="n">
         <v>39.12</v>
@@ -3974,7 +4046,7 @@
         </is>
       </c>
       <c r="D32" s="16" t="n">
-        <v>12.716956</v>
+        <v>12.687313</v>
       </c>
       <c r="E32" s="17" t="n">
         <v>38.1</v>
@@ -4002,7 +4074,7 @@
         </is>
       </c>
       <c r="D33" s="12" t="n">
-        <v>16.168224</v>
+        <v>16.130536</v>
       </c>
       <c r="E33" s="13" t="n">
         <v>48.44</v>
@@ -4030,7 +4102,7 @@
         </is>
       </c>
       <c r="D34" s="16" t="n">
-        <v>10.664219</v>
+        <v>10.639361</v>
       </c>
       <c r="E34" s="17" t="n">
         <v>31.95</v>
@@ -4086,7 +4158,7 @@
         </is>
       </c>
       <c r="D36" s="16" t="n">
-        <v>21.869159</v>
+        <v>21.818182</v>
       </c>
       <c r="E36" s="17" t="n">
         <v>65.52</v>
@@ -4114,7 +4186,7 @@
         </is>
       </c>
       <c r="D37" s="12" t="n">
-        <v>5.443925</v>
+        <v>5.431235</v>
       </c>
       <c r="E37" s="13" t="n">
         <v>16.31</v>
@@ -4142,7 +4214,7 @@
         </is>
       </c>
       <c r="D38" s="16" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E38" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4170,7 +4242,7 @@
         </is>
       </c>
       <c r="D39" s="12" t="n">
-        <v>16.281709</v>
+        <v>16.243756</v>
       </c>
       <c r="E39" s="13" t="n">
         <v>48.78</v>
@@ -4198,7 +4270,7 @@
         </is>
       </c>
       <c r="D40" s="16" t="n">
-        <v>10.550734</v>
+        <v>10.526141</v>
       </c>
       <c r="E40" s="17" t="n">
         <v>31.61</v>
@@ -4226,7 +4298,7 @@
         </is>
       </c>
       <c r="D41" s="12" t="n">
-        <v>32.363151</v>
+        <v>32.287712</v>
       </c>
       <c r="E41" s="13" t="n">
         <v>96.95999999999999</v>
@@ -4254,7 +4326,7 @@
         </is>
       </c>
       <c r="D42" s="16" t="n">
-        <v>35.390521</v>
+        <v>35.308025</v>
       </c>
       <c r="E42" s="17" t="n">
         <v>106.03</v>
@@ -4310,7 +4382,7 @@
         </is>
       </c>
       <c r="D44" s="16" t="n">
-        <v>38.321095</v>
+        <v>38.231768</v>
       </c>
       <c r="E44" s="17" t="n">
         <v>114.81</v>
@@ -4338,7 +4410,7 @@
         </is>
       </c>
       <c r="D45" s="12" t="n">
-        <v>5.317089</v>
+        <v>5.304695</v>
       </c>
       <c r="E45" s="13" t="n">
         <v>15.93</v>
@@ -4366,7 +4438,7 @@
         </is>
       </c>
       <c r="D46" s="16" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E46" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4394,7 +4466,7 @@
         </is>
       </c>
       <c r="D47" s="12" t="n">
-        <v>148.775033</v>
+        <v>148.428238</v>
       </c>
       <c r="E47" s="13" t="n">
         <v>445.73</v>
@@ -4422,7 +4494,7 @@
         </is>
       </c>
       <c r="D48" s="16" t="n">
-        <v>15.947931</v>
+        <v>15.910756</v>
       </c>
       <c r="E48" s="17" t="n">
         <v>47.78</v>
@@ -4450,7 +4522,7 @@
         </is>
       </c>
       <c r="D49" s="12" t="n">
-        <v>20.660881</v>
+        <v>20.612721</v>
       </c>
       <c r="E49" s="13" t="n">
         <v>61.9</v>
@@ -4478,7 +4550,7 @@
         </is>
       </c>
       <c r="D50" s="16" t="n">
-        <v>21.198264</v>
+        <v>21.148851</v>
       </c>
       <c r="E50" s="17" t="n">
         <v>63.51</v>
@@ -4506,7 +4578,7 @@
         </is>
       </c>
       <c r="D51" s="12" t="n">
-        <v>21.138184</v>
+        <v>21.088911</v>
       </c>
       <c r="E51" s="13" t="n">
         <v>63.33</v>
@@ -4534,7 +4606,7 @@
         </is>
       </c>
       <c r="D52" s="16" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E52" s="17" t="n">
         <v>49.9</v>
@@ -4590,7 +4662,7 @@
         </is>
       </c>
       <c r="D54" s="16" t="n">
-        <v>40.987984</v>
+        <v>40.892441</v>
       </c>
       <c r="E54" s="17" t="n">
         <v>122.8</v>
@@ -4618,7 +4690,7 @@
         </is>
       </c>
       <c r="D55" s="12" t="n">
-        <v>26.104806</v>
+        <v>26.043956</v>
       </c>
       <c r="E55" s="13" t="n">
         <v>78.20999999999999</v>
@@ -4646,7 +4718,7 @@
         </is>
       </c>
       <c r="D56" s="16" t="n">
-        <v>44.726302</v>
+        <v>44.622045</v>
       </c>
       <c r="E56" s="17" t="n">
         <v>134</v>
@@ -4674,7 +4746,7 @@
         </is>
       </c>
       <c r="D57" s="12" t="n">
-        <v>5.1502</v>
+        <v>5.138195</v>
       </c>
       <c r="E57" s="13" t="n">
         <v>15.43</v>
@@ -4702,7 +4774,7 @@
         </is>
       </c>
       <c r="D58" s="16" t="n">
-        <v>14.933244</v>
+        <v>14.898435</v>
       </c>
       <c r="E58" s="17" t="n">
         <v>44.74</v>
@@ -4730,7 +4802,7 @@
         </is>
       </c>
       <c r="D59" s="12" t="n">
-        <v>25.88785</v>
+        <v>25.827506</v>
       </c>
       <c r="E59" s="13" t="n">
         <v>77.56</v>
@@ -4758,7 +4830,7 @@
         </is>
       </c>
       <c r="D60" s="16" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E60" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4786,7 +4858,7 @@
         </is>
       </c>
       <c r="D61" s="12" t="n">
-        <v>32.5</v>
+        <v>32.424242</v>
       </c>
       <c r="E61" s="13" t="n">
         <v>97.37</v>
@@ -4814,7 +4886,7 @@
         </is>
       </c>
       <c r="D62" s="16" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E62" s="17" t="n">
         <v>49.9</v>
@@ -4842,7 +4914,7 @@
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>48.271028</v>
+        <v>48.158508</v>
       </c>
       <c r="E63" s="13" t="n">
         <v>144.62</v>
@@ -4870,7 +4942,7 @@
         </is>
       </c>
       <c r="D64" s="16" t="n">
-        <v>20.604139</v>
+        <v>20.556111</v>
       </c>
       <c r="E64" s="17" t="n">
         <v>61.73</v>
@@ -4898,7 +4970,7 @@
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>5.153538</v>
+        <v>5.141525</v>
       </c>
       <c r="E65" s="13" t="n">
         <v>15.44</v>
@@ -4954,7 +5026,7 @@
         </is>
       </c>
       <c r="D67" s="12" t="n">
-        <v>20.881175</v>
+        <v>20.832501</v>
       </c>
       <c r="E67" s="13" t="n">
         <v>62.56</v>
@@ -4982,7 +5054,7 @@
         </is>
       </c>
       <c r="D68" s="16" t="n">
-        <v>51.722296</v>
+        <v>51.601732</v>
       </c>
       <c r="E68" s="17" t="n">
         <v>154.96</v>
@@ -5010,7 +5082,7 @@
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>52.757009</v>
+        <v>52.634033</v>
       </c>
       <c r="E69" s="13" t="n">
         <v>158.06</v>
@@ -5038,7 +5110,7 @@
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>5.233645</v>
+        <v>5.221445</v>
       </c>
       <c r="E70" s="17" t="n">
         <v>15.68</v>
@@ -5066,7 +5138,7 @@
         </is>
       </c>
       <c r="D71" s="12" t="n">
-        <v>10.463952</v>
+        <v>10.43956</v>
       </c>
       <c r="E71" s="13" t="n">
         <v>31.35</v>
@@ -5094,7 +5166,7 @@
         </is>
       </c>
       <c r="D72" s="16" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E72" s="17" t="n">
         <v>75.90000000000001</v>
@@ -5122,7 +5194,7 @@
         </is>
       </c>
       <c r="D73" s="12" t="n">
-        <v>10.440587</v>
+        <v>10.41625</v>
       </c>
       <c r="E73" s="13" t="n">
         <v>31.28</v>
@@ -5150,7 +5222,7 @@
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>15.140187</v>
+        <v>15.104895</v>
       </c>
       <c r="E74" s="17" t="n">
         <v>45.36</v>
@@ -5178,7 +5250,7 @@
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E75" s="13" t="n">
         <v>75.90000000000001</v>
@@ -5206,7 +5278,7 @@
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>10.413885</v>
+        <v>10.38961</v>
       </c>
       <c r="E76" s="17" t="n">
         <v>31.2</v>
@@ -5234,7 +5306,7 @@
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>41.198264</v>
+        <v>41.102231</v>
       </c>
       <c r="E77" s="13" t="n">
         <v>123.43</v>
@@ -5262,7 +5334,7 @@
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E78" s="17" t="n">
         <v>49.9</v>
@@ -5290,7 +5362,7 @@
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>53.294393</v>
+        <v>53.170163</v>
       </c>
       <c r="E79" s="13" t="n">
         <v>159.67</v>
@@ -5318,7 +5390,7 @@
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>20.984646</v>
+        <v>20.935731</v>
       </c>
       <c r="E80" s="17" t="n">
         <v>62.87</v>
@@ -5374,7 +5446,7 @@
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E82" s="17" t="n">
         <v>49.9</v>
@@ -5402,7 +5474,7 @@
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>10.383845</v>
+        <v>10.35964</v>
       </c>
       <c r="E83" s="13" t="n">
         <v>31.11</v>
@@ -5430,7 +5502,7 @@
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>11.421896</v>
+        <v>11.395271</v>
       </c>
       <c r="E84" s="17" t="n">
         <v>34.22</v>
@@ -5486,7 +5558,7 @@
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>5.213618</v>
+        <v>5.201465</v>
       </c>
       <c r="E86" s="17" t="n">
         <v>15.62</v>
@@ -5542,7 +5614,7 @@
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>10.493992</v>
+        <v>10.46953</v>
       </c>
       <c r="E88" s="17" t="n">
         <v>31.44</v>
@@ -5570,7 +5642,7 @@
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E89" s="13" t="n">
         <v>75.90000000000001</v>
@@ -5598,7 +5670,7 @@
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>55.517356</v>
+        <v>55.387945</v>
       </c>
       <c r="E90" s="17" t="n">
         <v>166.33</v>
@@ -5654,7 +5726,7 @@
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>2.353138</v>
+        <v>2.347652</v>
       </c>
       <c r="E92" s="17" t="n">
         <v>7.05</v>
@@ -5682,7 +5754,7 @@
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>20.971295</v>
+        <v>20.922411</v>
       </c>
       <c r="E93" s="13" t="n">
         <v>62.83</v>
@@ -5710,7 +5782,7 @@
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E94" s="17" t="n">
         <v>49.9</v>
@@ -5741,7 +5813,7 @@
         <v>20</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
@@ -5769,7 +5841,7 @@
         <v>10</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>29.96</v>
+        <v>30.03</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -5797,7 +5869,7 @@
         <v>20</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -5822,7 +5894,7 @@
         </is>
       </c>
       <c r="D98" s="16" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E98" s="17" t="n">
         <v>49.9</v>
@@ -5853,7 +5925,7 @@
         <v>5</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>14.98</v>
+        <v>15.02</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
@@ -5864,91 +5936,91 @@
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D100" s="16" t="n">
-        <v>20</v>
+        <v>15.14</v>
       </c>
       <c r="E100" s="17" t="n">
-        <v>59.92</v>
+        <v>45.47</v>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D101" s="12" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="E101" s="13" t="n">
-        <v>59.92</v>
+        <v>30.03</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C102" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D102" s="16" t="n">
-        <v>20</v>
+        <v>10.15</v>
       </c>
       <c r="E102" s="17" t="n">
-        <v>59.92</v>
+        <v>30.48</v>
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -5965,18 +6037,18 @@
         <v>20</v>
       </c>
       <c r="E103" s="13" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
@@ -5993,18 +6065,18 @@
         <v>20</v>
       </c>
       <c r="E104" s="17" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
@@ -6021,18 +6093,18 @@
         <v>20</v>
       </c>
       <c r="E105" s="13" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B106" s="15" t="inlineStr">
@@ -6049,18 +6121,18 @@
         <v>20</v>
       </c>
       <c r="E106" s="17" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
@@ -6077,36 +6149,120 @@
         <v>20</v>
       </c>
       <c r="E107" s="13" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
+          <t>ספטמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B108" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C108" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D108" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E108" s="17" t="n">
+        <v>60.06</v>
+      </c>
+      <c r="F108" s="14" t="inlineStr">
+        <is>
+          <t>אוקטובר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="B109" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C109" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D109" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E109" s="13" t="n">
+        <v>60.06</v>
+      </c>
+      <c r="F109" s="10" t="inlineStr">
+        <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B110" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C110" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D110" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E110" s="17" t="n">
+        <v>60.06</v>
+      </c>
+      <c r="F110" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="18" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B108" s="19" t="n"/>
-      <c r="C108" s="19" t="n"/>
-      <c r="D108" s="20">
-        <f>SUM(D3:D107)</f>
-        <v/>
-      </c>
-      <c r="E108" s="21">
-        <f>SUM(E3:E107)</f>
-        <v/>
-      </c>
-      <c r="F108" s="19" t="n"/>
+      <c r="B111" s="19" t="n"/>
+      <c r="C111" s="19" t="n"/>
+      <c r="D111" s="20">
+        <f>SUM(D3:D110)</f>
+        <v/>
+      </c>
+      <c r="E111" s="21">
+        <f>SUM(E3:E110)</f>
+        <v/>
+      </c>
+      <c r="F111" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A111:C111"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A108:C108"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6197,7 +6353,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.92</v>
+        <v>60.06</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -10835,7 +10991,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>1.11482</v>
+        <v>1.112221</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>3.34</v>
@@ -10859,7 +11015,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>80.46729000000001</v>
+        <v>80.27972</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>241.08</v>
@@ -10883,7 +11039,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>11.695594</v>
+        <v>11.668332</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35.04</v>
@@ -10907,7 +11063,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>22.129506</v>
+        <v>22.077922</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>66.3</v>
@@ -10955,7 +11111,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>15.130174</v>
+        <v>15.094905</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>45.33</v>
@@ -10979,7 +11135,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>127.12283</v>
+        <v>126.826507</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>380.86</v>
@@ -11003,7 +11159,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>11.23498</v>
+        <v>11.208791</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>33.66</v>
@@ -11122,7 +11278,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>19.002003</v>
+        <v>18.957709</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11146,7 +11302,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>17.086115</v>
+        <v>17.046287</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>51.19</v>
@@ -11170,7 +11326,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>13.658211</v>
+        <v>13.626374</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>40.92</v>
@@ -11194,7 +11350,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>1.028037</v>
+        <v>1.025641</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>3.08</v>
@@ -11218,7 +11374,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>21.775701</v>
+        <v>21.724942</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>65.23999999999999</v>
@@ -11242,7 +11398,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>12.136182</v>
+        <v>12.107892</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>36.36</v>
@@ -11266,7 +11422,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>22.840454</v>
+        <v>22.787213</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>68.43000000000001</v>
@@ -11314,7 +11470,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>5.577437</v>
+        <v>5.564436</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>16.71</v>
@@ -11338,7 +11494,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>12.550067</v>
+        <v>12.520813</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>37.6</v>
@@ -11457,7 +11613,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>19.002003</v>
+        <v>18.957709</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11481,7 +11637,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>3.11749</v>
+        <v>3.110223</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>9.34</v>
@@ -11505,7 +11661,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>11.819092</v>
+        <v>11.791542</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35.41</v>
@@ -11553,7 +11709,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>22.316422</v>
+        <v>22.264402</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>66.86</v>
@@ -11577,7 +11733,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>5.510681</v>
+        <v>5.497835</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>16.51</v>
@@ -11696,7 +11852,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>19.002003</v>
+        <v>18.957709</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -11744,7 +11900,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>21.962617</v>
+        <v>21.911422</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>65.8</v>
@@ -11768,7 +11924,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>5.430574</v>
+        <v>5.417915</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>16.27</v>
@@ -11887,7 +12043,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>13.05741</v>
+        <v>13.026973</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>39.12</v>
@@ -11911,7 +12067,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>12.716956</v>
+        <v>12.687313</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>38.1</v>
@@ -11935,7 +12091,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>16.168224</v>
+        <v>16.130536</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>48.44</v>
@@ -11959,7 +12115,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>10.664219</v>
+        <v>10.639361</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>31.95</v>
@@ -12007,7 +12163,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>21.869159</v>
+        <v>21.818182</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>65.52</v>
@@ -12031,7 +12187,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5.443925</v>
+        <v>5.431235</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>16.31</v>
@@ -12150,7 +12306,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -12174,7 +12330,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>16.281709</v>
+        <v>16.243756</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>48.78</v>
@@ -12198,7 +12354,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>10.550734</v>
+        <v>10.526141</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>31.61</v>
@@ -12222,7 +12378,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>32.363151</v>
+        <v>32.287712</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>96.95999999999999</v>
@@ -12246,7 +12402,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>35.390521</v>
+        <v>35.308025</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>106.03</v>
@@ -12294,7 +12450,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>38.321095</v>
+        <v>38.231768</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>114.81</v>
@@ -12318,7 +12474,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>5.317089</v>
+        <v>5.304695</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>15.93</v>
@@ -12437,7 +12593,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.333778</v>
+        <v>25.274725</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -12461,7 +12617,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>148.775033</v>
+        <v>148.428238</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>445.73</v>
@@ -12485,7 +12641,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15.947931</v>
+        <v>15.910756</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>47.78</v>
@@ -12509,7 +12665,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>20.660881</v>
+        <v>20.612721</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>61.9</v>
@@ -12533,7 +12689,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>21.198264</v>
+        <v>21.148851</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>63.51</v>
@@ -12557,7 +12713,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>21.138184</v>
+        <v>21.088911</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>63.33</v>
@@ -12581,7 +12737,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.655541</v>
+        <v>16.616717</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -12629,7 +12785,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>40.987984</v>
+        <v>40.892441</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>122.8</v>
@@ -12653,7 +12809,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>26.104806</v>
+        <v>26.043956</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>78.20999999999999</v>
@@ -12677,7 +12833,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>44.726302</v>
+        <v>44.622045</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>134</v>
@@ -12701,7 +12857,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.1502</v>
+        <v>5.138195</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>15.43</v>
@@ -12725,7 +12881,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>14.933244</v>
+        <v>14.898435</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>44.74</v>

</xml_diff>

<commit_message>
Auto: add invoices – Supabase 2026-04-21, Anthropic 2026-04-21, Anthropic 2026-04-21, Anthropic 2026-04-21
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2297,27 +2297,123 @@
       </c>
       <c r="F18" s="24" t="n"/>
     </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="n">
+        <v>10.02</v>
+      </c>
+      <c r="E19" s="28" t="n">
+        <v>29.89</v>
+      </c>
+      <c r="F19" s="29" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D20" s="25" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="E20" s="26" t="n">
+        <v>31.32</v>
+      </c>
+      <c r="F20" s="24" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B21" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D21" s="27" t="n">
+        <v>11.17</v>
+      </c>
+      <c r="E21" s="28" t="n">
+        <v>33.32</v>
+      </c>
+      <c r="F21" s="29" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Supabase</t>
+        </is>
+      </c>
+      <c r="D22" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="E22" s="26" t="n">
+        <v>74.58</v>
+      </c>
+      <c r="F22" s="24" t="n"/>
+    </row>
+    <row r="23" ht="24" customHeight="1">
+      <c r="A23" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="31" t="n"/>
-      <c r="D19" s="20">
-        <f>SUM(D4:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="21">
-        <f>SUM(E4:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="31" t="n"/>
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="31" t="n"/>
+      <c r="D23" s="20">
+        <f>SUM(D4:D22)</f>
+        <v/>
+      </c>
+      <c r="E23" s="21">
+        <f>SUM(E4:E22)</f>
+        <v/>
+      </c>
+      <c r="F23" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3167,7 +3263,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F111"/>
+  <dimension ref="A1:F115"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6020,119 +6116,119 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D103" s="12" t="n">
-        <v>20</v>
+        <v>10.02</v>
       </c>
       <c r="E103" s="13" t="n">
-        <v>59.66</v>
+        <v>29.89</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B104" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C104" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D104" s="16" t="n">
-        <v>20</v>
+        <v>10.5</v>
       </c>
       <c r="E104" s="17" t="n">
-        <v>59.66</v>
+        <v>31.32</v>
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B105" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C105" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D105" s="12" t="n">
-        <v>20</v>
+        <v>11.17</v>
       </c>
       <c r="E105" s="13" t="n">
-        <v>59.66</v>
+        <v>33.32</v>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B106" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="C106" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="D106" s="16" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E106" s="17" t="n">
-        <v>59.66</v>
+        <v>74.58</v>
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
@@ -6153,14 +6249,14 @@
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B108" s="15" t="inlineStr">
@@ -6181,14 +6277,14 @@
       </c>
       <c r="F108" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
@@ -6209,14 +6305,14 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B110" s="15" t="inlineStr">
@@ -6237,31 +6333,143 @@
       </c>
       <c r="F110" s="14" t="inlineStr">
         <is>
+          <t>אוגוסט 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C111" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D111" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E111" s="13" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="F111" s="10" t="inlineStr">
+        <is>
+          <t>ספטמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B112" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C112" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D112" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E112" s="17" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="F112" s="14" t="inlineStr">
+        <is>
+          <t>אוקטובר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="B113" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C113" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D113" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E113" s="13" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="F113" s="10" t="inlineStr">
+        <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B114" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C114" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D114" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E114" s="17" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="F114" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" s="18" t="inlineStr">
+    <row r="115">
+      <c r="A115" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B111" s="19" t="n"/>
-      <c r="C111" s="19" t="n"/>
-      <c r="D111" s="20">
-        <f>SUM(D3:D110)</f>
-        <v/>
-      </c>
-      <c r="E111" s="21">
-        <f>SUM(E3:E110)</f>
-        <v/>
-      </c>
-      <c r="F111" s="19" t="n"/>
+      <c r="B115" s="19" t="n"/>
+      <c r="C115" s="19" t="n"/>
+      <c r="D115" s="20">
+        <f>SUM(D3:D114)</f>
+        <v/>
+      </c>
+      <c r="E115" s="21">
+        <f>SUM(E3:E114)</f>
+        <v/>
+      </c>
+      <c r="F115" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A111:C111"/>
+    <mergeCell ref="A115:C115"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6394,7 +6602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM26"/>
+  <dimension ref="A1:AM27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -9953,151 +10161,151 @@
     <row r="25">
       <c r="A25" s="36" t="inlineStr">
         <is>
-          <t>Timeless</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="B25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL25" s="39">
@@ -10109,162 +10317,321 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="30" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="41" t="inlineStr">
+        <is>
+          <t>Timeless</t>
+        </is>
+      </c>
+      <c r="B26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <v/>
+      </c>
+      <c r="C26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <v/>
+      </c>
+      <c r="D26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <v/>
+      </c>
+      <c r="E26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <v/>
+      </c>
+      <c r="F26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="G26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="H26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <v/>
+      </c>
+      <c r="I26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <v/>
+      </c>
+      <c r="J26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="K26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="L26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="M26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="N26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <v/>
+      </c>
+      <c r="O26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <v/>
+      </c>
+      <c r="P26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <v/>
+      </c>
+      <c r="Q26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <v/>
+      </c>
+      <c r="R26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <v/>
+      </c>
+      <c r="S26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <v/>
+      </c>
+      <c r="T26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <v/>
+      </c>
+      <c r="U26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <v/>
+      </c>
+      <c r="V26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <v/>
+      </c>
+      <c r="W26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <v/>
+      </c>
+      <c r="X26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <v/>
+      </c>
+      <c r="Y26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <v/>
+      </c>
+      <c r="Z26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <v/>
+      </c>
+      <c r="AA26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <v/>
+      </c>
+      <c r="AB26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <v/>
+      </c>
+      <c r="AC26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <v/>
+      </c>
+      <c r="AD26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AE26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AF26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <v/>
+      </c>
+      <c r="AG26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <v/>
+      </c>
+      <c r="AH26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AI26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AJ26" s="42">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AK26" s="43">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AL26" s="39">
+        <f>SUM(B26,D26,F26,H26,J26,L26,N26,P26,R26,T26,V26,X26,Z26,AB26,AD26,AF26,AH26,AJ26)</f>
+        <v/>
+      </c>
+      <c r="AM26" s="40">
+        <f>SUM(C26,E26,G26,I26,K26,M26,O26,Q26,S26,U26,W26,Y26,AA26,AC26,AE26,AG26,AI26,AK26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודשי</t>
         </is>
       </c>
-      <c r="B26" s="20">
-        <f>SUM(B5:B25)</f>
-        <v/>
-      </c>
-      <c r="C26" s="21">
-        <f>SUM(C5:C25)</f>
-        <v/>
-      </c>
-      <c r="D26" s="20">
-        <f>SUM(D5:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="21">
-        <f>SUM(E5:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="20">
-        <f>SUM(F5:F25)</f>
-        <v/>
-      </c>
-      <c r="G26" s="21">
-        <f>SUM(G5:G25)</f>
-        <v/>
-      </c>
-      <c r="H26" s="20">
-        <f>SUM(H5:H25)</f>
-        <v/>
-      </c>
-      <c r="I26" s="21">
-        <f>SUM(I5:I25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="20">
-        <f>SUM(J5:J25)</f>
-        <v/>
-      </c>
-      <c r="K26" s="21">
-        <f>SUM(K5:K25)</f>
-        <v/>
-      </c>
-      <c r="L26" s="20">
-        <f>SUM(L5:L25)</f>
-        <v/>
-      </c>
-      <c r="M26" s="21">
-        <f>SUM(M5:M25)</f>
-        <v/>
-      </c>
-      <c r="N26" s="20">
-        <f>SUM(N5:N25)</f>
-        <v/>
-      </c>
-      <c r="O26" s="21">
-        <f>SUM(O5:O25)</f>
-        <v/>
-      </c>
-      <c r="P26" s="20">
-        <f>SUM(P5:P25)</f>
-        <v/>
-      </c>
-      <c r="Q26" s="21">
-        <f>SUM(Q5:Q25)</f>
-        <v/>
-      </c>
-      <c r="R26" s="20">
-        <f>SUM(R5:R25)</f>
-        <v/>
-      </c>
-      <c r="S26" s="21">
-        <f>SUM(S5:S25)</f>
-        <v/>
-      </c>
-      <c r="T26" s="20">
-        <f>SUM(T5:T25)</f>
-        <v/>
-      </c>
-      <c r="U26" s="21">
-        <f>SUM(U5:U25)</f>
-        <v/>
-      </c>
-      <c r="V26" s="20">
-        <f>SUM(V5:V25)</f>
-        <v/>
-      </c>
-      <c r="W26" s="21">
-        <f>SUM(W5:W25)</f>
-        <v/>
-      </c>
-      <c r="X26" s="20">
-        <f>SUM(X5:X25)</f>
-        <v/>
-      </c>
-      <c r="Y26" s="21">
-        <f>SUM(Y5:Y25)</f>
-        <v/>
-      </c>
-      <c r="Z26" s="20">
-        <f>SUM(Z5:Z25)</f>
-        <v/>
-      </c>
-      <c r="AA26" s="21">
-        <f>SUM(AA5:AA25)</f>
-        <v/>
-      </c>
-      <c r="AB26" s="20">
-        <f>SUM(AB5:AB25)</f>
-        <v/>
-      </c>
-      <c r="AC26" s="21">
-        <f>SUM(AC5:AC25)</f>
-        <v/>
-      </c>
-      <c r="AD26" s="20">
-        <f>SUM(AD5:AD25)</f>
-        <v/>
-      </c>
-      <c r="AE26" s="21">
-        <f>SUM(AE5:AE25)</f>
-        <v/>
-      </c>
-      <c r="AF26" s="20">
-        <f>SUM(AF5:AF25)</f>
-        <v/>
-      </c>
-      <c r="AG26" s="21">
-        <f>SUM(AG5:AG25)</f>
-        <v/>
-      </c>
-      <c r="AH26" s="20">
-        <f>SUM(AH5:AH25)</f>
-        <v/>
-      </c>
-      <c r="AI26" s="21">
-        <f>SUM(AI5:AI25)</f>
-        <v/>
-      </c>
-      <c r="AJ26" s="20">
-        <f>SUM(AJ5:AJ25)</f>
-        <v/>
-      </c>
-      <c r="AK26" s="21">
-        <f>SUM(AK5:AK25)</f>
-        <v/>
-      </c>
-      <c r="AL26" s="44">
-        <f>SUM(AL5:AL25)</f>
-        <v/>
-      </c>
-      <c r="AM26" s="45">
-        <f>SUM(AM5:AM25)</f>
+      <c r="B27" s="20">
+        <f>SUM(B5:B26)</f>
+        <v/>
+      </c>
+      <c r="C27" s="21">
+        <f>SUM(C5:C26)</f>
+        <v/>
+      </c>
+      <c r="D27" s="20">
+        <f>SUM(D5:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="21">
+        <f>SUM(E5:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="20">
+        <f>SUM(F5:F26)</f>
+        <v/>
+      </c>
+      <c r="G27" s="21">
+        <f>SUM(G5:G26)</f>
+        <v/>
+      </c>
+      <c r="H27" s="20">
+        <f>SUM(H5:H26)</f>
+        <v/>
+      </c>
+      <c r="I27" s="21">
+        <f>SUM(I5:I26)</f>
+        <v/>
+      </c>
+      <c r="J27" s="20">
+        <f>SUM(J5:J26)</f>
+        <v/>
+      </c>
+      <c r="K27" s="21">
+        <f>SUM(K5:K26)</f>
+        <v/>
+      </c>
+      <c r="L27" s="20">
+        <f>SUM(L5:L26)</f>
+        <v/>
+      </c>
+      <c r="M27" s="21">
+        <f>SUM(M5:M26)</f>
+        <v/>
+      </c>
+      <c r="N27" s="20">
+        <f>SUM(N5:N26)</f>
+        <v/>
+      </c>
+      <c r="O27" s="21">
+        <f>SUM(O5:O26)</f>
+        <v/>
+      </c>
+      <c r="P27" s="20">
+        <f>SUM(P5:P26)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="21">
+        <f>SUM(Q5:Q26)</f>
+        <v/>
+      </c>
+      <c r="R27" s="20">
+        <f>SUM(R5:R26)</f>
+        <v/>
+      </c>
+      <c r="S27" s="21">
+        <f>SUM(S5:S26)</f>
+        <v/>
+      </c>
+      <c r="T27" s="20">
+        <f>SUM(T5:T26)</f>
+        <v/>
+      </c>
+      <c r="U27" s="21">
+        <f>SUM(U5:U26)</f>
+        <v/>
+      </c>
+      <c r="V27" s="20">
+        <f>SUM(V5:V26)</f>
+        <v/>
+      </c>
+      <c r="W27" s="21">
+        <f>SUM(W5:W26)</f>
+        <v/>
+      </c>
+      <c r="X27" s="20">
+        <f>SUM(X5:X26)</f>
+        <v/>
+      </c>
+      <c r="Y27" s="21">
+        <f>SUM(Y5:Y26)</f>
+        <v/>
+      </c>
+      <c r="Z27" s="20">
+        <f>SUM(Z5:Z26)</f>
+        <v/>
+      </c>
+      <c r="AA27" s="21">
+        <f>SUM(AA5:AA26)</f>
+        <v/>
+      </c>
+      <c r="AB27" s="20">
+        <f>SUM(AB5:AB26)</f>
+        <v/>
+      </c>
+      <c r="AC27" s="21">
+        <f>SUM(AC5:AC26)</f>
+        <v/>
+      </c>
+      <c r="AD27" s="20">
+        <f>SUM(AD5:AD26)</f>
+        <v/>
+      </c>
+      <c r="AE27" s="21">
+        <f>SUM(AE5:AE26)</f>
+        <v/>
+      </c>
+      <c r="AF27" s="20">
+        <f>SUM(AF5:AF26)</f>
+        <v/>
+      </c>
+      <c r="AG27" s="21">
+        <f>SUM(AG5:AG26)</f>
+        <v/>
+      </c>
+      <c r="AH27" s="20">
+        <f>SUM(AH5:AH26)</f>
+        <v/>
+      </c>
+      <c r="AI27" s="21">
+        <f>SUM(AI5:AI26)</f>
+        <v/>
+      </c>
+      <c r="AJ27" s="20">
+        <f>SUM(AJ5:AJ26)</f>
+        <v/>
+      </c>
+      <c r="AK27" s="21">
+        <f>SUM(AK5:AK26)</f>
+        <v/>
+      </c>
+      <c r="AL27" s="44">
+        <f>SUM(AL5:AL26)</f>
+        <v/>
+      </c>
+      <c r="AM27" s="45">
+        <f>SUM(AM5:AM26)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Stop auto-recurring entries from being suppressed by different-product manual entries
Dedup key was (month, tool), so a manual ChatGPT Pro upgrade on Apr 18
suppressed the recurring ChatGPT Plus charge on Apr 16. Add description
to the dedup key so distinct products in the same month coexist.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2156,24 +2156,24 @@
     <row r="13">
       <c r="A13" s="10" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Pro – Apr 2026 (₪49.90)</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>16.728126</v>
+        <v>20</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>49.9</v>
+        <v>59.66</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -2185,50 +2185,50 @@
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Pro Subscription</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>81.2</v>
+        <v>16.728126</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>242.22</v>
+        <v>49.9</v>
       </c>
       <c r="F14" s="24" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="10" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>ChatGPT Pro Subscription</t>
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5</v>
+        <v>81.2</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>14.92</v>
+        <v>242.22</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="14" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
@@ -2238,14 +2238,14 @@
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>15.14</v>
+        <v>5</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>45.16</v>
+        <v>14.92</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
@@ -2262,21 +2262,21 @@
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>10</v>
+        <v>15.14</v>
       </c>
       <c r="E17" s="28" t="n">
-        <v>29.83</v>
+        <v>45.16</v>
       </c>
       <c r="F17" s="29" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -2286,14 +2286,14 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D18" s="25" t="n">
-        <v>10.15</v>
+        <v>10</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>30.28</v>
+        <v>29.83</v>
       </c>
       <c r="F18" s="24" t="n"/>
     </row>
@@ -2314,10 +2314,10 @@
         </is>
       </c>
       <c r="D19" s="27" t="n">
-        <v>10.02</v>
+        <v>10.15</v>
       </c>
       <c r="E19" s="28" t="n">
-        <v>29.89</v>
+        <v>30.28</v>
       </c>
       <c r="F19" s="29" t="n"/>
     </row>
@@ -2338,10 +2338,10 @@
         </is>
       </c>
       <c r="D20" s="25" t="n">
-        <v>10.5</v>
+        <v>10.02</v>
       </c>
       <c r="E20" s="26" t="n">
-        <v>31.32</v>
+        <v>29.89</v>
       </c>
       <c r="F20" s="24" t="n"/>
     </row>
@@ -2362,10 +2362,10 @@
         </is>
       </c>
       <c r="D21" s="27" t="n">
-        <v>11.17</v>
+        <v>10.5</v>
       </c>
       <c r="E21" s="28" t="n">
-        <v>33.32</v>
+        <v>31.32</v>
       </c>
       <c r="F21" s="29" t="n"/>
     </row>
@@ -2377,43 +2377,67 @@
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D22" s="25" t="n">
+        <v>11.17</v>
+      </c>
+      <c r="E22" s="26" t="n">
+        <v>33.32</v>
+      </c>
+      <c r="F22" s="24" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-21</t>
+        </is>
+      </c>
+      <c r="B23" s="11" t="inlineStr">
+        <is>
           <t>Supabase</t>
         </is>
       </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>Supabase</t>
         </is>
       </c>
-      <c r="D22" s="25" t="n">
+      <c r="D23" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="E22" s="26" t="n">
+      <c r="E23" s="28" t="n">
         <v>74.58</v>
       </c>
-      <c r="F22" s="24" t="n"/>
-    </row>
-    <row r="23" ht="24" customHeight="1">
-      <c r="A23" s="30" t="inlineStr">
+      <c r="F23" s="29" t="n"/>
+    </row>
+    <row r="24" ht="24" customHeight="1">
+      <c r="A24" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B23" s="31" t="n"/>
-      <c r="C23" s="31" t="n"/>
-      <c r="D23" s="20">
-        <f>SUM(D4:D22)</f>
-        <v/>
-      </c>
-      <c r="E23" s="21">
-        <f>SUM(E4:E22)</f>
-        <v/>
-      </c>
-      <c r="F23" s="31" t="n"/>
+      <c r="B24" s="31" t="n"/>
+      <c r="C24" s="31" t="n"/>
+      <c r="D24" s="20">
+        <f>SUM(D4:D23)</f>
+        <v/>
+      </c>
+      <c r="E24" s="21">
+        <f>SUM(E4:E23)</f>
+        <v/>
+      </c>
+      <c r="F24" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3263,7 +3287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F115"/>
+  <dimension ref="A1:F116"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5948,24 +5972,24 @@
     <row r="97">
       <c r="A97" s="10" t="inlineStr">
         <is>
-          <t>2026-04-18</t>
+          <t>2026-04-16</t>
         </is>
       </c>
       <c r="B97" s="11" t="inlineStr">
         <is>
-          <t>CapCut</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Pro – Apr 2026 (₪49.90)</t>
+          <t>ChatGPT Plus</t>
         </is>
       </c>
       <c r="D97" s="12" t="n">
-        <v>16.728126</v>
+        <v>20</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>49.9</v>
+        <v>59.66</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -5981,19 +6005,19 @@
       </c>
       <c r="B98" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>CapCut</t>
         </is>
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Pro Subscription</t>
+          <t>Pro – Apr 2026 (₪49.90)</t>
         </is>
       </c>
       <c r="D98" s="16" t="n">
-        <v>81.2</v>
+        <v>16.728126</v>
       </c>
       <c r="E98" s="17" t="n">
-        <v>242.22</v>
+        <v>49.9</v>
       </c>
       <c r="F98" s="14" t="inlineStr">
         <is>
@@ -6004,24 +6028,24 @@
     <row r="99">
       <c r="A99" s="10" t="inlineStr">
         <is>
-          <t>2026-04-19</t>
+          <t>2026-04-18</t>
         </is>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="C99" s="11" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>ChatGPT Pro Subscription</t>
         </is>
       </c>
       <c r="D99" s="12" t="n">
-        <v>5</v>
+        <v>81.2</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>14.92</v>
+        <v>242.22</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
@@ -6032,7 +6056,7 @@
     <row r="100">
       <c r="A100" s="14" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B100" s="15" t="inlineStr">
@@ -6042,14 +6066,14 @@
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D100" s="16" t="n">
-        <v>15.14</v>
+        <v>5</v>
       </c>
       <c r="E100" s="17" t="n">
-        <v>45.16</v>
+        <v>14.92</v>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
@@ -6070,14 +6094,14 @@
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D101" s="12" t="n">
-        <v>10</v>
+        <v>15.14</v>
       </c>
       <c r="E101" s="13" t="n">
-        <v>29.83</v>
+        <v>45.16</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
@@ -6088,7 +6112,7 @@
     <row r="102">
       <c r="A102" s="14" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B102" s="15" t="inlineStr">
@@ -6098,14 +6122,14 @@
       </c>
       <c r="C102" s="15" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D102" s="16" t="n">
-        <v>10.15</v>
+        <v>10</v>
       </c>
       <c r="E102" s="17" t="n">
-        <v>30.28</v>
+        <v>29.83</v>
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
@@ -6130,10 +6154,10 @@
         </is>
       </c>
       <c r="D103" s="12" t="n">
-        <v>10.02</v>
+        <v>10.15</v>
       </c>
       <c r="E103" s="13" t="n">
-        <v>29.89</v>
+        <v>30.28</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
@@ -6158,10 +6182,10 @@
         </is>
       </c>
       <c r="D104" s="16" t="n">
-        <v>10.5</v>
+        <v>10.02</v>
       </c>
       <c r="E104" s="17" t="n">
-        <v>31.32</v>
+        <v>29.89</v>
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
@@ -6186,10 +6210,10 @@
         </is>
       </c>
       <c r="D105" s="12" t="n">
-        <v>11.17</v>
+        <v>10.5</v>
       </c>
       <c r="E105" s="13" t="n">
-        <v>33.32</v>
+        <v>31.32</v>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
@@ -6205,19 +6229,19 @@
       </c>
       <c r="B106" s="15" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C106" s="15" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D106" s="16" t="n">
-        <v>25</v>
+        <v>11.17</v>
       </c>
       <c r="E106" s="17" t="n">
-        <v>74.58</v>
+        <v>33.32</v>
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
@@ -6228,35 +6252,35 @@
     <row r="107">
       <c r="A107" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="D107" s="12" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="E107" s="13" t="n">
-        <v>59.66</v>
+        <v>74.58</v>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B108" s="15" t="inlineStr">
@@ -6277,14 +6301,14 @@
       </c>
       <c r="F108" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
@@ -6305,14 +6329,14 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B110" s="15" t="inlineStr">
@@ -6333,14 +6357,14 @@
       </c>
       <c r="F110" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
@@ -6361,14 +6385,14 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B112" s="15" t="inlineStr">
@@ -6389,14 +6413,14 @@
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
@@ -6417,14 +6441,14 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B114" s="15" t="inlineStr">
@@ -6445,32 +6469,60 @@
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B115" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C115" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D115" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E115" s="13" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="F115" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" s="18" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B115" s="19" t="n"/>
-      <c r="C115" s="19" t="n"/>
-      <c r="D115" s="20">
-        <f>SUM(D3:D114)</f>
-        <v/>
-      </c>
-      <c r="E115" s="21">
-        <f>SUM(E3:E114)</f>
-        <v/>
-      </c>
-      <c r="F115" s="19" t="n"/>
+      <c r="B116" s="19" t="n"/>
+      <c r="C116" s="19" t="n"/>
+      <c r="D116" s="20">
+        <f>SUM(D3:D115)</f>
+        <v/>
+      </c>
+      <c r="E116" s="21">
+        <f>SUM(E3:E115)</f>
+        <v/>
+      </c>
+      <c r="F116" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A115:C115"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A116:C116"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add client-side live refresh polling every 60s
New LiveRefresh component fetches /data.json on an interval and reloads
the page when built_at changes. build_report.py now writes a fresh
built_at timestamp on every build, so dashboard sees new data as soon as
CI republishes GitHub Pages (max ~1-2 min after scanner push).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2417,27 +2417,51 @@
       </c>
       <c r="F23" s="29" t="n"/>
     </row>
-    <row r="24" ht="24" customHeight="1">
-      <c r="A24" s="30" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-22</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D24" s="25" t="n">
+        <v>15.57</v>
+      </c>
+      <c r="E24" s="26" t="n">
+        <v>46.45</v>
+      </c>
+      <c r="F24" s="24" t="n"/>
+    </row>
+    <row r="25" ht="24" customHeight="1">
+      <c r="A25" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B24" s="31" t="n"/>
-      <c r="C24" s="31" t="n"/>
-      <c r="D24" s="20">
-        <f>SUM(D4:D23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="21">
-        <f>SUM(E4:E23)</f>
-        <v/>
-      </c>
-      <c r="F24" s="31" t="n"/>
+      <c r="B25" s="31" t="n"/>
+      <c r="C25" s="31" t="n"/>
+      <c r="D25" s="20">
+        <f>SUM(D4:D24)</f>
+        <v/>
+      </c>
+      <c r="E25" s="21">
+        <f>SUM(E4:E24)</f>
+        <v/>
+      </c>
+      <c r="F25" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="A25:C25"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3287,7 +3311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F116"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6280,35 +6304,35 @@
     <row r="108">
       <c r="A108" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B108" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C108" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D108" s="16" t="n">
-        <v>20</v>
+        <v>15.57</v>
       </c>
       <c r="E108" s="17" t="n">
-        <v>59.66</v>
+        <v>46.45</v>
       </c>
       <c r="F108" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B109" s="11" t="inlineStr">
@@ -6329,14 +6353,14 @@
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B110" s="15" t="inlineStr">
@@ -6357,14 +6381,14 @@
       </c>
       <c r="F110" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
@@ -6385,14 +6409,14 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B112" s="15" t="inlineStr">
@@ -6413,14 +6437,14 @@
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
@@ -6441,14 +6465,14 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B114" s="15" t="inlineStr">
@@ -6469,14 +6493,14 @@
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
@@ -6497,32 +6521,60 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B116" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C116" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D116" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E116" s="17" t="n">
+        <v>59.66</v>
+      </c>
+      <c r="F116" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="18" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B116" s="19" t="n"/>
-      <c r="C116" s="19" t="n"/>
-      <c r="D116" s="20">
-        <f>SUM(D3:D115)</f>
-        <v/>
-      </c>
-      <c r="E116" s="21">
-        <f>SUM(E3:E115)</f>
-        <v/>
-      </c>
-      <c r="F116" s="19" t="n"/>
+      <c r="B117" s="19" t="n"/>
+      <c r="C117" s="19" t="n"/>
+      <c r="D117" s="20">
+        <f>SUM(D3:D116)</f>
+        <v/>
+      </c>
+      <c r="E117" s="21">
+        <f>SUM(E3:E116)</f>
+        <v/>
+      </c>
+      <c r="F117" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A117:C117"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A116:C116"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-04-23
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F26"/>
+  <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2465,27 +2465,51 @@
       </c>
       <c r="F25" s="29" t="n"/>
     </row>
-    <row r="26" ht="24" customHeight="1">
-      <c r="A26" s="30" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-23</t>
+        </is>
+      </c>
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D26" s="25" t="n">
+        <v>10.16</v>
+      </c>
+      <c r="E26" s="26" t="n">
+        <v>30.53</v>
+      </c>
+      <c r="F26" s="24" t="n"/>
+    </row>
+    <row r="27" ht="24" customHeight="1">
+      <c r="A27" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B26" s="31" t="n"/>
-      <c r="C26" s="31" t="n"/>
-      <c r="D26" s="20">
-        <f>SUM(D4:D25)</f>
-        <v/>
-      </c>
-      <c r="E26" s="21">
-        <f>SUM(E4:E25)</f>
-        <v/>
-      </c>
-      <c r="F26" s="31" t="n"/>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="31" t="n"/>
+      <c r="D27" s="20">
+        <f>SUM(D4:D26)</f>
+        <v/>
+      </c>
+      <c r="E27" s="21">
+        <f>SUM(E4:E26)</f>
+        <v/>
+      </c>
+      <c r="F27" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A27:C27"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3335,7 +3359,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F118"/>
+  <dimension ref="A1:F119"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6384,35 +6408,35 @@
     <row r="110">
       <c r="A110" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B110" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C110" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D110" s="16" t="n">
-        <v>20</v>
+        <v>10.16</v>
       </c>
       <c r="E110" s="17" t="n">
-        <v>60.1</v>
+        <v>30.53</v>
       </c>
       <c r="F110" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
@@ -6433,14 +6457,14 @@
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B112" s="15" t="inlineStr">
@@ -6461,14 +6485,14 @@
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
@@ -6489,14 +6513,14 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B114" s="15" t="inlineStr">
@@ -6517,14 +6541,14 @@
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
@@ -6545,14 +6569,14 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B116" s="15" t="inlineStr">
@@ -6573,14 +6597,14 @@
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
@@ -6601,32 +6625,60 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B118" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C118" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D118" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E118" s="17" t="n">
+        <v>60.1</v>
+      </c>
+      <c r="F118" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="18" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B118" s="19" t="n"/>
-      <c r="C118" s="19" t="n"/>
-      <c r="D118" s="20">
-        <f>SUM(D3:D117)</f>
-        <v/>
-      </c>
-      <c r="E118" s="21">
-        <f>SUM(E3:E117)</f>
-        <v/>
-      </c>
-      <c r="F118" s="19" t="n"/>
+      <c r="B119" s="19" t="n"/>
+      <c r="C119" s="19" t="n"/>
+      <c r="D119" s="20">
+        <f>SUM(D3:D118)</f>
+        <v/>
+      </c>
+      <c r="E119" s="21">
+        <f>SUM(E3:E118)</f>
+        <v/>
+      </c>
+      <c r="F119" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A118:C118"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A119:C119"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Security: enforce CSP, add security.txt, harden headers
- CSP now enforcing via meta tag (GH Pages) + vercel.json (API).
  Report-Only removed. Tight allowlist for scripts/styles/connect.
- Added /.well-known/security.txt with roi@rt-ai.co.il contact.
- Added Cross-Origin-Opener-Policy + Cross-Origin-Resource-Policy
  to vercel.json for defense in depth.
- Postbuild preserves .well-known from the .txt cleanup pass.
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Security: switch manual import to secure Vercel gateway
Gateway now holds the GitHub PAT server-side (env vars on Vercel).
Dashboard no longer stores or transmits a token from the browser.
Config: https://ai-tools-expense-gateway.vercel.app
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Remove obsolete GitHub token card from settings page
Dashboard now runs in gateway mode - token lives on Vercel.
The token card was dead UI. Also clears any legacy localStorage
token on mount for users upgrading from the previous version.
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Auto: add invoices – Meta (Ads) 2026-04-26
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F27"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2489,27 +2489,51 @@
       </c>
       <c r="F26" s="24" t="n"/>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="30" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B27" s="11" t="inlineStr">
+        <is>
+          <t>Meta (Ads)</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Facebook Ads</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="n">
+        <v>51</v>
+      </c>
+      <c r="E27" s="28" t="n">
+        <v>153.15</v>
+      </c>
+      <c r="F27" s="29" t="n"/>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B27" s="31" t="n"/>
-      <c r="C27" s="31" t="n"/>
-      <c r="D27" s="20">
-        <f>SUM(D4:D26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="21">
-        <f>SUM(E4:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="31" t="n"/>
+      <c r="B28" s="31" t="n"/>
+      <c r="C28" s="31" t="n"/>
+      <c r="D28" s="20">
+        <f>SUM(D4:D27)</f>
+        <v/>
+      </c>
+      <c r="E28" s="21">
+        <f>SUM(E4:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="A28:C28"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3359,7 +3383,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F119"/>
+  <dimension ref="A1:F120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6436,35 +6460,35 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D111" s="12" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="E111" s="13" t="n">
-        <v>60.06</v>
+        <v>153.15</v>
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B112" s="15" t="inlineStr">
@@ -6485,14 +6509,14 @@
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
@@ -6513,14 +6537,14 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B114" s="15" t="inlineStr">
@@ -6541,14 +6565,14 @@
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
@@ -6569,14 +6593,14 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B116" s="15" t="inlineStr">
@@ -6597,14 +6621,14 @@
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
@@ -6625,14 +6649,14 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
@@ -6653,32 +6677,60 @@
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B119" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C119" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D119" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E119" s="13" t="n">
+        <v>60.06</v>
+      </c>
+      <c r="F119" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="18" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B119" s="19" t="n"/>
-      <c r="C119" s="19" t="n"/>
-      <c r="D119" s="20">
-        <f>SUM(D3:D118)</f>
-        <v/>
-      </c>
-      <c r="E119" s="21">
-        <f>SUM(E3:E118)</f>
-        <v/>
-      </c>
-      <c r="F119" s="19" t="n"/>
+      <c r="B120" s="19" t="n"/>
+      <c r="C120" s="19" t="n"/>
+      <c r="D120" s="20">
+        <f>SUM(D3:D119)</f>
+        <v/>
+      </c>
+      <c r="E120" s="21">
+        <f>SUM(E3:E119)</f>
+        <v/>
+      </c>
+      <c r="F120" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A120:C120"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A119:C119"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – Lovable 2026-04-26
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2497,43 +2497,67 @@
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
+          <t>Lovable</t>
+        </is>
+      </c>
+      <c r="C27" s="11" t="inlineStr">
+        <is>
+          <t>Lovable</t>
+        </is>
+      </c>
+      <c r="D27" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E27" s="28" t="n">
+        <v>15.02</v>
+      </c>
+      <c r="F27" s="29" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="B28" s="15" t="inlineStr">
+        <is>
           <t>Meta (Ads)</t>
         </is>
       </c>
-      <c r="C27" s="11" t="inlineStr">
+      <c r="C28" s="15" t="inlineStr">
         <is>
           <t>Facebook Ads</t>
         </is>
       </c>
-      <c r="D27" s="27" t="n">
+      <c r="D28" s="25" t="n">
         <v>51</v>
       </c>
-      <c r="E27" s="28" t="n">
+      <c r="E28" s="26" t="n">
         <v>153.15</v>
       </c>
-      <c r="F27" s="29" t="n"/>
-    </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="30" t="inlineStr">
+      <c r="F28" s="24" t="n"/>
+    </row>
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B28" s="31" t="n"/>
-      <c r="C28" s="31" t="n"/>
-      <c r="D28" s="20">
-        <f>SUM(D4:D27)</f>
-        <v/>
-      </c>
-      <c r="E28" s="21">
-        <f>SUM(E4:E27)</f>
-        <v/>
-      </c>
-      <c r="F28" s="31" t="n"/>
+      <c r="B29" s="31" t="n"/>
+      <c r="C29" s="31" t="n"/>
+      <c r="D29" s="20">
+        <f>SUM(D4:D28)</f>
+        <v/>
+      </c>
+      <c r="E29" s="21">
+        <f>SUM(E4:E28)</f>
+        <v/>
+      </c>
+      <c r="F29" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A28:C28"/>
+    <mergeCell ref="A29:C29"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3383,7 +3407,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F120"/>
+  <dimension ref="A1:F121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6465,19 +6489,19 @@
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="D111" s="12" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E111" s="13" t="n">
-        <v>153.15</v>
+        <v>15.02</v>
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
@@ -6488,35 +6512,35 @@
     <row r="112">
       <c r="A112" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B112" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C112" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D112" s="16" t="n">
-        <v>20</v>
+        <v>51</v>
       </c>
       <c r="E112" s="17" t="n">
-        <v>60.06</v>
+        <v>153.15</v>
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
@@ -6537,14 +6561,14 @@
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B114" s="15" t="inlineStr">
@@ -6565,14 +6589,14 @@
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
@@ -6593,14 +6617,14 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B116" s="15" t="inlineStr">
@@ -6621,14 +6645,14 @@
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
@@ -6649,14 +6673,14 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
@@ -6677,14 +6701,14 @@
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
@@ -6705,32 +6729,60 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B120" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C120" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D120" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E120" s="17" t="n">
+        <v>60.06</v>
+      </c>
+      <c r="F120" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="18" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B120" s="19" t="n"/>
-      <c r="C120" s="19" t="n"/>
-      <c r="D120" s="20">
-        <f>SUM(D3:D119)</f>
-        <v/>
-      </c>
-      <c r="E120" s="21">
-        <f>SUM(E3:E119)</f>
-        <v/>
-      </c>
-      <c r="F120" s="19" t="n"/>
+      <c r="B121" s="19" t="n"/>
+      <c r="C121" s="19" t="n"/>
+      <c r="D121" s="20">
+        <f>SUM(D3:D120)</f>
+        <v/>
+      </c>
+      <c r="E121" s="21">
+        <f>SUM(E3:E120)</f>
+        <v/>
+      </c>
+      <c r="F121" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A120:C120"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A121:C121"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-04-28
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F30"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2561,28 +2561,52 @@
       </c>
       <c r="F29" s="29" t="n"/>
     </row>
-    <row r="30" ht="24" customHeight="1">
-      <c r="A30" s="30" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="14" t="inlineStr">
+        <is>
+          <t>2026-04-28</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D30" s="25" t="n">
+        <v>10.56</v>
+      </c>
+      <c r="E30" s="26" t="n">
+        <v>31.58</v>
+      </c>
+      <c r="F30" s="24" t="n"/>
+    </row>
+    <row r="31" ht="24" customHeight="1">
+      <c r="A31" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B30" s="31" t="n"/>
-      <c r="C30" s="31" t="n"/>
-      <c r="D30" s="20">
-        <f>SUM(D4:D29)</f>
-        <v/>
-      </c>
-      <c r="E30" s="21">
-        <f>SUM(E4:E29)</f>
-        <v/>
-      </c>
-      <c r="F30" s="31" t="n"/>
+      <c r="B31" s="31" t="n"/>
+      <c r="C31" s="31" t="n"/>
+      <c r="D31" s="20">
+        <f>SUM(D4:D30)</f>
+        <v/>
+      </c>
+      <c r="E31" s="21">
+        <f>SUM(E4:E30)</f>
+        <v/>
+      </c>
+      <c r="F31" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A30:C30"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3431,7 +3455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F122"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6592,35 +6616,35 @@
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B114" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C114" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D114" s="16" t="n">
-        <v>20</v>
+        <v>10.56</v>
       </c>
       <c r="E114" s="17" t="n">
-        <v>59.82</v>
+        <v>31.58</v>
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
@@ -6641,14 +6665,14 @@
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B116" s="15" t="inlineStr">
@@ -6669,14 +6693,14 @@
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
@@ -6697,14 +6721,14 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
@@ -6725,14 +6749,14 @@
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
@@ -6753,14 +6777,14 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
@@ -6781,14 +6805,14 @@
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -6809,32 +6833,60 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B122" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C122" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D122" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E122" s="17" t="n">
+        <v>59.82</v>
+      </c>
+      <c r="F122" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="18" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B122" s="19" t="n"/>
-      <c r="C122" s="19" t="n"/>
-      <c r="D122" s="20">
-        <f>SUM(D3:D121)</f>
-        <v/>
-      </c>
-      <c r="E122" s="21">
-        <f>SUM(E3:E121)</f>
-        <v/>
-      </c>
-      <c r="F122" s="19" t="n"/>
+      <c r="B123" s="19" t="n"/>
+      <c r="C123" s="19" t="n"/>
+      <c r="D123" s="20">
+        <f>SUM(D3:D122)</f>
+        <v/>
+      </c>
+      <c r="E123" s="21">
+        <f>SUM(E3:E122)</f>
+        <v/>
+      </c>
+      <c r="F123" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A123:C123"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A122:C122"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-05-01
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2622,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2683,49 +2683,73 @@
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E4" s="26" t="n">
+        <v>30.66</v>
+      </c>
+      <c r="F4" s="24" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n">
+      <c r="D5" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E4" s="26" t="n">
+      <c r="E5" s="28" t="n">
         <v>58.96</v>
       </c>
-      <c r="F4" s="24" t="n"/>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="F5" s="29" t="n"/>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B5" s="31" t="n"/>
-      <c r="C5" s="31" t="n"/>
-      <c r="D5" s="20">
-        <f>SUM(D4:D4)</f>
-        <v/>
-      </c>
-      <c r="E5" s="21">
-        <f>SUM(E4:E4)</f>
-        <v/>
-      </c>
-      <c r="F5" s="31" t="n"/>
+      <c r="B6" s="31" t="n"/>
+      <c r="C6" s="31" t="n"/>
+      <c r="D6" s="20">
+        <f>SUM(D4:D5)</f>
+        <v/>
+      </c>
+      <c r="E6" s="21">
+        <f>SUM(E4:E5)</f>
+        <v/>
+      </c>
+      <c r="F6" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A5:C5"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A6:C6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3455,7 +3479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F123"/>
+  <dimension ref="A1:F124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6644,24 +6668,24 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D115" s="12" t="n">
-        <v>20</v>
+        <v>10.4</v>
       </c>
       <c r="E115" s="13" t="n">
-        <v>58.96</v>
+        <v>30.66</v>
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
@@ -6672,7 +6696,7 @@
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B116" s="15" t="inlineStr">
@@ -6693,14 +6717,14 @@
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
@@ -6721,14 +6745,14 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
@@ -6749,14 +6773,14 @@
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
@@ -6777,14 +6801,14 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
@@ -6805,14 +6829,14 @@
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -6833,14 +6857,14 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B122" s="15" t="inlineStr">
@@ -6861,31 +6885,59 @@
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D123" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E123" s="13" t="n">
+        <v>58.96</v>
+      </c>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="18" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B123" s="19" t="n"/>
-      <c r="C123" s="19" t="n"/>
-      <c r="D123" s="20">
-        <f>SUM(D3:D122)</f>
-        <v/>
-      </c>
-      <c r="E123" s="21">
-        <f>SUM(E3:E122)</f>
-        <v/>
-      </c>
-      <c r="F123" s="19" t="n"/>
+      <c r="B124" s="19" t="n"/>
+      <c r="C124" s="19" t="n"/>
+      <c r="D124" s="20">
+        <f>SUM(D3:D123)</f>
+        <v/>
+      </c>
+      <c r="E124" s="21">
+        <f>SUM(E3:E123)</f>
+        <v/>
+      </c>
+      <c r="F124" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A123:C123"/>
+    <mergeCell ref="A124:C124"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto: add invoices – Google Workspace 2026-05-01
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2622,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2707,49 +2707,73 @@
     <row r="5">
       <c r="A5" s="10" t="inlineStr">
         <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Google Workspace (₪75.90)</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>25.746269</v>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="F5" s="29" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B6" s="15" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C6" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D5" s="27" t="n">
+      <c r="D6" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E5" s="28" t="n">
+      <c r="E6" s="26" t="n">
         <v>58.96</v>
       </c>
-      <c r="F5" s="29" t="n"/>
-    </row>
-    <row r="6" ht="24" customHeight="1">
-      <c r="A6" s="30" t="inlineStr">
+      <c r="F6" s="24" t="n"/>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B6" s="31" t="n"/>
-      <c r="C6" s="31" t="n"/>
-      <c r="D6" s="20">
-        <f>SUM(D4:D5)</f>
-        <v/>
-      </c>
-      <c r="E6" s="21">
-        <f>SUM(E4:E5)</f>
-        <v/>
-      </c>
-      <c r="F6" s="31" t="n"/>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="31" t="n"/>
+      <c r="D7" s="20">
+        <f>SUM(D4:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="21">
+        <f>SUM(E4:E6)</f>
+        <v/>
+      </c>
+      <c r="F7" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A7:C7"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A6:C6"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3479,7 +3503,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6696,24 +6720,24 @@
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B116" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C116" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Google Workspace (₪75.90)</t>
         </is>
       </c>
       <c r="D116" s="16" t="n">
-        <v>20</v>
+        <v>25.746269</v>
       </c>
       <c r="E116" s="17" t="n">
-        <v>58.96</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
@@ -6724,7 +6748,7 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
@@ -6745,14 +6769,14 @@
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
@@ -6773,14 +6797,14 @@
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
@@ -6801,14 +6825,14 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
@@ -6829,14 +6853,14 @@
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -6857,14 +6881,14 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B122" s="15" t="inlineStr">
@@ -6885,14 +6909,14 @@
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
@@ -6913,32 +6937,60 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C124" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D124" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E124" s="17" t="n">
+        <v>58.96</v>
+      </c>
+      <c r="F124" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="18" t="inlineStr">
+    <row r="125">
+      <c r="A125" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B124" s="19" t="n"/>
-      <c r="C124" s="19" t="n"/>
-      <c r="D124" s="20">
-        <f>SUM(D3:D123)</f>
-        <v/>
-      </c>
-      <c r="E124" s="21">
-        <f>SUM(E3:E123)</f>
-        <v/>
-      </c>
-      <c r="F124" s="19" t="n"/>
+      <c r="B125" s="19" t="n"/>
+      <c r="C125" s="19" t="n"/>
+      <c r="D125" s="20">
+        <f>SUM(D3:D124)</f>
+        <v/>
+      </c>
+      <c r="E125" s="21">
+        <f>SUM(E3:E124)</f>
+        <v/>
+      </c>
+      <c r="F125" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A124:C124"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A125:C125"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix: detect Google Cloud payments and backfill missed ₪8.23 charge
The Gmail scanner mapped every payments-noreply@google.com email to
"Google Workspace" with source="pdf". Google Cloud's "התקבל תשלום"
confirmations have no PDF — the amount is in the body — so the scanner
returned None and silently marked the message as processed.

- auto_invoice.py: route payments-noreply@google.com by body content
  ("google cloud" → Google Cloud / body, otherwise → Google Workspace / pdf)
  and add a Google Cloud description.
- build_report.py: backfill the 2026-05-01 ₪8.23 Google Cloud Platform &
  APIs charge that was dropped by the old code path.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2622,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2712,67 +2712,91 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.90)</t>
+          <t>Google Cloud Platform &amp; APIs (₪8.23)</t>
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>25.746269</v>
+        <v>2.791723</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>75.90000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
         <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Google Workspace (₪75.90)</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>25.746269</v>
+      </c>
+      <c r="E6" s="26" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="F6" s="24" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B6" s="15" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D6" s="25" t="n">
+      <c r="D7" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E6" s="26" t="n">
+      <c r="E7" s="28" t="n">
         <v>58.96</v>
       </c>
-      <c r="F6" s="24" t="n"/>
-    </row>
-    <row r="7" ht="24" customHeight="1">
-      <c r="A7" s="30" t="inlineStr">
+      <c r="F7" s="29" t="n"/>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="31" t="n"/>
-      <c r="D7" s="20">
-        <f>SUM(D4:D6)</f>
-        <v/>
-      </c>
-      <c r="E7" s="21">
-        <f>SUM(E4:E6)</f>
-        <v/>
-      </c>
-      <c r="F7" s="31" t="n"/>
+      <c r="B8" s="31" t="n"/>
+      <c r="C8" s="31" t="n"/>
+      <c r="D8" s="20">
+        <f>SUM(D4:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="21">
+        <f>SUM(E4:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A8:C8"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3503,7 +3527,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F125"/>
+  <dimension ref="A1:F126"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6725,19 +6749,19 @@
       </c>
       <c r="B116" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="C116" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.90)</t>
+          <t>Google Cloud Platform &amp; APIs (₪8.23)</t>
         </is>
       </c>
       <c r="D116" s="16" t="n">
-        <v>25.746269</v>
+        <v>2.791723</v>
       </c>
       <c r="E116" s="17" t="n">
-        <v>75.90000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
@@ -6748,24 +6772,24 @@
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Google Workspace (₪75.90)</t>
         </is>
       </c>
       <c r="D117" s="12" t="n">
-        <v>20</v>
+        <v>25.746269</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>58.96</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
@@ -6776,7 +6800,7 @@
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
@@ -6797,14 +6821,14 @@
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
@@ -6825,14 +6849,14 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
@@ -6853,14 +6877,14 @@
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -6881,14 +6905,14 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B122" s="15" t="inlineStr">
@@ -6909,14 +6933,14 @@
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
@@ -6937,14 +6961,14 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B124" s="15" t="inlineStr">
@@ -6965,32 +6989,60 @@
       </c>
       <c r="F124" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D125" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E125" s="13" t="n">
+        <v>58.96</v>
+      </c>
+      <c r="F125" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="125">
-      <c r="A125" s="18" t="inlineStr">
+    <row r="126">
+      <c r="A126" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B125" s="19" t="n"/>
-      <c r="C125" s="19" t="n"/>
-      <c r="D125" s="20">
-        <f>SUM(D3:D124)</f>
-        <v/>
-      </c>
-      <c r="E125" s="21">
-        <f>SUM(E3:E124)</f>
-        <v/>
-      </c>
-      <c r="F125" s="19" t="n"/>
+      <c r="B126" s="19" t="n"/>
+      <c r="C126" s="19" t="n"/>
+      <c r="D126" s="20">
+        <f>SUM(D3:D125)</f>
+        <v/>
+      </c>
+      <c r="E126" s="21">
+        <f>SUM(E3:E125)</f>
+        <v/>
+      </c>
+      <c r="F126" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A126:C126"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A125:C125"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -7122,7 +7174,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AM27"/>
+  <dimension ref="A1:AM28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -8455,151 +8507,151 @@
     <row r="11">
       <c r="A11" s="36" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="B11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ11" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK11" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Cloud",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL11" s="39">
@@ -8614,151 +8666,151 @@
     <row r="12">
       <c r="A12" s="41" t="inlineStr">
         <is>
-          <t>Hedra</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="B12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ12" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK12" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Google Workspace",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL12" s="39">
@@ -8773,151 +8825,151 @@
     <row r="13">
       <c r="A13" s="36" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>Hedra</t>
         </is>
       </c>
       <c r="B13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ13" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK13" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Hedra",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL13" s="39">
@@ -8932,151 +8984,151 @@
     <row r="14">
       <c r="A14" s="41" t="inlineStr">
         <is>
-          <t>IONOS</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="B14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ14" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK14" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Higgsfield",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL14" s="39">
@@ -9091,151 +9143,151 @@
     <row r="15">
       <c r="A15" s="36" t="inlineStr">
         <is>
-          <t>Ideogram AI</t>
+          <t>IONOS</t>
         </is>
       </c>
       <c r="B15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ15" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK15" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"IONOS",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL15" s="39">
@@ -9250,151 +9302,151 @@
     <row r="16">
       <c r="A16" s="41" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Ideogram AI</t>
         </is>
       </c>
       <c r="B16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ16" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK16" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Ideogram AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL16" s="39">
@@ -9409,151 +9461,151 @@
     <row r="17">
       <c r="A17" s="36" t="inlineStr">
         <is>
-          <t>Make</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="B17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ17" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK17" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Lovable",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL17" s="39">
@@ -9568,151 +9620,151 @@
     <row r="18">
       <c r="A18" s="41" t="inlineStr">
         <is>
-          <t>Manus AI</t>
+          <t>Make</t>
         </is>
       </c>
       <c r="B18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ18" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK18" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Make",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL18" s="39">
@@ -9727,151 +9779,151 @@
     <row r="19">
       <c r="A19" s="36" t="inlineStr">
         <is>
-          <t>Manychat</t>
+          <t>Manus AI</t>
         </is>
       </c>
       <c r="B19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ19" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK19" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manus AI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL19" s="39">
@@ -9886,151 +9938,151 @@
     <row r="20">
       <c r="A20" s="41" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Manychat</t>
         </is>
       </c>
       <c r="B20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ20" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK20" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Manychat",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL20" s="39">
@@ -10045,151 +10097,151 @@
     <row r="21">
       <c r="A21" s="36" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="B21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ21" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK21" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Meta (Ads)",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL21" s="39">
@@ -10204,151 +10256,151 @@
     <row r="22">
       <c r="A22" s="41" t="inlineStr">
         <is>
-          <t>Recraft</t>
+          <t>OpenAI</t>
         </is>
       </c>
       <c r="B22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ22" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK22" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"OpenAI",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL22" s="39">
@@ -10363,151 +10415,151 @@
     <row r="23">
       <c r="A23" s="36" t="inlineStr">
         <is>
-          <t>Replicate</t>
+          <t>Recraft</t>
         </is>
       </c>
       <c r="B23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ23" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK23" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Recraft",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL23" s="39">
@@ -10522,151 +10574,151 @@
     <row r="24">
       <c r="A24" s="41" t="inlineStr">
         <is>
-          <t>Runway ML</t>
+          <t>Replicate</t>
         </is>
       </c>
       <c r="B24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ24" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK24" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Replicate",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL24" s="39">
@@ -10681,151 +10733,151 @@
     <row r="25">
       <c r="A25" s="36" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Runway ML</t>
         </is>
       </c>
       <c r="B25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ25" s="37">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK25" s="38">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Runway ML",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL25" s="39">
@@ -10840,151 +10892,151 @@
     <row r="26">
       <c r="A26" s="41" t="inlineStr">
         <is>
-          <t>Timeless</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="B26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="C26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
         <v/>
       </c>
       <c r="D26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="E26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
         <v/>
       </c>
       <c r="F26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="G26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
         <v/>
       </c>
       <c r="H26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="I26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
         <v/>
       </c>
       <c r="J26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="K26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
         <v/>
       </c>
       <c r="L26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="M26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
         <v/>
       </c>
       <c r="N26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="O26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
         <v/>
       </c>
       <c r="P26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="Q26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
         <v/>
       </c>
       <c r="R26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="S26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
         <v/>
       </c>
       <c r="T26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="U26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
         <v/>
       </c>
       <c r="V26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="W26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
         <v/>
       </c>
       <c r="X26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Y26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
         <v/>
       </c>
       <c r="Z26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AA26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
         <v/>
       </c>
       <c r="AB26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AC26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
         <v/>
       </c>
       <c r="AD26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AE26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
         <v/>
       </c>
       <c r="AF26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AG26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
         <v/>
       </c>
       <c r="AH26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AI26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
         <v/>
       </c>
       <c r="AJ26" s="42">
-        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AK26" s="43">
-        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Supabase",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
         <v/>
       </c>
       <c r="AL26" s="39">
@@ -10996,162 +11048,321 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="30" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="36" t="inlineStr">
+        <is>
+          <t>Timeless</t>
+        </is>
+      </c>
+      <c r="B27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <v/>
+      </c>
+      <c r="C27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2025")</f>
+        <v/>
+      </c>
+      <c r="D27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <v/>
+      </c>
+      <c r="E27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2025")</f>
+        <v/>
+      </c>
+      <c r="F27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="G27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="H27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <v/>
+      </c>
+      <c r="I27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2025")</f>
+        <v/>
+      </c>
+      <c r="J27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="K27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="L27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="M27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2025")</f>
+        <v/>
+      </c>
+      <c r="N27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <v/>
+      </c>
+      <c r="O27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ינואר 2026")</f>
+        <v/>
+      </c>
+      <c r="P27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <v/>
+      </c>
+      <c r="Q27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"פברואר 2026")</f>
+        <v/>
+      </c>
+      <c r="R27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <v/>
+      </c>
+      <c r="S27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מרץ 2026")</f>
+        <v/>
+      </c>
+      <c r="T27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <v/>
+      </c>
+      <c r="U27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אפריל 2026")</f>
+        <v/>
+      </c>
+      <c r="V27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <v/>
+      </c>
+      <c r="W27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"מאי 2026")</f>
+        <v/>
+      </c>
+      <c r="X27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <v/>
+      </c>
+      <c r="Y27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יוני 2026")</f>
+        <v/>
+      </c>
+      <c r="Z27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <v/>
+      </c>
+      <c r="AA27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"יולי 2026")</f>
+        <v/>
+      </c>
+      <c r="AB27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <v/>
+      </c>
+      <c r="AC27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוגוסט 2026")</f>
+        <v/>
+      </c>
+      <c r="AD27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AE27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"ספטמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AF27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <v/>
+      </c>
+      <c r="AG27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"אוקטובר 2026")</f>
+        <v/>
+      </c>
+      <c r="AH27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AI27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"נובמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AJ27" s="37">
+        <f>SUMIFS('כל ההוצאות'!$D:$D,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AK27" s="38">
+        <f>SUMIFS('כל ההוצאות'!$E:$E,'כל ההוצאות'!$B:$B,"Timeless",'כל ההוצאות'!$F:$F,"דצמבר 2026")</f>
+        <v/>
+      </c>
+      <c r="AL27" s="39">
+        <f>SUM(B27,D27,F27,H27,J27,L27,N27,P27,R27,T27,V27,X27,Z27,AB27,AD27,AF27,AH27,AJ27)</f>
+        <v/>
+      </c>
+      <c r="AM27" s="40">
+        <f>SUM(C27,E27,G27,I27,K27,M27,O27,Q27,S27,U27,W27,Y27,AA27,AC27,AE27,AG27,AI27,AK27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודשי</t>
         </is>
       </c>
-      <c r="B27" s="20">
-        <f>SUM(B5:B26)</f>
-        <v/>
-      </c>
-      <c r="C27" s="21">
-        <f>SUM(C5:C26)</f>
-        <v/>
-      </c>
-      <c r="D27" s="20">
-        <f>SUM(D5:D26)</f>
-        <v/>
-      </c>
-      <c r="E27" s="21">
-        <f>SUM(E5:E26)</f>
-        <v/>
-      </c>
-      <c r="F27" s="20">
-        <f>SUM(F5:F26)</f>
-        <v/>
-      </c>
-      <c r="G27" s="21">
-        <f>SUM(G5:G26)</f>
-        <v/>
-      </c>
-      <c r="H27" s="20">
-        <f>SUM(H5:H26)</f>
-        <v/>
-      </c>
-      <c r="I27" s="21">
-        <f>SUM(I5:I26)</f>
-        <v/>
-      </c>
-      <c r="J27" s="20">
-        <f>SUM(J5:J26)</f>
-        <v/>
-      </c>
-      <c r="K27" s="21">
-        <f>SUM(K5:K26)</f>
-        <v/>
-      </c>
-      <c r="L27" s="20">
-        <f>SUM(L5:L26)</f>
-        <v/>
-      </c>
-      <c r="M27" s="21">
-        <f>SUM(M5:M26)</f>
-        <v/>
-      </c>
-      <c r="N27" s="20">
-        <f>SUM(N5:N26)</f>
-        <v/>
-      </c>
-      <c r="O27" s="21">
-        <f>SUM(O5:O26)</f>
-        <v/>
-      </c>
-      <c r="P27" s="20">
-        <f>SUM(P5:P26)</f>
-        <v/>
-      </c>
-      <c r="Q27" s="21">
-        <f>SUM(Q5:Q26)</f>
-        <v/>
-      </c>
-      <c r="R27" s="20">
-        <f>SUM(R5:R26)</f>
-        <v/>
-      </c>
-      <c r="S27" s="21">
-        <f>SUM(S5:S26)</f>
-        <v/>
-      </c>
-      <c r="T27" s="20">
-        <f>SUM(T5:T26)</f>
-        <v/>
-      </c>
-      <c r="U27" s="21">
-        <f>SUM(U5:U26)</f>
-        <v/>
-      </c>
-      <c r="V27" s="20">
-        <f>SUM(V5:V26)</f>
-        <v/>
-      </c>
-      <c r="W27" s="21">
-        <f>SUM(W5:W26)</f>
-        <v/>
-      </c>
-      <c r="X27" s="20">
-        <f>SUM(X5:X26)</f>
-        <v/>
-      </c>
-      <c r="Y27" s="21">
-        <f>SUM(Y5:Y26)</f>
-        <v/>
-      </c>
-      <c r="Z27" s="20">
-        <f>SUM(Z5:Z26)</f>
-        <v/>
-      </c>
-      <c r="AA27" s="21">
-        <f>SUM(AA5:AA26)</f>
-        <v/>
-      </c>
-      <c r="AB27" s="20">
-        <f>SUM(AB5:AB26)</f>
-        <v/>
-      </c>
-      <c r="AC27" s="21">
-        <f>SUM(AC5:AC26)</f>
-        <v/>
-      </c>
-      <c r="AD27" s="20">
-        <f>SUM(AD5:AD26)</f>
-        <v/>
-      </c>
-      <c r="AE27" s="21">
-        <f>SUM(AE5:AE26)</f>
-        <v/>
-      </c>
-      <c r="AF27" s="20">
-        <f>SUM(AF5:AF26)</f>
-        <v/>
-      </c>
-      <c r="AG27" s="21">
-        <f>SUM(AG5:AG26)</f>
-        <v/>
-      </c>
-      <c r="AH27" s="20">
-        <f>SUM(AH5:AH26)</f>
-        <v/>
-      </c>
-      <c r="AI27" s="21">
-        <f>SUM(AI5:AI26)</f>
-        <v/>
-      </c>
-      <c r="AJ27" s="20">
-        <f>SUM(AJ5:AJ26)</f>
-        <v/>
-      </c>
-      <c r="AK27" s="21">
-        <f>SUM(AK5:AK26)</f>
-        <v/>
-      </c>
-      <c r="AL27" s="44">
-        <f>SUM(AL5:AL26)</f>
-        <v/>
-      </c>
-      <c r="AM27" s="45">
-        <f>SUM(AM5:AM26)</f>
+      <c r="B28" s="20">
+        <f>SUM(B5:B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="21">
+        <f>SUM(C5:C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="20">
+        <f>SUM(D5:D27)</f>
+        <v/>
+      </c>
+      <c r="E28" s="21">
+        <f>SUM(E5:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="20">
+        <f>SUM(F5:F27)</f>
+        <v/>
+      </c>
+      <c r="G28" s="21">
+        <f>SUM(G5:G27)</f>
+        <v/>
+      </c>
+      <c r="H28" s="20">
+        <f>SUM(H5:H27)</f>
+        <v/>
+      </c>
+      <c r="I28" s="21">
+        <f>SUM(I5:I27)</f>
+        <v/>
+      </c>
+      <c r="J28" s="20">
+        <f>SUM(J5:J27)</f>
+        <v/>
+      </c>
+      <c r="K28" s="21">
+        <f>SUM(K5:K27)</f>
+        <v/>
+      </c>
+      <c r="L28" s="20">
+        <f>SUM(L5:L27)</f>
+        <v/>
+      </c>
+      <c r="M28" s="21">
+        <f>SUM(M5:M27)</f>
+        <v/>
+      </c>
+      <c r="N28" s="20">
+        <f>SUM(N5:N27)</f>
+        <v/>
+      </c>
+      <c r="O28" s="21">
+        <f>SUM(O5:O27)</f>
+        <v/>
+      </c>
+      <c r="P28" s="20">
+        <f>SUM(P5:P27)</f>
+        <v/>
+      </c>
+      <c r="Q28" s="21">
+        <f>SUM(Q5:Q27)</f>
+        <v/>
+      </c>
+      <c r="R28" s="20">
+        <f>SUM(R5:R27)</f>
+        <v/>
+      </c>
+      <c r="S28" s="21">
+        <f>SUM(S5:S27)</f>
+        <v/>
+      </c>
+      <c r="T28" s="20">
+        <f>SUM(T5:T27)</f>
+        <v/>
+      </c>
+      <c r="U28" s="21">
+        <f>SUM(U5:U27)</f>
+        <v/>
+      </c>
+      <c r="V28" s="20">
+        <f>SUM(V5:V27)</f>
+        <v/>
+      </c>
+      <c r="W28" s="21">
+        <f>SUM(W5:W27)</f>
+        <v/>
+      </c>
+      <c r="X28" s="20">
+        <f>SUM(X5:X27)</f>
+        <v/>
+      </c>
+      <c r="Y28" s="21">
+        <f>SUM(Y5:Y27)</f>
+        <v/>
+      </c>
+      <c r="Z28" s="20">
+        <f>SUM(Z5:Z27)</f>
+        <v/>
+      </c>
+      <c r="AA28" s="21">
+        <f>SUM(AA5:AA27)</f>
+        <v/>
+      </c>
+      <c r="AB28" s="20">
+        <f>SUM(AB5:AB27)</f>
+        <v/>
+      </c>
+      <c r="AC28" s="21">
+        <f>SUM(AC5:AC27)</f>
+        <v/>
+      </c>
+      <c r="AD28" s="20">
+        <f>SUM(AD5:AD27)</f>
+        <v/>
+      </c>
+      <c r="AE28" s="21">
+        <f>SUM(AE5:AE27)</f>
+        <v/>
+      </c>
+      <c r="AF28" s="20">
+        <f>SUM(AF5:AF27)</f>
+        <v/>
+      </c>
+      <c r="AG28" s="21">
+        <f>SUM(AG5:AG27)</f>
+        <v/>
+      </c>
+      <c r="AH28" s="20">
+        <f>SUM(AH5:AH27)</f>
+        <v/>
+      </c>
+      <c r="AI28" s="21">
+        <f>SUM(AI5:AI27)</f>
+        <v/>
+      </c>
+      <c r="AJ28" s="20">
+        <f>SUM(AJ5:AJ27)</f>
+        <v/>
+      </c>
+      <c r="AK28" s="21">
+        <f>SUM(AK5:AK27)</f>
+        <v/>
+      </c>
+      <c r="AL28" s="44">
+        <f>SUM(AL5:AL27)</f>
+        <v/>
+      </c>
+      <c r="AM28" s="45">
+        <f>SUM(AM5:AM27)</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-05-02
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2622,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2755,48 +2755,72 @@
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Prepaid extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="28" t="n">
+        <v>14.74</v>
+      </c>
+      <c r="F7" s="29" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B8" s="15" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C8" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D7" s="27" t="n">
+      <c r="D8" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E7" s="28" t="n">
+      <c r="E8" s="26" t="n">
         <v>73</v>
       </c>
-      <c r="F7" s="29" t="n"/>
-    </row>
-    <row r="8" ht="24" customHeight="1">
-      <c r="A8" s="30" t="inlineStr">
+      <c r="F8" s="24" t="n"/>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B8" s="31" t="n"/>
-      <c r="C8" s="31" t="n"/>
-      <c r="D8" s="20">
-        <f>SUM(D4:D7)</f>
-        <v/>
-      </c>
-      <c r="E8" s="21">
-        <f>SUM(E4:E7)</f>
-        <v/>
-      </c>
-      <c r="F8" s="31" t="n"/>
+      <c r="B9" s="31" t="n"/>
+      <c r="C9" s="31" t="n"/>
+      <c r="D9" s="20">
+        <f>SUM(D4:D8)</f>
+        <v/>
+      </c>
+      <c r="E9" s="21">
+        <f>SUM(E4:E8)</f>
+        <v/>
+      </c>
+      <c r="F9" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A9:C9"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3527,7 +3551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F126"/>
+  <dimension ref="A1:F127"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6800,24 +6824,24 @@
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C118" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D118" s="16" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E118" s="17" t="n">
-        <v>73</v>
+        <v>14.74</v>
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
@@ -6828,7 +6852,7 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
@@ -6849,14 +6873,14 @@
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
@@ -6877,14 +6901,14 @@
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -6905,14 +6929,14 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B122" s="15" t="inlineStr">
@@ -6933,14 +6957,14 @@
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
@@ -6961,14 +6985,14 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B124" s="15" t="inlineStr">
@@ -6989,14 +7013,14 @@
       </c>
       <c r="F124" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B125" s="11" t="inlineStr">
@@ -7017,31 +7041,59 @@
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B126" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C126" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D126" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E126" s="17" t="n">
+        <v>73</v>
+      </c>
+      <c r="F126" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" s="18" t="inlineStr">
+    <row r="127">
+      <c r="A127" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B126" s="19" t="n"/>
-      <c r="C126" s="19" t="n"/>
-      <c r="D126" s="20">
-        <f>SUM(D3:D125)</f>
-        <v/>
-      </c>
-      <c r="E126" s="21">
-        <f>SUM(E3:E125)</f>
-        <v/>
-      </c>
-      <c r="F126" s="19" t="n"/>
+      <c r="B127" s="19" t="n"/>
+      <c r="C127" s="19" t="n"/>
+      <c r="D127" s="20">
+        <f>SUM(D3:D126)</f>
+        <v/>
+      </c>
+      <c r="E127" s="21">
+        <f>SUM(E3:E126)</f>
+        <v/>
+      </c>
+      <c r="F127" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A126:C126"/>
+    <mergeCell ref="A127:C127"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto: add invoices – Meta (Ads) 2026-05-03
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2622,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F9"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2779,48 +2779,72 @@
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Meta (Ads)</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Facebook Ads</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>27.279512</v>
+      </c>
+      <c r="E8" s="26" t="n">
+        <v>80.42</v>
+      </c>
+      <c r="F8" s="24" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B8" s="15" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D9" s="27" t="n">
         <v>20</v>
       </c>
-      <c r="E8" s="26" t="n">
+      <c r="E9" s="28" t="n">
         <v>73</v>
       </c>
-      <c r="F8" s="24" t="n"/>
-    </row>
-    <row r="9" ht="24" customHeight="1">
-      <c r="A9" s="30" t="inlineStr">
+      <c r="F9" s="29" t="n"/>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B9" s="31" t="n"/>
-      <c r="C9" s="31" t="n"/>
-      <c r="D9" s="20">
-        <f>SUM(D4:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="21">
-        <f>SUM(E4:E8)</f>
-        <v/>
-      </c>
-      <c r="F9" s="31" t="n"/>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="31" t="n"/>
+      <c r="D10" s="20">
+        <f>SUM(D4:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="21">
+        <f>SUM(E4:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A9:C9"/>
+    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3551,7 +3575,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F127"/>
+  <dimension ref="A1:F128"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6852,24 +6876,24 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D119" s="12" t="n">
-        <v>20</v>
+        <v>27.279512</v>
       </c>
       <c r="E119" s="13" t="n">
-        <v>73</v>
+        <v>80.42</v>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
@@ -6880,7 +6904,7 @@
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
@@ -6901,14 +6925,14 @@
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -6929,14 +6953,14 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B122" s="15" t="inlineStr">
@@ -6957,14 +6981,14 @@
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
@@ -6985,14 +7009,14 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B124" s="15" t="inlineStr">
@@ -7013,14 +7037,14 @@
       </c>
       <c r="F124" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B125" s="11" t="inlineStr">
@@ -7041,14 +7065,14 @@
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B126" s="15" t="inlineStr">
@@ -7069,31 +7093,59 @@
       </c>
       <c r="F126" s="14" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D127" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E127" s="13" t="n">
+        <v>73</v>
+      </c>
+      <c r="F127" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="127">
-      <c r="A127" s="18" t="inlineStr">
+    <row r="128">
+      <c r="A128" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B127" s="19" t="n"/>
-      <c r="C127" s="19" t="n"/>
-      <c r="D127" s="20">
-        <f>SUM(D3:D126)</f>
-        <v/>
-      </c>
-      <c r="E127" s="21">
-        <f>SUM(E3:E126)</f>
-        <v/>
-      </c>
-      <c r="F127" s="19" t="n"/>
+      <c r="B128" s="19" t="n"/>
+      <c r="C128" s="19" t="n"/>
+      <c r="D128" s="20">
+        <f>SUM(D3:D127)</f>
+        <v/>
+      </c>
+      <c r="E128" s="21">
+        <f>SUM(E3:E127)</f>
+        <v/>
+      </c>
+      <c r="F128" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A127:C127"/>
+    <mergeCell ref="A128:C128"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-05-03
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -2622,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F10"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2784,68 +2784,92 @@
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>27.279512</v>
+        <v>15.329037</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>80.42</v>
+        <v>45.19</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Meta (Ads)</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Facebook Ads</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>27.279512</v>
+      </c>
+      <c r="E9" s="28" t="n">
+        <v>80.42</v>
+      </c>
+      <c r="F9" s="29" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B10" s="15" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C10" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D9" s="27" t="n">
+      <c r="D10" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E9" s="28" t="n">
+      <c r="E10" s="26" t="n">
         <v>73</v>
       </c>
-      <c r="F9" s="29" t="n"/>
-    </row>
-    <row r="10" ht="24" customHeight="1">
-      <c r="A10" s="30" t="inlineStr">
+      <c r="F10" s="24" t="n"/>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B10" s="31" t="n"/>
-      <c r="C10" s="31" t="n"/>
-      <c r="D10" s="20">
-        <f>SUM(D4:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="21">
-        <f>SUM(E4:E9)</f>
-        <v/>
-      </c>
-      <c r="F10" s="31" t="n"/>
+      <c r="B11" s="31" t="n"/>
+      <c r="C11" s="31" t="n"/>
+      <c r="D11" s="20">
+        <f>SUM(D4:D10)</f>
+        <v/>
+      </c>
+      <c r="E11" s="21">
+        <f>SUM(E4:E10)</f>
+        <v/>
+      </c>
+      <c r="F11" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A10:C10"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A11:C11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3575,7 +3599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F128"/>
+  <dimension ref="A1:F129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6881,19 +6905,19 @@
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D119" s="12" t="n">
-        <v>27.279512</v>
+        <v>15.329037</v>
       </c>
       <c r="E119" s="13" t="n">
-        <v>80.42</v>
+        <v>45.19</v>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
@@ -6904,24 +6928,24 @@
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C120" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D120" s="16" t="n">
-        <v>20</v>
+        <v>27.279512</v>
       </c>
       <c r="E120" s="17" t="n">
-        <v>73</v>
+        <v>80.42</v>
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
@@ -6932,7 +6956,7 @@
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -6953,14 +6977,14 @@
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B122" s="15" t="inlineStr">
@@ -6981,14 +7005,14 @@
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
@@ -7009,14 +7033,14 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B124" s="15" t="inlineStr">
@@ -7037,14 +7061,14 @@
       </c>
       <c r="F124" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B125" s="11" t="inlineStr">
@@ -7065,14 +7089,14 @@
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B126" s="15" t="inlineStr">
@@ -7093,14 +7117,14 @@
       </c>
       <c r="F126" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B127" s="11" t="inlineStr">
@@ -7121,32 +7145,60 @@
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B128" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C128" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D128" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E128" s="17" t="n">
+        <v>73</v>
+      </c>
+      <c r="F128" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="128">
-      <c r="A128" s="18" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B128" s="19" t="n"/>
-      <c r="C128" s="19" t="n"/>
-      <c r="D128" s="20">
-        <f>SUM(D3:D127)</f>
-        <v/>
-      </c>
-      <c r="E128" s="21">
-        <f>SUM(E3:E127)</f>
-        <v/>
-      </c>
-      <c r="F128" s="19" t="n"/>
+      <c r="B129" s="19" t="n"/>
+      <c r="C129" s="19" t="n"/>
+      <c r="D129" s="20">
+        <f>SUM(D3:D128)</f>
+        <v/>
+      </c>
+      <c r="E129" s="21">
+        <f>SUM(E3:E128)</f>
+        <v/>
+      </c>
+      <c r="F129" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A128:C128"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A129:C129"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: scanner dropped duplicate-description Anthropic receipts on same day
Root cause: already_imported() matched only on date+tool+description, so when
Anthropic auto-recharge fired multiple times in one day (different USD amounts,
identical description), the 2nd and 3rd receipts were skipped as false-positive
duplicates. Three May 1 charges arrived ($10.40, $10.84, $10.82) but only the
first ($10.40) made it into MANUAL_TRANSACTIONS.

Fix:
- already_imported() now includes the amount in the dedup key (matches the USD
  comment for USD-source receipts and the ILS amount for ILS receipts).
- Backfilled the two missing May 1 receipts and converted the legacy USD-only
  entry to a 5-tuple ILS at the locked May 1 historical rate (2.9525).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -2622,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2697,7 +2697,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>10.4</v>
+        <v>10.367995</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>30.71</v>
@@ -2712,19 +2712,19 @@
       </c>
       <c r="B5" s="11" t="inlineStr">
         <is>
-          <t>Google Cloud</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C5" s="11" t="inlineStr">
         <is>
-          <t>Google Cloud Platform &amp; APIs (₪8.23)</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>2.778528</v>
+        <v>10.806887</v>
       </c>
       <c r="E5" s="28" t="n">
-        <v>8.23</v>
+        <v>32.01</v>
       </c>
       <c r="F5" s="29" t="n"/>
     </row>
@@ -2736,140 +2736,188 @@
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.90)</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>25.624578</v>
+        <v>10.786631</v>
       </c>
       <c r="E6" s="26" t="n">
-        <v>75.90000000000001</v>
+        <v>31.95</v>
       </c>
       <c r="F6" s="24" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="10" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="C7" s="11" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>Google Cloud Platform &amp; APIs (₪8.23)</t>
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>4.976367</v>
+        <v>2.778528</v>
       </c>
       <c r="E7" s="28" t="n">
-        <v>14.74</v>
+        <v>8.23</v>
       </c>
       <c r="F7" s="29" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="14" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Google Workspace (₪75.90)</t>
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>15.256583</v>
+        <v>25.624578</v>
       </c>
       <c r="E8" s="26" t="n">
-        <v>45.19</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F8" s="24" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="10" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>27.150574</v>
+        <v>4.976367</v>
       </c>
       <c r="E9" s="28" t="n">
-        <v>80.42</v>
+        <v>14.74</v>
       </c>
       <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="14" t="inlineStr">
         <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>15.256583</v>
+      </c>
+      <c r="E10" s="26" t="n">
+        <v>45.19</v>
+      </c>
+      <c r="F10" s="24" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Meta (Ads)</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Facebook Ads</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>27.150574</v>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>80.42</v>
+      </c>
+      <c r="F11" s="29" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B10" s="15" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D10" s="25" t="n">
+      <c r="D12" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E10" s="26" t="n">
+      <c r="E12" s="26" t="n">
         <v>73</v>
       </c>
-      <c r="F10" s="24" t="n"/>
-    </row>
-    <row r="11" ht="24" customHeight="1">
-      <c r="A11" s="30" t="inlineStr">
+      <c r="F12" s="24" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B11" s="31" t="n"/>
-      <c r="C11" s="31" t="n"/>
-      <c r="D11" s="20">
-        <f>SUM(D4:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="21">
-        <f>SUM(E4:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="31" t="n"/>
+      <c r="B13" s="31" t="n"/>
+      <c r="C13" s="31" t="n"/>
+      <c r="D13" s="20">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="21">
+        <f>SUM(E4:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A11:C11"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
@@ -3599,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F129"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6802,7 +6850,7 @@
         </is>
       </c>
       <c r="D115" s="12" t="n">
-        <v>10.4</v>
+        <v>10.367995</v>
       </c>
       <c r="E115" s="13" t="n">
         <v>30.71</v>
@@ -6821,19 +6869,19 @@
       </c>
       <c r="B116" s="15" t="inlineStr">
         <is>
-          <t>Google Cloud</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C116" s="15" t="inlineStr">
         <is>
-          <t>Google Cloud Platform &amp; APIs (₪8.23)</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D116" s="16" t="n">
-        <v>2.778528</v>
+        <v>10.806887</v>
       </c>
       <c r="E116" s="17" t="n">
-        <v>8.23</v>
+        <v>32.01</v>
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
@@ -6849,19 +6897,19 @@
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.90)</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D117" s="12" t="n">
-        <v>25.624578</v>
+        <v>10.786631</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>31.95</v>
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
@@ -6872,24 +6920,24 @@
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="C118" s="15" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>Google Cloud Platform &amp; APIs (₪8.23)</t>
         </is>
       </c>
       <c r="D118" s="16" t="n">
-        <v>4.976367</v>
+        <v>2.778528</v>
       </c>
       <c r="E118" s="17" t="n">
-        <v>14.74</v>
+        <v>8.23</v>
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
@@ -6900,24 +6948,24 @@
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Google Workspace (₪75.90)</t>
         </is>
       </c>
       <c r="D119" s="12" t="n">
-        <v>15.256583</v>
+        <v>25.624578</v>
       </c>
       <c r="E119" s="13" t="n">
-        <v>45.19</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
@@ -6928,24 +6976,24 @@
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C120" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D120" s="16" t="n">
-        <v>27.150574</v>
+        <v>4.976367</v>
       </c>
       <c r="E120" s="17" t="n">
-        <v>80.42</v>
+        <v>14.74</v>
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
@@ -6956,24 +7004,24 @@
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D121" s="12" t="n">
-        <v>20</v>
+        <v>15.256583</v>
       </c>
       <c r="E121" s="13" t="n">
-        <v>73</v>
+        <v>45.19</v>
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
@@ -6984,35 +7032,35 @@
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B122" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C122" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D122" s="16" t="n">
-        <v>20</v>
+        <v>27.150574</v>
       </c>
       <c r="E122" s="17" t="n">
-        <v>73</v>
+        <v>80.42</v>
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
@@ -7033,14 +7081,14 @@
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B124" s="15" t="inlineStr">
@@ -7061,14 +7109,14 @@
       </c>
       <c r="F124" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B125" s="11" t="inlineStr">
@@ -7089,14 +7137,14 @@
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B126" s="15" t="inlineStr">
@@ -7117,14 +7165,14 @@
       </c>
       <c r="F126" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B127" s="11" t="inlineStr">
@@ -7145,14 +7193,14 @@
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B128" s="15" t="inlineStr">
@@ -7173,32 +7221,88 @@
       </c>
       <c r="F128" s="14" t="inlineStr">
         <is>
+          <t>אוקטובר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D129" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E129" s="13" t="n">
+        <v>73</v>
+      </c>
+      <c r="F129" s="10" t="inlineStr">
+        <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C130" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D130" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E130" s="17" t="n">
+        <v>73</v>
+      </c>
+      <c r="F130" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="129">
-      <c r="A129" s="18" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B129" s="19" t="n"/>
-      <c r="C129" s="19" t="n"/>
-      <c r="D129" s="20">
-        <f>SUM(D3:D128)</f>
-        <v/>
-      </c>
-      <c r="E129" s="21">
-        <f>SUM(E3:E128)</f>
-        <v/>
-      </c>
-      <c r="F129" s="19" t="n"/>
+      <c r="B131" s="19" t="n"/>
+      <c r="C131" s="19" t="n"/>
+      <c r="D131" s="20">
+        <f>SUM(D3:D130)</f>
+        <v/>
+      </c>
+      <c r="E131" s="21">
+        <f>SUM(E3:E130)</f>
+        <v/>
+      </c>
+      <c r="F131" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A131:C131"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A129:C129"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-05-04
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1879,7 +1879,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F31"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2252,24 +2252,24 @@
     <row r="17">
       <c r="A17" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D17" s="27" t="n">
-        <v>15.14</v>
+        <v>4.996624</v>
       </c>
       <c r="E17" s="28" t="n">
-        <v>44.81</v>
+        <v>14.8</v>
       </c>
       <c r="F17" s="29" t="n"/>
     </row>
@@ -2286,21 +2286,21 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D18" s="25" t="n">
-        <v>10</v>
+        <v>15.14</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>29.6</v>
+        <v>44.81</v>
       </c>
       <c r="F18" s="24" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="10" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B19" s="11" t="inlineStr">
@@ -2310,14 +2310,14 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D19" s="27" t="n">
-        <v>10.15</v>
+        <v>10</v>
       </c>
       <c r="E19" s="28" t="n">
-        <v>30.34</v>
+        <v>29.6</v>
       </c>
       <c r="F19" s="29" t="n"/>
     </row>
@@ -2338,10 +2338,10 @@
         </is>
       </c>
       <c r="D20" s="25" t="n">
-        <v>10.02</v>
+        <v>10.15</v>
       </c>
       <c r="E20" s="26" t="n">
-        <v>29.95</v>
+        <v>30.34</v>
       </c>
       <c r="F20" s="24" t="n"/>
     </row>
@@ -2362,10 +2362,10 @@
         </is>
       </c>
       <c r="D21" s="27" t="n">
-        <v>10.5</v>
+        <v>10.02</v>
       </c>
       <c r="E21" s="28" t="n">
-        <v>31.38</v>
+        <v>29.95</v>
       </c>
       <c r="F21" s="29" t="n"/>
     </row>
@@ -2386,10 +2386,10 @@
         </is>
       </c>
       <c r="D22" s="25" t="n">
-        <v>11.17</v>
+        <v>10.5</v>
       </c>
       <c r="E22" s="26" t="n">
-        <v>33.39</v>
+        <v>31.38</v>
       </c>
       <c r="F22" s="24" t="n"/>
     </row>
@@ -2401,43 +2401,43 @@
       </c>
       <c r="B23" s="11" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D23" s="27" t="n">
-        <v>25</v>
+        <v>11.17</v>
       </c>
       <c r="E23" s="28" t="n">
-        <v>74.72</v>
+        <v>33.39</v>
       </c>
       <c r="F23" s="29" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="14" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="D24" s="25" t="n">
-        <v>15.57</v>
+        <v>25</v>
       </c>
       <c r="E24" s="26" t="n">
-        <v>46.79</v>
+        <v>74.72</v>
       </c>
       <c r="F24" s="24" t="n"/>
     </row>
@@ -2458,17 +2458,17 @@
         </is>
       </c>
       <c r="D25" s="27" t="n">
-        <v>10.74</v>
+        <v>15.57</v>
       </c>
       <c r="E25" s="28" t="n">
-        <v>32.27</v>
+        <v>46.79</v>
       </c>
       <c r="F25" s="29" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="14" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
@@ -2482,34 +2482,34 @@
         </is>
       </c>
       <c r="D26" s="25" t="n">
-        <v>10.16</v>
+        <v>10.74</v>
       </c>
       <c r="E26" s="26" t="n">
-        <v>30.47</v>
+        <v>32.27</v>
       </c>
       <c r="F26" s="24" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="10" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B27" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D27" s="27" t="n">
-        <v>5</v>
+        <v>10.16</v>
       </c>
       <c r="E27" s="28" t="n">
-        <v>14.93</v>
+        <v>30.47</v>
       </c>
       <c r="F27" s="29" t="n"/>
     </row>
@@ -2521,91 +2521,115 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="D28" s="25" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E28" s="26" t="n">
-        <v>152.29</v>
+        <v>14.93</v>
       </c>
       <c r="F28" s="24" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B29" s="11" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C29" s="11" t="inlineStr">
         <is>
-          <t>Credit Package</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D29" s="27" t="n">
-        <v>40.83052</v>
+        <v>51</v>
       </c>
       <c r="E29" s="28" t="n">
-        <v>120.94</v>
+        <v>152.29</v>
       </c>
       <c r="F29" s="29" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="14" t="inlineStr">
         <is>
+          <t>2026-04-27</t>
+        </is>
+      </c>
+      <c r="B30" s="15" t="inlineStr">
+        <is>
+          <t>Higgsfield</t>
+        </is>
+      </c>
+      <c r="C30" s="15" t="inlineStr">
+        <is>
+          <t>Credit Package</t>
+        </is>
+      </c>
+      <c r="D30" s="25" t="n">
+        <v>40.83052</v>
+      </c>
+      <c r="E30" s="26" t="n">
+        <v>120.94</v>
+      </c>
+      <c r="F30" s="24" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="10" t="inlineStr">
+        <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="B30" s="15" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Anthropic</t>
         </is>
       </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
-      <c r="D30" s="25" t="n">
+      <c r="D31" s="27" t="n">
         <v>10.56</v>
       </c>
-      <c r="E30" s="26" t="n">
+      <c r="E31" s="28" t="n">
         <v>31.42</v>
       </c>
-      <c r="F30" s="24" t="n"/>
-    </row>
-    <row r="31" ht="24" customHeight="1">
-      <c r="A31" s="30" t="inlineStr">
+      <c r="F31" s="29" t="n"/>
+    </row>
+    <row r="32" ht="24" customHeight="1">
+      <c r="A32" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B31" s="31" t="n"/>
-      <c r="C31" s="31" t="n"/>
-      <c r="D31" s="20">
-        <f>SUM(D4:D30)</f>
-        <v/>
-      </c>
-      <c r="E31" s="21">
-        <f>SUM(E4:E30)</f>
-        <v/>
-      </c>
-      <c r="F31" s="31" t="n"/>
+      <c r="B32" s="31" t="n"/>
+      <c r="C32" s="31" t="n"/>
+      <c r="D32" s="20">
+        <f>SUM(D4:D31)</f>
+        <v/>
+      </c>
+      <c r="E32" s="21">
+        <f>SUM(E4:E31)</f>
+        <v/>
+      </c>
+      <c r="F32" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="A32:C32"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -2622,7 +2646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2875,48 +2899,96 @@
     <row r="12">
       <c r="A12" s="14" t="inlineStr">
         <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B12" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C12" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D12" s="25" t="n">
+        <v>15.290344</v>
+      </c>
+      <c r="E12" s="26" t="n">
+        <v>45.29</v>
+      </c>
+      <c r="F12" s="24" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
+        <is>
+          <t>Eleven Labs</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
+        <is>
+          <t>Creator monthly</t>
+        </is>
+      </c>
+      <c r="D13" s="27" t="n">
+        <v>21.863606</v>
+      </c>
+      <c r="E13" s="28" t="n">
+        <v>64.76000000000001</v>
+      </c>
+      <c r="F13" s="29" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="14" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B12" s="15" t="inlineStr">
+      <c r="B14" s="15" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="C14" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D12" s="25" t="n">
+      <c r="D14" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E12" s="26" t="n">
+      <c r="E14" s="26" t="n">
         <v>73</v>
       </c>
-      <c r="F12" s="24" t="n"/>
-    </row>
-    <row r="13" ht="24" customHeight="1">
-      <c r="A13" s="30" t="inlineStr">
+      <c r="F14" s="24" t="n"/>
+    </row>
+    <row r="15" ht="24" customHeight="1">
+      <c r="A15" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B13" s="31" t="n"/>
-      <c r="C13" s="31" t="n"/>
-      <c r="D13" s="20">
-        <f>SUM(D4:D12)</f>
-        <v/>
-      </c>
-      <c r="E13" s="21">
-        <f>SUM(E4:E12)</f>
-        <v/>
-      </c>
-      <c r="F13" s="31" t="n"/>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="31" t="n"/>
+      <c r="D15" s="20">
+        <f>SUM(D4:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="21">
+        <f>SUM(E4:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A13:C13"/>
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3647,7 +3719,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F131"/>
+  <dimension ref="A1:F134"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6444,24 +6516,24 @@
     <row r="101">
       <c r="A101" s="10" t="inlineStr">
         <is>
-          <t>2026-04-20</t>
+          <t>2026-04-19</t>
         </is>
       </c>
       <c r="B101" s="11" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C101" s="11" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Starter monthly</t>
         </is>
       </c>
       <c r="D101" s="12" t="n">
-        <v>15.14</v>
+        <v>4.996624</v>
       </c>
       <c r="E101" s="13" t="n">
-        <v>44.81</v>
+        <v>14.8</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
@@ -6482,14 +6554,14 @@
       </c>
       <c r="C102" s="15" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D102" s="16" t="n">
-        <v>10</v>
+        <v>15.14</v>
       </c>
       <c r="E102" s="17" t="n">
-        <v>29.6</v>
+        <v>44.81</v>
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
@@ -6500,7 +6572,7 @@
     <row r="103">
       <c r="A103" s="10" t="inlineStr">
         <is>
-          <t>2026-04-21</t>
+          <t>2026-04-20</t>
         </is>
       </c>
       <c r="B103" s="11" t="inlineStr">
@@ -6510,14 +6582,14 @@
       </c>
       <c r="C103" s="11" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D103" s="12" t="n">
-        <v>10.15</v>
+        <v>10</v>
       </c>
       <c r="E103" s="13" t="n">
-        <v>30.34</v>
+        <v>29.6</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
@@ -6542,10 +6614,10 @@
         </is>
       </c>
       <c r="D104" s="16" t="n">
-        <v>10.02</v>
+        <v>10.15</v>
       </c>
       <c r="E104" s="17" t="n">
-        <v>29.95</v>
+        <v>30.34</v>
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
@@ -6570,10 +6642,10 @@
         </is>
       </c>
       <c r="D105" s="12" t="n">
-        <v>10.5</v>
+        <v>10.02</v>
       </c>
       <c r="E105" s="13" t="n">
-        <v>31.38</v>
+        <v>29.95</v>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
@@ -6598,10 +6670,10 @@
         </is>
       </c>
       <c r="D106" s="16" t="n">
-        <v>11.17</v>
+        <v>10.5</v>
       </c>
       <c r="E106" s="17" t="n">
-        <v>33.39</v>
+        <v>31.38</v>
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
@@ -6617,19 +6689,19 @@
       </c>
       <c r="B107" s="11" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C107" s="11" t="inlineStr">
         <is>
-          <t>Supabase</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D107" s="12" t="n">
-        <v>25</v>
+        <v>11.17</v>
       </c>
       <c r="E107" s="13" t="n">
-        <v>74.72</v>
+        <v>33.39</v>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
@@ -6640,24 +6712,24 @@
     <row r="108">
       <c r="A108" s="14" t="inlineStr">
         <is>
-          <t>2026-04-22</t>
+          <t>2026-04-21</t>
         </is>
       </c>
       <c r="B108" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="C108" s="15" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Supabase</t>
         </is>
       </c>
       <c r="D108" s="16" t="n">
-        <v>15.57</v>
+        <v>25</v>
       </c>
       <c r="E108" s="17" t="n">
-        <v>46.79</v>
+        <v>74.72</v>
       </c>
       <c r="F108" s="14" t="inlineStr">
         <is>
@@ -6682,10 +6754,10 @@
         </is>
       </c>
       <c r="D109" s="12" t="n">
-        <v>10.74</v>
+        <v>15.57</v>
       </c>
       <c r="E109" s="13" t="n">
-        <v>32.27</v>
+        <v>46.79</v>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
@@ -6696,7 +6768,7 @@
     <row r="110">
       <c r="A110" s="14" t="inlineStr">
         <is>
-          <t>2026-04-23</t>
+          <t>2026-04-22</t>
         </is>
       </c>
       <c r="B110" s="15" t="inlineStr">
@@ -6710,10 +6782,10 @@
         </is>
       </c>
       <c r="D110" s="16" t="n">
-        <v>10.16</v>
+        <v>10.74</v>
       </c>
       <c r="E110" s="17" t="n">
-        <v>30.47</v>
+        <v>32.27</v>
       </c>
       <c r="F110" s="14" t="inlineStr">
         <is>
@@ -6724,24 +6796,24 @@
     <row r="111">
       <c r="A111" s="10" t="inlineStr">
         <is>
-          <t>2026-04-26</t>
+          <t>2026-04-23</t>
         </is>
       </c>
       <c r="B111" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Lovable</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D111" s="12" t="n">
-        <v>5</v>
+        <v>10.16</v>
       </c>
       <c r="E111" s="13" t="n">
-        <v>14.93</v>
+        <v>30.47</v>
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
@@ -6757,19 +6829,19 @@
       </c>
       <c r="B112" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="C112" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Lovable</t>
         </is>
       </c>
       <c r="D112" s="16" t="n">
-        <v>51</v>
+        <v>5</v>
       </c>
       <c r="E112" s="17" t="n">
-        <v>152.29</v>
+        <v>14.93</v>
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
@@ -6780,24 +6852,24 @@
     <row r="113">
       <c r="A113" s="10" t="inlineStr">
         <is>
-          <t>2026-04-27</t>
+          <t>2026-04-26</t>
         </is>
       </c>
       <c r="B113" s="11" t="inlineStr">
         <is>
-          <t>Higgsfield</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Credit Package</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D113" s="12" t="n">
-        <v>40.83052</v>
+        <v>51</v>
       </c>
       <c r="E113" s="13" t="n">
-        <v>120.94</v>
+        <v>152.29</v>
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
@@ -6808,24 +6880,24 @@
     <row r="114">
       <c r="A114" s="14" t="inlineStr">
         <is>
-          <t>2026-04-28</t>
+          <t>2026-04-27</t>
         </is>
       </c>
       <c r="B114" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Higgsfield</t>
         </is>
       </c>
       <c r="C114" s="15" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Credit Package</t>
         </is>
       </c>
       <c r="D114" s="16" t="n">
-        <v>10.56</v>
+        <v>40.83052</v>
       </c>
       <c r="E114" s="17" t="n">
-        <v>31.42</v>
+        <v>120.94</v>
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
@@ -6836,7 +6908,7 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-04-28</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
@@ -6850,14 +6922,14 @@
         </is>
       </c>
       <c r="D115" s="12" t="n">
-        <v>10.367995</v>
+        <v>10.56</v>
       </c>
       <c r="E115" s="13" t="n">
-        <v>30.71</v>
+        <v>31.42</v>
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
-          <t>מאי 2026</t>
+          <t>אפריל 2026</t>
         </is>
       </c>
     </row>
@@ -6878,10 +6950,10 @@
         </is>
       </c>
       <c r="D116" s="16" t="n">
-        <v>10.806887</v>
+        <v>10.367995</v>
       </c>
       <c r="E116" s="17" t="n">
-        <v>32.01</v>
+        <v>30.71</v>
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
@@ -6906,10 +6978,10 @@
         </is>
       </c>
       <c r="D117" s="12" t="n">
-        <v>10.786631</v>
+        <v>10.806887</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>31.95</v>
+        <v>32.01</v>
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
@@ -6925,19 +6997,19 @@
       </c>
       <c r="B118" s="15" t="inlineStr">
         <is>
-          <t>Google Cloud</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C118" s="15" t="inlineStr">
         <is>
-          <t>Google Cloud Platform &amp; APIs (₪8.23)</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D118" s="16" t="n">
-        <v>2.778528</v>
+        <v>10.786631</v>
       </c>
       <c r="E118" s="17" t="n">
-        <v>8.23</v>
+        <v>31.95</v>
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
@@ -6953,19 +7025,19 @@
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace</t>
+          <t>Google Cloud</t>
         </is>
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>Google Workspace (₪75.90)</t>
+          <t>Google Cloud Platform &amp; APIs (₪8.23)</t>
         </is>
       </c>
       <c r="D119" s="12" t="n">
-        <v>25.624578</v>
+        <v>2.778528</v>
       </c>
       <c r="E119" s="13" t="n">
-        <v>75.90000000000001</v>
+        <v>8.23</v>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
@@ -6976,24 +7048,24 @@
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-05-02</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
         <is>
-          <t>Anthropic</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C120" s="15" t="inlineStr">
         <is>
-          <t>Prepaid extra usage, Individual plan</t>
+          <t>Google Workspace (₪75.90)</t>
         </is>
       </c>
       <c r="D120" s="16" t="n">
-        <v>4.976367</v>
+        <v>25.624578</v>
       </c>
       <c r="E120" s="17" t="n">
-        <v>14.74</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
@@ -7004,7 +7076,7 @@
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-05-03</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
@@ -7014,14 +7086,14 @@
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>Auto recharge extra usage, Individual plan</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D121" s="12" t="n">
-        <v>15.256583</v>
+        <v>4.976367</v>
       </c>
       <c r="E121" s="13" t="n">
-        <v>45.19</v>
+        <v>14.74</v>
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
@@ -7037,19 +7109,19 @@
       </c>
       <c r="B122" s="15" t="inlineStr">
         <is>
-          <t>Meta (Ads)</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C122" s="15" t="inlineStr">
         <is>
-          <t>Facebook Ads</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D122" s="16" t="n">
-        <v>27.150574</v>
+        <v>15.256583</v>
       </c>
       <c r="E122" s="17" t="n">
-        <v>80.42</v>
+        <v>45.19</v>
       </c>
       <c r="F122" s="14" t="inlineStr">
         <is>
@@ -7060,24 +7132,24 @@
     <row r="123">
       <c r="A123" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B123" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C123" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D123" s="12" t="n">
-        <v>20</v>
+        <v>27.150574</v>
       </c>
       <c r="E123" s="13" t="n">
-        <v>73</v>
+        <v>80.42</v>
       </c>
       <c r="F123" s="10" t="inlineStr">
         <is>
@@ -7088,63 +7160,63 @@
     <row r="124">
       <c r="A124" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B124" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C124" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D124" s="16" t="n">
-        <v>20</v>
+        <v>15.290344</v>
       </c>
       <c r="E124" s="17" t="n">
-        <v>73</v>
+        <v>45.29</v>
       </c>
       <c r="F124" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-05-04</t>
         </is>
       </c>
       <c r="B125" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Eleven Labs</t>
         </is>
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Creator monthly</t>
         </is>
       </c>
       <c r="D125" s="12" t="n">
-        <v>20</v>
+        <v>21.863606</v>
       </c>
       <c r="E125" s="13" t="n">
-        <v>73</v>
+        <v>64.76000000000001</v>
       </c>
       <c r="F125" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B126" s="15" t="inlineStr">
@@ -7165,14 +7237,14 @@
       </c>
       <c r="F126" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B127" s="11" t="inlineStr">
@@ -7193,14 +7265,14 @@
       </c>
       <c r="F127" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B128" s="15" t="inlineStr">
@@ -7221,14 +7293,14 @@
       </c>
       <c r="F128" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B129" s="11" t="inlineStr">
@@ -7249,14 +7321,14 @@
       </c>
       <c r="F129" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B130" s="15" t="inlineStr">
@@ -7277,31 +7349,115 @@
       </c>
       <c r="F130" s="14" t="inlineStr">
         <is>
+          <t>ספטמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="10" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B131" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C131" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D131" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E131" s="13" t="n">
+        <v>73</v>
+      </c>
+      <c r="F131" s="10" t="inlineStr">
+        <is>
+          <t>אוקטובר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="14" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="B132" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C132" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D132" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E132" s="17" t="n">
+        <v>73</v>
+      </c>
+      <c r="F132" s="14" t="inlineStr">
+        <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="10" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B133" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C133" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D133" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E133" s="13" t="n">
+        <v>73</v>
+      </c>
+      <c r="F133" s="10" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="18" t="inlineStr">
+    <row r="134">
+      <c r="A134" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B131" s="19" t="n"/>
-      <c r="C131" s="19" t="n"/>
-      <c r="D131" s="20">
-        <f>SUM(D3:D130)</f>
-        <v/>
-      </c>
-      <c r="E131" s="21">
-        <f>SUM(E3:E130)</f>
-        <v/>
-      </c>
-      <c r="F131" s="19" t="n"/>
+      <c r="B134" s="19" t="n"/>
+      <c r="C134" s="19" t="n"/>
+      <c r="D134" s="20">
+        <f>SUM(D3:D133)</f>
+        <v/>
+      </c>
+      <c r="E134" s="21">
+        <f>SUM(E3:E133)</f>
+        <v/>
+      </c>
+      <c r="F134" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A131:C131"/>
+    <mergeCell ref="A134:C134"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-05-04, Anthropic 2026-05-03, Meta (Ads) 2026-05-03, Anthropic 2026-05-02, Anthropic 2026-05-01, Anthropic 2026-05-01, Google Workspace 2026-05-01, Anthropic 2026-05-01
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -939,11 +939,11 @@
         </is>
       </c>
       <c r="B4" s="4" t="n">
-        <v>2.951</v>
+        <v>2.944</v>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>← מקור: Bank of Israel Public API | עודכן: 2026-04-30</t>
+          <t>← מקור: Bank of Israel Public API | עודכן: 2026-05-05</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>26.282616</v>
+        <v>26.345109</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>77.56</v>
@@ -1092,7 +1092,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1116,7 +1116,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>32.995595</v>
+        <v>33.074049</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>97.37</v>
@@ -1140,7 +1140,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>49.9</v>
@@ -1164,7 +1164,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>49.007116</v>
+        <v>49.123641</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>144.62</v>
@@ -1188,7 +1188,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>20.918333</v>
+        <v>20.968071</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>61.73</v>
@@ -1212,7 +1212,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5.232125</v>
+        <v>5.244565</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>15.44</v>
@@ -1260,7 +1260,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>21.199593</v>
+        <v>21.25</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>62.56</v>
@@ -1284,7 +1284,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>52.511013</v>
+        <v>52.63587</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>154.96</v>
@@ -1308,7 +1308,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>53.561505</v>
+        <v>53.688859</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>158.06</v>
@@ -1332,7 +1332,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.313453</v>
+        <v>5.326087</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>15.68</v>
@@ -1356,7 +1356,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>10.623517</v>
+        <v>10.648777</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>31.35</v>
@@ -1475,7 +1475,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -1499,7 +1499,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>10.599797</v>
+        <v>10.625</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>31.28</v>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>15.371061</v>
+        <v>15.407609</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>45.36</v>
@@ -1547,7 +1547,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>75.90000000000001</v>
@@ -1571,7 +1571,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>10.572687</v>
+        <v>10.597826</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>31.2</v>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>41.826499</v>
+        <v>41.925951</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>123.43</v>
@@ -1619,7 +1619,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -1643,7 +1643,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>54.107082</v>
+        <v>54.235734</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>159.67</v>
@@ -1667,7 +1667,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>21.304642</v>
+        <v>21.355299</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>62.87</v>
@@ -1715,7 +1715,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>49.9</v>
@@ -1739,7 +1739,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>10.542189</v>
+        <v>10.567255</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>31.11</v>
@@ -1763,7 +1763,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>11.596069</v>
+        <v>11.623641</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>34.22</v>
@@ -1811,7 +1811,7 @@
         </is>
       </c>
       <c r="D18" s="25" t="n">
-        <v>5.293121</v>
+        <v>5.305707</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>15.62</v>
@@ -1954,7 +1954,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>10.654016</v>
+        <v>10.679348</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>31.44</v>
@@ -1978,7 +1978,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>75.90000000000001</v>
@@ -2002,7 +2002,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>56.363944</v>
+        <v>56.497962</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>166.33</v>
@@ -2050,7 +2050,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>2.389021</v>
+        <v>2.394701</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>7.05</v>
@@ -2074,7 +2074,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>21.291088</v>
+        <v>21.341712</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>62.83</v>
@@ -2098,7 +2098,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -2125,7 +2125,7 @@
         <v>20</v>
       </c>
       <c r="E11" s="28" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F11" s="29" t="n"/>
     </row>
@@ -2149,7 +2149,7 @@
         <v>10</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>29.51</v>
+        <v>29.44</v>
       </c>
       <c r="F12" s="24" t="n"/>
     </row>
@@ -2173,7 +2173,7 @@
         <v>20</v>
       </c>
       <c r="E13" s="28" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F13" s="29" t="n"/>
     </row>
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>49.9</v>
@@ -2221,7 +2221,7 @@
         <v>81.2</v>
       </c>
       <c r="E15" s="28" t="n">
-        <v>239.62</v>
+        <v>239.05</v>
       </c>
       <c r="F15" s="29" t="n"/>
     </row>
@@ -2245,7 +2245,7 @@
         <v>5</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>14.76</v>
+        <v>14.72</v>
       </c>
       <c r="F16" s="24" t="n"/>
     </row>
@@ -2269,7 +2269,7 @@
         <v>15.14</v>
       </c>
       <c r="E17" s="28" t="n">
-        <v>44.68</v>
+        <v>44.57</v>
       </c>
       <c r="F17" s="29" t="n"/>
     </row>
@@ -2293,7 +2293,7 @@
         <v>10</v>
       </c>
       <c r="E18" s="26" t="n">
-        <v>29.51</v>
+        <v>29.44</v>
       </c>
       <c r="F18" s="24" t="n"/>
     </row>
@@ -2317,7 +2317,7 @@
         <v>10.15</v>
       </c>
       <c r="E19" s="28" t="n">
-        <v>29.95</v>
+        <v>29.88</v>
       </c>
       <c r="F19" s="29" t="n"/>
     </row>
@@ -2341,7 +2341,7 @@
         <v>10.02</v>
       </c>
       <c r="E20" s="26" t="n">
-        <v>29.57</v>
+        <v>29.5</v>
       </c>
       <c r="F20" s="24" t="n"/>
     </row>
@@ -2365,7 +2365,7 @@
         <v>10.5</v>
       </c>
       <c r="E21" s="28" t="n">
-        <v>30.99</v>
+        <v>30.91</v>
       </c>
       <c r="F21" s="29" t="n"/>
     </row>
@@ -2389,7 +2389,7 @@
         <v>11.17</v>
       </c>
       <c r="E22" s="26" t="n">
-        <v>32.96</v>
+        <v>32.88</v>
       </c>
       <c r="F22" s="24" t="n"/>
     </row>
@@ -2413,7 +2413,7 @@
         <v>25</v>
       </c>
       <c r="E23" s="28" t="n">
-        <v>73.78</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="F23" s="29" t="n"/>
     </row>
@@ -2437,7 +2437,7 @@
         <v>15.57</v>
       </c>
       <c r="E24" s="26" t="n">
-        <v>45.95</v>
+        <v>45.84</v>
       </c>
       <c r="F24" s="24" t="n"/>
     </row>
@@ -2461,7 +2461,7 @@
         <v>10.74</v>
       </c>
       <c r="E25" s="28" t="n">
-        <v>31.69</v>
+        <v>31.62</v>
       </c>
       <c r="F25" s="29" t="n"/>
     </row>
@@ -2485,7 +2485,7 @@
         <v>10.16</v>
       </c>
       <c r="E26" s="26" t="n">
-        <v>29.98</v>
+        <v>29.91</v>
       </c>
       <c r="F26" s="24" t="n"/>
     </row>
@@ -2509,7 +2509,7 @@
         <v>5</v>
       </c>
       <c r="E27" s="28" t="n">
-        <v>14.76</v>
+        <v>14.72</v>
       </c>
       <c r="F27" s="29" t="n"/>
     </row>
@@ -2533,7 +2533,7 @@
         <v>51</v>
       </c>
       <c r="E28" s="26" t="n">
-        <v>150.5</v>
+        <v>150.14</v>
       </c>
       <c r="F28" s="24" t="n"/>
     </row>
@@ -2557,7 +2557,7 @@
         <v>40.5</v>
       </c>
       <c r="E29" s="28" t="n">
-        <v>119.52</v>
+        <v>119.23</v>
       </c>
       <c r="F29" s="29" t="n"/>
     </row>
@@ -2581,7 +2581,7 @@
         <v>10.56</v>
       </c>
       <c r="E30" s="26" t="n">
-        <v>31.16</v>
+        <v>31.09</v>
       </c>
       <c r="F30" s="24" t="n"/>
     </row>
@@ -2622,7 +2622,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2683,48 +2683,240 @@
     <row r="4">
       <c r="A4" s="14" t="inlineStr">
         <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B4" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C4" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D4" s="25" t="n">
+        <v>10.82</v>
+      </c>
+      <c r="E4" s="26" t="n">
+        <v>31.85</v>
+      </c>
+      <c r="F4" s="24" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C5" s="11" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>10.84</v>
+      </c>
+      <c r="E5" s="28" t="n">
+        <v>31.91</v>
+      </c>
+      <c r="F5" s="29" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B6" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D6" s="25" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="E6" s="26" t="n">
+        <v>30.62</v>
+      </c>
+      <c r="F6" s="24" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-01</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Google Workspace</t>
+        </is>
+      </c>
+      <c r="C7" s="11" t="inlineStr">
+        <is>
+          <t>Google Workspace (₪75.90)</t>
+        </is>
+      </c>
+      <c r="D7" s="27" t="n">
+        <v>25.78125</v>
+      </c>
+      <c r="E7" s="28" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="F7" s="29" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-02</t>
+        </is>
+      </c>
+      <c r="B8" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C8" s="15" t="inlineStr">
+        <is>
+          <t>Prepaid extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D8" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="26" t="n">
+        <v>14.72</v>
+      </c>
+      <c r="F8" s="24" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D9" s="27" t="n">
+        <v>15.33</v>
+      </c>
+      <c r="E9" s="28" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="F9" s="29" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>2026-05-03</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>Meta (Ads)</t>
+        </is>
+      </c>
+      <c r="C10" s="15" t="inlineStr">
+        <is>
+          <t>Facebook Ads</t>
+        </is>
+      </c>
+      <c r="D10" s="25" t="n">
+        <v>27.28</v>
+      </c>
+      <c r="E10" s="26" t="n">
+        <v>80.31</v>
+      </c>
+      <c r="F10" s="24" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D11" s="27" t="n">
+        <v>15.29</v>
+      </c>
+      <c r="E11" s="28" t="n">
+        <v>45.01</v>
+      </c>
+      <c r="F11" s="29" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
           <t>2026-05-16</t>
         </is>
       </c>
-      <c r="B4" s="15" t="inlineStr">
+      <c r="B12" s="15" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="C12" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D4" s="25" t="n">
+      <c r="D12" s="25" t="n">
         <v>20</v>
       </c>
-      <c r="E4" s="26" t="n">
-        <v>59.02</v>
-      </c>
-      <c r="F4" s="24" t="n"/>
-    </row>
-    <row r="5" ht="24" customHeight="1">
-      <c r="A5" s="30" t="inlineStr">
+      <c r="E12" s="26" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F12" s="24" t="n"/>
+    </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="A13" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B5" s="31" t="n"/>
-      <c r="C5" s="31" t="n"/>
-      <c r="D5" s="20">
-        <f>SUM(D4:D4)</f>
-        <v/>
-      </c>
-      <c r="E5" s="21">
-        <f>SUM(E4:E4)</f>
-        <v/>
-      </c>
-      <c r="F5" s="31" t="n"/>
+      <c r="B13" s="31" t="n"/>
+      <c r="C13" s="31" t="n"/>
+      <c r="D13" s="20">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+      <c r="E13" s="21">
+        <f>SUM(E4:E12)</f>
+        <v/>
+      </c>
+      <c r="F13" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -2819,7 +3011,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -2938,7 +3130,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3057,7 +3249,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3176,7 +3368,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3295,7 +3487,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3414,7 +3606,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -3455,7 +3647,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F123"/>
+  <dimension ref="A1:F131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3522,7 +3714,7 @@
         </is>
       </c>
       <c r="D3" s="12" t="n">
-        <v>1.13182</v>
+        <v>1.134511</v>
       </c>
       <c r="E3" s="13" t="n">
         <v>3.34</v>
@@ -3550,7 +3742,7 @@
         </is>
       </c>
       <c r="D4" s="16" t="n">
-        <v>81.69434099999999</v>
+        <v>81.888587</v>
       </c>
       <c r="E4" s="17" t="n">
         <v>241.08</v>
@@ -3578,7 +3770,7 @@
         </is>
       </c>
       <c r="D5" s="12" t="n">
-        <v>11.873941</v>
+        <v>11.902174</v>
       </c>
       <c r="E5" s="13" t="n">
         <v>35.04</v>
@@ -3606,7 +3798,7 @@
         </is>
       </c>
       <c r="D6" s="16" t="n">
-        <v>22.46696</v>
+        <v>22.52038</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>66.3</v>
@@ -3662,7 +3854,7 @@
         </is>
       </c>
       <c r="D8" s="16" t="n">
-        <v>15.360895</v>
+        <v>15.397418</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>45.33</v>
@@ -3690,7 +3882,7 @@
         </is>
       </c>
       <c r="D9" s="12" t="n">
-        <v>129.061335</v>
+        <v>129.368207</v>
       </c>
       <c r="E9" s="13" t="n">
         <v>380.86</v>
@@ -3718,7 +3910,7 @@
         </is>
       </c>
       <c r="D10" s="16" t="n">
-        <v>11.406303</v>
+        <v>11.433424</v>
       </c>
       <c r="E10" s="17" t="n">
         <v>33.66</v>
@@ -3746,7 +3938,7 @@
         </is>
       </c>
       <c r="D11" s="12" t="n">
-        <v>19.291766</v>
+        <v>19.337636</v>
       </c>
       <c r="E11" s="13" t="n">
         <v>56.93</v>
@@ -3774,7 +3966,7 @@
         </is>
       </c>
       <c r="D12" s="16" t="n">
-        <v>17.346662</v>
+        <v>17.387908</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>51.19</v>
@@ -3802,7 +3994,7 @@
         </is>
       </c>
       <c r="D13" s="12" t="n">
-        <v>13.866486</v>
+        <v>13.899457</v>
       </c>
       <c r="E13" s="13" t="n">
         <v>40.92</v>
@@ -3830,7 +4022,7 @@
         </is>
       </c>
       <c r="D14" s="16" t="n">
-        <v>1.043714</v>
+        <v>1.046196</v>
       </c>
       <c r="E14" s="17" t="n">
         <v>3.08</v>
@@ -3858,7 +4050,7 @@
         </is>
       </c>
       <c r="D15" s="12" t="n">
-        <v>22.10776</v>
+        <v>22.160326</v>
       </c>
       <c r="E15" s="13" t="n">
         <v>65.23999999999999</v>
@@ -3886,7 +4078,7 @@
         </is>
       </c>
       <c r="D16" s="16" t="n">
-        <v>12.321247</v>
+        <v>12.350543</v>
       </c>
       <c r="E16" s="17" t="n">
         <v>36.36</v>
@@ -3914,7 +4106,7 @@
         </is>
       </c>
       <c r="D17" s="12" t="n">
-        <v>23.18875</v>
+        <v>23.243886</v>
       </c>
       <c r="E17" s="13" t="n">
         <v>68.43000000000001</v>
@@ -3970,7 +4162,7 @@
         </is>
       </c>
       <c r="D19" s="12" t="n">
-        <v>5.662487</v>
+        <v>5.675951</v>
       </c>
       <c r="E19" s="13" t="n">
         <v>16.71</v>
@@ -3998,7 +4190,7 @@
         </is>
       </c>
       <c r="D20" s="16" t="n">
-        <v>12.741444</v>
+        <v>12.771739</v>
       </c>
       <c r="E20" s="17" t="n">
         <v>37.6</v>
@@ -4026,7 +4218,7 @@
         </is>
       </c>
       <c r="D21" s="12" t="n">
-        <v>19.291766</v>
+        <v>19.337636</v>
       </c>
       <c r="E21" s="13" t="n">
         <v>56.93</v>
@@ -4054,7 +4246,7 @@
         </is>
       </c>
       <c r="D22" s="16" t="n">
-        <v>3.165029</v>
+        <v>3.172554</v>
       </c>
       <c r="E22" s="17" t="n">
         <v>9.34</v>
@@ -4082,7 +4274,7 @@
         </is>
       </c>
       <c r="D23" s="12" t="n">
-        <v>11.999322</v>
+        <v>12.027853</v>
       </c>
       <c r="E23" s="13" t="n">
         <v>35.41</v>
@@ -4138,7 +4330,7 @@
         </is>
       </c>
       <c r="D25" s="12" t="n">
-        <v>22.656727</v>
+        <v>22.710598</v>
       </c>
       <c r="E25" s="13" t="n">
         <v>66.86</v>
@@ -4166,7 +4358,7 @@
         </is>
       </c>
       <c r="D26" s="16" t="n">
-        <v>5.594714</v>
+        <v>5.608016</v>
       </c>
       <c r="E26" s="17" t="n">
         <v>16.51</v>
@@ -4194,7 +4386,7 @@
         </is>
       </c>
       <c r="D27" s="12" t="n">
-        <v>19.291766</v>
+        <v>19.337636</v>
       </c>
       <c r="E27" s="13" t="n">
         <v>56.93</v>
@@ -4250,7 +4442,7 @@
         </is>
       </c>
       <c r="D29" s="12" t="n">
-        <v>22.297526</v>
+        <v>22.350543</v>
       </c>
       <c r="E29" s="13" t="n">
         <v>65.8</v>
@@ -4278,7 +4470,7 @@
         </is>
       </c>
       <c r="D30" s="16" t="n">
-        <v>5.513385</v>
+        <v>5.526495</v>
       </c>
       <c r="E30" s="17" t="n">
         <v>16.27</v>
@@ -4306,7 +4498,7 @@
         </is>
       </c>
       <c r="D31" s="12" t="n">
-        <v>13.256523</v>
+        <v>13.288043</v>
       </c>
       <c r="E31" s="13" t="n">
         <v>39.12</v>
@@ -4334,7 +4526,7 @@
         </is>
       </c>
       <c r="D32" s="16" t="n">
-        <v>12.910878</v>
+        <v>12.941576</v>
       </c>
       <c r="E32" s="17" t="n">
         <v>38.1</v>
@@ -4362,7 +4554,7 @@
         </is>
       </c>
       <c r="D33" s="12" t="n">
-        <v>16.414775</v>
+        <v>16.453804</v>
       </c>
       <c r="E33" s="13" t="n">
         <v>48.44</v>
@@ -4390,7 +4582,7 @@
         </is>
       </c>
       <c r="D34" s="16" t="n">
-        <v>10.826838</v>
+        <v>10.852582</v>
       </c>
       <c r="E34" s="17" t="n">
         <v>31.95</v>
@@ -4446,7 +4638,7 @@
         </is>
       </c>
       <c r="D36" s="16" t="n">
-        <v>22.202643</v>
+        <v>22.255435</v>
       </c>
       <c r="E36" s="17" t="n">
         <v>65.52</v>
@@ -4474,7 +4666,7 @@
         </is>
       </c>
       <c r="D37" s="12" t="n">
-        <v>5.52694</v>
+        <v>5.540082</v>
       </c>
       <c r="E37" s="13" t="n">
         <v>16.31</v>
@@ -4502,7 +4694,7 @@
         </is>
       </c>
       <c r="D38" s="16" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E38" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4530,7 +4722,7 @@
         </is>
       </c>
       <c r="D39" s="12" t="n">
-        <v>16.52999</v>
+        <v>16.569293</v>
       </c>
       <c r="E39" s="13" t="n">
         <v>48.78</v>
@@ -4558,7 +4750,7 @@
         </is>
       </c>
       <c r="D40" s="16" t="n">
-        <v>10.711623</v>
+        <v>10.737092</v>
       </c>
       <c r="E40" s="17" t="n">
         <v>31.61</v>
@@ -4586,7 +4778,7 @@
         </is>
       </c>
       <c r="D41" s="12" t="n">
-        <v>32.856659</v>
+        <v>32.934783</v>
       </c>
       <c r="E41" s="13" t="n">
         <v>96.95999999999999</v>
@@ -4614,7 +4806,7 @@
         </is>
       </c>
       <c r="D42" s="16" t="n">
-        <v>35.930193</v>
+        <v>36.015625</v>
       </c>
       <c r="E42" s="17" t="n">
         <v>106.03</v>
@@ -4670,7 +4862,7 @@
         </is>
       </c>
       <c r="D44" s="16" t="n">
-        <v>38.905456</v>
+        <v>38.997962</v>
       </c>
       <c r="E44" s="17" t="n">
         <v>114.81</v>
@@ -4698,7 +4890,7 @@
         </is>
       </c>
       <c r="D45" s="12" t="n">
-        <v>5.39817</v>
+        <v>5.411005</v>
       </c>
       <c r="E45" s="13" t="n">
         <v>15.93</v>
@@ -4726,7 +4918,7 @@
         </is>
       </c>
       <c r="D46" s="16" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E46" s="17" t="n">
         <v>75.90000000000001</v>
@@ -4754,7 +4946,7 @@
         </is>
       </c>
       <c r="D47" s="12" t="n">
-        <v>151.043714</v>
+        <v>151.402853</v>
       </c>
       <c r="E47" s="13" t="n">
         <v>445.73</v>
@@ -4782,7 +4974,7 @@
         </is>
       </c>
       <c r="D48" s="16" t="n">
-        <v>16.191122</v>
+        <v>16.22962</v>
       </c>
       <c r="E48" s="17" t="n">
         <v>47.78</v>
@@ -4810,7 +5002,7 @@
         </is>
       </c>
       <c r="D49" s="12" t="n">
-        <v>20.97594</v>
+        <v>21.025815</v>
       </c>
       <c r="E49" s="13" t="n">
         <v>61.9</v>
@@ -4838,7 +5030,7 @@
         </is>
       </c>
       <c r="D50" s="16" t="n">
-        <v>21.521518</v>
+        <v>21.57269</v>
       </c>
       <c r="E50" s="17" t="n">
         <v>63.51</v>
@@ -4866,7 +5058,7 @@
         </is>
       </c>
       <c r="D51" s="12" t="n">
-        <v>21.460522</v>
+        <v>21.511549</v>
       </c>
       <c r="E51" s="13" t="n">
         <v>63.33</v>
@@ -4894,7 +5086,7 @@
         </is>
       </c>
       <c r="D52" s="16" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E52" s="17" t="n">
         <v>49.9</v>
@@ -4950,7 +5142,7 @@
         </is>
       </c>
       <c r="D54" s="16" t="n">
-        <v>41.613013</v>
+        <v>41.711957</v>
       </c>
       <c r="E54" s="17" t="n">
         <v>122.8</v>
@@ -4978,7 +5170,7 @@
         </is>
       </c>
       <c r="D55" s="12" t="n">
-        <v>26.50288</v>
+        <v>26.565897</v>
       </c>
       <c r="E55" s="13" t="n">
         <v>78.20999999999999</v>
@@ -5006,7 +5198,7 @@
         </is>
       </c>
       <c r="D56" s="16" t="n">
-        <v>45.408336</v>
+        <v>45.516304</v>
       </c>
       <c r="E56" s="17" t="n">
         <v>134</v>
@@ -5034,7 +5226,7 @@
         </is>
       </c>
       <c r="D57" s="12" t="n">
-        <v>5.228736</v>
+        <v>5.241168</v>
       </c>
       <c r="E57" s="13" t="n">
         <v>15.43</v>
@@ -5062,7 +5254,7 @@
         </is>
       </c>
       <c r="D58" s="16" t="n">
-        <v>15.160962</v>
+        <v>15.197011</v>
       </c>
       <c r="E58" s="17" t="n">
         <v>44.74</v>
@@ -5090,7 +5282,7 @@
         </is>
       </c>
       <c r="D59" s="12" t="n">
-        <v>26.282616</v>
+        <v>26.345109</v>
       </c>
       <c r="E59" s="13" t="n">
         <v>77.56</v>
@@ -5118,7 +5310,7 @@
         </is>
       </c>
       <c r="D60" s="16" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E60" s="17" t="n">
         <v>75.90000000000001</v>
@@ -5146,7 +5338,7 @@
         </is>
       </c>
       <c r="D61" s="12" t="n">
-        <v>32.995595</v>
+        <v>33.074049</v>
       </c>
       <c r="E61" s="13" t="n">
         <v>97.37</v>
@@ -5174,7 +5366,7 @@
         </is>
       </c>
       <c r="D62" s="16" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E62" s="17" t="n">
         <v>49.9</v>
@@ -5202,7 +5394,7 @@
         </is>
       </c>
       <c r="D63" s="12" t="n">
-        <v>49.007116</v>
+        <v>49.123641</v>
       </c>
       <c r="E63" s="13" t="n">
         <v>144.62</v>
@@ -5230,7 +5422,7 @@
         </is>
       </c>
       <c r="D64" s="16" t="n">
-        <v>20.918333</v>
+        <v>20.968071</v>
       </c>
       <c r="E64" s="17" t="n">
         <v>61.73</v>
@@ -5258,7 +5450,7 @@
         </is>
       </c>
       <c r="D65" s="12" t="n">
-        <v>5.232125</v>
+        <v>5.244565</v>
       </c>
       <c r="E65" s="13" t="n">
         <v>15.44</v>
@@ -5314,7 +5506,7 @@
         </is>
       </c>
       <c r="D67" s="12" t="n">
-        <v>21.199593</v>
+        <v>21.25</v>
       </c>
       <c r="E67" s="13" t="n">
         <v>62.56</v>
@@ -5342,7 +5534,7 @@
         </is>
       </c>
       <c r="D68" s="16" t="n">
-        <v>52.511013</v>
+        <v>52.63587</v>
       </c>
       <c r="E68" s="17" t="n">
         <v>154.96</v>
@@ -5370,7 +5562,7 @@
         </is>
       </c>
       <c r="D69" s="12" t="n">
-        <v>53.561505</v>
+        <v>53.688859</v>
       </c>
       <c r="E69" s="13" t="n">
         <v>158.06</v>
@@ -5398,7 +5590,7 @@
         </is>
       </c>
       <c r="D70" s="16" t="n">
-        <v>5.313453</v>
+        <v>5.326087</v>
       </c>
       <c r="E70" s="17" t="n">
         <v>15.68</v>
@@ -5426,7 +5618,7 @@
         </is>
       </c>
       <c r="D71" s="12" t="n">
-        <v>10.623517</v>
+        <v>10.648777</v>
       </c>
       <c r="E71" s="13" t="n">
         <v>31.35</v>
@@ -5454,7 +5646,7 @@
         </is>
       </c>
       <c r="D72" s="16" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E72" s="17" t="n">
         <v>75.90000000000001</v>
@@ -5482,7 +5674,7 @@
         </is>
       </c>
       <c r="D73" s="12" t="n">
-        <v>10.599797</v>
+        <v>10.625</v>
       </c>
       <c r="E73" s="13" t="n">
         <v>31.28</v>
@@ -5510,7 +5702,7 @@
         </is>
       </c>
       <c r="D74" s="16" t="n">
-        <v>15.371061</v>
+        <v>15.407609</v>
       </c>
       <c r="E74" s="17" t="n">
         <v>45.36</v>
@@ -5538,7 +5730,7 @@
         </is>
       </c>
       <c r="D75" s="12" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E75" s="13" t="n">
         <v>75.90000000000001</v>
@@ -5566,7 +5758,7 @@
         </is>
       </c>
       <c r="D76" s="16" t="n">
-        <v>10.572687</v>
+        <v>10.597826</v>
       </c>
       <c r="E76" s="17" t="n">
         <v>31.2</v>
@@ -5594,7 +5786,7 @@
         </is>
       </c>
       <c r="D77" s="12" t="n">
-        <v>41.826499</v>
+        <v>41.925951</v>
       </c>
       <c r="E77" s="13" t="n">
         <v>123.43</v>
@@ -5622,7 +5814,7 @@
         </is>
       </c>
       <c r="D78" s="16" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E78" s="17" t="n">
         <v>49.9</v>
@@ -5650,7 +5842,7 @@
         </is>
       </c>
       <c r="D79" s="12" t="n">
-        <v>54.107082</v>
+        <v>54.235734</v>
       </c>
       <c r="E79" s="13" t="n">
         <v>159.67</v>
@@ -5678,7 +5870,7 @@
         </is>
       </c>
       <c r="D80" s="16" t="n">
-        <v>21.304642</v>
+        <v>21.355299</v>
       </c>
       <c r="E80" s="17" t="n">
         <v>62.87</v>
@@ -5734,7 +5926,7 @@
         </is>
       </c>
       <c r="D82" s="16" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E82" s="17" t="n">
         <v>49.9</v>
@@ -5762,7 +5954,7 @@
         </is>
       </c>
       <c r="D83" s="12" t="n">
-        <v>10.542189</v>
+        <v>10.567255</v>
       </c>
       <c r="E83" s="13" t="n">
         <v>31.11</v>
@@ -5790,7 +5982,7 @@
         </is>
       </c>
       <c r="D84" s="16" t="n">
-        <v>11.596069</v>
+        <v>11.623641</v>
       </c>
       <c r="E84" s="17" t="n">
         <v>34.22</v>
@@ -5846,7 +6038,7 @@
         </is>
       </c>
       <c r="D86" s="16" t="n">
-        <v>5.293121</v>
+        <v>5.305707</v>
       </c>
       <c r="E86" s="17" t="n">
         <v>15.62</v>
@@ -5902,7 +6094,7 @@
         </is>
       </c>
       <c r="D88" s="16" t="n">
-        <v>10.654016</v>
+        <v>10.679348</v>
       </c>
       <c r="E88" s="17" t="n">
         <v>31.44</v>
@@ -5930,7 +6122,7 @@
         </is>
       </c>
       <c r="D89" s="12" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E89" s="13" t="n">
         <v>75.90000000000001</v>
@@ -5958,7 +6150,7 @@
         </is>
       </c>
       <c r="D90" s="16" t="n">
-        <v>56.363944</v>
+        <v>56.497962</v>
       </c>
       <c r="E90" s="17" t="n">
         <v>166.33</v>
@@ -6014,7 +6206,7 @@
         </is>
       </c>
       <c r="D92" s="16" t="n">
-        <v>2.389021</v>
+        <v>2.394701</v>
       </c>
       <c r="E92" s="17" t="n">
         <v>7.05</v>
@@ -6042,7 +6234,7 @@
         </is>
       </c>
       <c r="D93" s="12" t="n">
-        <v>21.291088</v>
+        <v>21.341712</v>
       </c>
       <c r="E93" s="13" t="n">
         <v>62.83</v>
@@ -6070,7 +6262,7 @@
         </is>
       </c>
       <c r="D94" s="16" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E94" s="17" t="n">
         <v>49.9</v>
@@ -6101,7 +6293,7 @@
         <v>20</v>
       </c>
       <c r="E95" s="13" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F95" s="10" t="inlineStr">
         <is>
@@ -6129,7 +6321,7 @@
         <v>10</v>
       </c>
       <c r="E96" s="17" t="n">
-        <v>29.51</v>
+        <v>29.44</v>
       </c>
       <c r="F96" s="14" t="inlineStr">
         <is>
@@ -6157,7 +6349,7 @@
         <v>20</v>
       </c>
       <c r="E97" s="13" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F97" s="10" t="inlineStr">
         <is>
@@ -6182,7 +6374,7 @@
         </is>
       </c>
       <c r="D98" s="16" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E98" s="17" t="n">
         <v>49.9</v>
@@ -6213,7 +6405,7 @@
         <v>81.2</v>
       </c>
       <c r="E99" s="13" t="n">
-        <v>239.62</v>
+        <v>239.05</v>
       </c>
       <c r="F99" s="10" t="inlineStr">
         <is>
@@ -6241,7 +6433,7 @@
         <v>5</v>
       </c>
       <c r="E100" s="17" t="n">
-        <v>14.76</v>
+        <v>14.72</v>
       </c>
       <c r="F100" s="14" t="inlineStr">
         <is>
@@ -6269,7 +6461,7 @@
         <v>15.14</v>
       </c>
       <c r="E101" s="13" t="n">
-        <v>44.68</v>
+        <v>44.57</v>
       </c>
       <c r="F101" s="10" t="inlineStr">
         <is>
@@ -6297,7 +6489,7 @@
         <v>10</v>
       </c>
       <c r="E102" s="17" t="n">
-        <v>29.51</v>
+        <v>29.44</v>
       </c>
       <c r="F102" s="14" t="inlineStr">
         <is>
@@ -6325,7 +6517,7 @@
         <v>10.15</v>
       </c>
       <c r="E103" s="13" t="n">
-        <v>29.95</v>
+        <v>29.88</v>
       </c>
       <c r="F103" s="10" t="inlineStr">
         <is>
@@ -6353,7 +6545,7 @@
         <v>10.02</v>
       </c>
       <c r="E104" s="17" t="n">
-        <v>29.57</v>
+        <v>29.5</v>
       </c>
       <c r="F104" s="14" t="inlineStr">
         <is>
@@ -6381,7 +6573,7 @@
         <v>10.5</v>
       </c>
       <c r="E105" s="13" t="n">
-        <v>30.99</v>
+        <v>30.91</v>
       </c>
       <c r="F105" s="10" t="inlineStr">
         <is>
@@ -6409,7 +6601,7 @@
         <v>11.17</v>
       </c>
       <c r="E106" s="17" t="n">
-        <v>32.96</v>
+        <v>32.88</v>
       </c>
       <c r="F106" s="14" t="inlineStr">
         <is>
@@ -6437,7 +6629,7 @@
         <v>25</v>
       </c>
       <c r="E107" s="13" t="n">
-        <v>73.78</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="F107" s="10" t="inlineStr">
         <is>
@@ -6465,7 +6657,7 @@
         <v>15.57</v>
       </c>
       <c r="E108" s="17" t="n">
-        <v>45.95</v>
+        <v>45.84</v>
       </c>
       <c r="F108" s="14" t="inlineStr">
         <is>
@@ -6493,7 +6685,7 @@
         <v>10.74</v>
       </c>
       <c r="E109" s="13" t="n">
-        <v>31.69</v>
+        <v>31.62</v>
       </c>
       <c r="F109" s="10" t="inlineStr">
         <is>
@@ -6521,7 +6713,7 @@
         <v>10.16</v>
       </c>
       <c r="E110" s="17" t="n">
-        <v>29.98</v>
+        <v>29.91</v>
       </c>
       <c r="F110" s="14" t="inlineStr">
         <is>
@@ -6549,7 +6741,7 @@
         <v>5</v>
       </c>
       <c r="E111" s="13" t="n">
-        <v>14.76</v>
+        <v>14.72</v>
       </c>
       <c r="F111" s="10" t="inlineStr">
         <is>
@@ -6577,7 +6769,7 @@
         <v>51</v>
       </c>
       <c r="E112" s="17" t="n">
-        <v>150.5</v>
+        <v>150.14</v>
       </c>
       <c r="F112" s="14" t="inlineStr">
         <is>
@@ -6605,7 +6797,7 @@
         <v>40.5</v>
       </c>
       <c r="E113" s="13" t="n">
-        <v>119.52</v>
+        <v>119.23</v>
       </c>
       <c r="F113" s="10" t="inlineStr">
         <is>
@@ -6633,7 +6825,7 @@
         <v>10.56</v>
       </c>
       <c r="E114" s="17" t="n">
-        <v>31.16</v>
+        <v>31.09</v>
       </c>
       <c r="F114" s="14" t="inlineStr">
         <is>
@@ -6644,24 +6836,24 @@
     <row r="115">
       <c r="A115" s="10" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B115" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C115" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D115" s="12" t="n">
-        <v>20</v>
+        <v>10.82</v>
       </c>
       <c r="E115" s="13" t="n">
-        <v>59.02</v>
+        <v>31.85</v>
       </c>
       <c r="F115" s="10" t="inlineStr">
         <is>
@@ -6672,220 +6864,444 @@
     <row r="116">
       <c r="A116" s="14" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B116" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C116" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D116" s="16" t="n">
-        <v>20</v>
+        <v>10.84</v>
       </c>
       <c r="E116" s="17" t="n">
-        <v>59.02</v>
+        <v>31.91</v>
       </c>
       <c r="F116" s="14" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="10" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B117" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C117" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D117" s="12" t="n">
-        <v>20</v>
+        <v>10.4</v>
       </c>
       <c r="E117" s="13" t="n">
-        <v>59.02</v>
+        <v>30.62</v>
       </c>
       <c r="F117" s="10" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="14" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-05-01</t>
         </is>
       </c>
       <c r="B118" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Google Workspace</t>
         </is>
       </c>
       <c r="C118" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Google Workspace (₪75.90)</t>
         </is>
       </c>
       <c r="D118" s="16" t="n">
-        <v>20</v>
+        <v>25.78125</v>
       </c>
       <c r="E118" s="17" t="n">
-        <v>59.02</v>
+        <v>75.90000000000001</v>
       </c>
       <c r="F118" s="14" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="10" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-05-02</t>
         </is>
       </c>
       <c r="B119" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C119" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Prepaid extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D119" s="12" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="E119" s="13" t="n">
-        <v>59.02</v>
+        <v>14.72</v>
       </c>
       <c r="F119" s="10" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="14" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B120" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C120" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Auto recharge extra usage, Individual plan</t>
         </is>
       </c>
       <c r="D120" s="16" t="n">
-        <v>20</v>
+        <v>15.33</v>
       </c>
       <c r="E120" s="17" t="n">
-        <v>59.02</v>
+        <v>45.13</v>
       </c>
       <c r="F120" s="14" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" s="10" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-05-03</t>
         </is>
       </c>
       <c r="B121" s="11" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Meta (Ads)</t>
         </is>
       </c>
       <c r="C121" s="11" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Facebook Ads</t>
         </is>
       </c>
       <c r="D121" s="12" t="n">
-        <v>20</v>
+        <v>27.28</v>
       </c>
       <c r="E121" s="13" t="n">
-        <v>59.02</v>
+        <v>80.31</v>
       </c>
       <c r="F121" s="10" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" s="14" t="inlineStr">
         <is>
+          <t>2026-05-04</t>
+        </is>
+      </c>
+      <c r="B122" s="15" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="C122" s="15" t="inlineStr">
+        <is>
+          <t>Auto recharge extra usage, Individual plan</t>
+        </is>
+      </c>
+      <c r="D122" s="16" t="n">
+        <v>15.29</v>
+      </c>
+      <c r="E122" s="17" t="n">
+        <v>45.01</v>
+      </c>
+      <c r="F122" s="14" t="inlineStr">
+        <is>
+          <t>מאי 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D123" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E123" s="13" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F123" s="10" t="inlineStr">
+        <is>
+          <t>מאי 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="inlineStr">
+        <is>
+          <t>2026-06-16</t>
+        </is>
+      </c>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C124" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D124" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E124" s="17" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F124" s="14" t="inlineStr">
+        <is>
+          <t>יוני 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="10" t="inlineStr">
+        <is>
+          <t>2026-07-16</t>
+        </is>
+      </c>
+      <c r="B125" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C125" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D125" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E125" s="13" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F125" s="10" t="inlineStr">
+        <is>
+          <t>יולי 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="14" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="B126" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C126" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D126" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E126" s="17" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F126" s="14" t="inlineStr">
+        <is>
+          <t>אוגוסט 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="10" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="B127" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C127" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D127" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E127" s="13" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F127" s="10" t="inlineStr">
+        <is>
+          <t>ספטמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="14" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B128" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C128" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D128" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E128" s="17" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F128" s="14" t="inlineStr">
+        <is>
+          <t>אוקטובר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="10" t="inlineStr">
+        <is>
+          <t>2026-11-16</t>
+        </is>
+      </c>
+      <c r="B129" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C129" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D129" s="12" t="n">
+        <v>20</v>
+      </c>
+      <c r="E129" s="13" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F129" s="10" t="inlineStr">
+        <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="14" t="inlineStr">
+        <is>
           <t>2026-12-16</t>
         </is>
       </c>
-      <c r="B122" s="15" t="inlineStr">
+      <c r="B130" s="15" t="inlineStr">
         <is>
           <t>OpenAI</t>
         </is>
       </c>
-      <c r="C122" s="15" t="inlineStr">
+      <c r="C130" s="15" t="inlineStr">
         <is>
           <t>ChatGPT Plus</t>
         </is>
       </c>
-      <c r="D122" s="16" t="n">
+      <c r="D130" s="16" t="n">
         <v>20</v>
       </c>
-      <c r="E122" s="17" t="n">
-        <v>59.02</v>
-      </c>
-      <c r="F122" s="14" t="inlineStr">
+      <c r="E130" s="17" t="n">
+        <v>58.88</v>
+      </c>
+      <c r="F130" s="14" t="inlineStr">
         <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="18" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B123" s="19" t="n"/>
-      <c r="C123" s="19" t="n"/>
-      <c r="D123" s="20">
-        <f>SUM(D3:D122)</f>
-        <v/>
-      </c>
-      <c r="E123" s="21">
-        <f>SUM(E3:E122)</f>
-        <v/>
-      </c>
-      <c r="F123" s="19" t="n"/>
+      <c r="B131" s="19" t="n"/>
+      <c r="C131" s="19" t="n"/>
+      <c r="D131" s="20">
+        <f>SUM(D3:D130)</f>
+        <v/>
+      </c>
+      <c r="E131" s="21">
+        <f>SUM(E3:E130)</f>
+        <v/>
+      </c>
+      <c r="F131" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A123:C123"/>
+    <mergeCell ref="A131:C131"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6977,7 +7393,7 @@
         <v>20</v>
       </c>
       <c r="E4" s="26" t="n">
-        <v>59.02</v>
+        <v>58.88</v>
       </c>
       <c r="F4" s="24" t="n"/>
     </row>
@@ -11774,7 +12190,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>1.13182</v>
+        <v>1.134511</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>3.34</v>
@@ -11798,7 +12214,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>81.69434099999999</v>
+        <v>81.888587</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>241.08</v>
@@ -11822,7 +12238,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>11.873941</v>
+        <v>11.902174</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35.04</v>
@@ -11846,7 +12262,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>22.46696</v>
+        <v>22.52038</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>66.3</v>
@@ -11894,7 +12310,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>15.360895</v>
+        <v>15.397418</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>45.33</v>
@@ -11918,7 +12334,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>129.061335</v>
+        <v>129.368207</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>380.86</v>
@@ -11942,7 +12358,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>11.406303</v>
+        <v>11.433424</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>33.66</v>
@@ -12061,7 +12477,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>19.291766</v>
+        <v>19.337636</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -12085,7 +12501,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>17.346662</v>
+        <v>17.387908</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>51.19</v>
@@ -12109,7 +12525,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>13.866486</v>
+        <v>13.899457</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>40.92</v>
@@ -12133,7 +12549,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>1.043714</v>
+        <v>1.046196</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>3.08</v>
@@ -12157,7 +12573,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>22.10776</v>
+        <v>22.160326</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>65.23999999999999</v>
@@ -12181,7 +12597,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>12.321247</v>
+        <v>12.350543</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>36.36</v>
@@ -12205,7 +12621,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>23.18875</v>
+        <v>23.243886</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>68.43000000000001</v>
@@ -12253,7 +12669,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>5.662487</v>
+        <v>5.675951</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>16.71</v>
@@ -12277,7 +12693,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>12.741444</v>
+        <v>12.771739</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>37.6</v>
@@ -12396,7 +12812,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>19.291766</v>
+        <v>19.337636</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -12420,7 +12836,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>3.165029</v>
+        <v>3.172554</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>9.34</v>
@@ -12444,7 +12860,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>11.999322</v>
+        <v>12.027853</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>35.41</v>
@@ -12492,7 +12908,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>22.656727</v>
+        <v>22.710598</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>66.86</v>
@@ -12516,7 +12932,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>5.594714</v>
+        <v>5.608016</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>16.51</v>
@@ -12635,7 +13051,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>19.291766</v>
+        <v>19.337636</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>56.93</v>
@@ -12683,7 +13099,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>22.297526</v>
+        <v>22.350543</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>65.8</v>
@@ -12707,7 +13123,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>5.513385</v>
+        <v>5.526495</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>16.27</v>
@@ -12826,7 +13242,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>13.256523</v>
+        <v>13.288043</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>39.12</v>
@@ -12850,7 +13266,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>12.910878</v>
+        <v>12.941576</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>38.1</v>
@@ -12874,7 +13290,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>16.414775</v>
+        <v>16.453804</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>48.44</v>
@@ -12898,7 +13314,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>10.826838</v>
+        <v>10.852582</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>31.95</v>
@@ -12946,7 +13362,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>22.202643</v>
+        <v>22.255435</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>65.52</v>
@@ -12970,7 +13386,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>5.52694</v>
+        <v>5.540082</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>16.31</v>
@@ -13089,7 +13505,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -13113,7 +13529,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>16.52999</v>
+        <v>16.569293</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>48.78</v>
@@ -13137,7 +13553,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>10.711623</v>
+        <v>10.737092</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>31.61</v>
@@ -13161,7 +13577,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>32.856659</v>
+        <v>32.934783</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>96.95999999999999</v>
@@ -13185,7 +13601,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>35.930193</v>
+        <v>36.015625</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>106.03</v>
@@ -13233,7 +13649,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>38.905456</v>
+        <v>38.997962</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>114.81</v>
@@ -13257,7 +13673,7 @@
         </is>
       </c>
       <c r="D11" s="27" t="n">
-        <v>5.39817</v>
+        <v>5.411005</v>
       </c>
       <c r="E11" s="28" t="n">
         <v>15.93</v>
@@ -13376,7 +13792,7 @@
         </is>
       </c>
       <c r="D4" s="25" t="n">
-        <v>25.720095</v>
+        <v>25.78125</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>75.90000000000001</v>
@@ -13400,7 +13816,7 @@
         </is>
       </c>
       <c r="D5" s="27" t="n">
-        <v>151.043714</v>
+        <v>151.402853</v>
       </c>
       <c r="E5" s="28" t="n">
         <v>445.73</v>
@@ -13424,7 +13840,7 @@
         </is>
       </c>
       <c r="D6" s="25" t="n">
-        <v>16.191122</v>
+        <v>16.22962</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>47.78</v>
@@ -13448,7 +13864,7 @@
         </is>
       </c>
       <c r="D7" s="27" t="n">
-        <v>20.97594</v>
+        <v>21.025815</v>
       </c>
       <c r="E7" s="28" t="n">
         <v>61.9</v>
@@ -13472,7 +13888,7 @@
         </is>
       </c>
       <c r="D8" s="25" t="n">
-        <v>21.521518</v>
+        <v>21.57269</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>63.51</v>
@@ -13496,7 +13912,7 @@
         </is>
       </c>
       <c r="D9" s="27" t="n">
-        <v>21.460522</v>
+        <v>21.511549</v>
       </c>
       <c r="E9" s="28" t="n">
         <v>63.33</v>
@@ -13520,7 +13936,7 @@
         </is>
       </c>
       <c r="D10" s="25" t="n">
-        <v>16.909522</v>
+        <v>16.949728</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>49.9</v>
@@ -13568,7 +13984,7 @@
         </is>
       </c>
       <c r="D12" s="25" t="n">
-        <v>41.613013</v>
+        <v>41.711957</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>122.8</v>
@@ -13592,7 +14008,7 @@
         </is>
       </c>
       <c r="D13" s="27" t="n">
-        <v>26.50288</v>
+        <v>26.565897</v>
       </c>
       <c r="E13" s="28" t="n">
         <v>78.20999999999999</v>
@@ -13616,7 +14032,7 @@
         </is>
       </c>
       <c r="D14" s="25" t="n">
-        <v>45.408336</v>
+        <v>45.516304</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>134</v>
@@ -13640,7 +14056,7 @@
         </is>
       </c>
       <c r="D15" s="27" t="n">
-        <v>5.228736</v>
+        <v>5.241168</v>
       </c>
       <c r="E15" s="28" t="n">
         <v>15.43</v>
@@ -13664,7 +14080,7 @@
         </is>
       </c>
       <c r="D16" s="25" t="n">
-        <v>15.160962</v>
+        <v>15.197011</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>44.74</v>

</xml_diff>

<commit_message>
Fix scanner publishing cache
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Fix scanner cadence status
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Align scanner status with task scheduler
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -1,34 +1,34 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="21" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
-    <sheet name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="הגדרות" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="כל ההוצאות" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2025" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2025" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2025" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2025" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2025" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2025" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ינואר 2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="פברואר 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מרץ 2026" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אפריל 2026" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="מאי 2026" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יוני 2026" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="יולי 2026" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוגוסט 2026" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ספטמבר 2026" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="אוקטובר 2026" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="נובמבר 2026" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דצמבר 2026" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="סיכום חודשי" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="דוח שנתי" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,14 +481,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -512,7 +512,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -540,8 +540,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -567,8 +567,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -594,7 +594,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>0</col>
@@ -609,9 +609,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>

</xml_diff>

<commit_message>
Auto: add invoices – Anthropic 2026-05-15
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/AI_Tools_Expenses_2025_2026.xlsx
+++ b/AI_Tools_Expenses_2025_2026.xlsx
@@ -2646,7 +2646,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3043,48 +3043,72 @@
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D18" s="25" t="n">
         <v>20</v>
       </c>
       <c r="E18" s="26" t="n">
+        <v>58.32</v>
+      </c>
+      <c r="F18" s="24" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="10" t="inlineStr">
+        <is>
+          <t>2026-05-16</t>
+        </is>
+      </c>
+      <c r="B19" s="11" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D19" s="27" t="n">
+        <v>20</v>
+      </c>
+      <c r="E19" s="28" t="n">
         <v>73</v>
       </c>
-      <c r="F18" s="24" t="n"/>
-    </row>
-    <row r="19" ht="24" customHeight="1">
-      <c r="A19" s="30" t="inlineStr">
+      <c r="F19" s="29" t="n"/>
+    </row>
+    <row r="20" ht="24" customHeight="1">
+      <c r="A20" s="30" t="inlineStr">
         <is>
           <t>סה"כ חודש"</t>
         </is>
       </c>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="31" t="n"/>
-      <c r="D19" s="20">
-        <f>SUM(D4:D18)</f>
-        <v/>
-      </c>
-      <c r="E19" s="21">
-        <f>SUM(E4:E18)</f>
-        <v/>
-      </c>
-      <c r="F19" s="31" t="n"/>
+      <c r="B20" s="31" t="n"/>
+      <c r="C20" s="31" t="n"/>
+      <c r="D20" s="20">
+        <f>SUM(D4:D19)</f>
+        <v/>
+      </c>
+      <c r="E20" s="21">
+        <f>SUM(E4:E19)</f>
+        <v/>
+      </c>
+      <c r="F20" s="31" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:C20"/>
     <mergeCell ref="A1:F1"/>
   </mergeCells>
   <hyperlinks>
@@ -3815,7 +3839,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -7424,24 +7448,24 @@
     <row r="130">
       <c r="A130" s="14" t="inlineStr">
         <is>
-          <t>2026-05-16</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="B130" s="15" t="inlineStr">
         <is>
-          <t>OpenAI</t>
+          <t>Anthropic</t>
         </is>
       </c>
       <c r="C130" s="15" t="inlineStr">
         <is>
-          <t>ChatGPT Plus</t>
+          <t>Claude Pro</t>
         </is>
       </c>
       <c r="D130" s="16" t="n">
         <v>20</v>
       </c>
       <c r="E130" s="17" t="n">
-        <v>73</v>
+        <v>58.32</v>
       </c>
       <c r="F130" s="14" t="inlineStr">
         <is>
@@ -7452,7 +7476,7 @@
     <row r="131">
       <c r="A131" s="10" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-05-16</t>
         </is>
       </c>
       <c r="B131" s="11" t="inlineStr">
@@ -7473,14 +7497,14 @@
       </c>
       <c r="F131" s="10" t="inlineStr">
         <is>
-          <t>יוני 2026</t>
+          <t>מאי 2026</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" s="14" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B132" s="15" t="inlineStr">
@@ -7501,14 +7525,14 @@
       </c>
       <c r="F132" s="14" t="inlineStr">
         <is>
-          <t>יולי 2026</t>
+          <t>יוני 2026</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" s="10" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B133" s="11" t="inlineStr">
@@ -7529,14 +7553,14 @@
       </c>
       <c r="F133" s="10" t="inlineStr">
         <is>
-          <t>אוגוסט 2026</t>
+          <t>יולי 2026</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" s="14" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B134" s="15" t="inlineStr">
@@ -7557,14 +7581,14 @@
       </c>
       <c r="F134" s="14" t="inlineStr">
         <is>
-          <t>ספטמבר 2026</t>
+          <t>אוגוסט 2026</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" s="10" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B135" s="11" t="inlineStr">
@@ -7585,14 +7609,14 @@
       </c>
       <c r="F135" s="10" t="inlineStr">
         <is>
-          <t>אוקטובר 2026</t>
+          <t>ספטמבר 2026</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" s="14" t="inlineStr">
         <is>
-          <t>2026-11-16</t>
+          <t>2026-10-16</t>
         </is>
       </c>
       <c r="B136" s="15" t="inlineStr">
@@ -7613,14 +7637,14 @@
       </c>
       <c r="F136" s="14" t="inlineStr">
         <is>
-          <t>נובמבר 2026</t>
+          <t>אוקטובר 2026</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" s="10" t="inlineStr">
         <is>
-          <t>2026-12-16</t>
+          <t>2026-11-16</t>
         </is>
       </c>
       <c r="B137" s="11" t="inlineStr">
@@ -7641,32 +7665,60 @@
       </c>
       <c r="F137" s="10" t="inlineStr">
         <is>
+          <t>נובמבר 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="14" t="inlineStr">
+        <is>
+          <t>2026-12-16</t>
+        </is>
+      </c>
+      <c r="B138" s="15" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="C138" s="15" t="inlineStr">
+        <is>
+          <t>ChatGPT Plus</t>
+        </is>
+      </c>
+      <c r="D138" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="E138" s="17" t="n">
+        <v>73</v>
+      </c>
+      <c r="F138" s="14" t="inlineStr">
+        <is>
           <t>דצמבר 2026</t>
         </is>
       </c>
     </row>
-    <row r="138">
-      <c r="A138" s="18" t="inlineStr">
+    <row r="139">
+      <c r="A139" s="18" t="inlineStr">
         <is>
           <t>סה"כ"</t>
         </is>
       </c>
-      <c r="B138" s="19" t="n"/>
-      <c r="C138" s="19" t="n"/>
-      <c r="D138" s="20">
-        <f>SUM(D3:D137)</f>
-        <v/>
-      </c>
-      <c r="E138" s="21">
-        <f>SUM(E3:E137)</f>
-        <v/>
-      </c>
-      <c r="F138" s="19" t="n"/>
+      <c r="B139" s="19" t="n"/>
+      <c r="C139" s="19" t="n"/>
+      <c r="D139" s="20">
+        <f>SUM(D3:D138)</f>
+        <v/>
+      </c>
+      <c r="E139" s="21">
+        <f>SUM(E3:E138)</f>
+        <v/>
+      </c>
+      <c r="F139" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
+    <mergeCell ref="A139:C139"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A138:C138"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>